<commit_message>
"Actualizo ipc marzo y opex 2025"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC1444C-785C-4B25-B7E3-358D53D8425E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8776FD2E-5FD7-4757-AE0D-7B215F69F12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -914,7 +914,7 @@
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -999,6 +999,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Euro" xfId="10" xr:uid="{8CA0DC4E-5AAC-43A0-AC51-59D877AC41AF}"/>
@@ -1330,7 +1332,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="1" customWidth="1"/>
@@ -3207,6 +3209,23 @@
       </c>
       <c r="E110">
         <v>2.4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="19">
+        <v>46054</v>
+      </c>
+      <c r="B111" s="1">
+        <v>2.9</v>
+      </c>
+      <c r="C111">
+        <v>-1.3</v>
+      </c>
+      <c r="D111">
+        <v>3.1</v>
+      </c>
+      <c r="E111">
+        <v>4.3</v>
       </c>
     </row>
   </sheetData>
@@ -5177,25 +5196,25 @@
         <v>121</v>
       </c>
       <c r="B2" s="37">
-        <v>2.2999999999999998</v>
+        <v>1.5</v>
       </c>
       <c r="C2" s="20">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="D2" s="20">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E2" s="20">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F2" s="20">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="G2" s="20">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="H2" s="16">
-        <v>1.8442869805313178</v>
+        <v>1.6092716037988009</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5203,25 +5222,25 @@
         <v>122</v>
       </c>
       <c r="B3" s="37">
-        <v>4.4000000000000004</v>
+        <v>7.2</v>
       </c>
       <c r="C3" s="20">
-        <v>4.4000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="D3" s="20">
-        <v>5.0999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="E3" s="20">
-        <v>4.4000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="F3" s="20">
-        <v>4.5</v>
+        <v>6.2</v>
       </c>
       <c r="G3" s="20">
-        <v>4.8</v>
+        <v>3.3</v>
       </c>
       <c r="H3" s="16">
-        <v>4.4683465770325226</v>
+        <v>6.2561659139136028</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5229,25 +5248,25 @@
         <v>123</v>
       </c>
       <c r="B4" s="37">
-        <v>0.9</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="C4" s="20">
-        <v>1.1000000000000001</v>
+        <v>1.9</v>
       </c>
       <c r="D4" s="20">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="E4" s="20">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="F4" s="20">
-        <v>-0.1</v>
+        <v>2.7</v>
       </c>
       <c r="G4" s="20">
-        <v>1.1000000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="H4" s="16">
-        <v>0.92599438765113007</v>
+        <v>1.8835946893488442</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5255,25 +5274,25 @@
         <v>124</v>
       </c>
       <c r="B5" s="37">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="C5" s="20">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="D5" s="20">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="E5" s="20">
-        <v>3.1</v>
+        <v>6</v>
       </c>
       <c r="F5" s="20">
-        <v>3.7</v>
+        <v>2</v>
       </c>
       <c r="G5" s="20">
-        <v>2.6</v>
+        <v>1.7</v>
       </c>
       <c r="H5" s="16">
-        <v>3.3549380560282005</v>
+        <v>2.390648530181938</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5281,25 +5300,25 @@
         <v>125</v>
       </c>
       <c r="B6" s="37">
-        <v>5.0999999999999996</v>
+        <v>-0.8</v>
       </c>
       <c r="C6" s="20">
-        <v>6.7</v>
+        <v>0.1</v>
       </c>
       <c r="D6" s="20">
-        <v>6.1</v>
+        <v>-0.5</v>
       </c>
       <c r="E6" s="20">
-        <v>2.6</v>
+        <v>0.5</v>
       </c>
       <c r="F6" s="20">
-        <v>5.6</v>
+        <v>-2.2999999999999998</v>
       </c>
       <c r="G6" s="20">
-        <v>6.3</v>
+        <v>4.2</v>
       </c>
       <c r="H6" s="16">
-        <v>5.5842296472066399</v>
+        <v>6.142693066479854E-2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5307,25 +5326,25 @@
         <v>126</v>
       </c>
       <c r="B7" s="37">
-        <v>28</v>
+        <v>-4.5</v>
       </c>
       <c r="C7" s="20">
-        <v>21.9</v>
+        <v>0.2</v>
       </c>
       <c r="D7" s="20">
-        <v>19</v>
+        <v>6.3</v>
       </c>
       <c r="E7" s="20">
-        <v>18.7</v>
+        <v>5.8</v>
       </c>
       <c r="F7" s="20">
-        <v>16.3</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="G7" s="20">
-        <v>5.4</v>
+        <v>2.1</v>
       </c>
       <c r="H7" s="16">
-        <v>23.180320578923542</v>
+        <v>0.17135374910239864</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5333,25 +5352,25 @@
         <v>127</v>
       </c>
       <c r="B8" s="37">
-        <v>4.2</v>
+        <v>2.4</v>
       </c>
       <c r="C8" s="20">
-        <v>3.4</v>
+        <v>2.9</v>
       </c>
       <c r="D8" s="20">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E8" s="20">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="F8" s="20">
-        <v>3.2</v>
+        <v>0.8</v>
       </c>
       <c r="G8" s="20">
-        <v>1.8</v>
+        <v>2.7</v>
       </c>
       <c r="H8" s="16">
-        <v>3.5858797340896809</v>
+        <v>2.8663193746377269</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5359,25 +5378,25 @@
         <v>128</v>
       </c>
       <c r="B9" s="37">
-        <v>2.2000000000000002</v>
+        <v>1.5</v>
       </c>
       <c r="C9" s="20">
         <v>1.1000000000000001</v>
       </c>
       <c r="D9" s="20">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E9" s="20">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F9" s="20">
-        <v>0.1</v>
+        <v>3.1</v>
       </c>
       <c r="G9" s="20">
-        <v>0.5</v>
+        <v>1.7</v>
       </c>
       <c r="H9" s="16">
-        <v>1.5389398617451588</v>
+        <v>1.0936481387725516</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5385,25 +5404,25 @@
         <v>129</v>
       </c>
       <c r="B10" s="37">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="C10" s="20">
-        <v>1.3</v>
+        <v>2.8</v>
       </c>
       <c r="D10" s="20">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E10" s="20">
-        <v>2.2000000000000002</v>
+        <v>3.1</v>
       </c>
       <c r="F10" s="20">
-        <v>0.9</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G10" s="20">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="H10" s="16">
-        <v>1.5771029464563879</v>
+        <v>2.7808829939621083</v>
       </c>
     </row>
   </sheetData>
@@ -5451,22 +5470,22 @@
         <v>2.9</v>
       </c>
       <c r="C2" s="24">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="D2" s="24">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="E2" s="24">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
       <c r="F2" s="24">
-        <v>2.8</v>
+        <v>3.5</v>
       </c>
       <c r="G2" s="24">
+        <v>3.4</v>
+      </c>
+      <c r="H2" s="24">
         <v>3</v>
-      </c>
-      <c r="H2" s="24">
-        <v>2.9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5474,25 +5493,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="22">
-        <v>4.7</v>
+        <v>3.3</v>
       </c>
       <c r="C3" s="22">
-        <v>5.0999999999999996</v>
+        <v>3</v>
       </c>
       <c r="D3" s="22">
+        <v>3.4</v>
+      </c>
+      <c r="E3" s="22">
         <v>4.5</v>
-      </c>
-      <c r="E3" s="22">
-        <v>4.8</v>
       </c>
       <c r="F3" s="22">
         <v>4.0999999999999996</v>
       </c>
       <c r="G3" s="22">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="H3" s="22">
-        <v>3.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5500,25 +5519,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="22">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="C4" s="22">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="D4" s="22">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="E4" s="22">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="F4" s="22">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="G4" s="22">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="H4" s="22">
-        <v>2.2000000000000002</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5526,25 +5545,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="22">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="C5" s="22">
-        <v>-1.5</v>
+        <v>-0.3</v>
       </c>
       <c r="D5" s="22">
+        <v>0</v>
+      </c>
+      <c r="E5" s="22">
+        <v>0.3</v>
+      </c>
+      <c r="F5" s="22">
         <v>0.4</v>
       </c>
-      <c r="E5" s="22">
-        <v>1.2</v>
-      </c>
-      <c r="F5" s="22">
-        <v>0</v>
-      </c>
       <c r="G5" s="22">
-        <v>-0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H5" s="22">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5552,25 +5571,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="22">
-        <v>3</v>
+        <v>6.8</v>
       </c>
       <c r="C6" s="22">
-        <v>2.1</v>
+        <v>6</v>
       </c>
       <c r="D6" s="22">
-        <v>3.3</v>
+        <v>6.6</v>
       </c>
       <c r="E6" s="22">
-        <v>9.4</v>
+        <v>3.4</v>
       </c>
       <c r="F6" s="22">
-        <v>2.7</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="G6" s="22">
-        <v>1.9</v>
+        <v>10.9</v>
       </c>
       <c r="H6" s="22">
-        <v>4.4000000000000004</v>
+        <v>9.3000000000000007</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5578,22 +5597,22 @@
         <v>17</v>
       </c>
       <c r="B7" s="22">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="C7" s="22">
-        <v>1.5</v>
+        <v>3.1</v>
       </c>
       <c r="D7" s="22">
-        <v>2.2000000000000002</v>
+        <v>2</v>
       </c>
       <c r="E7" s="22">
-        <v>1.5</v>
+        <v>2.7</v>
       </c>
       <c r="F7" s="22">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="G7" s="22">
-        <v>2.2000000000000002</v>
+        <v>2</v>
       </c>
       <c r="H7" s="22">
         <v>2</v>
@@ -5604,25 +5623,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="22">
+        <v>2.5</v>
+      </c>
+      <c r="C8" s="22">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C8" s="22">
-        <v>2.2000000000000002</v>
-      </c>
       <c r="D8" s="22">
+        <v>2.6</v>
+      </c>
+      <c r="E8" s="22">
+        <v>2.4</v>
+      </c>
+      <c r="F8" s="22">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="G8" s="22">
         <v>2.5</v>
       </c>
-      <c r="E8" s="22">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="F8" s="22">
-        <v>2.6</v>
-      </c>
-      <c r="G8" s="22">
-        <v>2.2999999999999998</v>
-      </c>
       <c r="H8" s="22">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5630,25 +5649,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="22">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="C9" s="22">
+        <v>2</v>
+      </c>
+      <c r="D9" s="22">
+        <v>1.9</v>
+      </c>
+      <c r="E9" s="22">
+        <v>2.5</v>
+      </c>
+      <c r="F9" s="22">
+        <v>3.6</v>
+      </c>
+      <c r="G9" s="22">
+        <v>0.8</v>
+      </c>
+      <c r="H9" s="22">
         <v>1.2</v>
-      </c>
-      <c r="D9" s="22">
-        <v>2</v>
-      </c>
-      <c r="E9" s="22">
-        <v>1.8</v>
-      </c>
-      <c r="F9" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="G9" s="22">
-        <v>4.5</v>
-      </c>
-      <c r="H9" s="22">
-        <v>2.7</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5656,25 +5675,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="22">
-        <v>3.6</v>
+        <v>1.8</v>
       </c>
       <c r="C10" s="22">
-        <v>3.9</v>
+        <v>2.1</v>
       </c>
       <c r="D10" s="22">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
       <c r="E10" s="22">
-        <v>3.4</v>
+        <v>1.7</v>
       </c>
       <c r="F10" s="22">
-        <v>3.3</v>
+        <v>1.8</v>
       </c>
       <c r="G10" s="22">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="H10" s="22">
-        <v>3.7</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -5682,25 +5701,25 @@
         <v>21</v>
       </c>
       <c r="B11" s="22">
-        <v>1</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="C11" s="22">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="D11" s="22">
-        <v>0.2</v>
+        <v>4.3</v>
       </c>
       <c r="E11" s="22">
-        <v>1.7</v>
+        <v>3.4</v>
       </c>
       <c r="F11" s="22">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
       <c r="G11" s="22">
-        <v>2.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H11" s="22">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -5708,25 +5727,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="22">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="C12" s="22">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="D12" s="22">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E12" s="22">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="F12" s="22">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="G12" s="22">
-        <v>0.9</v>
+        <v>2.5</v>
       </c>
       <c r="H12" s="22">
-        <v>-0.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -5734,25 +5753,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="22">
-        <v>4.0999999999999996</v>
+        <v>3</v>
       </c>
       <c r="C13" s="22">
-        <v>4.8</v>
+        <v>2.6</v>
       </c>
       <c r="D13" s="22">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E13" s="22">
-        <v>4.4000000000000004</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F13" s="22">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="G13" s="22">
-        <v>3.3</v>
+        <v>2.9</v>
       </c>
       <c r="H13" s="22">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -5760,22 +5779,22 @@
         <v>24</v>
       </c>
       <c r="B14" s="22">
+        <v>3.3</v>
+      </c>
+      <c r="C14" s="22">
+        <v>3.5</v>
+      </c>
+      <c r="D14" s="22">
+        <v>3.3</v>
+      </c>
+      <c r="E14" s="22">
+        <v>2.4</v>
+      </c>
+      <c r="F14" s="22">
         <v>2.7</v>
       </c>
-      <c r="C14" s="22">
-        <v>2.9</v>
-      </c>
-      <c r="D14" s="22">
-        <v>2.6</v>
-      </c>
-      <c r="E14" s="22">
-        <v>2.6</v>
-      </c>
-      <c r="F14" s="22">
-        <v>1.7</v>
-      </c>
       <c r="G14" s="22">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="H14" s="22">
         <v>2.5</v>
@@ -5822,338 +5841,338 @@
       <c r="A2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="33">
-        <v>32.4</v>
-      </c>
-      <c r="C2" s="33">
-        <v>32.700000000000003</v>
-      </c>
-      <c r="D2" s="33">
-        <v>32.200000000000003</v>
-      </c>
-      <c r="E2" s="33">
-        <v>30.5</v>
-      </c>
-      <c r="F2" s="33">
-        <v>31.8</v>
-      </c>
-      <c r="G2" s="33">
+      <c r="B2" s="50">
+        <v>33.1</v>
+      </c>
+      <c r="C2" s="50">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="D2" s="50">
+        <v>32.9</v>
+      </c>
+      <c r="E2" s="50">
+        <v>32.1</v>
+      </c>
+      <c r="F2" s="50">
         <v>33</v>
       </c>
-      <c r="H2" s="33">
-        <v>33.4</v>
+      <c r="G2" s="50">
+        <v>33.9</v>
+      </c>
+      <c r="H2" s="50">
+        <v>33.1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="34">
-        <v>35.9</v>
-      </c>
-      <c r="C3" s="34">
-        <v>37</v>
-      </c>
-      <c r="D3" s="34">
-        <v>35</v>
-      </c>
-      <c r="E3" s="34">
-        <v>36.5</v>
-      </c>
-      <c r="F3" s="34">
+      <c r="B3" s="51">
         <v>36</v>
       </c>
-      <c r="G3" s="34">
-        <v>37.9</v>
-      </c>
-      <c r="H3" s="34">
-        <v>30</v>
+      <c r="C3" s="51">
+        <v>36.700000000000003</v>
+      </c>
+      <c r="D3" s="51">
+        <v>35.4</v>
+      </c>
+      <c r="E3" s="51">
+        <v>38.9</v>
+      </c>
+      <c r="F3" s="51">
+        <v>36.700000000000003</v>
+      </c>
+      <c r="G3" s="51">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="H3" s="51">
+        <v>27.6</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="34">
-        <v>24.1</v>
-      </c>
-      <c r="C4" s="34">
-        <v>24.3</v>
-      </c>
-      <c r="D4" s="34">
-        <v>24.3</v>
-      </c>
-      <c r="E4" s="34">
-        <v>18.8</v>
-      </c>
-      <c r="F4" s="34">
+      <c r="B4" s="51">
+        <v>23.3</v>
+      </c>
+      <c r="C4" s="51">
         <v>23.6</v>
       </c>
-      <c r="G4" s="34">
-        <v>24</v>
-      </c>
-      <c r="H4" s="34">
-        <v>27.6</v>
+      <c r="D4" s="51">
+        <v>23.1</v>
+      </c>
+      <c r="E4" s="51">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="F4" s="51">
+        <v>22.1</v>
+      </c>
+      <c r="G4" s="51">
+        <v>23.3</v>
+      </c>
+      <c r="H4" s="51">
+        <v>26.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="34">
-        <v>15.6</v>
-      </c>
-      <c r="C5" s="34">
-        <v>16</v>
-      </c>
-      <c r="D5" s="34">
-        <v>14.3</v>
-      </c>
-      <c r="E5" s="34">
-        <v>14.5</v>
-      </c>
-      <c r="F5" s="34">
-        <v>17.5</v>
-      </c>
-      <c r="G5" s="34">
-        <v>15.7</v>
-      </c>
-      <c r="H5" s="34">
-        <v>18</v>
+      <c r="B5" s="51">
+        <v>15.1</v>
+      </c>
+      <c r="C5" s="51">
+        <v>15.1</v>
+      </c>
+      <c r="D5" s="51">
+        <v>13.8</v>
+      </c>
+      <c r="E5" s="51">
+        <v>15</v>
+      </c>
+      <c r="F5" s="51">
+        <v>17.2</v>
+      </c>
+      <c r="G5" s="51">
+        <v>16.8</v>
+      </c>
+      <c r="H5" s="51">
+        <v>19.3</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="34">
-        <v>40.200000000000003</v>
-      </c>
-      <c r="C6" s="34">
-        <v>37</v>
-      </c>
-      <c r="D6" s="34">
-        <v>43.5</v>
-      </c>
-      <c r="E6" s="34">
+      <c r="B6" s="51">
+        <v>44.3</v>
+      </c>
+      <c r="C6" s="51">
+        <v>40.700000000000003</v>
+      </c>
+      <c r="D6" s="51">
+        <v>46.8</v>
+      </c>
+      <c r="E6" s="51">
+        <v>43.1</v>
+      </c>
+      <c r="F6" s="51">
         <v>42.1</v>
       </c>
-      <c r="F6" s="34">
-        <v>33.700000000000003</v>
-      </c>
-      <c r="G6" s="34">
-        <v>40.299999999999997</v>
-      </c>
-      <c r="H6" s="34">
-        <v>59.5</v>
+      <c r="G6" s="51">
+        <v>47</v>
+      </c>
+      <c r="H6" s="51">
+        <v>62.5</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="34">
-        <v>19.5</v>
-      </c>
-      <c r="C7" s="34">
-        <v>21</v>
-      </c>
-      <c r="D7" s="34">
-        <v>18.600000000000001</v>
-      </c>
-      <c r="E7" s="34">
-        <v>12.7</v>
-      </c>
-      <c r="F7" s="34">
-        <v>18.399999999999999</v>
-      </c>
-      <c r="G7" s="34">
+      <c r="B7" s="51">
+        <v>21.4</v>
+      </c>
+      <c r="C7" s="51">
+        <v>23.2</v>
+      </c>
+      <c r="D7" s="51">
         <v>20.3</v>
       </c>
-      <c r="H7" s="34">
-        <v>20.100000000000001</v>
+      <c r="E7" s="51">
+        <v>14.6</v>
+      </c>
+      <c r="F7" s="51">
+        <v>20.3</v>
+      </c>
+      <c r="G7" s="51">
+        <v>21.3</v>
+      </c>
+      <c r="H7" s="51">
+        <v>20.6</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="34">
-        <v>28.2</v>
-      </c>
-      <c r="C8" s="34">
-        <v>27.9</v>
-      </c>
-      <c r="D8" s="34">
-        <v>28.6</v>
-      </c>
-      <c r="E8" s="34">
-        <v>26.7</v>
-      </c>
-      <c r="F8" s="34">
+      <c r="B8" s="51">
         <v>28.7</v>
       </c>
-      <c r="G8" s="34">
-        <v>26.1</v>
-      </c>
-      <c r="H8" s="34">
-        <v>30.6</v>
+      <c r="C8" s="51">
+        <v>28.3</v>
+      </c>
+      <c r="D8" s="51">
+        <v>29.1</v>
+      </c>
+      <c r="E8" s="51">
+        <v>27.1</v>
+      </c>
+      <c r="F8" s="51">
+        <v>29.3</v>
+      </c>
+      <c r="G8" s="51">
+        <v>26.6</v>
+      </c>
+      <c r="H8" s="51">
+        <v>32.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="34">
-        <v>32.799999999999997</v>
-      </c>
-      <c r="C9" s="34">
-        <v>33.5</v>
-      </c>
-      <c r="D9" s="34">
+      <c r="B9" s="51">
+        <v>33.1</v>
+      </c>
+      <c r="C9" s="51">
+        <v>34</v>
+      </c>
+      <c r="D9" s="51">
         <v>31.5</v>
       </c>
-      <c r="E9" s="34">
-        <v>26</v>
-      </c>
-      <c r="F9" s="34">
-        <v>32.9</v>
-      </c>
-      <c r="G9" s="34">
-        <v>35.6</v>
-      </c>
-      <c r="H9" s="34">
-        <v>38.200000000000003</v>
+      <c r="E9" s="51">
+        <v>27.1</v>
+      </c>
+      <c r="F9" s="51">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="G9" s="51">
+        <v>34.9</v>
+      </c>
+      <c r="H9" s="51">
+        <v>38.299999999999997</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="34">
-        <v>36.700000000000003</v>
-      </c>
-      <c r="C10" s="34">
-        <v>39</v>
-      </c>
-      <c r="D10" s="34">
-        <v>34.6</v>
-      </c>
-      <c r="E10" s="34">
-        <v>32.700000000000003</v>
-      </c>
-      <c r="F10" s="34">
+      <c r="B10" s="51">
+        <v>36.1</v>
+      </c>
+      <c r="C10" s="51">
+        <v>38.4</v>
+      </c>
+      <c r="D10" s="51">
         <v>34.299999999999997</v>
       </c>
-      <c r="G10" s="34">
-        <v>35</v>
-      </c>
-      <c r="H10" s="34">
-        <v>38</v>
+      <c r="E10" s="51">
+        <v>32</v>
+      </c>
+      <c r="F10" s="51">
+        <v>33.5</v>
+      </c>
+      <c r="G10" s="51">
+        <v>33.9</v>
+      </c>
+      <c r="H10" s="51">
+        <v>35.799999999999997</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="34">
-        <v>28.6</v>
-      </c>
-      <c r="C11" s="34">
-        <v>27.1</v>
-      </c>
-      <c r="D11" s="34">
-        <v>32.9</v>
-      </c>
-      <c r="E11" s="34">
-        <v>24.5</v>
-      </c>
-      <c r="F11" s="34">
-        <v>26.4</v>
-      </c>
-      <c r="G11" s="34">
-        <v>27.4</v>
-      </c>
-      <c r="H11" s="34">
-        <v>22.6</v>
+      <c r="B11" s="51">
+        <v>27.9</v>
+      </c>
+      <c r="C11" s="51">
+        <v>25.5</v>
+      </c>
+      <c r="D11" s="51">
+        <v>33</v>
+      </c>
+      <c r="E11" s="51">
+        <v>26.6</v>
+      </c>
+      <c r="F11" s="51">
+        <v>25.3</v>
+      </c>
+      <c r="G11" s="51">
+        <v>27.2</v>
+      </c>
+      <c r="H11" s="51">
+        <v>22.2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="34">
-        <v>52.4</v>
-      </c>
-      <c r="C12" s="34">
-        <v>41.4</v>
-      </c>
-      <c r="D12" s="34">
-        <v>58.8</v>
-      </c>
-      <c r="E12" s="34">
-        <v>62.1</v>
-      </c>
-      <c r="F12" s="34">
-        <v>76.099999999999994</v>
-      </c>
-      <c r="G12" s="34">
-        <v>61</v>
-      </c>
-      <c r="H12" s="34">
-        <v>82.5</v>
+      <c r="B12" s="51">
+        <v>50.7</v>
+      </c>
+      <c r="C12" s="51">
+        <v>40.9</v>
+      </c>
+      <c r="D12" s="51">
+        <v>56.4</v>
+      </c>
+      <c r="E12" s="51">
+        <v>47.6</v>
+      </c>
+      <c r="F12" s="51">
+        <v>74.5</v>
+      </c>
+      <c r="G12" s="51">
+        <v>63.3</v>
+      </c>
+      <c r="H12" s="51">
+        <v>74.099999999999994</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="34">
-        <v>40.6</v>
-      </c>
-      <c r="C13" s="34">
-        <v>39.700000000000003</v>
-      </c>
-      <c r="D13" s="34">
-        <v>42.7</v>
-      </c>
-      <c r="E13" s="34">
-        <v>43.3</v>
-      </c>
-      <c r="F13" s="34">
-        <v>36.700000000000003</v>
-      </c>
-      <c r="G13" s="34">
-        <v>38.700000000000003</v>
-      </c>
-      <c r="H13" s="34">
-        <v>40.299999999999997</v>
+      <c r="B13" s="51">
+        <v>41.6</v>
+      </c>
+      <c r="C13" s="51">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="D13" s="51">
+        <v>44.1</v>
+      </c>
+      <c r="E13" s="51">
+        <v>47.3</v>
+      </c>
+      <c r="F13" s="51">
+        <v>37.299999999999997</v>
+      </c>
+      <c r="G13" s="51">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="H13" s="51">
+        <v>37.4</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="34">
-        <v>33.200000000000003</v>
-      </c>
-      <c r="C14" s="34">
-        <v>37</v>
-      </c>
-      <c r="D14" s="34">
-        <v>30.8</v>
-      </c>
-      <c r="E14" s="34">
-        <v>28.1</v>
-      </c>
-      <c r="F14" s="34">
-        <v>26.6</v>
-      </c>
-      <c r="G14" s="34">
-        <v>34.299999999999997</v>
-      </c>
-      <c r="H14" s="34">
-        <v>29.8</v>
+      <c r="B14" s="51">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="C14" s="51">
+        <v>37.5</v>
+      </c>
+      <c r="D14" s="51">
+        <v>31.6</v>
+      </c>
+      <c r="E14" s="51">
+        <v>27.9</v>
+      </c>
+      <c r="F14" s="51">
+        <v>26.7</v>
+      </c>
+      <c r="G14" s="51">
+        <v>34.4</v>
+      </c>
+      <c r="H14" s="51">
+        <v>28.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
"Agrego dato res. fiscal y comex feb26, PIB y VAB 4t26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8776FD2E-5FD7-4757-AE0D-7B215F69F12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92C0314-FC8C-41BE-BED4-DD5F6AF8E953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="225">
   <si>
     <t>Período</t>
   </si>
@@ -914,7 +914,7 @@
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -994,13 +994,18 @@
     <xf numFmtId="3" fontId="11" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Euro" xfId="10" xr:uid="{8CA0DC4E-5AAC-43A0-AC51-59D877AC41AF}"/>
@@ -3259,10 +3264,10 @@
         <v>93</v>
       </c>
       <c r="B2">
-        <v>601774.37183884543</v>
+        <v>599983.70014805021</v>
       </c>
       <c r="C2">
-        <v>2.0679847015510067</v>
+        <v>1.3240439045926866</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3270,10 +3275,10 @@
         <v>94</v>
       </c>
       <c r="B3">
-        <v>35745.52874742214</v>
+        <v>38842.924521107714</v>
       </c>
       <c r="C3">
-        <v>0.75515798166041481</v>
+        <v>16.089218460720023</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3281,10 +3286,10 @@
         <v>95</v>
       </c>
       <c r="B4">
-        <v>2885.6963476257092</v>
+        <v>1545.6270924291682</v>
       </c>
       <c r="C4">
-        <v>-20.190472912503587</v>
+        <v>10.567832179756099</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3292,10 +3297,10 @@
         <v>96</v>
       </c>
       <c r="B5">
-        <v>30883.247444069126</v>
+        <v>30755.076629366038</v>
       </c>
       <c r="C5">
-        <v>10.277229912305597</v>
+        <v>8.0983822641656378</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3303,10 +3308,10 @@
         <v>97</v>
       </c>
       <c r="B6">
-        <v>113577.88788301843</v>
+        <v>112761.23165011391</v>
       </c>
       <c r="C6">
-        <v>-2.4055655465160419</v>
+        <v>-5.0381313317373388</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3314,10 +3319,10 @@
         <v>98</v>
       </c>
       <c r="B7">
-        <v>13164.81247256164</v>
+        <v>12673.907286977306</v>
       </c>
       <c r="C7">
-        <v>-0.81974073762508537</v>
+        <v>4.6886508068879618</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3325,10 +3330,10 @@
         <v>99</v>
       </c>
       <c r="B8">
-        <v>20296.837836281982</v>
+        <v>19017.800104434555</v>
       </c>
       <c r="C8">
-        <v>1.0237817598343968</v>
+        <v>0.92123335642904092</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3336,10 +3341,10 @@
         <v>100</v>
       </c>
       <c r="B9">
-        <v>93343.614986502551</v>
+        <v>91872.245634525272</v>
       </c>
       <c r="C9">
-        <v>0.619094181924984</v>
+        <v>-2.2069029193928613</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3347,10 +3352,10 @@
         <v>101</v>
       </c>
       <c r="B10">
-        <v>11853.533818035672</v>
+        <v>13022.400979766842</v>
       </c>
       <c r="C10">
-        <v>7.1428768688438504</v>
+        <v>-0.66957849547361059</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3358,10 +3363,10 @@
         <v>102</v>
       </c>
       <c r="B11">
-        <v>55332.186087353206</v>
+        <v>55633.327772916178</v>
       </c>
       <c r="C11">
-        <v>1.7728968233303721</v>
+        <v>2.1967051692507011</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3369,10 +3374,10 @@
         <v>103</v>
       </c>
       <c r="B12">
-        <v>31025.390068801698</v>
+        <v>30381.126773097683</v>
       </c>
       <c r="C12">
-        <v>28.354908519955814</v>
+        <v>17.24588178668942</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3380,10 +3385,10 @@
         <v>104</v>
       </c>
       <c r="B13">
-        <v>84710.173468865076</v>
+        <v>85939.774708283672</v>
       </c>
       <c r="C13">
-        <v>3.6890093504288846</v>
+        <v>2.0043316406221923</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3391,10 +3396,10 @@
         <v>105</v>
       </c>
       <c r="B14">
-        <v>35107.740864300358</v>
+        <v>34900.492729780119</v>
       </c>
       <c r="C14">
-        <v>-0.57065650406127322</v>
+        <v>-1.0550626738513924</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3402,10 +3407,10 @@
         <v>106</v>
       </c>
       <c r="B15">
-        <v>29948.638227285704</v>
+        <v>29912.893832996058</v>
       </c>
       <c r="C15">
-        <v>1.3503828666152184</v>
+        <v>0.64148026369161837</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -3413,10 +3418,10 @@
         <v>107</v>
       </c>
       <c r="B16">
-        <v>24349.209293840257</v>
+        <v>23085.607234226565</v>
       </c>
       <c r="C16">
-        <v>7.1541632982685677E-2</v>
+        <v>0.28721826490549773</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3424,10 +3429,10 @@
         <v>108</v>
       </c>
       <c r="B17">
-        <v>15566.748781195141</v>
+        <v>15478.186568411322</v>
       </c>
       <c r="C17">
-        <v>0.5659234061553553</v>
+        <v>1.0991937461104273</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -3435,10 +3440,10 @@
         <v>109</v>
       </c>
       <c r="B18">
-        <v>3983.1255116867405</v>
+        <v>4161.0766296179845</v>
       </c>
       <c r="C18">
-        <v>-0.48787459513544018</v>
+        <v>2.7585257742845926E-2</v>
       </c>
     </row>
   </sheetData>
@@ -5841,25 +5846,25 @@
       <c r="A2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="50">
+      <c r="B2" s="33">
         <v>33.1</v>
       </c>
-      <c r="C2" s="50">
+      <c r="C2" s="33">
         <v>33.200000000000003</v>
       </c>
-      <c r="D2" s="50">
+      <c r="D2" s="33">
         <v>32.9</v>
       </c>
-      <c r="E2" s="50">
+      <c r="E2" s="33">
         <v>32.1</v>
       </c>
-      <c r="F2" s="50">
+      <c r="F2" s="33">
         <v>33</v>
       </c>
-      <c r="G2" s="50">
+      <c r="G2" s="33">
         <v>33.9</v>
       </c>
-      <c r="H2" s="50">
+      <c r="H2" s="33">
         <v>33.1</v>
       </c>
     </row>
@@ -5867,25 +5872,25 @@
       <c r="A3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="51">
+      <c r="B3" s="34">
         <v>36</v>
       </c>
-      <c r="C3" s="51">
+      <c r="C3" s="34">
         <v>36.700000000000003</v>
       </c>
-      <c r="D3" s="51">
+      <c r="D3" s="34">
         <v>35.4</v>
       </c>
-      <c r="E3" s="51">
+      <c r="E3" s="34">
         <v>38.9</v>
       </c>
-      <c r="F3" s="51">
+      <c r="F3" s="34">
         <v>36.700000000000003</v>
       </c>
-      <c r="G3" s="51">
+      <c r="G3" s="34">
         <v>38.299999999999997</v>
       </c>
-      <c r="H3" s="51">
+      <c r="H3" s="34">
         <v>27.6</v>
       </c>
     </row>
@@ -5893,25 +5898,25 @@
       <c r="A4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="51">
+      <c r="B4" s="34">
         <v>23.3</v>
       </c>
-      <c r="C4" s="51">
+      <c r="C4" s="34">
         <v>23.6</v>
       </c>
-      <c r="D4" s="51">
+      <c r="D4" s="34">
         <v>23.1</v>
       </c>
-      <c r="E4" s="51">
+      <c r="E4" s="34">
         <v>20.399999999999999</v>
       </c>
-      <c r="F4" s="51">
+      <c r="F4" s="34">
         <v>22.1</v>
       </c>
-      <c r="G4" s="51">
+      <c r="G4" s="34">
         <v>23.3</v>
       </c>
-      <c r="H4" s="51">
+      <c r="H4" s="34">
         <v>26.4</v>
       </c>
     </row>
@@ -5919,25 +5924,25 @@
       <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="51">
+      <c r="B5" s="34">
         <v>15.1</v>
       </c>
-      <c r="C5" s="51">
+      <c r="C5" s="34">
         <v>15.1</v>
       </c>
-      <c r="D5" s="51">
+      <c r="D5" s="34">
         <v>13.8</v>
       </c>
-      <c r="E5" s="51">
+      <c r="E5" s="34">
         <v>15</v>
       </c>
-      <c r="F5" s="51">
+      <c r="F5" s="34">
         <v>17.2</v>
       </c>
-      <c r="G5" s="51">
+      <c r="G5" s="34">
         <v>16.8</v>
       </c>
-      <c r="H5" s="51">
+      <c r="H5" s="34">
         <v>19.3</v>
       </c>
     </row>
@@ -5945,25 +5950,25 @@
       <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="51">
+      <c r="B6" s="34">
         <v>44.3</v>
       </c>
-      <c r="C6" s="51">
+      <c r="C6" s="34">
         <v>40.700000000000003</v>
       </c>
-      <c r="D6" s="51">
+      <c r="D6" s="34">
         <v>46.8</v>
       </c>
-      <c r="E6" s="51">
+      <c r="E6" s="34">
         <v>43.1</v>
       </c>
-      <c r="F6" s="51">
+      <c r="F6" s="34">
         <v>42.1</v>
       </c>
-      <c r="G6" s="51">
+      <c r="G6" s="34">
         <v>47</v>
       </c>
-      <c r="H6" s="51">
+      <c r="H6" s="34">
         <v>62.5</v>
       </c>
     </row>
@@ -5971,25 +5976,25 @@
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="51">
+      <c r="B7" s="34">
         <v>21.4</v>
       </c>
-      <c r="C7" s="51">
+      <c r="C7" s="34">
         <v>23.2</v>
       </c>
-      <c r="D7" s="51">
+      <c r="D7" s="34">
         <v>20.3</v>
       </c>
-      <c r="E7" s="51">
+      <c r="E7" s="34">
         <v>14.6</v>
       </c>
-      <c r="F7" s="51">
+      <c r="F7" s="34">
         <v>20.3</v>
       </c>
-      <c r="G7" s="51">
+      <c r="G7" s="34">
         <v>21.3</v>
       </c>
-      <c r="H7" s="51">
+      <c r="H7" s="34">
         <v>20.6</v>
       </c>
     </row>
@@ -5997,25 +6002,25 @@
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="51">
+      <c r="B8" s="34">
         <v>28.7</v>
       </c>
-      <c r="C8" s="51">
+      <c r="C8" s="34">
         <v>28.3</v>
       </c>
-      <c r="D8" s="51">
+      <c r="D8" s="34">
         <v>29.1</v>
       </c>
-      <c r="E8" s="51">
+      <c r="E8" s="34">
         <v>27.1</v>
       </c>
-      <c r="F8" s="51">
+      <c r="F8" s="34">
         <v>29.3</v>
       </c>
-      <c r="G8" s="51">
+      <c r="G8" s="34">
         <v>26.6</v>
       </c>
-      <c r="H8" s="51">
+      <c r="H8" s="34">
         <v>32.4</v>
       </c>
     </row>
@@ -6023,25 +6028,25 @@
       <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="51">
+      <c r="B9" s="34">
         <v>33.1</v>
       </c>
-      <c r="C9" s="51">
+      <c r="C9" s="34">
         <v>34</v>
       </c>
-      <c r="D9" s="51">
+      <c r="D9" s="34">
         <v>31.5</v>
       </c>
-      <c r="E9" s="51">
+      <c r="E9" s="34">
         <v>27.1</v>
       </c>
-      <c r="F9" s="51">
+      <c r="F9" s="34">
         <v>34.299999999999997</v>
       </c>
-      <c r="G9" s="51">
+      <c r="G9" s="34">
         <v>34.9</v>
       </c>
-      <c r="H9" s="51">
+      <c r="H9" s="34">
         <v>38.299999999999997</v>
       </c>
     </row>
@@ -6049,25 +6054,25 @@
       <c r="A10" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="51">
+      <c r="B10" s="34">
         <v>36.1</v>
       </c>
-      <c r="C10" s="51">
+      <c r="C10" s="34">
         <v>38.4</v>
       </c>
-      <c r="D10" s="51">
+      <c r="D10" s="34">
         <v>34.299999999999997</v>
       </c>
-      <c r="E10" s="51">
+      <c r="E10" s="34">
         <v>32</v>
       </c>
-      <c r="F10" s="51">
+      <c r="F10" s="34">
         <v>33.5</v>
       </c>
-      <c r="G10" s="51">
+      <c r="G10" s="34">
         <v>33.9</v>
       </c>
-      <c r="H10" s="51">
+      <c r="H10" s="34">
         <v>35.799999999999997</v>
       </c>
     </row>
@@ -6075,25 +6080,25 @@
       <c r="A11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="51">
+      <c r="B11" s="34">
         <v>27.9</v>
       </c>
-      <c r="C11" s="51">
+      <c r="C11" s="34">
         <v>25.5</v>
       </c>
-      <c r="D11" s="51">
+      <c r="D11" s="34">
         <v>33</v>
       </c>
-      <c r="E11" s="51">
+      <c r="E11" s="34">
         <v>26.6</v>
       </c>
-      <c r="F11" s="51">
+      <c r="F11" s="34">
         <v>25.3</v>
       </c>
-      <c r="G11" s="51">
+      <c r="G11" s="34">
         <v>27.2</v>
       </c>
-      <c r="H11" s="51">
+      <c r="H11" s="34">
         <v>22.2</v>
       </c>
     </row>
@@ -6101,25 +6106,25 @@
       <c r="A12" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="51">
+      <c r="B12" s="34">
         <v>50.7</v>
       </c>
-      <c r="C12" s="51">
+      <c r="C12" s="34">
         <v>40.9</v>
       </c>
-      <c r="D12" s="51">
+      <c r="D12" s="34">
         <v>56.4</v>
       </c>
-      <c r="E12" s="51">
+      <c r="E12" s="34">
         <v>47.6</v>
       </c>
-      <c r="F12" s="51">
+      <c r="F12" s="34">
         <v>74.5</v>
       </c>
-      <c r="G12" s="51">
+      <c r="G12" s="34">
         <v>63.3</v>
       </c>
-      <c r="H12" s="51">
+      <c r="H12" s="34">
         <v>74.099999999999994</v>
       </c>
     </row>
@@ -6127,25 +6132,25 @@
       <c r="A13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="51">
+      <c r="B13" s="34">
         <v>41.6</v>
       </c>
-      <c r="C13" s="51">
+      <c r="C13" s="34">
         <v>40.799999999999997</v>
       </c>
-      <c r="D13" s="51">
+      <c r="D13" s="34">
         <v>44.1</v>
       </c>
-      <c r="E13" s="51">
+      <c r="E13" s="34">
         <v>47.3</v>
       </c>
-      <c r="F13" s="51">
+      <c r="F13" s="34">
         <v>37.299999999999997</v>
       </c>
-      <c r="G13" s="51">
+      <c r="G13" s="34">
         <v>38.299999999999997</v>
       </c>
-      <c r="H13" s="51">
+      <c r="H13" s="34">
         <v>37.4</v>
       </c>
     </row>
@@ -6153,25 +6158,25 @@
       <c r="A14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="51">
+      <c r="B14" s="34">
         <v>33.700000000000003</v>
       </c>
-      <c r="C14" s="51">
+      <c r="C14" s="34">
         <v>37.5</v>
       </c>
-      <c r="D14" s="51">
+      <c r="D14" s="34">
         <v>31.6</v>
       </c>
-      <c r="E14" s="51">
+      <c r="E14" s="34">
         <v>27.9</v>
       </c>
-      <c r="F14" s="51">
+      <c r="F14" s="34">
         <v>26.7</v>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="34">
         <v>34.4</v>
       </c>
-      <c r="H14" s="51">
+      <c r="H14" s="34">
         <v>28.8</v>
       </c>
     </row>
@@ -6183,7 +6188,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="11.42578125" style="10" customWidth="1"/>
@@ -6211,7 +6216,7 @@
         <v>29</v>
       </c>
       <c r="C2" s="11">
-        <v>476076.35591188457</v>
+        <v>476036.52687146427</v>
       </c>
       <c r="D2" s="11">
         <v>460369.44223294902</v>
@@ -6225,7 +6230,7 @@
         <v>30</v>
       </c>
       <c r="C3" s="11">
-        <v>470012.80022148089</v>
+        <v>470010.06614707055</v>
       </c>
       <c r="D3" s="11">
         <v>514395.68177236198</v>
@@ -6239,7 +6244,7 @@
         <v>31</v>
       </c>
       <c r="C4" s="11">
-        <v>493891.12238798192</v>
+        <v>493895.12091097509</v>
       </c>
       <c r="D4" s="11">
         <v>481151.97994350799</v>
@@ -6253,7 +6258,7 @@
         <v>32</v>
       </c>
       <c r="C5" s="11">
-        <v>500480.50233110512</v>
+        <v>500519.06692598236</v>
       </c>
       <c r="D5" s="11">
         <v>484543.67687656201</v>
@@ -6267,7 +6272,7 @@
         <v>29</v>
       </c>
       <c r="C6" s="11">
-        <v>514983.24764611531</v>
+        <v>514918.45889096794</v>
       </c>
       <c r="D6" s="11">
         <v>493602.53057785501</v>
@@ -6281,7 +6286,7 @@
         <v>30</v>
       </c>
       <c r="C7" s="11">
-        <v>527064.5782008057</v>
+        <v>527084.19831498002</v>
       </c>
       <c r="D7" s="11">
         <v>581668.24987960199</v>
@@ -6295,7 +6300,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="11">
-        <v>530103.2878765451</v>
+        <v>530101.95784154162</v>
       </c>
       <c r="D8" s="11">
         <v>514697.78950542799</v>
@@ -6309,7 +6314,7 @@
         <v>32</v>
       </c>
       <c r="C9" s="11">
-        <v>540072.65629019018</v>
+        <v>540119.15496616694</v>
       </c>
       <c r="D9" s="11">
         <v>522255.20005077199</v>
@@ -6323,7 +6328,7 @@
         <v>29</v>
       </c>
       <c r="C10" s="11">
-        <v>554499.36072981206</v>
+        <v>554455.77230754215</v>
       </c>
       <c r="D10" s="11">
         <v>532348.21201691695</v>
@@ -6337,7 +6342,7 @@
         <v>30</v>
       </c>
       <c r="C11" s="11">
-        <v>561170.97269354202</v>
+        <v>561157.22299964982</v>
       </c>
       <c r="D11" s="11">
         <v>614076.39260854397</v>
@@ -6351,7 +6356,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="11">
-        <v>577074.9473486176</v>
+        <v>577088.45820131898</v>
       </c>
       <c r="D12" s="11">
         <v>562978.96562687703</v>
@@ -6365,7 +6370,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="11">
-        <v>589452.33611095417</v>
+        <v>589496.16337441502</v>
       </c>
       <c r="D13" s="11">
         <v>572794.04663058801</v>
@@ -6379,7 +6384,7 @@
         <v>29</v>
       </c>
       <c r="C14" s="11">
-        <v>603536.53953781037</v>
+        <v>603483.20680705283</v>
       </c>
       <c r="D14" s="11">
         <v>576846.88569942699</v>
@@ -6393,7 +6398,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="11">
-        <v>616075.60945719469</v>
+        <v>616073.36568713211</v>
       </c>
       <c r="D15" s="11">
         <v>674620.563006485</v>
@@ -6407,7 +6412,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="11">
-        <v>624421.53581424942</v>
+        <v>624446.89492768422</v>
       </c>
       <c r="D16" s="11">
         <v>610425.69401485403</v>
@@ -6421,7 +6426,7 @@
         <v>32</v>
       </c>
       <c r="C17" s="11">
-        <v>643736.32577510865</v>
+        <v>643766.54316249432</v>
       </c>
       <c r="D17" s="11">
         <v>625876.867863597</v>
@@ -6435,7 +6440,7 @@
         <v>29</v>
       </c>
       <c r="C18" s="11">
-        <v>650156.81326832587</v>
+        <v>650003.25715436717</v>
       </c>
       <c r="D18" s="11">
         <v>616720.35706447798</v>
@@ -6449,7 +6454,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="11">
-        <v>653370.04317222571</v>
+        <v>653467.95396695228</v>
       </c>
       <c r="D19" s="11">
         <v>711405.50045523304</v>
@@ -6463,7 +6468,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="11">
-        <v>657667.74583037221</v>
+        <v>657695.28402587795</v>
       </c>
       <c r="D20" s="11">
         <v>647087.95974249404</v>
@@ -6477,7 +6482,7 @@
         <v>32</v>
       </c>
       <c r="C21" s="11">
-        <v>627510.03669392434</v>
+        <v>627538.1438176519</v>
       </c>
       <c r="D21" s="11">
         <v>613490.82170264097</v>
@@ -6491,7 +6496,7 @@
         <v>29</v>
       </c>
       <c r="C22" s="11">
-        <v>604984.05052486621</v>
+        <v>604940.28395197983</v>
       </c>
       <c r="D22" s="11">
         <v>578553.04424240498</v>
@@ -6505,7 +6510,7 @@
         <v>30</v>
       </c>
       <c r="C23" s="11">
-        <v>590520.62462346</v>
+        <v>590529.02806835552</v>
       </c>
       <c r="D23" s="11">
         <v>631197.75186006899</v>
@@ -6519,7 +6524,7 @@
         <v>31</v>
       </c>
       <c r="C24" s="11">
-        <v>613784.10582940001</v>
+        <v>613800.25653562765</v>
       </c>
       <c r="D24" s="11">
         <v>610519.85461172694</v>
@@ -6533,7 +6538,7 @@
         <v>32</v>
       </c>
       <c r="C25" s="11">
-        <v>626202.7246737713</v>
+        <v>626221.93709553429</v>
       </c>
       <c r="D25" s="11">
         <v>615220.85493729694</v>
@@ -6547,7 +6552,7 @@
         <v>29</v>
       </c>
       <c r="C26" s="11">
-        <v>645567.1335175815</v>
+        <v>645513.99738394632</v>
       </c>
       <c r="D26" s="11">
         <v>611607.33658973</v>
@@ -6561,7 +6566,7 @@
         <v>30</v>
       </c>
       <c r="C27" s="11">
-        <v>674129.37854994042</v>
+        <v>674164.23542403907</v>
       </c>
       <c r="D27" s="11">
         <v>733730.773968903</v>
@@ -6575,7 +6580,7 @@
         <v>31</v>
       </c>
       <c r="C28" s="11">
-        <v>676987.62755641807</v>
+        <v>676995.53972733335</v>
       </c>
       <c r="D28" s="11">
         <v>668566.50948898599</v>
@@ -6589,7 +6594,7 @@
         <v>32</v>
       </c>
       <c r="C29" s="11">
-        <v>685410.57814325311</v>
+        <v>685420.94523187377</v>
       </c>
       <c r="D29" s="11">
         <v>668190.097719574</v>
@@ -6603,7 +6608,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="11">
-        <v>701719.95832865476</v>
+        <v>701686.92075505713</v>
       </c>
       <c r="D30" s="11">
         <v>662325.58597269503</v>
@@ -6617,7 +6622,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="11">
-        <v>710310.00486147264</v>
+        <v>710326.15459237562</v>
       </c>
       <c r="D31" s="11">
         <v>766332.95457161299</v>
@@ -6631,7 +6636,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="11">
-        <v>715887.66436332592</v>
+        <v>715883.91149126994</v>
       </c>
       <c r="D32" s="11">
         <v>711417.39193010505</v>
@@ -6645,7 +6650,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="11">
-        <v>715208.76132895402</v>
+        <v>715229.40204370406</v>
       </c>
       <c r="D33" s="11">
         <v>703050.45640799298</v>
@@ -6659,7 +6664,7 @@
         <v>29</v>
       </c>
       <c r="C34" s="11">
-        <v>708376.22005569842</v>
+        <v>708348.86146128085</v>
       </c>
       <c r="D34" s="11">
         <v>672685.993630504</v>
@@ -6673,7 +6678,7 @@
         <v>30</v>
       </c>
       <c r="C35" s="11">
-        <v>683605.99878134322</v>
+        <v>683593.31589575845</v>
       </c>
       <c r="D35" s="11">
         <v>730838.27259277599</v>
@@ -6687,7 +6692,7 @@
         <v>31</v>
       </c>
       <c r="C36" s="11">
-        <v>705285.22539860196</v>
+        <v>705293.74411482143</v>
       </c>
       <c r="D36" s="11">
         <v>703461.65253019601</v>
@@ -6701,7 +6706,7 @@
         <v>32</v>
       </c>
       <c r="C37" s="11">
-        <v>716676.51360015152</v>
+        <v>716708.03636393591</v>
       </c>
       <c r="D37" s="11">
         <v>706958.03908231901</v>
@@ -6715,7 +6720,7 @@
         <v>29</v>
       </c>
       <c r="C38" s="11">
-        <v>716063.69146123226</v>
+        <v>715943.73773188714</v>
       </c>
       <c r="D38" s="11">
         <v>677085.52917315101</v>
@@ -6729,7 +6734,7 @@
         <v>30</v>
       </c>
       <c r="C39" s="11">
-        <v>720808.83227209072</v>
+        <v>720882.8515662452</v>
       </c>
       <c r="D39" s="11">
         <v>776486.60279942001</v>
@@ -6743,7 +6748,7 @@
         <v>31</v>
       </c>
       <c r="C40" s="11">
-        <v>725573.2191300554</v>
+        <v>725588.38163084479</v>
       </c>
       <c r="D40" s="11">
         <v>721458.94421618199</v>
@@ -6757,7 +6762,7 @@
         <v>32</v>
       </c>
       <c r="C41" s="11">
-        <v>719182.67834788037</v>
+        <v>719213.4502822801</v>
       </c>
       <c r="D41" s="11">
         <v>706597.34502250701</v>
@@ -6771,7 +6776,7 @@
         <v>29</v>
       </c>
       <c r="C42" s="11">
-        <v>708315.37698831095</v>
+        <v>708278.97258087643</v>
       </c>
       <c r="D42" s="11">
         <v>671066.04663506302</v>
@@ -6785,7 +6790,7 @@
         <v>30</v>
       </c>
       <c r="C43" s="11">
-        <v>702913.19880550797</v>
+        <v>702914.57152322109</v>
       </c>
       <c r="D43" s="11">
         <v>760576.86834800395</v>
@@ -6799,7 +6804,7 @@
         <v>31</v>
       </c>
       <c r="C44" s="11">
-        <v>697283.51011195104</v>
+        <v>697281.49261729233</v>
       </c>
       <c r="D44" s="11">
         <v>690879.79825168301</v>
@@ -6813,7 +6818,7 @@
         <v>32</v>
       </c>
       <c r="C45" s="11">
-        <v>700712.09794769145</v>
+        <v>700749.14713207202</v>
       </c>
       <c r="D45" s="11">
         <v>686701.47061871097</v>
@@ -6827,7 +6832,7 @@
         <v>29</v>
       </c>
       <c r="C46" s="11">
-        <v>710751.90614638862</v>
+        <v>710714.75219443382</v>
       </c>
       <c r="D46" s="11">
         <v>672749.81139169901</v>
@@ -6841,7 +6846,7 @@
         <v>30</v>
       </c>
       <c r="C47" s="11">
-        <v>728932.58641636837</v>
+        <v>728934.83476324868</v>
       </c>
       <c r="D47" s="11">
         <v>791235.96554166998</v>
@@ -6855,7 +6860,7 @@
         <v>31</v>
       </c>
       <c r="C48" s="11">
-        <v>727453.28403633856</v>
+        <v>727453.63885899587</v>
       </c>
       <c r="D48" s="11">
         <v>718281.26544978202</v>
@@ -6869,7 +6874,7 @@
         <v>32</v>
       </c>
       <c r="C49" s="11">
-        <v>718810.80995306326</v>
+        <v>718845.360735483</v>
       </c>
       <c r="D49" s="11">
         <v>703681.54416900803</v>
@@ -6883,7 +6888,7 @@
         <v>29</v>
       </c>
       <c r="C50" s="11">
-        <v>713509.00776950188</v>
+        <v>713388.1069145425</v>
       </c>
       <c r="D50" s="11">
         <v>677652.08911570301</v>
@@ -6897,7 +6902,7 @@
         <v>30</v>
       </c>
       <c r="C51" s="11">
-        <v>701417.69900093763</v>
+        <v>701514.77320906788</v>
       </c>
       <c r="D51" s="11">
         <v>760703.28015165601</v>
@@ -6911,7 +6916,7 @@
         <v>31</v>
       </c>
       <c r="C52" s="11">
-        <v>703218.45737271302</v>
+        <v>703211.858554565</v>
       </c>
       <c r="D52" s="11">
         <v>694382.47577623103</v>
@@ -6925,7 +6930,7 @@
         <v>32</v>
       </c>
       <c r="C53" s="11">
-        <v>707766.23024749616</v>
+        <v>707796.65571247344</v>
       </c>
       <c r="D53" s="11">
         <v>693173.54934705805</v>
@@ -6939,7 +6944,7 @@
         <v>29</v>
       </c>
       <c r="C54" s="11">
-        <v>714739.75730170158</v>
+        <v>714701.00378393335</v>
       </c>
       <c r="D54" s="11">
         <v>681444.76611022197</v>
@@ -6953,7 +6958,7 @@
         <v>30</v>
       </c>
       <c r="C55" s="11">
-        <v>721738.8931862677</v>
+        <v>721713.65757954179</v>
       </c>
       <c r="D55" s="11">
         <v>778401.67644931702</v>
@@ -6967,7 +6972,7 @@
         <v>31</v>
       </c>
       <c r="C56" s="11">
-        <v>731047.79495902965</v>
+        <v>731047.00599477056</v>
       </c>
       <c r="D56" s="11">
         <v>721120.42685279401</v>
@@ -6981,7 +6986,7 @@
         <v>32</v>
       </c>
       <c r="C57" s="11">
-        <v>738033.34560429957</v>
+        <v>738098.12369305</v>
       </c>
       <c r="D57" s="11">
         <v>724592.92163896305</v>
@@ -6995,7 +7000,7 @@
         <v>29</v>
       </c>
       <c r="C58" s="11">
-        <v>734123.80379438028</v>
+        <v>734098.41115135164</v>
       </c>
       <c r="D58" s="11">
         <v>707324.26805721398</v>
@@ -7009,7 +7014,7 @@
         <v>30</v>
       </c>
       <c r="C59" s="11">
-        <v>703511.92695430492</v>
+        <v>703426.52003617655</v>
       </c>
       <c r="D59" s="11">
         <v>747428.29995457502</v>
@@ -7023,7 +7028,7 @@
         <v>31</v>
       </c>
       <c r="C60" s="11">
-        <v>701395.88870482845</v>
+        <v>701416.02106970118</v>
       </c>
       <c r="D60" s="11">
         <v>696101.58352180803</v>
@@ -7037,7 +7042,7 @@
         <v>32</v>
       </c>
       <c r="C61" s="11">
-        <v>690478.15246453509</v>
+        <v>690568.81966081902</v>
       </c>
       <c r="D61" s="11">
         <v>678655.62038445403</v>
@@ -7051,7 +7056,7 @@
         <v>29</v>
       </c>
       <c r="C62" s="11">
-        <v>693093.70549915161</v>
+        <v>692977.78815745737</v>
       </c>
       <c r="D62">
         <v>665848.71529970889</v>
@@ -7065,7 +7070,7 @@
         <v>30</v>
       </c>
       <c r="C63" s="11">
-        <v>696861.35118506756</v>
+        <v>696856.65350922232</v>
       </c>
       <c r="D63">
         <v>751784.46077713254</v>
@@ -7079,13 +7084,13 @@
         <v>31</v>
       </c>
       <c r="C64" s="11">
-        <v>696314.14262671897</v>
+        <v>696337.7406497316</v>
       </c>
       <c r="D64">
         <v>683900.89855257841</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="10">
         <v>2019</v>
       </c>
@@ -7093,13 +7098,13 @@
         <v>32</v>
       </c>
       <c r="C65" s="11">
-        <v>686626.01504090067</v>
+        <v>686723.03203542822</v>
       </c>
       <c r="D65">
         <v>671361.13972242002</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="10">
         <v>2020</v>
       </c>
@@ -7107,13 +7112,13 @@
         <v>29</v>
       </c>
       <c r="C66" s="10">
-        <v>656444.50206127646</v>
+        <v>656405.46191031951</v>
       </c>
       <c r="D66" s="10">
         <v>632389.35353461001</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="10">
         <v>2020</v>
       </c>
@@ -7121,13 +7126,13 @@
         <v>30</v>
       </c>
       <c r="C67" s="10">
-        <v>563576.4456951567</v>
+        <v>563484.6621608017</v>
       </c>
       <c r="D67" s="10">
         <v>609379.98946480127</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="10">
         <v>2020</v>
       </c>
@@ -7135,13 +7140,13 @@
         <v>31</v>
       </c>
       <c r="C68" s="10">
-        <v>623894.19861283677</v>
+        <v>623894.44182136783</v>
       </c>
       <c r="D68" s="10">
         <v>614192.47840422287</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="10">
         <v>2020</v>
       </c>
@@ -7149,13 +7154,13 @@
         <v>32</v>
       </c>
       <c r="C69" s="10">
-        <v>654449.99823231436</v>
+        <v>654580.57870909641</v>
       </c>
       <c r="D69" s="10">
         <v>642403.32319795026</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="10">
         <v>2021</v>
       </c>
@@ -7163,13 +7168,13 @@
         <v>29</v>
       </c>
       <c r="C70" s="10">
-        <v>677250.47982575209</v>
+        <v>677169.13791920443</v>
       </c>
       <c r="D70">
         <v>652831.97670632158</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="10">
         <v>2021</v>
       </c>
@@ -7177,13 +7182,13 @@
         <v>30</v>
       </c>
       <c r="C71" s="10">
-        <v>679149.09279086394</v>
+        <v>679096.31371864828</v>
       </c>
       <c r="D71">
         <v>723516.62249067484</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="10">
         <v>2021</v>
       </c>
@@ -7191,13 +7196,13 @@
         <v>31</v>
       </c>
       <c r="C72" s="10">
-        <v>693044.47480042151</v>
+        <v>693100.33574559912</v>
       </c>
       <c r="D72" s="10">
         <v>686756.46782667423</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="10">
         <v>2021</v>
       </c>
@@ -7205,13 +7210,13 @@
         <v>32</v>
       </c>
       <c r="C73" s="10">
-        <v>709795.68871874886</v>
+        <v>709873.94875233434</v>
       </c>
       <c r="D73" s="10">
         <v>696134.66911211505</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="10">
         <v>2022</v>
       </c>
@@ -7219,13 +7224,13 @@
         <v>29</v>
       </c>
       <c r="C74" s="10">
-        <v>727217.19021071692</v>
+        <v>726931.81776528095</v>
       </c>
       <c r="D74">
         <v>697625.28466635814</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="10">
         <v>2022</v>
       </c>
@@ -7233,13 +7238,13 @@
         <v>30</v>
       </c>
       <c r="C75" s="10">
-        <v>741248.85874275723</v>
+        <v>741189.8641333899</v>
       </c>
       <c r="D75">
         <v>782338.62853373506</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="10">
         <v>2022</v>
       </c>
@@ -7247,13 +7252,13 @@
         <v>31</v>
       </c>
       <c r="C76" s="10">
-        <v>735357.63471055031</v>
+        <v>735605.99139607733</v>
       </c>
       <c r="D76" s="10">
         <v>732662.16387550125</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="10">
         <v>2022</v>
       </c>
@@ -7261,13 +7266,13 @@
         <v>32</v>
       </c>
       <c r="C77" s="10">
-        <v>721542.85124030802</v>
+        <v>721638.86160958419</v>
       </c>
       <c r="D77" s="10">
         <v>712740.45782873826</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="10">
         <v>2023</v>
       </c>
@@ -7275,15 +7280,14 @@
         <v>29</v>
       </c>
       <c r="C78" s="10">
-        <v>728411.03637298418</v>
+        <v>727949.28499660653</v>
       </c>
       <c r="D78" s="10">
         <v>703987.50432157726</v>
       </c>
       <c r="E78" s="39"/>
-      <c r="F78" s="39"/>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="10">
         <v>2023</v>
       </c>
@@ -7291,15 +7295,14 @@
         <v>30</v>
       </c>
       <c r="C79" s="10">
-        <v>710604.35007449426</v>
+        <v>710424.84865227621</v>
       </c>
       <c r="D79" s="10">
         <v>737941.90937407222</v>
       </c>
       <c r="E79" s="40"/>
-      <c r="F79" s="40"/>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="10">
         <v>2023</v>
       </c>
@@ -7307,7 +7310,7 @@
         <v>31</v>
       </c>
       <c r="C80" s="10">
-        <v>724360.15045882703</v>
+        <v>725091.04020458832</v>
       </c>
       <c r="D80" s="10">
         <v>728638.58456868224</v>
@@ -7322,7 +7325,7 @@
         <v>32</v>
       </c>
       <c r="C81" s="10">
-        <v>707702.39593034761</v>
+        <v>707612.75898318249</v>
       </c>
       <c r="D81" s="10">
         <v>700509.93457232334</v>
@@ -7336,7 +7339,7 @@
         <v>29</v>
       </c>
       <c r="C82" s="10">
-        <v>696359.28899467527</v>
+        <v>696039.64182027197</v>
       </c>
       <c r="D82" s="10">
         <v>669057.73338516685</v>
@@ -7350,7 +7353,7 @@
         <v>30</v>
       </c>
       <c r="C83" s="10">
-        <v>690619.26110419934</v>
+        <v>690565.59876287449</v>
       </c>
       <c r="D83">
         <v>729947.78527455311</v>
@@ -7364,7 +7367,7 @@
         <v>31</v>
       </c>
       <c r="C84" s="10">
-        <v>715761.56016933941</v>
+        <v>717175.74805169622</v>
       </c>
       <c r="D84">
         <v>714524.36554995924</v>
@@ -7378,7 +7381,7 @@
         <v>32</v>
       </c>
       <c r="C85" s="10">
-        <v>729781.23766831763</v>
+        <v>728740.35651141696</v>
       </c>
       <c r="D85" s="10">
         <v>718991.4609365795</v>
@@ -7392,7 +7395,7 @@
         <v>29</v>
       </c>
       <c r="C86" s="10">
-        <v>737836.57234611677</v>
+        <v>736261.04995951243</v>
       </c>
       <c r="D86" s="10">
         <v>708113.80567017628</v>
@@ -7406,7 +7409,7 @@
         <v>30</v>
       </c>
       <c r="C87" s="10">
-        <v>737449.93857344822</v>
+        <v>735534.38226519676</v>
       </c>
       <c r="D87" s="10">
         <v>776528.77609078528</v>
@@ -7420,10 +7423,24 @@
         <v>31</v>
       </c>
       <c r="C88" s="10">
-        <v>739523.51945228642</v>
-      </c>
-      <c r="D88" s="10">
-        <v>737868.04979272792</v>
+        <v>739903.77331731853</v>
+      </c>
+      <c r="D88">
+        <v>737795.74161343137</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="10">
+        <v>2025</v>
+      </c>
+      <c r="B89" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C89" s="10">
+        <v>744527.7879887321</v>
+      </c>
+      <c r="D89">
+        <v>733788.66978506034</v>
       </c>
     </row>
   </sheetData>
@@ -7444,14 +7461,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="49" t="s">
+      <c r="B1" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49" t="s">
+      <c r="C1" s="47"/>
+      <c r="D1" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="49"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8050,14 +8067,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="49" t="s">
+      <c r="B1" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49" t="s">
+      <c r="C1" s="47"/>
+      <c r="D1" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="49"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8228,390 +8245,390 @@
       <c r="A2" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="47">
-        <v>936.27410860999998</v>
-      </c>
-      <c r="C2" s="47">
-        <v>1076.3037140900001</v>
+      <c r="B2" s="48">
+        <v>2055.8357156299999</v>
+      </c>
+      <c r="C2" s="48">
+        <v>2644.1434920199999</v>
       </c>
       <c r="D2" s="27">
         <f>B2-C2</f>
-        <v>-140.0296054800001</v>
+        <v>-588.30777639000007</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="B3" s="45">
-        <v>650.75628898000002</v>
-      </c>
-      <c r="C3" s="45">
-        <v>943.80559072999995</v>
+      <c r="B3" s="49">
+        <v>1564.1559994900001</v>
+      </c>
+      <c r="C3" s="49">
+        <v>2088.58644116</v>
       </c>
       <c r="D3" s="27">
         <f t="shared" ref="D3:D27" si="0">B3-C3</f>
-        <v>-293.04930174999993</v>
+        <v>-524.43044166999994</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
         <v>217</v>
       </c>
-      <c r="B4" s="45">
-        <v>109.07318960000001</v>
-      </c>
-      <c r="C4" s="45">
-        <v>74.930277520000004</v>
+      <c r="B4" s="49">
+        <v>196.73058093</v>
+      </c>
+      <c r="C4" s="49">
+        <v>470.6189273</v>
       </c>
       <c r="D4" s="27">
         <f t="shared" si="0"/>
-        <v>34.142912080000002</v>
+        <v>-273.88834637000002</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B5" s="45">
-        <v>158.72932526</v>
-      </c>
-      <c r="C5" s="45">
-        <v>56.913766340000002</v>
+      <c r="B5" s="49">
+        <v>265.86702915000001</v>
+      </c>
+      <c r="C5" s="49">
+        <v>84.09820406</v>
       </c>
       <c r="D5" s="27">
         <f t="shared" si="0"/>
-        <v>101.81555892</v>
+        <v>181.76882509000001</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="47">
-        <v>669.28620208999996</v>
-      </c>
-      <c r="C6" s="47">
-        <v>162.97711426000001</v>
+      <c r="B6" s="48">
+        <v>1506.7852195400001</v>
+      </c>
+      <c r="C6" s="48">
+        <v>302.49792280000003</v>
       </c>
       <c r="D6" s="27">
         <f t="shared" si="0"/>
-        <v>506.30908782999995</v>
+        <v>1204.2872967400001</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="45">
-        <v>299.05721779999999</v>
-      </c>
-      <c r="C7" s="45">
-        <v>68.793103239999994</v>
+      <c r="B7" s="49">
+        <v>752.27831757000001</v>
+      </c>
+      <c r="C7" s="49">
+        <v>130.65088157</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" si="0"/>
-        <v>230.26411456</v>
+        <v>621.62743599999999</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="B8" s="45">
-        <v>218.94576251000001</v>
-      </c>
-      <c r="C8" s="45">
-        <v>30.344938930000001</v>
+      <c r="B8" s="49">
+        <v>383.64015707999999</v>
+      </c>
+      <c r="C8" s="49">
+        <v>52.942879079999997</v>
       </c>
       <c r="D8" s="27">
         <f t="shared" si="0"/>
-        <v>188.60082358</v>
+        <v>330.69727799999998</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="47">
-        <v>1132.17603093</v>
-      </c>
-      <c r="C9" s="47">
-        <v>614.56651895000005</v>
+      <c r="B9" s="48">
+        <v>1732.70458177</v>
+      </c>
+      <c r="C9" s="48">
+        <v>1207.4340521300001</v>
       </c>
       <c r="D9" s="27">
         <f t="shared" si="0"/>
-        <v>517.60951197999998</v>
+        <v>525.27052963999995</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="32" t="s">
         <v>214</v>
       </c>
-      <c r="B10" s="45">
-        <v>941.11897670999997</v>
-      </c>
-      <c r="C10" s="45">
-        <v>476.35405560999999</v>
+      <c r="B10" s="49">
+        <v>1371.16275774</v>
+      </c>
+      <c r="C10" s="49">
+        <v>893.34532280999997</v>
       </c>
       <c r="D10" s="27">
         <f t="shared" si="0"/>
-        <v>464.76492109999998</v>
+        <v>477.81743492999999</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="B11" s="47">
-        <v>603.67978519999997</v>
-      </c>
-      <c r="C11" s="47">
-        <v>770.61897223999995</v>
+      <c r="B11" s="48">
+        <v>1203.6026445499999</v>
+      </c>
+      <c r="C11" s="48">
+        <v>1426.6886535399999</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" si="0"/>
-        <v>-166.93918703999998</v>
+        <v>-223.08600898999998</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="32" t="s">
         <v>221</v>
       </c>
-      <c r="B12" s="45">
-        <v>100.13218195</v>
-      </c>
-      <c r="C12" s="45">
-        <v>240.88989505999999</v>
+      <c r="B12" s="49">
+        <v>186.15408069</v>
+      </c>
+      <c r="C12" s="49">
+        <v>410.40748841999999</v>
       </c>
       <c r="D12" s="27">
         <f t="shared" si="0"/>
-        <v>-140.75771311</v>
+        <v>-224.25340772999999</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="32" t="s">
         <v>222</v>
       </c>
-      <c r="B13" s="45">
-        <v>97.572028630000005</v>
-      </c>
-      <c r="C13" s="45">
-        <v>103.3571518</v>
+      <c r="B13" s="49">
+        <v>168.55518856</v>
+      </c>
+      <c r="C13" s="49">
+        <v>177.82558041999999</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>-5.7851231699999914</v>
+        <v>-9.2703918599999895</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="B14" s="45">
-        <v>78.72847797</v>
-      </c>
-      <c r="C14" s="45">
-        <v>128.12472002999999</v>
+      <c r="B14" s="49">
+        <v>141.62651867</v>
+      </c>
+      <c r="C14" s="49">
+        <v>227.27655566999999</v>
       </c>
       <c r="D14" s="27">
         <f t="shared" si="0"/>
-        <v>-49.396242059999992</v>
+        <v>-85.650036999999998</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="B15" s="45">
-        <v>117.57978384</v>
-      </c>
-      <c r="C15" s="45">
-        <v>29.658874579999999</v>
+      <c r="B15" s="49">
+        <v>234.33700390999999</v>
+      </c>
+      <c r="C15" s="49">
+        <v>43.005741749999999</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>87.920909260000002</v>
+        <v>191.33126215999999</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="B16" s="47">
-        <v>414.42415140000003</v>
-      </c>
-      <c r="C16" s="47">
-        <v>1436.0215764300001</v>
+      <c r="B16" s="48">
+        <v>1071.0758428199999</v>
+      </c>
+      <c r="C16" s="48">
+        <v>2707.4913193900002</v>
       </c>
       <c r="D16" s="27">
         <f t="shared" si="0"/>
-        <v>-1021.5974250300001</v>
+        <v>-1636.4154765700002</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="B17" s="47">
-        <v>422.07484118999997</v>
-      </c>
-      <c r="C17" s="47">
-        <v>90.872460450000005</v>
+      <c r="B17" s="48">
+        <v>817.57811244000004</v>
+      </c>
+      <c r="C17" s="48">
+        <v>178.81806847999999</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>331.20238073999997</v>
+        <v>638.76004396000008</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="47">
-        <v>804.18947652999998</v>
-      </c>
-      <c r="C18" s="47">
-        <v>335.62233985</v>
+      <c r="B18" s="48">
+        <v>1304.6751968799999</v>
+      </c>
+      <c r="C18" s="48">
+        <v>687.25814527</v>
       </c>
       <c r="D18" s="27">
         <f t="shared" si="0"/>
-        <v>468.56713667999998</v>
+        <v>617.41705160999993</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="32" t="s">
         <v>216</v>
       </c>
-      <c r="B19" s="45">
-        <v>204.91412288999999</v>
-      </c>
-      <c r="C19" s="45">
-        <v>35.77621276</v>
+      <c r="B19" s="49">
+        <v>335.11905289999999</v>
+      </c>
+      <c r="C19" s="49">
+        <v>76.667375160000006</v>
       </c>
       <c r="D19" s="27">
         <f t="shared" si="0"/>
-        <v>169.13791012999999</v>
+        <v>258.45167773999998</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="32" t="s">
         <v>219</v>
       </c>
-      <c r="B20" s="45">
-        <v>147.75539094000001</v>
-      </c>
-      <c r="C20" s="45">
-        <v>18.419799250000001</v>
+      <c r="B20" s="49">
+        <v>212.96472790000001</v>
+      </c>
+      <c r="C20" s="49">
+        <v>39.044309120000001</v>
       </c>
       <c r="D20" s="27">
         <f t="shared" si="0"/>
-        <v>129.33559169</v>
+        <v>173.92041878000001</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="B21" s="45">
-        <v>115.91342023999999</v>
-      </c>
-      <c r="C21" s="45">
-        <v>153.29953037000001</v>
+      <c r="B21" s="49">
+        <v>160.86447251999999</v>
+      </c>
+      <c r="C21" s="49">
+        <v>341.33399687999997</v>
       </c>
       <c r="D21" s="27">
         <f t="shared" si="0"/>
-        <v>-37.38611013000002</v>
+        <v>-180.46952435999998</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="B22" s="45">
-        <v>291.15369507999998</v>
-      </c>
-      <c r="C22" s="45">
-        <v>97.179907150000005</v>
+      <c r="B22" s="49">
+        <v>538.16199499000004</v>
+      </c>
+      <c r="C22" s="49">
+        <v>176.45890802</v>
       </c>
       <c r="D22" s="27">
         <f t="shared" si="0"/>
-        <v>193.97378792999996</v>
+        <v>361.70308697000007</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="47">
-        <v>556.74258235000002</v>
-      </c>
-      <c r="C23" s="47">
-        <v>24.729357950000001</v>
+      <c r="B23" s="48">
+        <v>806.12336928000002</v>
+      </c>
+      <c r="C23" s="48">
+        <v>37.451314670000002</v>
       </c>
       <c r="D23" s="27">
         <f t="shared" si="0"/>
-        <v>532.01322440000001</v>
+        <v>768.67205461000003</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="B24" s="47">
-        <v>347.18862567999997</v>
-      </c>
-      <c r="C24" s="47">
-        <v>24.756080520000001</v>
+      <c r="B24" s="48">
+        <v>586.03007229000002</v>
+      </c>
+      <c r="C24" s="48">
+        <v>41.090413150000003</v>
       </c>
       <c r="D24" s="27">
         <f t="shared" si="0"/>
-        <v>322.43254515999996</v>
+        <v>544.93965914</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="47">
-        <v>42.086978520000002</v>
-      </c>
-      <c r="C25" s="47">
-        <v>10.31719768</v>
+      <c r="B25" s="48">
+        <v>75.301730789999993</v>
+      </c>
+      <c r="C25" s="48">
+        <v>33.193095450000001</v>
       </c>
       <c r="D25" s="27">
         <f t="shared" si="0"/>
-        <v>31.769780840000003</v>
+        <v>42.108635339999992</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="47">
-        <v>66.496588680000002</v>
-      </c>
-      <c r="C26" s="47">
-        <v>34.240716859999999</v>
+      <c r="B26" s="48">
+        <v>170.99937065</v>
+      </c>
+      <c r="C26" s="48">
+        <v>44.496689160000003</v>
       </c>
       <c r="D26" s="27">
         <f t="shared" si="0"/>
-        <v>32.255871820000003</v>
+        <v>126.50268149</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="B27" s="48">
-        <v>1062.6406108799999</v>
-      </c>
-      <c r="C27" s="48">
-        <v>489.26552715000003</v>
+      <c r="B27" s="50">
+        <v>1876.8735020900001</v>
+      </c>
+      <c r="C27" s="50">
+        <v>920.36887134000006</v>
       </c>
       <c r="D27" s="27">
         <f t="shared" si="0"/>
-        <v>573.37508372999991</v>
+        <v>956.50463075000005</v>
       </c>
     </row>
   </sheetData>
@@ -8641,7 +8658,7 @@
         <v>181</v>
       </c>
       <c r="B2" s="43">
-        <v>7057.2599820599999</v>
+        <v>13207.585358730001</v>
       </c>
       <c r="D2" s="29"/>
     </row>
@@ -8650,7 +8667,7 @@
         <v>177</v>
       </c>
       <c r="B3" s="43">
-        <v>2056.55148452</v>
+        <v>3838.3825559400002</v>
       </c>
       <c r="D3" s="29"/>
     </row>
@@ -8659,7 +8676,7 @@
         <v>130</v>
       </c>
       <c r="B4" s="44">
-        <v>2.9708269999999999</v>
+        <v>4.3860492899999999</v>
       </c>
       <c r="D4" s="30"/>
     </row>
@@ -8668,7 +8685,7 @@
         <v>131</v>
       </c>
       <c r="B5" s="44">
-        <v>158.99370970000001</v>
+        <v>358.34224784999998</v>
       </c>
       <c r="D5" s="30"/>
     </row>
@@ -8677,7 +8694,7 @@
         <v>132</v>
       </c>
       <c r="B6" s="44">
-        <v>13.966239590000001</v>
+        <v>34.741751530000002</v>
       </c>
       <c r="D6" s="30"/>
     </row>
@@ -8686,7 +8703,7 @@
         <v>133</v>
       </c>
       <c r="B7" s="44">
-        <v>77.170994999999991</v>
+        <v>143.80485421</v>
       </c>
       <c r="D7" s="30"/>
     </row>
@@ -8695,7 +8712,7 @@
         <v>134</v>
       </c>
       <c r="B8" s="44">
-        <v>27.232516050000001</v>
+        <v>78.934716230000006</v>
       </c>
       <c r="D8" s="30"/>
     </row>
@@ -8704,7 +8721,7 @@
         <v>135</v>
       </c>
       <c r="B9" s="44">
-        <v>1450.6090971399999</v>
+        <v>2488.1987099299999</v>
       </c>
       <c r="D9" s="30"/>
     </row>
@@ -8713,7 +8730,7 @@
         <v>136</v>
       </c>
       <c r="B10" s="44">
-        <v>172.96834376000001</v>
+        <v>405.68594094000002</v>
       </c>
       <c r="D10" s="30"/>
     </row>
@@ -8722,7 +8739,7 @@
         <v>137</v>
       </c>
       <c r="B11" s="44">
-        <v>7.6785863699999997</v>
+        <v>27.567491919999998</v>
       </c>
       <c r="D11" s="30"/>
     </row>
@@ -8731,7 +8748,7 @@
         <v>138</v>
       </c>
       <c r="B12" s="44">
-        <v>8.2910350600000005</v>
+        <v>15.39608967</v>
       </c>
       <c r="D12" s="30"/>
     </row>
@@ -8740,7 +8757,7 @@
         <v>139</v>
       </c>
       <c r="B13" s="44">
-        <v>8.6803353199999993</v>
+        <v>18.001209469999999</v>
       </c>
       <c r="D13" s="30"/>
     </row>
@@ -8749,7 +8766,7 @@
         <v>140</v>
       </c>
       <c r="B14" s="44">
-        <v>100.95532219</v>
+        <v>216.01886056000001</v>
       </c>
       <c r="D14" s="30"/>
     </row>
@@ -8758,7 +8775,7 @@
         <v>141</v>
       </c>
       <c r="B15" s="44">
-        <v>27.034477339999999</v>
+        <v>47.30463434</v>
       </c>
       <c r="D15" s="30"/>
     </row>
@@ -8767,7 +8784,7 @@
         <v>178</v>
       </c>
       <c r="B16" s="43">
-        <v>2280.59335874</v>
+        <v>4108.9096855199996</v>
       </c>
       <c r="D16" s="29"/>
     </row>
@@ -8776,7 +8793,7 @@
         <v>142</v>
       </c>
       <c r="B17" s="44">
-        <v>383.31608292999999</v>
+        <v>743.04116016</v>
       </c>
       <c r="D17" s="30"/>
     </row>
@@ -8785,7 +8802,7 @@
         <v>143</v>
       </c>
       <c r="B18" s="44">
-        <v>20.354449949999999</v>
+        <v>39.849933989999997</v>
       </c>
       <c r="D18" s="30"/>
     </row>
@@ -8794,7 +8811,7 @@
         <v>144</v>
       </c>
       <c r="B19" s="44">
-        <v>129.75591433</v>
+        <v>237.56029172000001</v>
       </c>
       <c r="D19" s="30"/>
     </row>
@@ -8803,7 +8820,7 @@
         <v>145</v>
       </c>
       <c r="B20" s="44">
-        <v>7.9936328100000003</v>
+        <v>14.170199390000001</v>
       </c>
       <c r="D20" s="30"/>
     </row>
@@ -8812,7 +8829,7 @@
         <v>146</v>
       </c>
       <c r="B21" s="44">
-        <v>5.4211407300000003</v>
+        <v>11.336348060000001</v>
       </c>
       <c r="D21" s="30"/>
     </row>
@@ -8821,7 +8838,7 @@
         <v>147</v>
       </c>
       <c r="B22" s="44">
-        <v>13.86635018</v>
+        <v>26.981322290000001</v>
       </c>
       <c r="D22" s="30"/>
     </row>
@@ -8830,7 +8847,7 @@
         <v>148</v>
       </c>
       <c r="B23" s="44">
-        <v>65.188714099999999</v>
+        <v>120.61129541</v>
       </c>
       <c r="D23" s="30"/>
     </row>
@@ -8839,7 +8856,7 @@
         <v>149</v>
       </c>
       <c r="B24" s="44">
-        <v>690.54856474999997</v>
+        <v>1216.4536875700001</v>
       </c>
       <c r="D24" s="30"/>
     </row>
@@ -8848,7 +8865,7 @@
         <v>150</v>
       </c>
       <c r="B25" s="44">
-        <v>44.376118079999998</v>
+        <v>71.898552679999995</v>
       </c>
       <c r="D25" s="30"/>
     </row>
@@ -8857,7 +8874,7 @@
         <v>151</v>
       </c>
       <c r="B26" s="44">
-        <v>70.995134980000003</v>
+        <v>141.62678188000001</v>
       </c>
       <c r="D26" s="30"/>
     </row>
@@ -8866,7 +8883,7 @@
         <v>152</v>
       </c>
       <c r="B27" s="44">
-        <v>51.462848469999997</v>
+        <v>111.2139683</v>
       </c>
       <c r="D27" s="30"/>
     </row>
@@ -8875,7 +8892,7 @@
         <v>153</v>
       </c>
       <c r="B28" s="44">
-        <v>666.64309023999999</v>
+        <v>1128.21193786</v>
       </c>
       <c r="D28" s="30"/>
     </row>
@@ -8884,7 +8901,7 @@
         <v>154</v>
       </c>
       <c r="B29" s="44">
-        <v>23.963101810000001</v>
+        <v>47.049963599999998</v>
       </c>
       <c r="D29" s="30"/>
     </row>
@@ -8893,7 +8910,7 @@
         <v>155</v>
       </c>
       <c r="B30" s="44">
-        <v>26.787494339999999</v>
+        <v>50.140863359999997</v>
       </c>
       <c r="D30" s="30"/>
     </row>
@@ -8902,7 +8919,7 @@
         <v>156</v>
       </c>
       <c r="B31" s="44">
-        <v>9.2576955699999992</v>
+        <v>18.130049110000002</v>
       </c>
       <c r="D31" s="30"/>
     </row>
@@ -8911,7 +8928,7 @@
         <v>157</v>
       </c>
       <c r="B32" s="44">
-        <v>70.663025469999994</v>
+        <v>130.63333014</v>
       </c>
       <c r="D32" s="30"/>
     </row>
@@ -8920,7 +8937,7 @@
         <v>179</v>
       </c>
       <c r="B33" s="43">
-        <v>1938.9244339899999</v>
+        <v>3697.3168202500001</v>
       </c>
       <c r="D33" s="29"/>
     </row>
@@ -8929,7 +8946,7 @@
         <v>158</v>
       </c>
       <c r="B34" s="44">
-        <v>378.24464881</v>
+        <v>849.9980276</v>
       </c>
       <c r="D34" s="30"/>
     </row>
@@ -8938,7 +8955,7 @@
         <v>159</v>
       </c>
       <c r="B35" s="44">
-        <v>80.583972500000002</v>
+        <v>155.27257409000001</v>
       </c>
       <c r="D35" s="30"/>
     </row>
@@ -8947,7 +8964,7 @@
         <v>160</v>
       </c>
       <c r="B36" s="44">
-        <v>14.423540320000001</v>
+        <v>25.470443889999999</v>
       </c>
       <c r="D36" s="30"/>
     </row>
@@ -8956,7 +8973,7 @@
         <v>161</v>
       </c>
       <c r="B37" s="44">
-        <v>1.62437415</v>
+        <v>2.7287990299999998</v>
       </c>
       <c r="D37" s="30"/>
     </row>
@@ -8965,7 +8982,7 @@
         <v>162</v>
       </c>
       <c r="B38" s="44">
-        <v>34.611767479999997</v>
+        <v>67.649627609999996</v>
       </c>
       <c r="D38" s="30"/>
     </row>
@@ -8974,7 +8991,7 @@
         <v>163</v>
       </c>
       <c r="B39" s="44">
-        <v>8.4366099699999992</v>
+        <v>16.198883989999999</v>
       </c>
       <c r="D39" s="30"/>
     </row>
@@ -8983,7 +9000,7 @@
         <v>164</v>
       </c>
       <c r="B40" s="44">
-        <v>0.92599301000000001</v>
+        <v>1.43051251</v>
       </c>
       <c r="D40" s="30"/>
     </row>
@@ -8992,7 +9009,7 @@
         <v>165</v>
       </c>
       <c r="B41" s="44">
-        <v>9.2802341500000001</v>
+        <v>19.168406239999999</v>
       </c>
       <c r="D41" s="30"/>
     </row>
@@ -9001,7 +9018,7 @@
         <v>166</v>
       </c>
       <c r="B42" s="44">
-        <v>583.58031032999997</v>
+        <v>1053.352331</v>
       </c>
       <c r="D42" s="30"/>
     </row>
@@ -9010,7 +9027,7 @@
         <v>167</v>
       </c>
       <c r="B43" s="44">
-        <v>219.88986378000001</v>
+        <v>298.25986130000001</v>
       </c>
       <c r="D43" s="30"/>
     </row>
@@ -9019,7 +9036,7 @@
         <v>168</v>
       </c>
       <c r="B44" s="44">
-        <v>96.342121090000006</v>
+        <v>185.25430915000001</v>
       </c>
       <c r="D44" s="30"/>
     </row>
@@ -9028,7 +9045,7 @@
         <v>169</v>
       </c>
       <c r="B45" s="44">
-        <v>274.79163116000001</v>
+        <v>751.51911275999998</v>
       </c>
       <c r="D45" s="30"/>
     </row>
@@ -9037,7 +9054,7 @@
         <v>170</v>
       </c>
       <c r="B46" s="44">
-        <v>21.460628440000001</v>
+        <v>22.685022549999999</v>
       </c>
       <c r="D46" s="30"/>
     </row>
@@ -9046,7 +9063,7 @@
         <v>171</v>
       </c>
       <c r="B47" s="44">
-        <v>214.7287388</v>
+        <v>248.32890853000001</v>
       </c>
       <c r="D47" s="30"/>
     </row>
@@ -9055,7 +9072,7 @@
         <v>180</v>
       </c>
       <c r="B48" s="43">
-        <v>781.19070481000006</v>
+        <v>1562.9762970199999</v>
       </c>
       <c r="D48" s="29"/>
     </row>
@@ -9064,7 +9081,7 @@
         <v>172</v>
       </c>
       <c r="B49" s="44">
-        <v>402.22015691000001</v>
+        <v>849.42092487000002</v>
       </c>
       <c r="D49" s="30"/>
     </row>
@@ -9073,7 +9090,7 @@
         <v>173</v>
       </c>
       <c r="B50" s="44">
-        <v>205.48592647000001</v>
+        <v>380.88709162999999</v>
       </c>
       <c r="D50" s="30"/>
     </row>
@@ -9082,7 +9099,7 @@
         <v>174</v>
       </c>
       <c r="B51" s="44">
-        <v>4.4941127999999999</v>
+        <v>9.4532592100000006</v>
       </c>
       <c r="D51" s="30"/>
     </row>
@@ -9091,7 +9108,7 @@
         <v>175</v>
       </c>
       <c r="B52" s="45">
-        <v>122.18674315</v>
+        <v>237.53615798999999</v>
       </c>
       <c r="D52" s="30"/>
     </row>
@@ -9100,7 +9117,7 @@
         <v>176</v>
       </c>
       <c r="B53" s="46">
-        <v>46.803765480000003</v>
+        <v>85.678863320000005</v>
       </c>
     </row>
   </sheetData>
@@ -9130,7 +9147,7 @@
         <v>186</v>
       </c>
       <c r="B2" s="29">
-        <v>5070.2915764299996</v>
+        <v>10230.9320374</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -9138,7 +9155,7 @@
         <v>187</v>
       </c>
       <c r="B3" s="29">
-        <v>1088.1157404200001</v>
+        <v>2149.1071075599998</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -9146,7 +9163,7 @@
         <v>188</v>
       </c>
       <c r="B4" s="30">
-        <v>830.04616043999999</v>
+        <v>1626.06836828</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -9154,7 +9171,7 @@
         <v>189</v>
       </c>
       <c r="B5" s="30">
-        <v>103.24359586</v>
+        <v>231.20314798999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -9162,7 +9179,7 @@
         <v>190</v>
       </c>
       <c r="B6" s="30">
-        <v>154.82598411999999</v>
+        <v>291.83559129000002</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -9170,7 +9187,7 @@
         <v>191</v>
       </c>
       <c r="B7" s="29">
-        <v>1495.2751218599999</v>
+        <v>3274.6054727000001</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -9178,7 +9195,7 @@
         <v>192</v>
       </c>
       <c r="B8" s="30">
-        <v>28.576074370000001</v>
+        <v>397.57618968999998</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -9186,7 +9203,7 @@
         <v>193</v>
       </c>
       <c r="B9" s="30">
-        <v>44.326431210000003</v>
+        <v>90.548557709999997</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -9194,7 +9211,7 @@
         <v>194</v>
       </c>
       <c r="B10" s="30">
-        <v>73.95033291</v>
+        <v>151.71123872000001</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -9202,7 +9219,7 @@
         <v>195</v>
       </c>
       <c r="B11" s="30">
-        <v>1178.5225770300001</v>
+        <v>2310.3730725700002</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -9210,7 +9227,7 @@
         <v>196</v>
       </c>
       <c r="B12" s="30">
-        <v>169.89970633999999</v>
+        <v>324.39641401</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -9218,7 +9235,7 @@
         <v>197</v>
       </c>
       <c r="B13" s="29">
-        <v>162.73177154999999</v>
+        <v>294.49078997999999</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -9226,7 +9243,7 @@
         <v>198</v>
       </c>
       <c r="B14" s="30">
-        <v>22.253619669999999</v>
+        <v>36.16919438</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -9234,7 +9251,7 @@
         <v>199</v>
       </c>
       <c r="B15" s="30">
-        <v>140.47815188000001</v>
+        <v>258.32159560000002</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -9242,7 +9259,7 @@
         <v>200</v>
       </c>
       <c r="B16" s="29">
-        <v>890.83407714999998</v>
+        <v>1811.6569512200001</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -9250,7 +9267,7 @@
         <v>201</v>
       </c>
       <c r="B17" s="30">
-        <v>364.49208435999998</v>
+        <v>722.65841826999997</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9258,7 +9275,7 @@
         <v>202</v>
       </c>
       <c r="B18" s="30">
-        <v>65.938425159999994</v>
+        <v>123.39147755</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -9266,7 +9283,7 @@
         <v>203</v>
       </c>
       <c r="B19" s="30">
-        <v>460.40356763</v>
+        <v>965.60705540000004</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -9274,7 +9291,7 @@
         <v>204</v>
       </c>
       <c r="B20" s="29">
-        <v>855.43711072999997</v>
+        <v>1657.2453018199999</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -9282,7 +9299,7 @@
         <v>205</v>
       </c>
       <c r="B21" s="30">
-        <v>74.441761029999995</v>
+        <v>140.91804273</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -9290,7 +9307,7 @@
         <v>206</v>
       </c>
       <c r="B22" s="30">
-        <v>110.66903169</v>
+        <v>206.74287163</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -9298,7 +9315,7 @@
         <v>207</v>
       </c>
       <c r="B23" s="30">
-        <v>69.664696860000006</v>
+        <v>128.47421363000001</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -9306,7 +9323,7 @@
         <v>208</v>
       </c>
       <c r="B24" s="30">
-        <v>98.354433929999999</v>
+        <v>176.62252258999999</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -9314,7 +9331,7 @@
         <v>209</v>
       </c>
       <c r="B25" s="30">
-        <v>235.81053366</v>
+        <v>467.40797422999998</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -9322,7 +9339,7 @@
         <v>210</v>
       </c>
       <c r="B26" s="30">
-        <v>139.80675395</v>
+        <v>264.96412925999999</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -9330,7 +9347,7 @@
         <v>196</v>
       </c>
       <c r="B27" s="30">
-        <v>126.68989961</v>
+        <v>272.11554775000002</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -9338,7 +9355,7 @@
         <v>211</v>
       </c>
       <c r="B28" s="29">
-        <v>483.70625353999998</v>
+        <v>853.95577985</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -9346,7 +9363,7 @@
         <v>182</v>
       </c>
       <c r="B29" s="38">
-        <v>94.191501180000003</v>
+        <v>189.87063427000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
"actualizo dato emae enero26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92C0314-FC8C-41BE-BED4-DD5F6AF8E953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941369A6-41D1-4204-983C-6A5A2F07767E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -994,9 +994,6 @@
     <xf numFmtId="3" fontId="11" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1005,6 +1002,9 @@
     </xf>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -3454,7 +3454,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:D122"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -3484,10 +3484,10 @@
         <v>134.74645041349706</v>
       </c>
       <c r="C2" s="36">
-        <v>147.98565231936306</v>
+        <v>147.98416443521199</v>
       </c>
       <c r="D2" s="36">
-        <v>147.10226693661878</v>
+        <v>147.12594096702841</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3498,10 +3498,10 @@
         <v>134.23236103862521</v>
       </c>
       <c r="C3" s="36">
-        <v>147.0606349800521</v>
+        <v>147.0735309036678</v>
       </c>
       <c r="D3" s="36">
-        <v>146.52566019178045</v>
+        <v>146.54748831828914</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3512,10 +3512,10 @@
         <v>150.0878942366954</v>
       </c>
       <c r="C4" s="36">
-        <v>146.11460983094</v>
+        <v>146.10851463731433</v>
       </c>
       <c r="D4" s="36">
-        <v>145.97647775132208</v>
+        <v>145.99672295993258</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3526,10 +3526,10 @@
         <v>153.25067436662908</v>
       </c>
       <c r="C5" s="36">
-        <v>144.93846889580914</v>
+        <v>144.92921584007314</v>
       </c>
       <c r="D5" s="36">
-        <v>145.48976299838353</v>
+        <v>145.50904554873608</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3540,10 +3540,10 @@
         <v>163.51360808690507</v>
       </c>
       <c r="C6" s="36">
-        <v>144.61035739785015</v>
+        <v>144.60979068880104</v>
       </c>
       <c r="D6" s="36">
-        <v>145.092593948836</v>
+        <v>145.11168805200137</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3554,10 +3554,10 @@
         <v>153.66209524099784</v>
       </c>
       <c r="C7" s="36">
-        <v>144.27838482831481</v>
+        <v>144.28461730121603</v>
       </c>
       <c r="D7" s="36">
-        <v>144.8057480982049</v>
+        <v>144.82538456264692</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3568,10 +3568,10 @@
         <v>143.73110098180126</v>
       </c>
       <c r="C8" s="36">
-        <v>144.45294665379353</v>
+        <v>144.44230222025726</v>
       </c>
       <c r="D8" s="36">
-        <v>144.64144659149576</v>
+        <v>144.6621397657425</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3582,10 +3582,10 @@
         <v>143.6741026486049</v>
       </c>
       <c r="C9" s="36">
-        <v>145.51468699442697</v>
+        <v>145.51658654598589</v>
       </c>
       <c r="D9" s="36">
-        <v>144.60720711888763</v>
+        <v>144.62918087773434</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3596,10 +3596,10 @@
         <v>142.00773744282046</v>
       </c>
       <c r="C10" s="36">
-        <v>144.91042633469948</v>
+        <v>144.91422930495111</v>
       </c>
       <c r="D10" s="36">
-        <v>144.7072726915203</v>
+        <v>144.73037937674931</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3610,10 +3610,10 @@
         <v>141.13686329808141</v>
       </c>
       <c r="C11" s="36">
-        <v>144.97397699515963</v>
+        <v>145.0099426627921</v>
       </c>
       <c r="D11" s="36">
-        <v>144.93793492190531</v>
+        <v>144.96158361546256</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3624,10 +3624,10 @@
         <v>144.93832064073018</v>
       </c>
       <c r="C12" s="36">
-        <v>145.66810806965714</v>
+        <v>145.71579727175728</v>
       </c>
       <c r="D12" s="36">
-        <v>145.28801417462043</v>
+        <v>145.31113330135875</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3638,10 +3638,10 @@
         <v>142.59014516031914</v>
       </c>
       <c r="C13" s="36">
-        <v>147.06310022883548</v>
+        <v>146.9826617165933</v>
       </c>
       <c r="D13" s="36">
-        <v>145.74439481826263</v>
+        <v>145.7658942195805</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3652,10 +3652,10 @@
         <v>136.63265948316217</v>
       </c>
       <c r="C14" s="36">
-        <v>147.27180504104768</v>
+        <v>147.28783054174625</v>
       </c>
       <c r="D14" s="36">
-        <v>146.28941776855942</v>
+        <v>146.30854552394575</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3666,10 +3666,10 @@
         <v>132.15851633982282</v>
       </c>
       <c r="C15" s="36">
-        <v>146.92648244741355</v>
+        <v>146.93413462664321</v>
       </c>
       <c r="D15" s="36">
-        <v>146.90122151947429</v>
+        <v>146.91759868504354</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3680,10 +3680,10 @@
         <v>152.62095855905741</v>
       </c>
       <c r="C16" s="36">
-        <v>147.76638715481141</v>
+        <v>147.75615312299135</v>
       </c>
       <c r="D16" s="36">
-        <v>147.55626001125702</v>
+        <v>147.57012884683868</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3694,10 +3694,10 @@
         <v>151.94634480448744</v>
       </c>
       <c r="C17" s="36">
-        <v>147.65808668666747</v>
+        <v>147.64422761579598</v>
       </c>
       <c r="D17" s="36">
-        <v>148.22949923104082</v>
+        <v>148.24183922410623</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3708,10 +3708,10 @@
         <v>168.3892094693679</v>
       </c>
       <c r="C18" s="36">
-        <v>148.50221834124534</v>
+        <v>148.506517670411</v>
       </c>
       <c r="D18" s="36">
-        <v>148.89054036244306</v>
+        <v>148.90276577033757</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3722,10 +3722,10 @@
         <v>161.03568546945243</v>
       </c>
       <c r="C19" s="36">
-        <v>150.16642701678867</v>
+        <v>150.16406696867037</v>
       </c>
       <c r="D19" s="36">
-        <v>149.50579969832361</v>
+        <v>149.51953400295426</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3736,10 +3736,10 @@
         <v>150.3060501239201</v>
       </c>
       <c r="C20" s="36">
-        <v>150.4306782326756</v>
+        <v>150.41944165359786</v>
       </c>
       <c r="D20" s="36">
-        <v>150.03989571220691</v>
+        <v>150.05662690671261</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3750,10 +3750,10 @@
         <v>149.25534277384119</v>
       </c>
       <c r="C21" s="36">
-        <v>150.4502680720656</v>
+        <v>150.44302122832045</v>
       </c>
       <c r="D21" s="36">
-        <v>150.45766319857549</v>
+        <v>150.4783661838681</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3764,10 +3764,10 @@
         <v>146.38655965775396</v>
       </c>
       <c r="C22" s="36">
-        <v>151.21639137002231</v>
+        <v>151.22418367580548</v>
       </c>
       <c r="D22" s="36">
-        <v>150.72633931610724</v>
+        <v>150.75111225813859</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3778,10 +3778,10 @@
         <v>149.38594966601465</v>
       </c>
       <c r="C23" s="36">
-        <v>151.71479321242282</v>
+        <v>151.758219009497</v>
       </c>
       <c r="D23" s="36">
-        <v>150.82163519816061</v>
+        <v>150.84979048866137</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3792,10 +3792,10 @@
         <v>151.92604285202702</v>
       </c>
       <c r="C24" s="36">
-        <v>152.52037968344413</v>
+        <v>152.57421307554173</v>
       </c>
       <c r="D24" s="36">
-        <v>150.72432777361735</v>
+        <v>150.75430898737324</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3806,10 +3806,10 @@
         <v>146.78338490922457</v>
       </c>
       <c r="C25" s="36">
-        <v>152.20278682195942</v>
+        <v>152.11469489125977</v>
       </c>
       <c r="D25" s="36">
-        <v>150.42670927736398</v>
+        <v>150.4567340837346</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3820,10 +3820,10 @@
         <v>142.74091260617232</v>
       </c>
       <c r="C26" s="36">
-        <v>150.70497030143636</v>
+        <v>150.73526012195717</v>
       </c>
       <c r="D26" s="36">
-        <v>149.93719930253161</v>
+        <v>149.96567876832358</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3834,10 +3834,10 @@
         <v>138.81804035165752</v>
       </c>
       <c r="C27" s="36">
-        <v>151.89592692838517</v>
+        <v>151.90328057084443</v>
       </c>
       <c r="D27" s="36">
-        <v>149.27881762261703</v>
+        <v>149.30435008530588</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3848,10 +3848,10 @@
         <v>155.85731953576982</v>
       </c>
       <c r="C28" s="36">
-        <v>151.35486205273259</v>
+        <v>151.33512477508165</v>
       </c>
       <c r="D28" s="36">
-        <v>148.48706016801756</v>
+        <v>148.50864233651453</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3862,10 +3862,10 @@
         <v>151.52454398394349</v>
       </c>
       <c r="C29" s="36">
-        <v>146.84017770222033</v>
+        <v>146.83545544273494</v>
       </c>
       <c r="D29" s="36">
-        <v>147.60596969693657</v>
+        <v>147.62333168581083</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3876,10 +3876,10 @@
         <v>159.56669237791675</v>
       </c>
       <c r="C30" s="36">
-        <v>144.74513301972749</v>
+        <v>144.73606068174158</v>
       </c>
       <c r="D30" s="36">
-        <v>146.68643140915174</v>
+        <v>146.69981092291601</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3890,10 +3890,10 @@
         <v>151.1257632334553</v>
       </c>
       <c r="C31" s="36">
-        <v>143.4397973151531</v>
+        <v>143.43435071467957</v>
       </c>
       <c r="D31" s="36">
-        <v>145.78147715447952</v>
+        <v>145.79150750165263</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -3904,10 +3904,10 @@
         <v>145.9635244300047</v>
       </c>
       <c r="C32" s="36">
-        <v>143.87003314549</v>
+        <v>143.8593540054695</v>
       </c>
       <c r="D32" s="36">
-        <v>144.94014208130514</v>
+        <v>144.94779112366157</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3918,10 +3918,10 @@
         <v>146.76596003413977</v>
       </c>
       <c r="C33" s="36">
-        <v>146.68494289698566</v>
+        <v>146.6868146054301</v>
       </c>
       <c r="D33" s="36">
-        <v>144.20703284367139</v>
+        <v>144.21330657798896</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -3932,10 +3932,10 @@
         <v>137.74656971864809</v>
       </c>
       <c r="C34" s="36">
-        <v>143.22938772747611</v>
+        <v>143.21638592657462</v>
       </c>
       <c r="D34" s="36">
-        <v>143.61304042591726</v>
+        <v>143.6187013418222</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3946,10 +3946,10 @@
         <v>142.84327598456773</v>
       </c>
       <c r="C35" s="36">
-        <v>143.43940727925798</v>
+        <v>143.46264585114906</v>
       </c>
       <c r="D35" s="36">
-        <v>143.17215190761056</v>
+        <v>143.17761282979643</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -3960,10 +3960,10 @@
         <v>140.59240732533573</v>
       </c>
       <c r="C36" s="36">
-        <v>141.57478839535472</v>
+        <v>141.5857201570667</v>
       </c>
       <c r="D36" s="36">
-        <v>142.88558211426778</v>
+        <v>142.8909948083799</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -3974,10 +3974,10 @@
         <v>136.25161596905645</v>
       </c>
       <c r="C37" s="36">
-        <v>142.01719875961422</v>
+        <v>142.00617267082225</v>
       </c>
       <c r="D37" s="36">
-        <v>142.74164624253009</v>
+        <v>142.74711270118166</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -3988,10 +3988,10 @@
         <v>134.53623985669589</v>
       </c>
       <c r="C38" s="36">
-        <v>141.77247294316507</v>
+        <v>141.79432368279794</v>
       </c>
       <c r="D38" s="36">
-        <v>142.71398469689075</v>
+        <v>142.71947890740492</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4002,10 +4002,10 @@
         <v>132.2678886127367</v>
       </c>
       <c r="C39" s="36">
-        <v>144.15295347345267</v>
+        <v>144.15550670865235</v>
       </c>
       <c r="D39" s="36">
-        <v>142.76516293583052</v>
+        <v>142.77094533098327</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4016,10 +4016,10 @@
         <v>144.96325495574922</v>
       </c>
       <c r="C40" s="36">
-        <v>142.60326134847173</v>
+        <v>142.59443805924374</v>
       </c>
       <c r="D40" s="36">
-        <v>142.85600117098957</v>
+        <v>142.86225149941299</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4030,10 +4030,10 @@
         <v>149.9162214035228</v>
       </c>
       <c r="C41" s="36">
-        <v>142.60072395871825</v>
+        <v>142.60231019450458</v>
       </c>
       <c r="D41" s="36">
-        <v>142.94487748131402</v>
+        <v>142.95153273177766</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4044,10 +4044,10 @@
         <v>164.13569907592046</v>
       </c>
       <c r="C42" s="36">
-        <v>144.61887520451666</v>
+        <v>144.6132395614579</v>
       </c>
       <c r="D42" s="36">
-        <v>142.9943822997449</v>
+        <v>143.00113542926778</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4058,10 +4058,10 @@
         <v>150.85897174113131</v>
       </c>
       <c r="C43" s="36">
-        <v>143.7462781420308</v>
+        <v>143.72744711431142</v>
       </c>
       <c r="D43" s="36">
-        <v>142.97194493326145</v>
+        <v>142.97836557235004</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4072,10 +4072,10 @@
         <v>146.77702964007042</v>
       </c>
       <c r="C44" s="36">
-        <v>145.55429967455612</v>
+        <v>145.55248976350893</v>
       </c>
       <c r="D44" s="36">
-        <v>142.8510332193604</v>
+        <v>142.85657834248337</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4086,10 +4086,10 @@
         <v>141.27693468084041</v>
       </c>
       <c r="C45" s="36">
-        <v>144.63578980785942</v>
+        <v>144.6185374108843</v>
       </c>
       <c r="D45" s="36">
-        <v>142.61493732207171</v>
+        <v>142.61906386804452</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4100,10 +4100,10 @@
         <v>134.87706647993659</v>
       </c>
       <c r="C46" s="36">
-        <v>140.4627721847196</v>
+        <v>140.45106888843378</v>
       </c>
       <c r="D46" s="36">
-        <v>142.25730921810464</v>
+        <v>142.25955618378433</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -4114,10 +4114,10 @@
         <v>141.63933661701387</v>
       </c>
       <c r="C47" s="36">
-        <v>143.72560878687943</v>
+        <v>143.74226390099199</v>
       </c>
       <c r="D47" s="36">
-        <v>141.78179696601291</v>
+        <v>141.78183838434097</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -4128,10 +4128,10 @@
         <v>137.77182966933154</v>
       </c>
       <c r="C48" s="36">
-        <v>140.81426938873403</v>
+        <v>140.82638022720951</v>
       </c>
       <c r="D48" s="36">
-        <v>141.2022371231624</v>
+        <v>141.19987367454414</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4142,10 +4142,10 @@
         <v>135.7651545276351</v>
       </c>
       <c r="C49" s="36">
-        <v>140.09832232120701</v>
+        <v>140.10762172203482</v>
       </c>
       <c r="D49" s="36">
-        <v>140.54325906623276</v>
+        <v>140.53870161865993</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -4156,10 +4156,10 @@
         <v>133.89108608957252</v>
       </c>
       <c r="C50" s="36">
-        <v>140.57610652652261</v>
+        <v>140.6036798183564</v>
       </c>
       <c r="D50" s="36">
-        <v>139.83382759371713</v>
+        <v>139.82772013200128</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -4170,10 +4170,10 @@
         <v>128.97363874659834</v>
       </c>
       <c r="C51" s="36">
-        <v>139.35087605981357</v>
+        <v>139.35074093412922</v>
       </c>
       <c r="D51" s="36">
-        <v>139.1074344313368</v>
+        <v>139.10085474883599</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -4184,10 +4184,10 @@
         <v>128.21106074025664</v>
       </c>
       <c r="C52" s="36">
-        <v>125.98411164237771</v>
+        <v>125.97316204831111</v>
       </c>
       <c r="D52" s="36">
-        <v>138.39978288630601</v>
+        <v>138.39412945530478</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -4198,10 +4198,10 @@
         <v>113.29503444580129</v>
       </c>
       <c r="C53" s="36">
-        <v>106.1832465160599</v>
+        <v>106.18032476382055</v>
       </c>
       <c r="D53" s="36">
-        <v>137.74746485856258</v>
+        <v>137.74419083130718</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -4212,10 +4212,10 @@
         <v>131.02956919734908</v>
       </c>
       <c r="C54" s="36">
-        <v>117.58476119194647</v>
+        <v>117.56499589517145</v>
       </c>
       <c r="D54" s="36">
-        <v>137.18555622740527</v>
+        <v>137.18583559564087</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -4226,10 +4226,10 @@
         <v>132.52196526648828</v>
       </c>
       <c r="C55" s="36">
-        <v>124.72243664639063</v>
+        <v>124.71912720009033</v>
       </c>
       <c r="D55" s="36">
-        <v>136.74288112201</v>
+        <v>136.74753207589245</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -4240,10 +4240,10 @@
         <v>127.46368946979557</v>
       </c>
       <c r="C56" s="36">
-        <v>126.26814413288902</v>
+        <v>126.26766306255661</v>
       </c>
       <c r="D56" s="36">
-        <v>136.44033585735122</v>
+        <v>136.44960639816946</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -4254,10 +4254,10 @@
         <v>125.18389375984724</v>
       </c>
       <c r="C57" s="36">
-        <v>128.88427192913926</v>
+        <v>128.86297264851027</v>
       </c>
       <c r="D57" s="36">
-        <v>136.29190792850508</v>
+        <v>136.30545816098535</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -4268,10 +4268,10 @@
         <v>127.17507609335082</v>
       </c>
       <c r="C58" s="36">
-        <v>130.70780259882406</v>
+        <v>130.69181304546765</v>
       </c>
       <c r="D58" s="36">
-        <v>136.30090374918049</v>
+        <v>136.31800121280813</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -4282,10 +4282,10 @@
         <v>131.34550189452142</v>
       </c>
       <c r="C59" s="36">
-        <v>133.25227237007618</v>
+        <v>133.26525897935591</v>
       </c>
       <c r="D59" s="36">
-        <v>136.46264215825943</v>
+        <v>136.48223855035084</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -4296,10 +4296,10 @@
         <v>132.06865525299401</v>
       </c>
       <c r="C60" s="36">
-        <v>134.68136236486615</v>
+        <v>134.71071040246167</v>
       </c>
       <c r="D60" s="36">
-        <v>136.76266506176555</v>
+        <v>136.78361152018331</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -4310,10 +4310,10 @@
         <v>133.85436559461567</v>
       </c>
       <c r="C61" s="36">
-        <v>136.81814454866745</v>
+        <v>136.82308772906509</v>
       </c>
       <c r="D61" s="36">
-        <v>137.18101614550551</v>
+        <v>137.20224637216864</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -4324,10 +4324,10 @@
         <v>131.52153739734899</v>
       </c>
       <c r="C62" s="36">
-        <v>139.61902323053997</v>
+        <v>139.63894578986631</v>
       </c>
       <c r="D62" s="36">
-        <v>137.69673254587158</v>
+        <v>137.71736457026788</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -4338,10 +4338,10 @@
         <v>126.2392669683769</v>
       </c>
       <c r="C63" s="36">
-        <v>138.09347901414276</v>
+        <v>138.09511409430371</v>
       </c>
       <c r="D63" s="36">
-        <v>138.29394853992895</v>
+        <v>138.31354130774039</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -4352,10 +4352,10 @@
         <v>145.95690010360465</v>
       </c>
       <c r="C64" s="36">
-        <v>141.03910751615138</v>
+        <v>141.03398403621657</v>
       </c>
       <c r="D64" s="36">
-        <v>138.96185876230584</v>
+        <v>138.97963431850297</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -4366,10 +4366,10 @@
         <v>147.28084401862384</v>
       </c>
       <c r="C65" s="36">
-        <v>139.46424638264449</v>
+        <v>139.45903788617423</v>
       </c>
       <c r="D65" s="36">
-        <v>139.69371868628528</v>
+        <v>139.70889552256895</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -4380,10 +4380,10 @@
         <v>151.16932233869107</v>
       </c>
       <c r="C66" s="36">
-        <v>138.99016198991799</v>
+        <v>138.97237834209403</v>
       </c>
       <c r="D66" s="36">
-        <v>140.4868358387069</v>
+        <v>140.49863799043612</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -4394,10 +4394,10 @@
         <v>148.97961710860557</v>
       </c>
       <c r="C67" s="36">
-        <v>141.52106671218871</v>
+        <v>141.52841212917215</v>
       </c>
       <c r="D67" s="36">
-        <v>141.33771815514032</v>
+        <v>141.34543253573938</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -4405,13 +4405,13 @@
         <v>44378</v>
       </c>
       <c r="B68" s="17">
-        <v>142.42591306097333</v>
+        <v>142.42591306097327</v>
       </c>
       <c r="C68" s="36">
-        <v>141.35886000493807</v>
+        <v>141.34508748860509</v>
       </c>
       <c r="D68" s="36">
-        <v>142.24716223716493</v>
+        <v>142.25037642214357</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -4422,10 +4422,10 @@
         <v>140.9749407280367</v>
       </c>
       <c r="C69" s="36">
-        <v>143.26923602769929</v>
+        <v>143.24815928365717</v>
       </c>
       <c r="D69" s="36">
-        <v>143.21623712158012</v>
+        <v>143.21506248206509</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -4433,13 +4433,13 @@
         <v>44440</v>
       </c>
       <c r="B70" s="17">
-        <v>141.29608908940978</v>
+        <v>141.2960890894098</v>
       </c>
       <c r="C70" s="36">
-        <v>144.0368021137991</v>
+        <v>144.02680631022127</v>
       </c>
       <c r="D70" s="36">
-        <v>144.23922266173949</v>
+        <v>144.2342680385934</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -4447,13 +4447,13 @@
         <v>44470</v>
       </c>
       <c r="B71" s="17">
-        <v>139.51475869689301</v>
+        <v>139.51475869689307</v>
       </c>
       <c r="C71" s="36">
-        <v>143.31697692936714</v>
+        <v>143.34148953752734</v>
       </c>
       <c r="D71" s="36">
-        <v>145.30407282411397</v>
+        <v>145.29648583611456</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -4461,13 +4461,13 @@
         <v>44501</v>
       </c>
       <c r="B72" s="17">
-        <v>143.75187761771426</v>
+        <v>143.75187761771429</v>
       </c>
       <c r="C72" s="36">
-        <v>145.8290703588618</v>
+        <v>145.88334396965624</v>
       </c>
       <c r="D72" s="36">
-        <v>146.38659975145896</v>
+        <v>146.37775470607781</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -4475,13 +4475,13 @@
         <v>44531</v>
       </c>
       <c r="B73" s="17">
-        <v>147.22987832209449</v>
+        <v>147.22987832209441</v>
       </c>
       <c r="C73" s="36">
-        <v>149.80291514399599</v>
+        <v>149.76818655647341</v>
       </c>
       <c r="D73" s="36">
-        <v>147.45002634916275</v>
+        <v>147.44135970192912</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -4489,13 +4489,13 @@
         <v>44562</v>
       </c>
       <c r="B74" s="17">
-        <v>139.63796162490004</v>
+        <v>139.63796162489982</v>
       </c>
       <c r="C74" s="36">
-        <v>148.41357071668713</v>
+        <v>148.43728728335583</v>
       </c>
       <c r="D74" s="36">
-        <v>148.45136367214639</v>
+        <v>148.44426449318115</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -4503,13 +4503,13 @@
         <v>44593</v>
       </c>
       <c r="B75" s="17">
-        <v>137.849513530395</v>
+        <v>137.84951353039492</v>
       </c>
       <c r="C75" s="36">
-        <v>150.64216289946913</v>
+        <v>150.63289440752891</v>
       </c>
       <c r="D75" s="36">
-        <v>149.34555610364404</v>
+        <v>149.34108732013675</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -4517,13 +4517,13 @@
         <v>44621</v>
       </c>
       <c r="B76" s="17">
-        <v>153.93085077631517</v>
+        <v>153.93085077631551</v>
       </c>
       <c r="C76" s="36">
-        <v>150.48070700030922</v>
+        <v>150.47159205926275</v>
       </c>
       <c r="D76" s="36">
-        <v>150.09176613492505</v>
+        <v>150.0904916491825</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -4531,13 +4531,13 @@
         <v>44652</v>
       </c>
       <c r="B77" s="17">
-        <v>157.66169211629358</v>
+        <v>157.66169211629463</v>
       </c>
       <c r="C77" s="36">
-        <v>152.00968915217322</v>
+        <v>152.0034071839209</v>
       </c>
       <c r="D77" s="36">
-        <v>150.66184136619867</v>
+        <v>150.66390513843072</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -4545,13 +4545,13 @@
         <v>44682</v>
       </c>
       <c r="B78" s="17">
-        <v>164.68936308999201</v>
+        <v>164.68936308999244</v>
       </c>
       <c r="C78" s="36">
-        <v>152.17393942829094</v>
+        <v>152.16490263017786</v>
       </c>
       <c r="D78" s="36">
-        <v>151.04041258621987</v>
+        <v>151.04562504327819</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -4559,13 +4559,13 @@
         <v>44713</v>
       </c>
       <c r="B79" s="17">
-        <v>161.45483436245846</v>
+        <v>161.45483436245701</v>
       </c>
       <c r="C79" s="36">
-        <v>154.18153206874666</v>
+        <v>154.19077980789419</v>
       </c>
       <c r="D79" s="36">
-        <v>151.22579993660898</v>
+        <v>151.23368190379077</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -4573,13 +4573,13 @@
         <v>44743</v>
       </c>
       <c r="B80" s="17">
-        <v>152.44538769472058</v>
+        <v>152.44538769471595</v>
       </c>
       <c r="C80" s="36">
-        <v>152.47453334212534</v>
+        <v>152.47346331942649</v>
       </c>
       <c r="D80" s="36">
-        <v>151.23244314795454</v>
+        <v>151.24235287224582</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4587,13 +4587,13 @@
         <v>44774</v>
       </c>
       <c r="B81" s="17">
-        <v>151.46573902518026</v>
+        <v>151.46573902517829</v>
       </c>
       <c r="C81" s="36">
-        <v>151.66127370680593</v>
+        <v>151.65743372718188</v>
       </c>
       <c r="D81" s="36">
-        <v>151.0881229409818</v>
+        <v>151.09940874223366</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4601,13 +4601,13 @@
         <v>44805</v>
       </c>
       <c r="B82" s="17">
-        <v>149.17434933730379</v>
+        <v>149.17434933731033</v>
       </c>
       <c r="C82" s="36">
-        <v>150.8093117481032</v>
+        <v>150.7750708473458</v>
       </c>
       <c r="D82" s="36">
-        <v>150.8288767259952</v>
+        <v>150.8408611686215</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4615,13 +4615,13 @@
         <v>44835</v>
       </c>
       <c r="B83" s="17">
-        <v>146.55439498927336</v>
+        <v>146.55439498929425</v>
       </c>
       <c r="C83" s="36">
-        <v>149.23258112206847</v>
+        <v>149.23974308318589</v>
       </c>
       <c r="D83" s="36">
-        <v>150.49379232882674</v>
+        <v>150.50583574647703</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4629,13 +4629,13 @@
         <v>44866</v>
       </c>
       <c r="B84" s="17">
-        <v>148.0304944353044</v>
+        <v>148.03049443531322</v>
       </c>
       <c r="C84" s="36">
-        <v>148.48437616415652</v>
+        <v>148.50749990138871</v>
       </c>
       <c r="D84" s="36">
-        <v>150.11916703714238</v>
+        <v>150.13081034108305</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -4643,13 +4643,13 @@
         <v>44896</v>
       </c>
       <c r="B85" s="17">
-        <v>146.18080800461092</v>
+        <v>146.18080800458125</v>
       </c>
       <c r="C85" s="36">
-        <v>148.51171161009415</v>
+        <v>148.5213147080778</v>
       </c>
       <c r="D85" s="36">
-        <v>149.73698303674897</v>
+        <v>149.74796080882658</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -4657,13 +4657,13 @@
         <v>44927</v>
       </c>
       <c r="B86" s="17">
-        <v>143.03019028689684</v>
+        <v>143.03019028680231</v>
       </c>
       <c r="C86" s="36">
-        <v>149.69384943224711</v>
+        <v>149.69317822957683</v>
       </c>
       <c r="D86" s="36">
-        <v>149.36915378269097</v>
+        <v>149.37939009446657</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4671,13 +4671,13 @@
         <v>44958</v>
       </c>
       <c r="B87" s="17">
-        <v>137.26202711168159</v>
+        <v>137.26202711164171</v>
       </c>
       <c r="C87" s="36">
-        <v>149.65607321238184</v>
+        <v>149.64274747212693</v>
       </c>
       <c r="D87" s="36">
-        <v>149.0262067096653</v>
+        <v>149.03501410197069</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -4685,13 +4685,13 @@
         <v>44986</v>
       </c>
       <c r="B88" s="17">
-        <v>155.06056763764474</v>
+        <v>155.06056763777909</v>
       </c>
       <c r="C88" s="36">
-        <v>150.84064294251075</v>
+        <v>150.83505977466785</v>
       </c>
       <c r="D88" s="36">
-        <v>148.70190523252708</v>
+        <v>148.70890535647786</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -4699,13 +4699,13 @@
         <v>45017</v>
       </c>
       <c r="B89" s="17">
-        <v>150.02108492527952</v>
+        <v>150.02108492570758</v>
       </c>
       <c r="C89" s="36">
-        <v>147.38227763492009</v>
+        <v>147.36470885338534</v>
       </c>
       <c r="D89" s="36">
-        <v>148.37987455016355</v>
+        <v>148.38532978945474</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4713,13 +4713,13 @@
         <v>45047</v>
       </c>
       <c r="B90" s="17">
-        <v>153.7724057047094</v>
+        <v>153.77240570488985</v>
       </c>
       <c r="C90" s="36">
-        <v>145.64450323043363</v>
+        <v>145.67210800721972</v>
       </c>
       <c r="D90" s="36">
-        <v>148.0369899043362</v>
+        <v>148.04175321375715</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4727,13 +4727,13 @@
         <v>45078</v>
       </c>
       <c r="B91" s="17">
-        <v>152.55703188468178</v>
+        <v>152.55703188407324</v>
       </c>
       <c r="C91" s="36">
-        <v>146.29805793736915</v>
+        <v>146.29688511039032</v>
       </c>
       <c r="D91" s="36">
-        <v>147.6525836973035</v>
+        <v>147.65804453750539</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -4741,13 +4741,13 @@
         <v>45108</v>
       </c>
       <c r="B92" s="17">
-        <v>150.22297368979832</v>
+        <v>150.22297368785945</v>
       </c>
       <c r="C92" s="36">
-        <v>148.73208391206597</v>
+        <v>148.75232261473298</v>
       </c>
       <c r="D92" s="36">
-        <v>147.21476937430103</v>
+        <v>147.22280669257339</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -4755,13 +4755,13 @@
         <v>45139</v>
       </c>
       <c r="B93" s="17">
-        <v>151.94203814961483</v>
+        <v>151.94203814879756</v>
       </c>
       <c r="C93" s="36">
-        <v>150.10312383995364</v>
+        <v>150.0926319307934</v>
       </c>
       <c r="D93" s="36">
-        <v>146.72058809932821</v>
+        <v>146.73320547539899</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -4769,13 +4769,13 @@
         <v>45170</v>
       </c>
       <c r="B94" s="17">
-        <v>148.43224326744129</v>
+        <v>148.4322432701974</v>
       </c>
       <c r="C94" s="36">
-        <v>149.60731738090746</v>
+        <v>149.55846428674684</v>
       </c>
       <c r="D94" s="36">
-        <v>146.18069891848586</v>
+        <v>146.19967388150923</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4783,13 +4783,13 @@
         <v>45200</v>
       </c>
       <c r="B95" s="17">
-        <v>147.50696065166397</v>
+        <v>147.50696066044537</v>
       </c>
       <c r="C95" s="36">
-        <v>148.12949905103457</v>
+        <v>148.14029444558713</v>
       </c>
       <c r="D95" s="36">
-        <v>145.61919826344177</v>
+        <v>145.64577732617855</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -4797,13 +4797,13 @@
         <v>45231</v>
       </c>
       <c r="B96" s="17">
-        <v>146.35949532813629</v>
+        <v>146.35949533183793</v>
       </c>
       <c r="C96" s="36">
-        <v>146.49639509016845</v>
+        <v>146.51277382726593</v>
       </c>
       <c r="D96" s="36">
-        <v>145.07027660458857</v>
+        <v>145.10423503691078</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -4811,13 +4811,13 @@
         <v>45261</v>
       </c>
       <c r="B97" s="17">
-        <v>139.33576577766939</v>
+        <v>139.33576576518632</v>
       </c>
       <c r="C97" s="36">
-        <v>142.91896072403381</v>
+        <v>142.94160983525137</v>
       </c>
       <c r="D97" s="36">
-        <v>144.57840813557522</v>
+        <v>144.61838048925998</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -4825,13 +4825,13 @@
         <v>45292</v>
       </c>
       <c r="B98" s="17">
-        <v>137.5460273956858</v>
+        <v>137.54602735591297</v>
       </c>
       <c r="C98" s="36">
-        <v>143.8048130224725</v>
+        <v>143.76883369012882</v>
       </c>
       <c r="D98" s="36">
-        <v>144.19114953173016</v>
+        <v>144.23481395740316</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4839,13 +4839,13 @@
         <v>45323</v>
       </c>
       <c r="B99" s="17">
-        <v>133.63722385882616</v>
+        <v>133.63722384206051</v>
       </c>
       <c r="C99" s="36">
-        <v>143.94365107974818</v>
+        <v>143.89465322280864</v>
       </c>
       <c r="D99" s="36">
-        <v>143.95316685235136</v>
+        <v>143.99752040583331</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4853,13 +4853,13 @@
         <v>45352</v>
       </c>
       <c r="B100" s="17">
-        <v>142.5686204636574</v>
+        <v>142.56862052019582</v>
       </c>
       <c r="C100" s="36">
-        <v>142.80172295472559</v>
+        <v>142.77426190677184</v>
       </c>
       <c r="D100" s="36">
-        <v>143.90155716196381</v>
+        <v>143.9433434259976</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4867,13 +4867,13 @@
         <v>45383</v>
       </c>
       <c r="B101" s="17">
-        <v>147.26512436842066</v>
+        <v>147.26512454856004</v>
       </c>
       <c r="C101" s="36">
-        <v>140.91047867078075</v>
+        <v>140.89793664197632</v>
       </c>
       <c r="D101" s="36">
-        <v>144.05833279235353</v>
+        <v>144.09459659939233</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4881,13 +4881,13 @@
         <v>45413</v>
       </c>
       <c r="B102" s="17">
-        <v>156.7765836855713</v>
+        <v>156.7765837615064</v>
       </c>
       <c r="C102" s="36">
-        <v>142.46056503407371</v>
+        <v>142.51215427525324</v>
       </c>
       <c r="D102" s="36">
-        <v>144.42400245702649</v>
+        <v>144.45245702311871</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4895,13 +4895,13 @@
         <v>45444</v>
       </c>
       <c r="B103" s="17">
-        <v>147.3651696242483</v>
+        <v>147.36516936817381</v>
       </c>
       <c r="C103" s="36">
-        <v>143.63784831454871</v>
+        <v>143.64245592690298</v>
       </c>
       <c r="D103" s="36">
-        <v>144.98130919698767</v>
+        <v>145.00036065680248</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -4909,13 +4909,13 @@
         <v>45474</v>
       </c>
       <c r="B104" s="17">
-        <v>149.69752779125386</v>
+        <v>149.69752697536458</v>
       </c>
       <c r="C104" s="36">
-        <v>147.39198036178112</v>
+        <v>147.44117252611102</v>
       </c>
       <c r="D104" s="36">
-        <v>145.69247130919078</v>
+        <v>145.70198490469494</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -4923,13 +4923,13 @@
         <v>45505</v>
       </c>
       <c r="B105" s="17">
-        <v>147.32757382665579</v>
+        <v>147.32757348272975</v>
       </c>
       <c r="C105" s="36">
-        <v>148.15892003568277</v>
+        <v>148.15608489238346</v>
       </c>
       <c r="D105" s="36">
-        <v>146.50587539534538</v>
+        <v>146.50738235925428</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -4937,13 +4937,13 @@
         <v>45536</v>
       </c>
       <c r="B106" s="17">
-        <v>144.84378186204515</v>
+        <v>144.84378302186047</v>
       </c>
       <c r="C106" s="36">
-        <v>147.97127077921914</v>
+        <v>147.91126702726274</v>
       </c>
       <c r="D106" s="36">
-        <v>147.36492384683075</v>
+        <v>147.36100464411041</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -4951,13 +4951,13 @@
         <v>45566</v>
       </c>
       <c r="B107" s="17">
-        <v>147.99465868829566</v>
+        <v>147.99466238363041</v>
       </c>
       <c r="C107" s="36">
-        <v>148.84493121948327</v>
+        <v>148.87494748794492</v>
       </c>
       <c r="D107" s="36">
-        <v>148.21165580461383</v>
+        <v>148.20558224385911</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -4965,13 +4965,13 @@
         <v>45597</v>
       </c>
       <c r="B108" s="17">
-        <v>148.06937327842638</v>
+        <v>148.06937483613993</v>
       </c>
       <c r="C108" s="36">
-        <v>150.47396476873647</v>
+        <v>150.49590003515124</v>
       </c>
       <c r="D108" s="36">
-        <v>149.000562573357</v>
+        <v>148.99585556290131</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -4979,13 +4979,13 @@
         <v>45627</v>
       </c>
       <c r="B109" s="17">
-        <v>148.56734716216033</v>
+        <v>148.56734190911206</v>
       </c>
       <c r="C109" s="36">
-        <v>151.25886573718373</v>
+        <v>151.28934434546181</v>
       </c>
       <c r="D109" s="36">
-        <v>149.69926988117098</v>
+        <v>149.69917389113817</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -4993,13 +4993,13 @@
         <v>45658</v>
       </c>
       <c r="B110" s="17">
-        <v>146.29581848082546</v>
+        <v>146.29580174387476</v>
       </c>
       <c r="C110" s="36">
-        <v>151.90987559671504</v>
+        <v>151.84835710402444</v>
       </c>
       <c r="D110" s="36">
-        <v>150.29132919043107</v>
+        <v>150.2980988059023</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -5007,13 +5007,13 @@
         <v>45689</v>
       </c>
       <c r="B111" s="17">
-        <v>141.20217650743407</v>
+        <v>141.2021694522208</v>
       </c>
       <c r="C111" s="36">
-        <v>153.23750040470952</v>
+        <v>153.14243736157638</v>
       </c>
       <c r="D111" s="36">
-        <v>150.77569197704591</v>
+        <v>150.79011026457874</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -5021,13 +5021,13 @@
         <v>45717</v>
       </c>
       <c r="B112" s="17">
-        <v>150.40653531756544</v>
+        <v>150.40655910972941</v>
       </c>
       <c r="C112" s="36">
-        <v>150.34594805837466</v>
+        <v>150.32026807591762</v>
       </c>
       <c r="D112" s="36">
-        <v>151.16296602103316</v>
+        <v>151.18446463534534</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -5035,13 +5035,13 @@
         <v>45748</v>
       </c>
       <c r="B113" s="17">
-        <v>158.74102716126998</v>
+        <v>158.74110296645111</v>
       </c>
       <c r="C113" s="36">
-        <v>151.92804205623708</v>
+        <v>151.92898883643196</v>
       </c>
       <c r="D113" s="36">
-        <v>151.47566780434084</v>
+        <v>151.50055430850293</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -5049,13 +5049,13 @@
         <v>45778</v>
       </c>
       <c r="B114" s="17">
-        <v>164.87786600141825</v>
+        <v>164.8778979559678</v>
       </c>
       <c r="C114" s="36">
-        <v>151.60071689216284</v>
+        <v>151.68489734200023</v>
       </c>
       <c r="D114" s="36">
-        <v>151.74177147605752</v>
+        <v>151.76412995400179</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -5063,13 +5063,13 @@
         <v>45809</v>
       </c>
       <c r="B115" s="17">
-        <v>156.59412660913381</v>
+        <v>156.59401884940311</v>
       </c>
       <c r="C115" s="36">
-        <v>151.19579768566436</v>
+        <v>151.24779792587231</v>
       </c>
       <c r="D115" s="36">
-        <v>151.98950085972618</v>
+        <v>152.00191650731665</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -5077,13 +5077,13 @@
         <v>45839</v>
       </c>
       <c r="B116" s="17">
-        <v>153.92340824679954</v>
+        <v>153.90772081429063</v>
       </c>
       <c r="C116" s="36">
-        <v>151.46103596143544</v>
+        <v>151.51469569017755</v>
       </c>
       <c r="D116" s="36">
-        <v>152.24319343111716</v>
+        <v>152.23763361792382</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -5091,13 +5091,13 @@
         <v>45870</v>
       </c>
       <c r="B117" s="17">
-        <v>150.52771937643857</v>
+        <v>150.51256572733467</v>
       </c>
       <c r="C117" s="36">
-        <v>152.53658488531468</v>
+        <v>152.55472207534925</v>
       </c>
       <c r="D117" s="36">
-        <v>152.51976167916609</v>
+        <v>152.48849687213487</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -5105,13 +5105,13 @@
         <v>45901</v>
       </c>
       <c r="B118" s="17">
-        <v>151.85371940111096</v>
+        <v>151.83984439466224</v>
       </c>
       <c r="C118" s="36">
-        <v>153.53890201952643</v>
+        <v>153.4943406678635</v>
       </c>
       <c r="D118" s="36">
-        <v>152.8285919289664</v>
+        <v>152.76457799839011</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -5119,13 +5119,13 @@
         <v>45931</v>
       </c>
       <c r="B119" s="17">
-        <v>152.68993540896943</v>
+        <v>152.59573745863372</v>
       </c>
       <c r="C119" s="36">
-        <v>152.80038570770361</v>
+        <v>152.65435605342799</v>
       </c>
       <c r="D119" s="36">
-        <v>153.17394234767983</v>
+        <v>153.07088380818087</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -5133,27 +5133,41 @@
         <v>45962</v>
       </c>
       <c r="B120" s="17">
-        <v>147.87681054545467</v>
+        <v>147.72352773408562</v>
       </c>
       <c r="C120" s="36">
-        <v>152.68550791321741</v>
+        <v>152.48907642385822</v>
       </c>
       <c r="D120" s="36">
-        <v>153.55434669880731</v>
+        <v>153.41081353041972</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
         <v>45992</v>
       </c>
-      <c r="B121" s="41">
-        <v>153.73541944556123</v>
-      </c>
-      <c r="C121" s="42">
-        <v>155.48426552052715</v>
-      </c>
-      <c r="D121" s="42">
-        <v>153.96730244004959</v>
+      <c r="B121" s="17">
+        <v>153.46285317997496</v>
+      </c>
+      <c r="C121" s="36">
+        <v>155.2798620314735</v>
+      </c>
+      <c r="D121" s="36">
+        <v>153.78425609353792</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="4">
+        <v>46023</v>
+      </c>
+      <c r="B122" s="41">
+        <v>149.04090209242113</v>
+      </c>
+      <c r="C122" s="42">
+        <v>155.93678506834027</v>
+      </c>
+      <c r="D122" s="42">
+        <v>154.19106810873225</v>
       </c>
     </row>
   </sheetData>
@@ -7461,14 +7475,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="47" t="s">
+      <c r="B1" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47" t="s">
+      <c r="C1" s="50"/>
+      <c r="D1" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="47"/>
+      <c r="E1" s="50"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8067,14 +8081,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="47" t="s">
+      <c r="B1" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47" t="s">
+      <c r="C1" s="50"/>
+      <c r="D1" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="47"/>
+      <c r="E1" s="50"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8245,10 +8259,10 @@
       <c r="A2" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="48">
+      <c r="B2" s="47">
         <v>2055.8357156299999</v>
       </c>
-      <c r="C2" s="48">
+      <c r="C2" s="47">
         <v>2644.1434920199999</v>
       </c>
       <c r="D2" s="27">
@@ -8260,10 +8274,10 @@
       <c r="A3" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="B3" s="49">
+      <c r="B3" s="48">
         <v>1564.1559994900001</v>
       </c>
-      <c r="C3" s="49">
+      <c r="C3" s="48">
         <v>2088.58644116</v>
       </c>
       <c r="D3" s="27">
@@ -8275,10 +8289,10 @@
       <c r="A4" s="32" t="s">
         <v>217</v>
       </c>
-      <c r="B4" s="49">
+      <c r="B4" s="48">
         <v>196.73058093</v>
       </c>
-      <c r="C4" s="49">
+      <c r="C4" s="48">
         <v>470.6189273</v>
       </c>
       <c r="D4" s="27">
@@ -8290,10 +8304,10 @@
       <c r="A5" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="B5" s="49">
+      <c r="B5" s="48">
         <v>265.86702915000001</v>
       </c>
-      <c r="C5" s="49">
+      <c r="C5" s="48">
         <v>84.09820406</v>
       </c>
       <c r="D5" s="27">
@@ -8305,10 +8319,10 @@
       <c r="A6" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="48">
+      <c r="B6" s="47">
         <v>1506.7852195400001</v>
       </c>
-      <c r="C6" s="48">
+      <c r="C6" s="47">
         <v>302.49792280000003</v>
       </c>
       <c r="D6" s="27">
@@ -8320,10 +8334,10 @@
       <c r="A7" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="49">
+      <c r="B7" s="48">
         <v>752.27831757000001</v>
       </c>
-      <c r="C7" s="49">
+      <c r="C7" s="48">
         <v>130.65088157</v>
       </c>
       <c r="D7" s="27">
@@ -8335,10 +8349,10 @@
       <c r="A8" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="B8" s="49">
+      <c r="B8" s="48">
         <v>383.64015707999999</v>
       </c>
-      <c r="C8" s="49">
+      <c r="C8" s="48">
         <v>52.942879079999997</v>
       </c>
       <c r="D8" s="27">
@@ -8350,10 +8364,10 @@
       <c r="A9" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="48">
+      <c r="B9" s="47">
         <v>1732.70458177</v>
       </c>
-      <c r="C9" s="48">
+      <c r="C9" s="47">
         <v>1207.4340521300001</v>
       </c>
       <c r="D9" s="27">
@@ -8365,10 +8379,10 @@
       <c r="A10" s="32" t="s">
         <v>214</v>
       </c>
-      <c r="B10" s="49">
+      <c r="B10" s="48">
         <v>1371.16275774</v>
       </c>
-      <c r="C10" s="49">
+      <c r="C10" s="48">
         <v>893.34532280999997</v>
       </c>
       <c r="D10" s="27">
@@ -8380,10 +8394,10 @@
       <c r="A11" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="B11" s="48">
+      <c r="B11" s="47">
         <v>1203.6026445499999</v>
       </c>
-      <c r="C11" s="48">
+      <c r="C11" s="47">
         <v>1426.6886535399999</v>
       </c>
       <c r="D11" s="27">
@@ -8395,10 +8409,10 @@
       <c r="A12" s="32" t="s">
         <v>221</v>
       </c>
-      <c r="B12" s="49">
+      <c r="B12" s="48">
         <v>186.15408069</v>
       </c>
-      <c r="C12" s="49">
+      <c r="C12" s="48">
         <v>410.40748841999999</v>
       </c>
       <c r="D12" s="27">
@@ -8410,10 +8424,10 @@
       <c r="A13" s="32" t="s">
         <v>222</v>
       </c>
-      <c r="B13" s="49">
+      <c r="B13" s="48">
         <v>168.55518856</v>
       </c>
-      <c r="C13" s="49">
+      <c r="C13" s="48">
         <v>177.82558041999999</v>
       </c>
       <c r="D13" s="27">
@@ -8425,10 +8439,10 @@
       <c r="A14" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="B14" s="49">
+      <c r="B14" s="48">
         <v>141.62651867</v>
       </c>
-      <c r="C14" s="49">
+      <c r="C14" s="48">
         <v>227.27655566999999</v>
       </c>
       <c r="D14" s="27">
@@ -8440,10 +8454,10 @@
       <c r="A15" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="B15" s="49">
+      <c r="B15" s="48">
         <v>234.33700390999999</v>
       </c>
-      <c r="C15" s="49">
+      <c r="C15" s="48">
         <v>43.005741749999999</v>
       </c>
       <c r="D15" s="27">
@@ -8455,10 +8469,10 @@
       <c r="A16" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="B16" s="48">
+      <c r="B16" s="47">
         <v>1071.0758428199999</v>
       </c>
-      <c r="C16" s="48">
+      <c r="C16" s="47">
         <v>2707.4913193900002</v>
       </c>
       <c r="D16" s="27">
@@ -8470,10 +8484,10 @@
       <c r="A17" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="B17" s="48">
+      <c r="B17" s="47">
         <v>817.57811244000004</v>
       </c>
-      <c r="C17" s="48">
+      <c r="C17" s="47">
         <v>178.81806847999999</v>
       </c>
       <c r="D17" s="27">
@@ -8485,10 +8499,10 @@
       <c r="A18" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="48">
+      <c r="B18" s="47">
         <v>1304.6751968799999</v>
       </c>
-      <c r="C18" s="48">
+      <c r="C18" s="47">
         <v>687.25814527</v>
       </c>
       <c r="D18" s="27">
@@ -8500,10 +8514,10 @@
       <c r="A19" s="32" t="s">
         <v>216</v>
       </c>
-      <c r="B19" s="49">
+      <c r="B19" s="48">
         <v>335.11905289999999</v>
       </c>
-      <c r="C19" s="49">
+      <c r="C19" s="48">
         <v>76.667375160000006</v>
       </c>
       <c r="D19" s="27">
@@ -8515,10 +8529,10 @@
       <c r="A20" s="32" t="s">
         <v>219</v>
       </c>
-      <c r="B20" s="49">
+      <c r="B20" s="48">
         <v>212.96472790000001</v>
       </c>
-      <c r="C20" s="49">
+      <c r="C20" s="48">
         <v>39.044309120000001</v>
       </c>
       <c r="D20" s="27">
@@ -8530,10 +8544,10 @@
       <c r="A21" s="32" t="s">
         <v>220</v>
       </c>
-      <c r="B21" s="49">
+      <c r="B21" s="48">
         <v>160.86447251999999</v>
       </c>
-      <c r="C21" s="49">
+      <c r="C21" s="48">
         <v>341.33399687999997</v>
       </c>
       <c r="D21" s="27">
@@ -8545,10 +8559,10 @@
       <c r="A22" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="B22" s="49">
+      <c r="B22" s="48">
         <v>538.16199499000004</v>
       </c>
-      <c r="C22" s="49">
+      <c r="C22" s="48">
         <v>176.45890802</v>
       </c>
       <c r="D22" s="27">
@@ -8560,10 +8574,10 @@
       <c r="A23" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="48">
+      <c r="B23" s="47">
         <v>806.12336928000002</v>
       </c>
-      <c r="C23" s="48">
+      <c r="C23" s="47">
         <v>37.451314670000002</v>
       </c>
       <c r="D23" s="27">
@@ -8575,10 +8589,10 @@
       <c r="A24" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="B24" s="48">
+      <c r="B24" s="47">
         <v>586.03007229000002</v>
       </c>
-      <c r="C24" s="48">
+      <c r="C24" s="47">
         <v>41.090413150000003</v>
       </c>
       <c r="D24" s="27">
@@ -8590,10 +8604,10 @@
       <c r="A25" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="48">
+      <c r="B25" s="47">
         <v>75.301730789999993</v>
       </c>
-      <c r="C25" s="48">
+      <c r="C25" s="47">
         <v>33.193095450000001</v>
       </c>
       <c r="D25" s="27">
@@ -8605,10 +8619,10 @@
       <c r="A26" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="48">
+      <c r="B26" s="47">
         <v>170.99937065</v>
       </c>
-      <c r="C26" s="48">
+      <c r="C26" s="47">
         <v>44.496689160000003</v>
       </c>
       <c r="D26" s="27">
@@ -8620,10 +8634,10 @@
       <c r="A27" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="B27" s="50">
+      <c r="B27" s="49">
         <v>1876.8735020900001</v>
       </c>
-      <c r="C27" s="50">
+      <c r="C27" s="49">
         <v>920.36887134000006</v>
       </c>
       <c r="D27" s="27">

</xml_diff>

<commit_message>
"Agrego dato pobreza e indigencia 2dno semestre 2026"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941369A6-41D1-4204-983C-6A5A2F07767E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D681577D-33B3-4500-92B5-0E1640FF3E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -166,12 +166,6 @@
     <t>Partidos del GBA</t>
   </si>
   <si>
-    <t xml:space="preserve">Gran Mendoza </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gran San Juan </t>
-  </si>
-  <si>
     <t>Gran San Luis</t>
   </si>
   <si>
@@ -181,9 +175,6 @@
     <t>Formosa</t>
   </si>
   <si>
-    <t xml:space="preserve">Gran Resistencia </t>
-  </si>
-  <si>
     <t>Posadas</t>
   </si>
   <si>
@@ -202,15 +193,9 @@
     <t>Salta</t>
   </si>
   <si>
-    <t xml:space="preserve">Santiago del Estero - La Banda </t>
-  </si>
-  <si>
     <t>Bahía Blanca - Cerri</t>
   </si>
   <si>
-    <t xml:space="preserve">Concordia </t>
-  </si>
-  <si>
     <t>Gran Córdoba</t>
   </si>
   <si>
@@ -220,9 +205,6 @@
     <t>Gran Rosario</t>
   </si>
   <si>
-    <t xml:space="preserve">Gran Paraná </t>
-  </si>
-  <si>
     <t>Gran Santa Fe</t>
   </si>
   <si>
@@ -235,24 +217,15 @@
     <t>Santa Rosa - Toay</t>
   </si>
   <si>
-    <t xml:space="preserve">San Nicolás - Villa Constitución </t>
-  </si>
-  <si>
     <t>Comodoro Rivadavia - Rada Tilly</t>
   </si>
   <si>
-    <t>Neuquen - Plottier</t>
-  </si>
-  <si>
     <t>Río Gallegos</t>
   </si>
   <si>
     <t>Ushuaia - Río Grande</t>
   </si>
   <si>
-    <t xml:space="preserve">Rawson - Trelew </t>
-  </si>
-  <si>
     <t>Viedma - Carmen de Patagones</t>
   </si>
   <si>
@@ -716,6 +689,33 @@
   </si>
   <si>
     <t xml:space="preserve"> Países Bajos</t>
+  </si>
+  <si>
+    <t>Gran Mendoza</t>
+  </si>
+  <si>
+    <t>Gran San Juan</t>
+  </si>
+  <si>
+    <t>Gran Resistencia</t>
+  </si>
+  <si>
+    <t>Santiago del Estero - La Banda</t>
+  </si>
+  <si>
+    <t>Concordia</t>
+  </si>
+  <si>
+    <t>Gran Paraná</t>
+  </si>
+  <si>
+    <t>San Nicolás - Villa Constitución</t>
+  </si>
+  <si>
+    <t>Neuquén - Plottier</t>
+  </si>
+  <si>
+    <t>Rawson - Trelew</t>
   </si>
 </sst>
 </file>
@@ -3250,18 +3250,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="B2">
         <v>599983.70014805021</v>
@@ -3272,7 +3272,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B3">
         <v>38842.924521107714</v>
@@ -3283,7 +3283,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B4">
         <v>1545.6270924291682</v>
@@ -3294,7 +3294,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="B5">
         <v>30755.076629366038</v>
@@ -3305,7 +3305,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="B6">
         <v>112761.23165011391</v>
@@ -3316,7 +3316,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="B7">
         <v>12673.907286977306</v>
@@ -3327,7 +3327,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B8">
         <v>19017.800104434555</v>
@@ -3338,7 +3338,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="B9">
         <v>91872.245634525272</v>
@@ -3349,7 +3349,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B10">
         <v>13022.400979766842</v>
@@ -3360,7 +3360,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="B11">
         <v>55633.327772916178</v>
@@ -3371,7 +3371,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="B12">
         <v>30381.126773097683</v>
@@ -3382,7 +3382,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="B13">
         <v>85939.774708283672</v>
@@ -3393,7 +3393,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="B14">
         <v>34900.492729780119</v>
@@ -3404,7 +3404,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="B15">
         <v>29912.893832996058</v>
@@ -3415,7 +3415,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="B16">
         <v>23085.607234226565</v>
@@ -3426,7 +3426,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="B17">
         <v>15478.186568411322</v>
@@ -3437,7 +3437,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="B18">
         <v>4161.0766296179845</v>
@@ -3464,16 +3464,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -5186,33 +5186,33 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="B2" s="37">
         <v>1.5</v>
@@ -5238,7 +5238,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="B3" s="37">
         <v>7.2</v>
@@ -5264,7 +5264,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="B4" s="37">
         <v>2.2000000000000002</v>
@@ -5290,7 +5290,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="B5" s="37">
         <v>3.3</v>
@@ -5316,7 +5316,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B6" s="37">
         <v>-0.8</v>
@@ -5342,7 +5342,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B7" s="37">
         <v>-4.5</v>
@@ -5368,7 +5368,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="B8" s="37">
         <v>2.4</v>
@@ -5394,7 +5394,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="B9" s="37">
         <v>1.5</v>
@@ -5420,7 +5420,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="B10" s="37">
         <v>2</v>
@@ -7503,16 +7503,16 @@
         <v>38</v>
       </c>
       <c r="B3">
-        <v>24.1</v>
+        <v>21</v>
       </c>
       <c r="C3">
-        <v>31.6</v>
+        <v>28.2</v>
       </c>
       <c r="D3">
-        <v>5.6</v>
+        <v>4.8</v>
       </c>
       <c r="E3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -7520,16 +7520,16 @@
         <v>39</v>
       </c>
       <c r="B4">
-        <v>11.3</v>
+        <v>7.3</v>
       </c>
       <c r="C4">
-        <v>15.1</v>
+        <v>9.6</v>
       </c>
       <c r="D4">
-        <v>3.3</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E4">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -7537,526 +7537,526 @@
         <v>40</v>
       </c>
       <c r="B5">
-        <v>28.8</v>
+        <v>25.5</v>
       </c>
       <c r="C5">
-        <v>35.299999999999997</v>
+        <v>32.6</v>
       </c>
       <c r="D5">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="E5">
-        <v>8.8000000000000007</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>216</v>
       </c>
       <c r="B6">
-        <v>25.3</v>
+        <v>23.5</v>
       </c>
       <c r="C6">
-        <v>33.5</v>
+        <v>31.9</v>
       </c>
       <c r="D6">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="E6">
-        <v>4.7</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>217</v>
       </c>
       <c r="B7">
-        <v>26.3</v>
+        <v>25.5</v>
       </c>
       <c r="C7">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D7">
-        <v>4.7</v>
+        <v>2.9</v>
       </c>
       <c r="E7">
-        <v>5.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B8">
-        <v>23.1</v>
+        <v>23.2</v>
       </c>
       <c r="C8">
-        <v>30.3</v>
+        <v>30.1</v>
       </c>
       <c r="D8">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E8">
-        <v>2.5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B9">
-        <v>25.4</v>
+        <v>23.5</v>
       </c>
       <c r="C9">
-        <v>37.4</v>
+        <v>31.3</v>
       </c>
       <c r="D9">
-        <v>4.8</v>
+        <v>5.6</v>
       </c>
       <c r="E9">
-        <v>6.5</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B10">
-        <v>24</v>
+        <v>19.7</v>
       </c>
       <c r="C10">
-        <v>28.3</v>
+        <v>27.9</v>
       </c>
       <c r="D10">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="E10">
-        <v>2.7</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>218</v>
       </c>
       <c r="B11">
-        <v>39.1</v>
+        <v>34</v>
       </c>
       <c r="C11">
-        <v>48.1</v>
+        <v>42.2</v>
       </c>
       <c r="D11">
-        <v>12.6</v>
+        <v>10.6</v>
       </c>
       <c r="E11">
-        <v>15.5</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B12">
-        <v>29.8</v>
+        <v>22.2</v>
       </c>
       <c r="C12">
-        <v>38.1</v>
+        <v>27.3</v>
       </c>
       <c r="D12">
-        <v>6.8</v>
+        <v>2.9</v>
       </c>
       <c r="E12">
-        <v>6.8</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B13">
-        <v>26.2</v>
+        <v>26.9</v>
       </c>
       <c r="C13" s="28">
-        <v>34</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="D13">
-        <v>5.8</v>
+        <v>3.7</v>
       </c>
       <c r="E13">
-        <v>7.3</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B14">
-        <v>24.3</v>
+        <v>17.8</v>
       </c>
       <c r="C14">
-        <v>30.8</v>
+        <v>23.6</v>
       </c>
       <c r="D14">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="E14">
-        <v>4.0999999999999996</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B15">
-        <v>24.7</v>
+        <v>20.3</v>
       </c>
       <c r="C15">
-        <v>31.2</v>
+        <v>26.6</v>
       </c>
       <c r="D15">
-        <v>4.4000000000000004</v>
+        <v>2.9</v>
       </c>
       <c r="E15">
-        <v>4.5999999999999996</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B16">
-        <v>22.2</v>
+        <v>26.2</v>
       </c>
       <c r="C16">
-        <v>32.4</v>
+        <v>36.700000000000003</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="E16">
-        <v>2.9</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B17">
-        <v>23</v>
+        <v>22.5</v>
       </c>
       <c r="C17">
-        <v>29.5</v>
+        <v>29.7</v>
       </c>
       <c r="D17">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="E17">
-        <v>4.0999999999999996</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>219</v>
       </c>
       <c r="B18">
-        <v>23.9</v>
+        <v>20.6</v>
       </c>
       <c r="C18">
-        <v>32.5</v>
+        <v>29.4</v>
       </c>
       <c r="D18">
-        <v>3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="E18">
-        <v>4.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B19">
-        <v>17.100000000000001</v>
+        <v>15.4</v>
       </c>
       <c r="C19">
-        <v>23.5</v>
+        <v>22.6</v>
       </c>
       <c r="D19">
-        <v>5.9</v>
+        <v>4.3</v>
       </c>
       <c r="E19">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>220</v>
       </c>
       <c r="B20">
-        <v>38.5</v>
+        <v>39.299999999999997</v>
       </c>
       <c r="C20">
-        <v>49.2</v>
+        <v>49.9</v>
       </c>
       <c r="D20">
-        <v>9.5</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="E20">
-        <v>12.3</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B21">
-        <v>20.6</v>
+        <v>16.8</v>
       </c>
       <c r="C21">
-        <v>29.5</v>
+        <v>23.2</v>
       </c>
       <c r="D21">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="E21">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B22">
-        <v>25.1</v>
+        <v>23.6</v>
       </c>
       <c r="C22">
-        <v>35.200000000000003</v>
+        <v>31.5</v>
       </c>
       <c r="D22">
-        <v>4.7</v>
+        <v>6.5</v>
       </c>
       <c r="E22">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B23">
-        <v>21.7</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="C23">
-        <v>28.1</v>
+        <v>22.3</v>
       </c>
       <c r="D23">
-        <v>6</v>
+        <v>3.1</v>
       </c>
       <c r="E23">
-        <v>6.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>221</v>
       </c>
       <c r="B24">
-        <v>21.6</v>
+        <v>21.7</v>
       </c>
       <c r="C24">
-        <v>29.9</v>
+        <v>31.1</v>
       </c>
       <c r="D24">
-        <v>4.4000000000000004</v>
+        <v>6.2</v>
       </c>
       <c r="E24">
-        <v>6.1</v>
+        <v>8.8000000000000007</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B25">
-        <v>26.5</v>
+        <v>22.8</v>
       </c>
       <c r="C25">
-        <v>35.799999999999997</v>
+        <v>30.6</v>
       </c>
       <c r="D25">
-        <v>4.5999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="E25">
-        <v>6.3</v>
+        <v>9.3000000000000007</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B26">
-        <v>18.399999999999999</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="C26">
-        <v>27.5</v>
+        <v>22.8</v>
       </c>
       <c r="D26">
         <v>4.3</v>
       </c>
       <c r="E26">
-        <v>6.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B27">
-        <v>18.3</v>
+        <v>17.2</v>
       </c>
       <c r="C27">
-        <v>24.4</v>
+        <v>22.8</v>
       </c>
       <c r="D27">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
       <c r="E27">
-        <v>3.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B28">
-        <v>18.899999999999999</v>
+        <v>17.2</v>
       </c>
       <c r="C28">
         <v>25.6</v>
       </c>
       <c r="D28">
-        <v>6.7</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="E28">
-        <v>9.6999999999999993</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>64</v>
+        <v>222</v>
       </c>
       <c r="B29">
-        <v>24.1</v>
+        <v>25</v>
       </c>
       <c r="C29">
-        <v>34.5</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="D29">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="E29">
-        <v>8.6999999999999993</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B30">
-        <v>20.3</v>
+        <v>19</v>
       </c>
       <c r="C30">
-        <v>26.9</v>
+        <v>27.1</v>
       </c>
       <c r="D30">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E30">
-        <v>3.6</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>223</v>
       </c>
       <c r="B31">
-        <v>21</v>
+        <v>18.3</v>
       </c>
       <c r="C31">
-        <v>26</v>
+        <v>22.4</v>
       </c>
       <c r="D31">
-        <v>4.0999999999999996</v>
+        <v>3.2</v>
       </c>
       <c r="E31">
-        <v>4.5999999999999996</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B32">
-        <v>23.7</v>
+        <v>16.5</v>
       </c>
       <c r="C32">
-        <v>32.299999999999997</v>
+        <v>23.6</v>
       </c>
       <c r="D32">
-        <v>2.8</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="E32">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B33">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="C33">
-        <v>22.3</v>
+        <v>22.6</v>
       </c>
       <c r="D33">
-        <v>2.5</v>
+        <v>3.4</v>
       </c>
       <c r="E33">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>224</v>
       </c>
       <c r="B34">
-        <v>21.8</v>
+        <v>25.4</v>
       </c>
       <c r="C34">
-        <v>30.1</v>
+        <v>32.9</v>
       </c>
       <c r="D34">
-        <v>3</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="E34">
-        <v>3.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B35">
-        <v>18.3</v>
+        <v>19.8</v>
       </c>
       <c r="C35">
-        <v>26.7</v>
+        <v>26.5</v>
       </c>
       <c r="D35">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E35">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
   </sheetData>
@@ -8106,19 +8106,19 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B3">
-        <v>24.1</v>
+        <v>21</v>
       </c>
       <c r="C3">
-        <v>31.6</v>
+        <v>28.2</v>
       </c>
       <c r="D3">
-        <v>5.6</v>
+        <v>4.8</v>
       </c>
       <c r="E3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -8126,33 +8126,33 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>24.7</v>
+        <v>24</v>
       </c>
       <c r="C4">
-        <v>31.5</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="D4">
-        <v>6.4</v>
+        <v>3.7</v>
       </c>
       <c r="E4">
-        <v>7.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B5">
-        <v>25.3</v>
+        <v>21.2</v>
       </c>
       <c r="C5">
-        <v>33.799999999999997</v>
+        <v>28.3</v>
       </c>
       <c r="D5">
-        <v>3.9</v>
+        <v>5.4</v>
       </c>
       <c r="E5">
-        <v>4.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -8160,16 +8160,16 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>30.2</v>
+        <v>25.5</v>
       </c>
       <c r="C6">
-        <v>39</v>
+        <v>32.700000000000003</v>
       </c>
       <c r="D6">
-        <v>7.2</v>
+        <v>5.8</v>
       </c>
       <c r="E6">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -8177,50 +8177,50 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>24</v>
+        <v>21.1</v>
       </c>
       <c r="C7">
-        <v>31.2</v>
+        <v>28.4</v>
       </c>
       <c r="D7">
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
       <c r="E7">
-        <v>4.4000000000000004</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="B8">
-        <v>22</v>
+        <v>19.3</v>
       </c>
       <c r="C8">
-        <v>30.5</v>
+        <v>26.2</v>
       </c>
       <c r="D8">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
       <c r="E8">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="B9">
-        <v>20.3</v>
+        <v>19</v>
       </c>
       <c r="C9">
-        <v>27</v>
+        <v>25.4</v>
       </c>
       <c r="D9">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="E9">
-        <v>3.8</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -8243,21 +8243,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C1" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D1" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="31" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="B2" s="47">
         <v>2055.8357156299999</v>
@@ -8272,7 +8272,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="B3" s="48">
         <v>1564.1559994900001</v>
@@ -8287,7 +8287,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B4" s="48">
         <v>196.73058093</v>
@@ -8302,7 +8302,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="B5" s="48">
         <v>265.86702915000001</v>
@@ -8317,7 +8317,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B6" s="47">
         <v>1506.7852195400001</v>
@@ -8332,7 +8332,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="B7" s="48">
         <v>752.27831757000001</v>
@@ -8347,7 +8347,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="32" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B8" s="48">
         <v>383.64015707999999</v>
@@ -8362,7 +8362,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="B9" s="47">
         <v>1732.70458177</v>
@@ -8377,7 +8377,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="32" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="B10" s="48">
         <v>1371.16275774</v>
@@ -8392,7 +8392,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="B11" s="47">
         <v>1203.6026445499999</v>
@@ -8407,7 +8407,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="32" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="B12" s="48">
         <v>186.15408069</v>
@@ -8422,7 +8422,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="32" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="B13" s="48">
         <v>168.55518856</v>
@@ -8437,7 +8437,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="32" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="B14" s="48">
         <v>141.62651867</v>
@@ -8452,7 +8452,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="B15" s="48">
         <v>234.33700390999999</v>
@@ -8467,7 +8467,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B16" s="47">
         <v>1071.0758428199999</v>
@@ -8482,7 +8482,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="B17" s="47">
         <v>817.57811244000004</v>
@@ -8497,7 +8497,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B18" s="47">
         <v>1304.6751968799999</v>
@@ -8512,7 +8512,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="32" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="B19" s="48">
         <v>335.11905289999999</v>
@@ -8527,7 +8527,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="32" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="B20" s="48">
         <v>212.96472790000001</v>
@@ -8542,7 +8542,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="32" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B21" s="48">
         <v>160.86447251999999</v>
@@ -8557,7 +8557,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B22" s="48">
         <v>538.16199499000004</v>
@@ -8572,7 +8572,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B23" s="47">
         <v>806.12336928000002</v>
@@ -8587,7 +8587,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B24" s="47">
         <v>586.03007229000002</v>
@@ -8602,7 +8602,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B25" s="47">
         <v>75.301730789999993</v>
@@ -8617,7 +8617,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B26" s="47">
         <v>170.99937065</v>
@@ -8632,7 +8632,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B27" s="49">
         <v>1876.8735020900001</v>
@@ -8661,15 +8661,15 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="B2" s="43">
         <v>13207.585358730001</v>
@@ -8678,7 +8678,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="B3" s="43">
         <v>3838.3825559400002</v>
@@ -8687,7 +8687,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B4" s="44">
         <v>4.3860492899999999</v>
@@ -8696,7 +8696,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="B5" s="44">
         <v>358.34224784999998</v>
@@ -8705,7 +8705,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B6" s="44">
         <v>34.741751530000002</v>
@@ -8714,7 +8714,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="B7" s="44">
         <v>143.80485421</v>
@@ -8723,7 +8723,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B8" s="44">
         <v>78.934716230000006</v>
@@ -8732,7 +8732,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B9" s="44">
         <v>2488.1987099299999</v>
@@ -8741,7 +8741,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="22" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B10" s="44">
         <v>405.68594094000002</v>
@@ -8750,7 +8750,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="B11" s="44">
         <v>27.567491919999998</v>
@@ -8759,7 +8759,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="B12" s="44">
         <v>15.39608967</v>
@@ -8768,7 +8768,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="22" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="B13" s="44">
         <v>18.001209469999999</v>
@@ -8777,7 +8777,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="22" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="B14" s="44">
         <v>216.01886056000001</v>
@@ -8786,7 +8786,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="22" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="B15" s="44">
         <v>47.30463434</v>
@@ -8795,7 +8795,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="B16" s="43">
         <v>4108.9096855199996</v>
@@ -8804,7 +8804,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="22" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B17" s="44">
         <v>743.04116016</v>
@@ -8813,7 +8813,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="22" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="B18" s="44">
         <v>39.849933989999997</v>
@@ -8822,7 +8822,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="22" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="B19" s="44">
         <v>237.56029172000001</v>
@@ -8831,7 +8831,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="22" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="B20" s="44">
         <v>14.170199390000001</v>
@@ -8840,7 +8840,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="B21" s="44">
         <v>11.336348060000001</v>
@@ -8849,7 +8849,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="22" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="B22" s="44">
         <v>26.981322290000001</v>
@@ -8858,7 +8858,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="22" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="B23" s="44">
         <v>120.61129541</v>
@@ -8867,7 +8867,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="22" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B24" s="44">
         <v>1216.4536875700001</v>
@@ -8876,7 +8876,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="22" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="B25" s="44">
         <v>71.898552679999995</v>
@@ -8885,7 +8885,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="22" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="B26" s="44">
         <v>141.62678188000001</v>
@@ -8894,7 +8894,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="22" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="B27" s="44">
         <v>111.2139683</v>
@@ -8903,7 +8903,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="22" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="B28" s="44">
         <v>1128.21193786</v>
@@ -8912,7 +8912,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="22" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="B29" s="44">
         <v>47.049963599999998</v>
@@ -8921,7 +8921,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="22" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="B30" s="44">
         <v>50.140863359999997</v>
@@ -8930,7 +8930,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="22" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="B31" s="44">
         <v>18.130049110000002</v>
@@ -8939,7 +8939,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="22" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="B32" s="44">
         <v>130.63333014</v>
@@ -8948,7 +8948,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="24" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="B33" s="43">
         <v>3697.3168202500001</v>
@@ -8957,7 +8957,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="22" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B34" s="44">
         <v>849.9980276</v>
@@ -8966,7 +8966,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="22" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="B35" s="44">
         <v>155.27257409000001</v>
@@ -8975,7 +8975,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="22" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="B36" s="44">
         <v>25.470443889999999</v>
@@ -8984,7 +8984,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="22" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="B37" s="44">
         <v>2.7287990299999998</v>
@@ -8993,7 +8993,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="22" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="B38" s="44">
         <v>67.649627609999996</v>
@@ -9002,7 +9002,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="22" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="B39" s="44">
         <v>16.198883989999999</v>
@@ -9011,7 +9011,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="22" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="B40" s="44">
         <v>1.43051251</v>
@@ -9020,7 +9020,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="22" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="B41" s="44">
         <v>19.168406239999999</v>
@@ -9029,7 +9029,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="22" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="B42" s="44">
         <v>1053.352331</v>
@@ -9038,7 +9038,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="22" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="B43" s="44">
         <v>298.25986130000001</v>
@@ -9047,7 +9047,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="22" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="B44" s="44">
         <v>185.25430915000001</v>
@@ -9056,7 +9056,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="22" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="B45" s="44">
         <v>751.51911275999998</v>
@@ -9065,7 +9065,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="22" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="B46" s="44">
         <v>22.685022549999999</v>
@@ -9074,7 +9074,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="22" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="B47" s="44">
         <v>248.32890853000001</v>
@@ -9083,7 +9083,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="24" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="B48" s="43">
         <v>1562.9762970199999</v>
@@ -9092,7 +9092,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="22" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B49" s="44">
         <v>849.42092487000002</v>
@@ -9101,7 +9101,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="22" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="B50" s="44">
         <v>380.88709162999999</v>
@@ -9110,7 +9110,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="22" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="B51" s="44">
         <v>9.4532592100000006</v>
@@ -9119,7 +9119,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="22" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="B52" s="45">
         <v>237.53615798999999</v>
@@ -9128,7 +9128,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="23" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="B53" s="46">
         <v>85.678863320000005</v>
@@ -9150,15 +9150,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="B2" s="29">
         <v>10230.9320374</v>
@@ -9166,7 +9166,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="B3" s="29">
         <v>2149.1071075599998</v>
@@ -9174,7 +9174,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="B4" s="30">
         <v>1626.06836828</v>
@@ -9182,7 +9182,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="B5" s="30">
         <v>231.20314798999999</v>
@@ -9190,7 +9190,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="B6" s="30">
         <v>291.83559129000002</v>
@@ -9198,7 +9198,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="B7" s="29">
         <v>3274.6054727000001</v>
@@ -9206,7 +9206,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="B8" s="30">
         <v>397.57618968999998</v>
@@ -9214,7 +9214,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B9" s="30">
         <v>90.548557709999997</v>
@@ -9222,7 +9222,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="B10" s="30">
         <v>151.71123872000001</v>
@@ -9230,7 +9230,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="B11" s="30">
         <v>2310.3730725700002</v>
@@ -9238,7 +9238,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="34" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="B12" s="30">
         <v>324.39641401</v>
@@ -9246,7 +9246,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B13" s="29">
         <v>294.49078997999999</v>
@@ -9254,7 +9254,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="34" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="B14" s="30">
         <v>36.16919438</v>
@@ -9262,7 +9262,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="B15" s="30">
         <v>258.32159560000002</v>
@@ -9270,7 +9270,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B16" s="29">
         <v>1811.6569512200001</v>
@@ -9278,7 +9278,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="34" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B17" s="30">
         <v>722.65841826999997</v>
@@ -9286,7 +9286,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="34" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="B18" s="30">
         <v>123.39147755</v>
@@ -9294,7 +9294,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="34" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B19" s="30">
         <v>965.60705540000004</v>
@@ -9302,7 +9302,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="B20" s="29">
         <v>1657.2453018199999</v>
@@ -9310,7 +9310,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="34" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="B21" s="30">
         <v>140.91804273</v>
@@ -9318,7 +9318,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="34" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="B22" s="30">
         <v>206.74287163</v>
@@ -9326,7 +9326,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="34" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="B23" s="30">
         <v>128.47421363000001</v>
@@ -9334,7 +9334,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="34" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="B24" s="30">
         <v>176.62252258999999</v>
@@ -9342,7 +9342,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="34" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="B25" s="30">
         <v>467.40797422999998</v>
@@ -9350,7 +9350,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="34" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B26" s="30">
         <v>264.96412925999999</v>
@@ -9358,7 +9358,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="34" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="B27" s="30">
         <v>272.11554775000002</v>
@@ -9366,7 +9366,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="33" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B28" s="29">
         <v>853.95577985</v>
@@ -9374,7 +9374,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="35" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="B29" s="38">
         <v>189.87063427000001</v>

</xml_diff>

<commit_message>
"Agrego IPC y comex marzo26, emae feb26 y coef gini 4T25"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D681577D-33B3-4500-92B5-0E1640FF3E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F43B7A4-1AA6-4B09-AF65-4F90D395EFE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -1337,7 +1337,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="1" customWidth="1"/>
@@ -3231,6 +3231,23 @@
       </c>
       <c r="E111">
         <v>4.3</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="19">
+        <v>46082</v>
+      </c>
+      <c r="B112" s="1">
+        <v>3.4</v>
+      </c>
+      <c r="C112">
+        <v>1</v>
+      </c>
+      <c r="D112">
+        <v>3.2</v>
+      </c>
+      <c r="E112">
+        <v>5.0999999999999996</v>
       </c>
     </row>
   </sheetData>
@@ -3454,7 +3471,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -3484,10 +3501,10 @@
         <v>134.74645041349706</v>
       </c>
       <c r="C2" s="36">
-        <v>147.98416443521199</v>
+        <v>148.01098759830978</v>
       </c>
       <c r="D2" s="36">
-        <v>147.12594096702841</v>
+        <v>147.12086271528273</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3498,10 +3515,10 @@
         <v>134.23236103862521</v>
       </c>
       <c r="C3" s="36">
-        <v>147.0735309036678</v>
+        <v>147.04192648038881</v>
       </c>
       <c r="D3" s="36">
-        <v>146.54748831828914</v>
+        <v>146.54143624974256</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3512,10 +3529,10 @@
         <v>150.0878942366954</v>
       </c>
       <c r="C4" s="36">
-        <v>146.10851463731433</v>
+        <v>146.11329589755002</v>
       </c>
       <c r="D4" s="36">
-        <v>145.99672295993258</v>
+        <v>145.98963189840191</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3526,10 +3543,10 @@
         <v>153.25067436662908</v>
       </c>
       <c r="C5" s="36">
-        <v>144.92921584007314</v>
+        <v>144.91144960260394</v>
       </c>
       <c r="D5" s="36">
-        <v>145.50904554873608</v>
+        <v>145.50096500309323</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3540,10 +3557,10 @@
         <v>163.51360808690507</v>
       </c>
       <c r="C6" s="36">
-        <v>144.60979068880104</v>
+        <v>144.62489626653098</v>
       </c>
       <c r="D6" s="36">
-        <v>145.11168805200137</v>
+        <v>145.10292112863843</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3554,10 +3571,10 @@
         <v>153.66209524099784</v>
       </c>
       <c r="C7" s="36">
-        <v>144.28461730121603</v>
+        <v>144.28727796100659</v>
       </c>
       <c r="D7" s="36">
-        <v>144.82538456264692</v>
+        <v>144.81635266378433</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3568,10 +3585,10 @@
         <v>143.73110098180126</v>
       </c>
       <c r="C8" s="36">
-        <v>144.44230222025726</v>
+        <v>144.45235172541018</v>
       </c>
       <c r="D8" s="36">
-        <v>144.6621397657425</v>
+        <v>144.65327709197499</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3582,10 +3599,10 @@
         <v>143.6741026486049</v>
       </c>
       <c r="C9" s="36">
-        <v>145.51658654598589</v>
+        <v>145.52363655941912</v>
       </c>
       <c r="D9" s="36">
-        <v>144.62918087773434</v>
+        <v>144.62092576805313</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3596,10 +3613,10 @@
         <v>142.00773744282046</v>
       </c>
       <c r="C10" s="36">
-        <v>144.91422930495111</v>
+        <v>144.89712978641674</v>
       </c>
       <c r="D10" s="36">
-        <v>144.73037937674931</v>
+        <v>144.7231248780077</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3610,10 +3627,10 @@
         <v>141.13686329808141</v>
       </c>
       <c r="C11" s="36">
-        <v>145.0099426627921</v>
+        <v>145.01500612592429</v>
       </c>
       <c r="D11" s="36">
-        <v>144.96158361546256</v>
+        <v>144.95565947551708</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3624,10 +3641,10 @@
         <v>144.93832064073018</v>
       </c>
       <c r="C12" s="36">
-        <v>145.71579727175728</v>
+        <v>145.73745860567124</v>
       </c>
       <c r="D12" s="36">
-        <v>145.31113330135875</v>
+        <v>145.30662076547225</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3638,10 +3655,10 @@
         <v>142.59014516031914</v>
       </c>
       <c r="C13" s="36">
-        <v>146.9826617165933</v>
+        <v>146.95593691960002</v>
       </c>
       <c r="D13" s="36">
-        <v>145.7658942195805</v>
+        <v>145.76254941479078</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3652,10 +3669,10 @@
         <v>136.63265948316217</v>
       </c>
       <c r="C14" s="36">
-        <v>147.28783054174625</v>
+        <v>147.28111363140778</v>
       </c>
       <c r="D14" s="36">
-        <v>146.30854552394575</v>
+        <v>146.30616240170187</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3666,10 +3683,10 @@
         <v>132.15851633982282</v>
       </c>
       <c r="C15" s="36">
-        <v>146.93413462664321</v>
+        <v>146.93713499433917</v>
       </c>
       <c r="D15" s="36">
-        <v>146.91759868504354</v>
+        <v>146.91600896710906</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3680,10 +3697,10 @@
         <v>152.62095855905741</v>
       </c>
       <c r="C16" s="36">
-        <v>147.75615312299135</v>
+        <v>147.75986966568857</v>
       </c>
       <c r="D16" s="36">
-        <v>147.57012884683868</v>
+        <v>147.56917267380467</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3694,10 +3711,10 @@
         <v>151.94634480448744</v>
       </c>
       <c r="C17" s="36">
-        <v>147.64422761579598</v>
+        <v>147.625262164101</v>
       </c>
       <c r="D17" s="36">
-        <v>148.24183922410623</v>
+        <v>148.24128807548888</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3708,10 +3725,10 @@
         <v>168.3892094693679</v>
       </c>
       <c r="C18" s="36">
-        <v>148.506517670411</v>
+        <v>148.51681898705647</v>
       </c>
       <c r="D18" s="36">
-        <v>148.90276577033757</v>
+        <v>148.90252215418158</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3722,10 +3739,10 @@
         <v>161.03568546945243</v>
       </c>
       <c r="C19" s="36">
-        <v>150.16406696867037</v>
+        <v>150.17273110377675</v>
       </c>
       <c r="D19" s="36">
-        <v>149.51953400295426</v>
+        <v>149.51965525841922</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3736,10 +3753,10 @@
         <v>150.3060501239201</v>
       </c>
       <c r="C20" s="36">
-        <v>150.41944165359786</v>
+        <v>150.41984345111493</v>
       </c>
       <c r="D20" s="36">
-        <v>150.05662690671261</v>
+        <v>150.05730416267465</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3750,10 +3767,10 @@
         <v>149.25534277384119</v>
       </c>
       <c r="C21" s="36">
-        <v>150.44302122832045</v>
+        <v>150.44687754301867</v>
       </c>
       <c r="D21" s="36">
-        <v>150.4783661838681</v>
+        <v>150.47980534569041</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3764,10 +3781,10 @@
         <v>146.38655965775396</v>
       </c>
       <c r="C22" s="36">
-        <v>151.22418367580548</v>
+        <v>151.21992556364921</v>
       </c>
       <c r="D22" s="36">
-        <v>150.75111225813859</v>
+        <v>150.75328935366625</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3778,10 +3795,10 @@
         <v>149.38594966601465</v>
       </c>
       <c r="C23" s="36">
-        <v>151.758219009497</v>
+        <v>151.77525571571192</v>
       </c>
       <c r="D23" s="36">
-        <v>150.84979048866137</v>
+        <v>150.85247794964803</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3792,10 +3809,10 @@
         <v>151.92604285202702</v>
       </c>
       <c r="C24" s="36">
-        <v>152.57421307554173</v>
+        <v>152.55842394576581</v>
       </c>
       <c r="D24" s="36">
-        <v>150.75430898737324</v>
+        <v>150.75676025442888</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3806,10 +3823,10 @@
         <v>146.78338490922457</v>
       </c>
       <c r="C25" s="36">
-        <v>152.11469489125977</v>
+        <v>152.11344731488316</v>
       </c>
       <c r="D25" s="36">
-        <v>150.4567340837346</v>
+        <v>150.45819990243763</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3820,10 +3837,10 @@
         <v>142.74091260617232</v>
       </c>
       <c r="C26" s="36">
-        <v>150.73526012195717</v>
+        <v>150.73320475690605</v>
       </c>
       <c r="D26" s="36">
-        <v>149.96567876832358</v>
+        <v>149.96566368423788</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3834,10 +3851,10 @@
         <v>138.81804035165752</v>
       </c>
       <c r="C27" s="36">
-        <v>151.90328057084443</v>
+        <v>151.92718912792515</v>
       </c>
       <c r="D27" s="36">
-        <v>149.30435008530588</v>
+        <v>149.30251169045846</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3845,13 +3862,13 @@
         <v>43160</v>
       </c>
       <c r="B28" s="17">
-        <v>155.85731953576982</v>
+        <v>155.85731953576979</v>
       </c>
       <c r="C28" s="36">
-        <v>151.33512477508165</v>
+        <v>151.31327158311342</v>
       </c>
       <c r="D28" s="36">
-        <v>148.50864233651453</v>
+        <v>148.50478054472566</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3862,10 +3879,10 @@
         <v>151.52454398394349</v>
       </c>
       <c r="C29" s="36">
-        <v>146.83545544273494</v>
+        <v>146.85430728092382</v>
       </c>
       <c r="D29" s="36">
-        <v>147.62333168581083</v>
+        <v>147.61775834167585</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3876,10 +3893,10 @@
         <v>159.56669237791675</v>
       </c>
       <c r="C30" s="36">
-        <v>144.73606068174158</v>
+        <v>144.71989342594935</v>
       </c>
       <c r="D30" s="36">
-        <v>146.69981092291601</v>
+        <v>146.69282260219174</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3890,10 +3907,10 @@
         <v>151.1257632334553</v>
       </c>
       <c r="C31" s="36">
-        <v>143.43435071467957</v>
+        <v>143.43166613233919</v>
       </c>
       <c r="D31" s="36">
-        <v>145.79150750165263</v>
+        <v>145.78314209846303</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -3904,10 +3921,10 @@
         <v>145.9635244300047</v>
       </c>
       <c r="C32" s="36">
-        <v>143.8593540054695</v>
+        <v>143.86286163426718</v>
       </c>
       <c r="D32" s="36">
-        <v>144.94779112366157</v>
+        <v>144.93788535540864</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3918,10 +3935,10 @@
         <v>146.76596003413977</v>
       </c>
       <c r="C33" s="36">
-        <v>146.6868146054301</v>
+        <v>146.70287267918201</v>
       </c>
       <c r="D33" s="36">
-        <v>144.21330657798896</v>
+        <v>144.20160832192963</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -3932,10 +3949,10 @@
         <v>137.74656971864809</v>
       </c>
       <c r="C34" s="36">
-        <v>143.21638592657462</v>
+        <v>143.19682022408026</v>
       </c>
       <c r="D34" s="36">
-        <v>143.6187013418222</v>
+        <v>143.60495466908517</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3946,10 +3963,10 @@
         <v>142.84327598456773</v>
       </c>
       <c r="C35" s="36">
-        <v>143.46264585114906</v>
+        <v>143.4972382881202</v>
       </c>
       <c r="D35" s="36">
-        <v>143.17761282979643</v>
+        <v>143.16169375878408</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -3960,10 +3977,10 @@
         <v>140.59240732533573</v>
       </c>
       <c r="C36" s="36">
-        <v>141.5857201570667</v>
+        <v>141.5817162286825</v>
       </c>
       <c r="D36" s="36">
-        <v>142.8909948083799</v>
+        <v>142.87298762422233</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -3974,10 +3991,10 @@
         <v>136.25161596905645</v>
       </c>
       <c r="C37" s="36">
-        <v>142.00617267082225</v>
+        <v>141.97558416228699</v>
       </c>
       <c r="D37" s="36">
-        <v>142.74711270118166</v>
+        <v>142.72746019426879</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -3988,10 +4005,10 @@
         <v>134.53623985669589</v>
       </c>
       <c r="C38" s="36">
-        <v>141.79432368279794</v>
+        <v>141.75823528596922</v>
       </c>
       <c r="D38" s="36">
-        <v>142.71947890740492</v>
+        <v>142.69890452556666</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4002,10 +4019,10 @@
         <v>132.2678886127367</v>
       </c>
       <c r="C39" s="36">
-        <v>144.15550670865235</v>
+        <v>144.16801805361411</v>
       </c>
       <c r="D39" s="36">
-        <v>142.77094533098327</v>
+        <v>142.7504499028754</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4016,10 +4033,10 @@
         <v>144.96325495574922</v>
       </c>
       <c r="C40" s="36">
-        <v>142.59443805924374</v>
+        <v>142.61801511116187</v>
       </c>
       <c r="D40" s="36">
-        <v>142.86225149941299</v>
+        <v>142.84288102132973</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4030,10 +4047,10 @@
         <v>149.9162214035228</v>
       </c>
       <c r="C41" s="36">
-        <v>142.60231019450458</v>
+        <v>142.59377058595626</v>
       </c>
       <c r="D41" s="36">
-        <v>142.95153273177766</v>
+        <v>142.93420960376099</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4044,10 +4061,10 @@
         <v>164.13569907592046</v>
       </c>
       <c r="C42" s="36">
-        <v>144.6132395614579</v>
+        <v>144.62746246123709</v>
       </c>
       <c r="D42" s="36">
-        <v>143.00113542926778</v>
+        <v>142.98646106092323</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4058,10 +4075,10 @@
         <v>150.85897174113131</v>
       </c>
       <c r="C43" s="36">
-        <v>143.72744711431142</v>
+        <v>143.72176382313401</v>
       </c>
       <c r="D43" s="36">
-        <v>142.97836557235004</v>
+        <v>142.96653648496644</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4072,10 +4089,10 @@
         <v>146.77702964007042</v>
       </c>
       <c r="C44" s="36">
-        <v>145.55248976350893</v>
+        <v>145.57608841723237</v>
       </c>
       <c r="D44" s="36">
-        <v>142.85657834248337</v>
+        <v>142.84734942480696</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4086,10 +4103,10 @@
         <v>141.27693468084041</v>
       </c>
       <c r="C45" s="36">
-        <v>144.6185374108843</v>
+        <v>144.5867230373083</v>
       </c>
       <c r="D45" s="36">
-        <v>142.61906386804452</v>
+        <v>142.6115037562007</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4100,10 +4117,10 @@
         <v>134.87706647993659</v>
       </c>
       <c r="C46" s="36">
-        <v>140.45106888843378</v>
+        <v>140.45928460833969</v>
       </c>
       <c r="D46" s="36">
-        <v>142.25955618378433</v>
+        <v>142.25208700368466</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -4114,10 +4131,10 @@
         <v>141.63933661701387</v>
       </c>
       <c r="C47" s="36">
-        <v>143.74226390099199</v>
+        <v>143.76929914815295</v>
       </c>
       <c r="D47" s="36">
-        <v>141.78183838434097</v>
+        <v>141.77251793986341</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -4128,10 +4145,10 @@
         <v>137.77182966933154</v>
       </c>
       <c r="C48" s="36">
-        <v>140.82638022720951</v>
+        <v>140.82581612981005</v>
       </c>
       <c r="D48" s="36">
-        <v>141.19987367454414</v>
+        <v>141.18696366988326</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4142,10 +4159,10 @@
         <v>135.7651545276351</v>
       </c>
       <c r="C49" s="36">
-        <v>140.10762172203482</v>
+        <v>140.08115057232507</v>
       </c>
       <c r="D49" s="36">
-        <v>140.53870161865993</v>
+        <v>140.52126707298086</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -4156,10 +4173,10 @@
         <v>133.89108608957252</v>
       </c>
       <c r="C50" s="36">
-        <v>140.6036798183564</v>
+        <v>140.59146066606024</v>
       </c>
       <c r="D50" s="36">
-        <v>139.82772013200128</v>
+        <v>139.80572745278548</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -4170,10 +4187,10 @@
         <v>128.97363874659834</v>
       </c>
       <c r="C51" s="36">
-        <v>139.35074093412922</v>
+        <v>139.32585337854485</v>
       </c>
       <c r="D51" s="36">
-        <v>139.10085474883599</v>
+        <v>139.07535965654986</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -4184,10 +4201,10 @@
         <v>128.21106074025664</v>
       </c>
       <c r="C52" s="36">
-        <v>125.97316204831111</v>
+        <v>126.0102687562371</v>
       </c>
       <c r="D52" s="36">
-        <v>138.39412945530478</v>
+        <v>138.36706322033021</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -4198,10 +4215,10 @@
         <v>113.29503444580129</v>
       </c>
       <c r="C53" s="36">
-        <v>106.18032476382055</v>
+        <v>106.18849056621826</v>
       </c>
       <c r="D53" s="36">
-        <v>137.74419083130718</v>
+        <v>137.71823989965426</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -4212,10 +4229,10 @@
         <v>131.02956919734908</v>
       </c>
       <c r="C54" s="36">
-        <v>117.56499589517145</v>
+        <v>117.57694156274655</v>
       </c>
       <c r="D54" s="36">
-        <v>137.18583559564087</v>
+        <v>137.1638590138501</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -4226,10 +4243,10 @@
         <v>132.52196526648828</v>
       </c>
       <c r="C55" s="36">
-        <v>124.71912720009033</v>
+        <v>124.69901573014316</v>
       </c>
       <c r="D55" s="36">
-        <v>136.74753207589245</v>
+        <v>136.73238309407228</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -4240,10 +4257,10 @@
         <v>127.46368946979557</v>
       </c>
       <c r="C56" s="36">
-        <v>126.26766306255661</v>
+        <v>126.29154844608678</v>
       </c>
       <c r="D56" s="36">
-        <v>136.44960639816946</v>
+        <v>136.44366799252003</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -4254,10 +4271,10 @@
         <v>125.18389375984724</v>
       </c>
       <c r="C57" s="36">
-        <v>128.86297264851027</v>
+        <v>128.83848661323916</v>
       </c>
       <c r="D57" s="36">
-        <v>136.30545816098535</v>
+        <v>136.31017846543881</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -4268,10 +4285,10 @@
         <v>127.17507609335082</v>
       </c>
       <c r="C58" s="36">
-        <v>130.69181304546765</v>
+        <v>130.69241369724585</v>
       </c>
       <c r="D58" s="36">
-        <v>136.31800121280813</v>
+        <v>136.33359196995013</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -4282,10 +4299,10 @@
         <v>131.34550189452142</v>
       </c>
       <c r="C59" s="36">
-        <v>133.26525897935591</v>
+        <v>133.27900105390182</v>
       </c>
       <c r="D59" s="36">
-        <v>136.48223855035084</v>
+        <v>136.5076983356185</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -4296,10 +4313,10 @@
         <v>132.06865525299401</v>
       </c>
       <c r="C60" s="36">
-        <v>134.71071040246167</v>
+        <v>134.75761608382544</v>
       </c>
       <c r="D60" s="36">
-        <v>136.78361152018331</v>
+        <v>136.81700503430804</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -4310,10 +4327,10 @@
         <v>133.85436559461567</v>
       </c>
       <c r="C61" s="36">
-        <v>136.82308772906509</v>
+        <v>136.76243997319986</v>
       </c>
       <c r="D61" s="36">
-        <v>137.20224637216864</v>
+        <v>137.24099515867724</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -4324,10 +4341,10 @@
         <v>131.52153739734899</v>
       </c>
       <c r="C62" s="36">
-        <v>139.63894578986631</v>
+        <v>139.53110165499149</v>
       </c>
       <c r="D62" s="36">
-        <v>137.71736457026788</v>
+        <v>137.75854128313458</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -4338,10 +4355,10 @@
         <v>126.2392669683769</v>
       </c>
       <c r="C63" s="36">
-        <v>138.09511409430371</v>
+        <v>138.17596709188399</v>
       </c>
       <c r="D63" s="36">
-        <v>138.31354130774039</v>
+        <v>138.35309338301954</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -4352,10 +4369,10 @@
         <v>145.95690010360465</v>
       </c>
       <c r="C64" s="36">
-        <v>141.03398403621657</v>
+        <v>141.06097517355974</v>
       </c>
       <c r="D64" s="36">
-        <v>138.97963431850297</v>
+        <v>139.01403257617207</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -4366,10 +4383,10 @@
         <v>147.28084401862384</v>
       </c>
       <c r="C65" s="36">
-        <v>139.45903788617423</v>
+        <v>139.46258508049939</v>
       </c>
       <c r="D65" s="36">
-        <v>139.70889552256895</v>
+        <v>139.73547944088494</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -4380,10 +4397,10 @@
         <v>151.16932233869107</v>
       </c>
       <c r="C66" s="36">
-        <v>138.97237834209403</v>
+        <v>138.96189928358311</v>
       </c>
       <c r="D66" s="36">
-        <v>140.49863799043612</v>
+        <v>140.51647056125293</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -4394,10 +4411,10 @@
         <v>148.97961710860557</v>
       </c>
       <c r="C67" s="36">
-        <v>141.52841212917215</v>
+        <v>141.53534399340631</v>
       </c>
       <c r="D67" s="36">
-        <v>141.34543253573938</v>
+        <v>141.35549240580593</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -4408,10 +4425,10 @@
         <v>142.42591306097327</v>
       </c>
       <c r="C68" s="36">
-        <v>141.34508748860509</v>
+        <v>141.33257195041091</v>
       </c>
       <c r="D68" s="36">
-        <v>142.25037642214357</v>
+        <v>142.25463334833978</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -4422,10 +4439,10 @@
         <v>140.9749407280367</v>
       </c>
       <c r="C69" s="36">
-        <v>143.24815928365717</v>
+        <v>143.26416810434233</v>
       </c>
       <c r="D69" s="36">
-        <v>143.21506248206509</v>
+        <v>143.21562429899168</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -4436,10 +4453,10 @@
         <v>141.2960890894098</v>
       </c>
       <c r="C70" s="36">
-        <v>144.02680631022127</v>
+        <v>144.02331302778106</v>
       </c>
       <c r="D70" s="36">
-        <v>144.2342680385934</v>
+        <v>144.23310771308283</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -4450,10 +4467,10 @@
         <v>139.51475869689307</v>
       </c>
       <c r="C71" s="36">
-        <v>143.34148953752734</v>
+        <v>143.40092987390815</v>
       </c>
       <c r="D71" s="36">
-        <v>145.29648583611456</v>
+        <v>145.29515450919925</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -4464,10 +4481,10 @@
         <v>143.75187761771429</v>
       </c>
       <c r="C72" s="36">
-        <v>145.88334396965624</v>
+        <v>145.89876196548934</v>
       </c>
       <c r="D72" s="36">
-        <v>146.37775470607781</v>
+        <v>146.37689934669191</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -4478,10 +4495,10 @@
         <v>147.22987832209441</v>
       </c>
       <c r="C73" s="36">
-        <v>149.76818655647341</v>
+        <v>149.69332822431508</v>
       </c>
       <c r="D73" s="36">
-        <v>147.44135970192912</v>
+        <v>147.44067363818939</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -4492,10 +4509,10 @@
         <v>139.63796162489982</v>
       </c>
       <c r="C74" s="36">
-        <v>148.43728728335583</v>
+        <v>148.25393324162565</v>
       </c>
       <c r="D74" s="36">
-        <v>148.44426449318115</v>
+        <v>148.44293480400648</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -4506,10 +4523,10 @@
         <v>137.84951353039492</v>
       </c>
       <c r="C75" s="36">
-        <v>150.63289440752891</v>
+        <v>150.74905390996096</v>
       </c>
       <c r="D75" s="36">
-        <v>149.34108732013675</v>
+        <v>149.33967081502831</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -4520,10 +4537,10 @@
         <v>153.93085077631551</v>
       </c>
       <c r="C76" s="36">
-        <v>150.47159205926275</v>
+        <v>150.53878659862093</v>
       </c>
       <c r="D76" s="36">
-        <v>150.0904916491825</v>
+        <v>150.09051948711567</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -4534,10 +4551,10 @@
         <v>157.66169211629463</v>
       </c>
       <c r="C77" s="36">
-        <v>152.0034071839209</v>
+        <v>152.03583935458209</v>
       </c>
       <c r="D77" s="36">
-        <v>150.66390513843072</v>
+        <v>150.66598837212686</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -4548,10 +4565,10 @@
         <v>164.68936308999244</v>
       </c>
       <c r="C78" s="36">
-        <v>152.16490263017786</v>
+        <v>152.17839451373504</v>
       </c>
       <c r="D78" s="36">
-        <v>151.04562504327819</v>
+        <v>151.04875880297126</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -4562,10 +4579,10 @@
         <v>161.45483436245701</v>
       </c>
       <c r="C79" s="36">
-        <v>154.19077980789419</v>
+        <v>154.14485575373874</v>
       </c>
       <c r="D79" s="36">
-        <v>151.23368190379077</v>
+        <v>151.23555238684673</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -4576,10 +4593,10 @@
         <v>152.44538769471595</v>
       </c>
       <c r="C80" s="36">
-        <v>152.47346331942649</v>
+        <v>152.47891898224907</v>
       </c>
       <c r="D80" s="36">
-        <v>151.24235287224582</v>
+        <v>151.24029427871656</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4590,10 +4607,10 @@
         <v>151.46573902517829</v>
       </c>
       <c r="C81" s="36">
-        <v>151.65743372718188</v>
+        <v>151.65757904386837</v>
       </c>
       <c r="D81" s="36">
-        <v>151.09940874223366</v>
+        <v>151.09123715918429</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4604,10 +4621,10 @@
         <v>149.17434933731033</v>
       </c>
       <c r="C82" s="36">
-        <v>150.7750708473458</v>
+        <v>150.76946986790088</v>
       </c>
       <c r="D82" s="36">
-        <v>150.8408611686215</v>
+        <v>150.82557137519984</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4618,10 +4635,10 @@
         <v>146.55439498929425</v>
       </c>
       <c r="C83" s="36">
-        <v>149.23974308318589</v>
+        <v>149.29210589362691</v>
       </c>
       <c r="D83" s="36">
-        <v>150.50583574647703</v>
+        <v>150.4839717644017</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4632,10 +4649,10 @@
         <v>148.03049443531322</v>
       </c>
       <c r="C84" s="36">
-        <v>148.50749990138871</v>
+        <v>148.59272305832613</v>
       </c>
       <c r="D84" s="36">
-        <v>150.13081034108305</v>
+        <v>150.10423203431668</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -4646,10 +4663,10 @@
         <v>146.18080800458125</v>
       </c>
       <c r="C85" s="36">
-        <v>148.5213147080778</v>
+        <v>148.38372874076049</v>
       </c>
       <c r="D85" s="36">
-        <v>149.74796080882658</v>
+        <v>149.71925893214558</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -4660,10 +4677,10 @@
         <v>143.03019028680231</v>
       </c>
       <c r="C86" s="36">
-        <v>149.69317822957683</v>
+        <v>149.42540329357686</v>
       </c>
       <c r="D86" s="36">
-        <v>149.37939009446657</v>
+        <v>149.35136782035747</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4674,10 +4691,10 @@
         <v>137.26202711164171</v>
       </c>
       <c r="C87" s="36">
-        <v>149.64274747212693</v>
+        <v>149.80041668986829</v>
       </c>
       <c r="D87" s="36">
-        <v>149.03501410197069</v>
+        <v>149.0095174095525</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -4688,10 +4705,10 @@
         <v>155.06056763777909</v>
       </c>
       <c r="C88" s="36">
-        <v>150.83505977466785</v>
+        <v>150.94516549298999</v>
       </c>
       <c r="D88" s="36">
-        <v>148.70890535647786</v>
+        <v>148.68844544834684</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -4702,10 +4719,10 @@
         <v>150.02108492570758</v>
       </c>
       <c r="C89" s="36">
-        <v>147.36470885338534</v>
+        <v>147.40208090995787</v>
       </c>
       <c r="D89" s="36">
-        <v>148.38532978945474</v>
+        <v>148.37307500824281</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4716,10 +4733,10 @@
         <v>153.77240570488985</v>
       </c>
       <c r="C90" s="36">
-        <v>145.67210800721972</v>
+        <v>145.7072010721923</v>
       </c>
       <c r="D90" s="36">
-        <v>148.04175321375715</v>
+        <v>148.04177512445932</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4730,10 +4747,10 @@
         <v>152.55703188407324</v>
       </c>
       <c r="C91" s="36">
-        <v>146.29688511039032</v>
+        <v>146.22441998890517</v>
       </c>
       <c r="D91" s="36">
-        <v>147.65804453750539</v>
+        <v>147.67373495905306</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -4744,10 +4761,10 @@
         <v>150.22297368785945</v>
       </c>
       <c r="C92" s="36">
-        <v>148.75232261473298</v>
+        <v>148.73770721655438</v>
       </c>
       <c r="D92" s="36">
-        <v>147.22280669257339</v>
+        <v>147.25561082099853</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -4758,10 +4775,10 @@
         <v>151.94203814879756</v>
       </c>
       <c r="C93" s="36">
-        <v>150.0926319307934</v>
+        <v>150.0818844307978</v>
       </c>
       <c r="D93" s="36">
-        <v>146.73320547539899</v>
+        <v>146.78226017689644</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -4772,10 +4789,10 @@
         <v>148.4322432701974</v>
       </c>
       <c r="C94" s="36">
-        <v>149.55846428674684</v>
+        <v>149.58382718498399</v>
       </c>
       <c r="D94" s="36">
-        <v>146.19967388150923</v>
+        <v>146.26176608811957</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4786,10 +4803,10 @@
         <v>147.50696066044537</v>
       </c>
       <c r="C95" s="36">
-        <v>148.14029444558713</v>
+        <v>148.22226335986232</v>
       </c>
       <c r="D95" s="36">
-        <v>145.64577732617855</v>
+        <v>145.71558877455374</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -4800,10 +4817,10 @@
         <v>146.35949533183793</v>
       </c>
       <c r="C96" s="36">
-        <v>146.51277382726593</v>
+        <v>146.58267269019237</v>
       </c>
       <c r="D96" s="36">
-        <v>145.10423503691078</v>
+        <v>145.17544035724288</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -4814,10 +4831,10 @@
         <v>139.33576576518632</v>
       </c>
       <c r="C97" s="36">
-        <v>142.94160983525137</v>
+        <v>142.78974205810835</v>
       </c>
       <c r="D97" s="36">
-        <v>144.61838048925998</v>
+        <v>144.68575924389799</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -4828,10 +4845,10 @@
         <v>137.54602735591297</v>
       </c>
       <c r="C98" s="36">
-        <v>143.76883369012882</v>
+        <v>143.48265454112794</v>
       </c>
       <c r="D98" s="36">
-        <v>144.23481395740316</v>
+        <v>144.29356237988557</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4842,10 +4859,10 @@
         <v>133.63722384206051</v>
       </c>
       <c r="C99" s="36">
-        <v>143.89465322280864</v>
+        <v>144.05255219339068</v>
       </c>
       <c r="D99" s="36">
-        <v>143.99752040583331</v>
+        <v>144.04387119805276</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4856,10 +4873,10 @@
         <v>142.56862052019582</v>
       </c>
       <c r="C100" s="36">
-        <v>142.77426190677184</v>
+        <v>142.90254208524681</v>
       </c>
       <c r="D100" s="36">
-        <v>143.9433434259976</v>
+        <v>143.97650870009548</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4870,10 +4887,10 @@
         <v>147.26512454856004</v>
       </c>
       <c r="C101" s="36">
-        <v>140.89793664197632</v>
+        <v>140.96025044219942</v>
       </c>
       <c r="D101" s="36">
-        <v>144.09459659939233</v>
+        <v>144.11805717758716</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4884,10 +4901,10 @@
         <v>156.7765837615064</v>
       </c>
       <c r="C102" s="36">
-        <v>142.51215427525324</v>
+        <v>142.54498400140477</v>
       </c>
       <c r="D102" s="36">
-        <v>144.45245702311871</v>
+        <v>144.47473787248018</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4895,13 +4912,13 @@
         <v>45444</v>
       </c>
       <c r="B103" s="17">
-        <v>147.36516936817381</v>
+        <v>147.36516936817389</v>
       </c>
       <c r="C103" s="36">
-        <v>143.64245592690298</v>
+        <v>143.54731240058413</v>
       </c>
       <c r="D103" s="36">
-        <v>145.00036065680248</v>
+        <v>145.03374266011252</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -4912,10 +4929,10 @@
         <v>149.69752697536458</v>
       </c>
       <c r="C104" s="36">
-        <v>147.44117252611102</v>
+        <v>147.40216831223594</v>
       </c>
       <c r="D104" s="36">
-        <v>145.70198490469494</v>
+        <v>145.75946892808861</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -4926,10 +4943,10 @@
         <v>147.32757348272975</v>
       </c>
       <c r="C105" s="36">
-        <v>148.15608489238346</v>
+        <v>148.11129841137603</v>
       </c>
       <c r="D105" s="36">
-        <v>146.50738235925428</v>
+        <v>146.60018857621711</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -4940,10 +4957,10 @@
         <v>144.84378302186047</v>
       </c>
       <c r="C106" s="36">
-        <v>147.91126702726274</v>
+        <v>147.99505772220581</v>
       </c>
       <c r="D106" s="36">
-        <v>147.36100464411041</v>
+        <v>147.4957731698471</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -4954,10 +4971,10 @@
         <v>147.99466238363041</v>
       </c>
       <c r="C107" s="36">
-        <v>148.87494748794492</v>
+        <v>148.99241120605578</v>
       </c>
       <c r="D107" s="36">
-        <v>148.20558224385911</v>
+        <v>148.38637355757476</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -4968,10 +4985,10 @@
         <v>148.06937483613993</v>
       </c>
       <c r="C108" s="36">
-        <v>150.49590003515124</v>
+        <v>150.61267185225518</v>
       </c>
       <c r="D108" s="36">
-        <v>148.99585556290131</v>
+        <v>149.21958681063214</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -4982,10 +4999,10 @@
         <v>148.56734190911206</v>
       </c>
       <c r="C109" s="36">
-        <v>151.28934434546181</v>
+        <v>151.05510881031032</v>
       </c>
       <c r="D109" s="36">
-        <v>149.69917389113817</v>
+        <v>149.95705141918856</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -4996,10 +5013,10 @@
         <v>146.29580174387476</v>
       </c>
       <c r="C110" s="36">
-        <v>151.84835710402444</v>
+        <v>151.5018205088835</v>
       </c>
       <c r="D110" s="36">
-        <v>150.2980988059023</v>
+        <v>150.57471839371709</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -5010,10 +5027,10 @@
         <v>141.2021694522208</v>
       </c>
       <c r="C111" s="36">
-        <v>153.14243736157638</v>
+        <v>153.43664475077557</v>
       </c>
       <c r="D111" s="36">
-        <v>150.79011026457874</v>
+        <v>151.064343973592</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -5024,10 +5041,10 @@
         <v>150.40655910972941</v>
       </c>
       <c r="C112" s="36">
-        <v>150.32026807591762</v>
+        <v>150.37259728192413</v>
       </c>
       <c r="D112" s="36">
-        <v>151.18446463534534</v>
+        <v>151.43218413570568</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -5038,10 +5055,10 @@
         <v>158.74110296645111</v>
       </c>
       <c r="C113" s="36">
-        <v>151.92898883643196</v>
+        <v>152.04459357205783</v>
       </c>
       <c r="D113" s="36">
-        <v>151.50055430850293</v>
+        <v>151.69557736720424</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -5052,10 +5069,10 @@
         <v>164.8778979559678</v>
       </c>
       <c r="C114" s="36">
-        <v>151.68489734200023</v>
+        <v>151.67363016442619</v>
       </c>
       <c r="D114" s="36">
-        <v>151.76412995400179</v>
+        <v>151.87853516462113</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -5066,10 +5083,10 @@
         <v>156.59401884940311</v>
       </c>
       <c r="C115" s="36">
-        <v>151.24779792587231</v>
+        <v>151.14346036788424</v>
       </c>
       <c r="D115" s="36">
-        <v>152.00191650731665</v>
+        <v>152.00690826247319</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -5080,10 +5097,10 @@
         <v>153.90772081429063</v>
       </c>
       <c r="C116" s="36">
-        <v>151.51469569017755</v>
+        <v>151.4558141653047</v>
       </c>
       <c r="D116" s="36">
-        <v>152.23763361792382</v>
+        <v>152.10424327522946</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -5094,10 +5111,10 @@
         <v>150.51256572733467</v>
       </c>
       <c r="C117" s="36">
-        <v>152.55472207534925</v>
+        <v>152.57027083830084</v>
       </c>
       <c r="D117" s="36">
-        <v>152.48849687213487</v>
+        <v>152.1874781401736</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -5108,10 +5125,10 @@
         <v>151.83984439466224</v>
       </c>
       <c r="C118" s="36">
-        <v>153.4943406678635</v>
+        <v>153.53767342984943</v>
       </c>
       <c r="D118" s="36">
-        <v>152.76457799839011</v>
+        <v>152.26910227199022</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -5119,13 +5136,13 @@
         <v>45931</v>
       </c>
       <c r="B119" s="17">
-        <v>152.59573745863372</v>
+        <v>152.56798377141189</v>
       </c>
       <c r="C119" s="36">
-        <v>152.65435605342799</v>
+        <v>152.71748568104624</v>
       </c>
       <c r="D119" s="36">
-        <v>153.07088380818087</v>
+        <v>152.35630280996764</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -5133,13 +5150,13 @@
         <v>45962</v>
       </c>
       <c r="B120" s="17">
-        <v>147.72352773408562</v>
+        <v>147.69977298929118</v>
       </c>
       <c r="C120" s="36">
-        <v>152.48907642385822</v>
+        <v>152.54463449254752</v>
       </c>
       <c r="D120" s="36">
-        <v>153.41081353041972</v>
+        <v>152.45253676119401</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -5147,27 +5164,41 @@
         <v>45992</v>
       </c>
       <c r="B121" s="17">
-        <v>153.46285317997496</v>
+        <v>153.51436161199129</v>
       </c>
       <c r="C121" s="36">
-        <v>155.2798620314735</v>
+        <v>155.16117433523141</v>
       </c>
       <c r="D121" s="36">
-        <v>153.78425609353792</v>
+        <v>152.55859752385459</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
         <v>46023</v>
       </c>
-      <c r="B122" s="41">
-        <v>149.04090209242113</v>
-      </c>
-      <c r="C122" s="42">
-        <v>155.93678506834027</v>
-      </c>
-      <c r="D122" s="42">
-        <v>154.19106810873225</v>
+      <c r="B122" s="17">
+        <v>148.78601868878062</v>
+      </c>
+      <c r="C122" s="36">
+        <v>155.70506528002818</v>
+      </c>
+      <c r="D122" s="36">
+        <v>152.67173720221635</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="4">
+        <v>46054</v>
+      </c>
+      <c r="B123" s="41">
+        <v>138.20389337039899</v>
+      </c>
+      <c r="C123" s="42">
+        <v>151.68243919385438</v>
+      </c>
+      <c r="D123" s="42">
+        <v>152.7934630987927</v>
       </c>
     </row>
   </sheetData>
@@ -5215,22 +5246,22 @@
         <v>112</v>
       </c>
       <c r="B2" s="37">
-        <v>1.5</v>
+        <v>1.9401324373755413</v>
       </c>
       <c r="C2" s="20">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="D2" s="20">
-        <v>1.7</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="20">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="F2" s="20">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="G2" s="20">
-        <v>2</v>
+        <v>2.7</v>
       </c>
       <c r="H2" s="16">
         <v>1.6092716037988009</v>
@@ -5241,22 +5272,22 @@
         <v>113</v>
       </c>
       <c r="B3" s="37">
+        <v>6.9838686395306659</v>
+      </c>
+      <c r="C3" s="20">
+        <v>7.1</v>
+      </c>
+      <c r="D3" s="20">
+        <v>7.6</v>
+      </c>
+      <c r="E3" s="20">
         <v>7.2</v>
       </c>
-      <c r="C3" s="20">
-        <v>6.3</v>
-      </c>
-      <c r="D3" s="20">
-        <v>6.2</v>
-      </c>
-      <c r="E3" s="20">
-        <v>6.7</v>
-      </c>
       <c r="F3" s="20">
-        <v>6.2</v>
+        <v>7.9</v>
       </c>
       <c r="G3" s="20">
-        <v>3.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="H3" s="16">
         <v>6.2561659139136028</v>
@@ -5267,22 +5298,22 @@
         <v>114</v>
       </c>
       <c r="B4" s="37">
-        <v>2.2000000000000002</v>
+        <v>1.9506961730765271</v>
       </c>
       <c r="C4" s="20">
         <v>1.9</v>
       </c>
       <c r="D4" s="20">
-        <v>1.4</v>
+        <v>3.9</v>
       </c>
       <c r="E4" s="20">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="F4" s="20">
-        <v>2.7</v>
+        <v>1.2</v>
       </c>
       <c r="G4" s="20">
-        <v>1.5</v>
+        <v>2.8</v>
       </c>
       <c r="H4" s="16">
         <v>1.8835946893488442</v>
@@ -5293,22 +5324,22 @@
         <v>115</v>
       </c>
       <c r="B5" s="37">
-        <v>3.3</v>
+        <v>2.4837275383298829</v>
       </c>
       <c r="C5" s="20">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="D5" s="20">
-        <v>3.4</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E5" s="20">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="F5" s="20">
-        <v>2</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G5" s="20">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="H5" s="16">
         <v>2.390648530181938</v>
@@ -5319,22 +5350,22 @@
         <v>116</v>
       </c>
       <c r="B6" s="37">
+        <v>-2.0205470524042202</v>
+      </c>
+      <c r="C6" s="20">
+        <v>-1.6</v>
+      </c>
+      <c r="D6" s="20">
+        <v>3.5</v>
+      </c>
+      <c r="E6" s="20">
+        <v>2.1</v>
+      </c>
+      <c r="F6" s="20">
         <v>-0.8</v>
       </c>
-      <c r="C6" s="20">
-        <v>0.1</v>
-      </c>
-      <c r="D6" s="20">
-        <v>-0.5</v>
-      </c>
-      <c r="E6" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="F6" s="20">
-        <v>-2.2999999999999998</v>
-      </c>
       <c r="G6" s="20">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="H6" s="16">
         <v>6.142693066479854E-2</v>
@@ -5345,22 +5376,22 @@
         <v>117</v>
       </c>
       <c r="B7" s="37">
-        <v>-4.5</v>
+        <v>-2.21134951799693</v>
       </c>
       <c r="C7" s="20">
-        <v>0.2</v>
+        <v>-1.6</v>
       </c>
       <c r="D7" s="20">
-        <v>6.3</v>
+        <v>-0.8</v>
       </c>
       <c r="E7" s="20">
-        <v>5.8</v>
+        <v>2.5</v>
       </c>
       <c r="F7" s="20">
-        <v>8.8000000000000007</v>
+        <v>-0.8</v>
       </c>
       <c r="G7" s="20">
-        <v>2.1</v>
+        <v>0.5</v>
       </c>
       <c r="H7" s="16">
         <v>0.17135374910239864</v>
@@ -5371,22 +5402,22 @@
         <v>118</v>
       </c>
       <c r="B8" s="37">
-        <v>2.4</v>
+        <v>2.139369389265422</v>
       </c>
       <c r="C8" s="20">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="D8" s="20">
         <v>2.9</v>
       </c>
       <c r="E8" s="20">
-        <v>3.1</v>
+        <v>2.1</v>
       </c>
       <c r="F8" s="20">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="G8" s="20">
-        <v>2.7</v>
+        <v>1.2</v>
       </c>
       <c r="H8" s="16">
         <v>2.8663193746377269</v>
@@ -5397,22 +5428,22 @@
         <v>119</v>
       </c>
       <c r="B9" s="37">
-        <v>1.5</v>
+        <v>1.1770100060511268</v>
       </c>
       <c r="C9" s="20">
-        <v>1.1000000000000001</v>
+        <v>0.3</v>
       </c>
       <c r="D9" s="20">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="E9" s="20">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="F9" s="20">
-        <v>3.1</v>
+        <v>-0.2</v>
       </c>
       <c r="G9" s="20">
-        <v>1.7</v>
+        <v>0.5</v>
       </c>
       <c r="H9" s="16">
         <v>1.0936481387725516</v>
@@ -5423,22 +5454,22 @@
         <v>120</v>
       </c>
       <c r="B10" s="37">
-        <v>2</v>
+        <v>2.1981704342407093</v>
       </c>
       <c r="C10" s="20">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="D10" s="20">
         <v>2.9</v>
       </c>
       <c r="E10" s="20">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="F10" s="20">
-        <v>2.2999999999999998</v>
+        <v>1.6</v>
       </c>
       <c r="G10" s="20">
-        <v>1.9</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="H10" s="16">
         <v>2.7808829939621083</v>
@@ -5486,25 +5517,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="24">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="C2" s="24">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="D2" s="24">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="E2" s="24">
-        <v>3.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="F2" s="24">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="G2" s="24">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="H2" s="24">
-        <v>3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5512,25 +5543,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="22">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="C3" s="22">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="D3" s="22">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="E3" s="22">
         <v>4.5</v>
       </c>
       <c r="F3" s="22">
-        <v>4.0999999999999996</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="G3" s="22">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="H3" s="22">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5538,25 +5569,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="22">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="C4" s="22">
-        <v>0.3</v>
+        <v>2.1</v>
       </c>
       <c r="D4" s="22">
-        <v>0.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E4" s="22">
-        <v>2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F4" s="22">
-        <v>0.4</v>
+        <v>2.4</v>
       </c>
       <c r="G4" s="22">
-        <v>0.9</v>
+        <v>2.1</v>
       </c>
       <c r="H4" s="22">
-        <v>1.1000000000000001</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5564,25 +5595,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="22">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="C5" s="22">
-        <v>-0.3</v>
+        <v>4.2</v>
       </c>
       <c r="D5" s="22">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="E5" s="22">
-        <v>0.3</v>
+        <v>2.5</v>
       </c>
       <c r="F5" s="22">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="G5" s="22">
-        <v>0.2</v>
+        <v>1.9</v>
       </c>
       <c r="H5" s="22">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5590,25 +5621,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="22">
-        <v>6.8</v>
+        <v>3.7</v>
       </c>
       <c r="C6" s="22">
-        <v>6</v>
+        <v>3.6</v>
       </c>
       <c r="D6" s="22">
-        <v>6.6</v>
+        <v>3.2</v>
       </c>
       <c r="E6" s="22">
-        <v>3.4</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="F6" s="22">
-        <v>9.1999999999999993</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="G6" s="22">
-        <v>10.9</v>
+        <v>3.2</v>
       </c>
       <c r="H6" s="22">
-        <v>9.3000000000000007</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5616,25 +5647,25 @@
         <v>17</v>
       </c>
       <c r="B7" s="22">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="C7" s="22">
-        <v>3.1</v>
+        <v>1.3</v>
       </c>
       <c r="D7" s="22">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E7" s="22">
-        <v>2.7</v>
+        <v>0.9</v>
       </c>
       <c r="F7" s="22">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
       <c r="G7" s="22">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="H7" s="22">
-        <v>2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5642,25 +5673,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="22">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="C8" s="22">
-        <v>2.2999999999999998</v>
+        <v>3</v>
       </c>
       <c r="D8" s="22">
+        <v>2.4</v>
+      </c>
+      <c r="E8" s="22">
+        <v>2</v>
+      </c>
+      <c r="F8" s="22">
+        <v>2.4</v>
+      </c>
+      <c r="G8" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="H8" s="22">
         <v>2.6</v>
-      </c>
-      <c r="E8" s="22">
-        <v>2.4</v>
-      </c>
-      <c r="F8" s="22">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="G8" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="H8" s="22">
-        <v>3.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5668,25 +5699,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="22">
-        <v>2</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="C9" s="22">
-        <v>2</v>
+        <v>4.7</v>
       </c>
       <c r="D9" s="22">
-        <v>1.9</v>
+        <v>3.6</v>
       </c>
       <c r="E9" s="22">
         <v>2.5</v>
       </c>
       <c r="F9" s="22">
-        <v>3.6</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="G9" s="22">
-        <v>0.8</v>
+        <v>3.8</v>
       </c>
       <c r="H9" s="22">
-        <v>1.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5694,25 +5725,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="22">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="C10" s="22">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="D10" s="22">
-        <v>1.6</v>
+        <v>2.9</v>
       </c>
       <c r="E10" s="22">
-        <v>1.7</v>
+        <v>2.8</v>
       </c>
       <c r="F10" s="22">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="G10" s="22">
-        <v>1.5</v>
+        <v>2.8</v>
       </c>
       <c r="H10" s="22">
-        <v>1.4</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -5720,25 +5751,25 @@
         <v>21</v>
       </c>
       <c r="B11" s="22">
-        <v>2.2999999999999998</v>
+        <v>3.6</v>
       </c>
       <c r="C11" s="22">
-        <v>1.3</v>
+        <v>3.2</v>
       </c>
       <c r="D11" s="22">
-        <v>4.3</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="E11" s="22">
-        <v>3.4</v>
+        <v>1.2</v>
       </c>
       <c r="F11" s="22">
-        <v>0.3</v>
+        <v>4.8</v>
       </c>
       <c r="G11" s="22">
-        <v>1.1000000000000001</v>
+        <v>3.1</v>
       </c>
       <c r="H11" s="22">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -5746,25 +5777,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="22">
-        <v>1.2</v>
+        <v>12.1</v>
       </c>
       <c r="C12" s="22">
-        <v>1.2</v>
+        <v>10.7</v>
       </c>
       <c r="D12" s="22">
-        <v>0.3</v>
+        <v>12.1</v>
       </c>
       <c r="E12" s="22">
-        <v>1.4</v>
+        <v>22.7</v>
       </c>
       <c r="F12" s="22">
-        <v>1.4</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="G12" s="22">
-        <v>2.5</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="H12" s="22">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -5772,25 +5803,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="22">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="C13" s="22">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="D13" s="22">
+        <v>3.8</v>
+      </c>
+      <c r="E13" s="22">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="F13" s="22">
         <v>3.5</v>
-      </c>
-      <c r="E13" s="22">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="F13" s="22">
-        <v>3.7</v>
       </c>
       <c r="G13" s="22">
         <v>2.9</v>
       </c>
       <c r="H13" s="22">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -5798,25 +5829,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="22">
-        <v>3.3</v>
+        <v>1.7</v>
       </c>
       <c r="C14" s="22">
-        <v>3.5</v>
+        <v>1.8</v>
       </c>
       <c r="D14" s="22">
-        <v>3.3</v>
+        <v>1.6</v>
       </c>
       <c r="E14" s="22">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="F14" s="22">
-        <v>2.7</v>
+        <v>1.9</v>
       </c>
       <c r="G14" s="22">
-        <v>3.1</v>
+        <v>1.4</v>
       </c>
       <c r="H14" s="22">
-        <v>2.5</v>
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>
@@ -5861,25 +5892,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="33">
-        <v>33.1</v>
+        <v>32.6</v>
       </c>
       <c r="C2" s="33">
-        <v>33.200000000000003</v>
+        <v>32.6</v>
       </c>
       <c r="D2" s="33">
-        <v>32.9</v>
+        <v>32.4</v>
       </c>
       <c r="E2" s="33">
+        <v>33.4</v>
+      </c>
+      <c r="F2" s="33">
+        <v>32.5</v>
+      </c>
+      <c r="G2" s="33">
+        <v>33.5</v>
+      </c>
+      <c r="H2" s="33">
         <v>32.1</v>
-      </c>
-      <c r="F2" s="33">
-        <v>33</v>
-      </c>
-      <c r="G2" s="33">
-        <v>33.9</v>
-      </c>
-      <c r="H2" s="33">
-        <v>33.1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5887,25 +5918,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="34">
+        <v>32.700000000000003</v>
+      </c>
+      <c r="C3" s="34">
+        <v>32.4</v>
+      </c>
+      <c r="D3" s="34">
+        <v>32.5</v>
+      </c>
+      <c r="E3" s="34">
+        <v>37.299999999999997</v>
+      </c>
+      <c r="F3" s="34">
+        <v>34.6</v>
+      </c>
+      <c r="G3" s="34">
         <v>36</v>
       </c>
-      <c r="C3" s="34">
-        <v>36.700000000000003</v>
-      </c>
-      <c r="D3" s="34">
-        <v>35.4</v>
-      </c>
-      <c r="E3" s="34">
-        <v>38.9</v>
-      </c>
-      <c r="F3" s="34">
-        <v>36.700000000000003</v>
-      </c>
-      <c r="G3" s="34">
-        <v>38.299999999999997</v>
-      </c>
       <c r="H3" s="34">
-        <v>27.6</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5913,25 +5944,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="34">
-        <v>23.3</v>
+        <v>24.9</v>
       </c>
       <c r="C4" s="34">
-        <v>23.6</v>
+        <v>24.9</v>
       </c>
       <c r="D4" s="34">
-        <v>23.1</v>
+        <v>24.9</v>
       </c>
       <c r="E4" s="34">
-        <v>20.399999999999999</v>
+        <v>23.4</v>
       </c>
       <c r="F4" s="34">
-        <v>22.1</v>
+        <v>24.5</v>
       </c>
       <c r="G4" s="34">
-        <v>23.3</v>
+        <v>24.9</v>
       </c>
       <c r="H4" s="34">
-        <v>26.4</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5939,25 +5970,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="34">
-        <v>15.1</v>
+        <v>13.4</v>
       </c>
       <c r="C5" s="34">
-        <v>15.1</v>
+        <v>13.6</v>
       </c>
       <c r="D5" s="34">
-        <v>13.8</v>
+        <v>12</v>
       </c>
       <c r="E5" s="34">
-        <v>15</v>
+        <v>16.8</v>
       </c>
       <c r="F5" s="34">
-        <v>17.2</v>
+        <v>15.5</v>
       </c>
       <c r="G5" s="34">
-        <v>16.8</v>
+        <v>13.5</v>
       </c>
       <c r="H5" s="34">
-        <v>19.3</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5965,25 +5996,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="34">
-        <v>44.3</v>
+        <v>45.5</v>
       </c>
       <c r="C6" s="34">
-        <v>40.700000000000003</v>
+        <v>41.5</v>
       </c>
       <c r="D6" s="34">
-        <v>46.8</v>
+        <v>47.7</v>
       </c>
       <c r="E6" s="34">
-        <v>43.1</v>
+        <v>54.1</v>
       </c>
       <c r="F6" s="34">
-        <v>42.1</v>
+        <v>44.4</v>
       </c>
       <c r="G6" s="34">
-        <v>47</v>
+        <v>47.1</v>
       </c>
       <c r="H6" s="34">
-        <v>62.5</v>
+        <v>58.4</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5991,25 +6022,25 @@
         <v>17</v>
       </c>
       <c r="B7" s="34">
+        <v>21.1</v>
+      </c>
+      <c r="C7" s="34">
+        <v>23.1</v>
+      </c>
+      <c r="D7" s="34">
+        <v>20</v>
+      </c>
+      <c r="E7" s="34">
+        <v>15</v>
+      </c>
+      <c r="F7" s="34">
+        <v>19.8</v>
+      </c>
+      <c r="G7" s="34">
         <v>21.4</v>
       </c>
-      <c r="C7" s="34">
-        <v>23.2</v>
-      </c>
-      <c r="D7" s="34">
-        <v>20.3</v>
-      </c>
-      <c r="E7" s="34">
-        <v>14.6</v>
-      </c>
-      <c r="F7" s="34">
-        <v>20.3</v>
-      </c>
-      <c r="G7" s="34">
-        <v>21.3</v>
-      </c>
       <c r="H7" s="34">
-        <v>20.6</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6017,25 +6048,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="34">
-        <v>28.7</v>
+        <v>29.7</v>
       </c>
       <c r="C8" s="34">
-        <v>28.3</v>
+        <v>29.7</v>
       </c>
       <c r="D8" s="34">
-        <v>29.1</v>
+        <v>30.2</v>
       </c>
       <c r="E8" s="34">
-        <v>27.1</v>
+        <v>26.9</v>
       </c>
       <c r="F8" s="34">
         <v>29.3</v>
       </c>
       <c r="G8" s="34">
-        <v>26.6</v>
+        <v>27.4</v>
       </c>
       <c r="H8" s="34">
-        <v>32.4</v>
+        <v>32.200000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -6043,25 +6074,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="34">
-        <v>33.1</v>
+        <v>36.200000000000003</v>
       </c>
       <c r="C9" s="34">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D9" s="34">
-        <v>31.5</v>
+        <v>33.6</v>
       </c>
       <c r="E9" s="34">
-        <v>27.1</v>
+        <v>29.6</v>
       </c>
       <c r="F9" s="34">
-        <v>34.299999999999997</v>
+        <v>38.5</v>
       </c>
       <c r="G9" s="34">
-        <v>34.9</v>
+        <v>38.5</v>
       </c>
       <c r="H9" s="34">
-        <v>38.299999999999997</v>
+        <v>40.6</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -6069,25 +6100,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="34">
-        <v>36.1</v>
+        <v>36.6</v>
       </c>
       <c r="C10" s="34">
-        <v>38.4</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="D10" s="34">
-        <v>34.299999999999997</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="E10" s="34">
-        <v>32</v>
+        <v>33.1</v>
       </c>
       <c r="F10" s="34">
-        <v>33.5</v>
+        <v>35.5</v>
       </c>
       <c r="G10" s="34">
-        <v>33.9</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="H10" s="34">
-        <v>35.799999999999997</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -6095,22 +6126,22 @@
         <v>21</v>
       </c>
       <c r="B11" s="34">
-        <v>27.9</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="C11" s="34">
-        <v>25.5</v>
+        <v>29.8</v>
       </c>
       <c r="D11" s="34">
-        <v>33</v>
+        <v>38.6</v>
       </c>
       <c r="E11" s="34">
-        <v>26.6</v>
+        <v>26.8</v>
       </c>
       <c r="F11" s="34">
-        <v>25.3</v>
+        <v>30.1</v>
       </c>
       <c r="G11" s="34">
-        <v>27.2</v>
+        <v>29.7</v>
       </c>
       <c r="H11" s="34">
         <v>22.2</v>
@@ -6121,25 +6152,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="34">
-        <v>50.7</v>
+        <v>38.9</v>
       </c>
       <c r="C12" s="34">
-        <v>40.9</v>
+        <v>34.5</v>
       </c>
       <c r="D12" s="34">
-        <v>56.4</v>
+        <v>38.5</v>
       </c>
       <c r="E12" s="34">
-        <v>47.6</v>
+        <v>45.5</v>
       </c>
       <c r="F12" s="34">
-        <v>74.5</v>
+        <v>56.3</v>
       </c>
       <c r="G12" s="34">
-        <v>63.3</v>
+        <v>42.4</v>
       </c>
       <c r="H12" s="34">
-        <v>74.099999999999994</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -6147,25 +6178,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="34">
-        <v>41.6</v>
+        <v>41</v>
       </c>
       <c r="C13" s="34">
-        <v>40.799999999999997</v>
+        <v>40.1</v>
       </c>
       <c r="D13" s="34">
         <v>44.1</v>
       </c>
       <c r="E13" s="34">
-        <v>47.3</v>
+        <v>49.4</v>
       </c>
       <c r="F13" s="34">
-        <v>37.299999999999997</v>
+        <v>34.299999999999997</v>
       </c>
       <c r="G13" s="34">
-        <v>38.299999999999997</v>
+        <v>39.299999999999997</v>
       </c>
       <c r="H13" s="34">
-        <v>37.4</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -6173,25 +6204,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="34">
-        <v>33.700000000000003</v>
+        <v>31.8</v>
       </c>
       <c r="C14" s="34">
-        <v>37.5</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="D14" s="34">
-        <v>31.6</v>
+        <v>30.8</v>
       </c>
       <c r="E14" s="34">
-        <v>27.9</v>
+        <v>26.8</v>
       </c>
       <c r="F14" s="34">
-        <v>26.7</v>
+        <v>26.5</v>
       </c>
       <c r="G14" s="34">
-        <v>34.4</v>
+        <v>33</v>
       </c>
       <c r="H14" s="34">
-        <v>28.8</v>
+        <v>27.8</v>
       </c>
     </row>
   </sheetData>
@@ -8260,14 +8291,14 @@
         <v>70</v>
       </c>
       <c r="B2" s="47">
-        <v>2055.8357156299999</v>
+        <v>3642.0849776</v>
       </c>
       <c r="C2" s="47">
-        <v>2644.1434920199999</v>
+        <v>4599.8744133099999</v>
       </c>
       <c r="D2" s="27">
         <f>B2-C2</f>
-        <v>-588.30777639000007</v>
+        <v>-957.78943570999991</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -8275,14 +8306,14 @@
         <v>203</v>
       </c>
       <c r="B3" s="48">
-        <v>1564.1559994900001</v>
+        <v>2720.7819912800001</v>
       </c>
       <c r="C3" s="48">
-        <v>2088.58644116</v>
+        <v>3534.7605033300001</v>
       </c>
       <c r="D3" s="27">
         <f t="shared" ref="D3:D27" si="0">B3-C3</f>
-        <v>-524.43044166999994</v>
+        <v>-813.97851205000006</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -8290,14 +8321,14 @@
         <v>208</v>
       </c>
       <c r="B4" s="48">
-        <v>196.73058093</v>
+        <v>364.63594053000003</v>
       </c>
       <c r="C4" s="48">
-        <v>470.6189273</v>
+        <v>931.43666941000004</v>
       </c>
       <c r="D4" s="27">
         <f t="shared" si="0"/>
-        <v>-273.88834637000002</v>
+        <v>-566.80072887999995</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -8305,14 +8336,14 @@
         <v>209</v>
       </c>
       <c r="B5" s="48">
-        <v>265.86702915000001</v>
+        <v>460.54735755000002</v>
       </c>
       <c r="C5" s="48">
-        <v>84.09820406</v>
+        <v>132.83453276</v>
       </c>
       <c r="D5" s="27">
         <f t="shared" si="0"/>
-        <v>181.76882509000001</v>
+        <v>327.71282479000001</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -8320,14 +8351,14 @@
         <v>72</v>
       </c>
       <c r="B6" s="47">
-        <v>1506.7852195400001</v>
+        <v>2388.6359809800001</v>
       </c>
       <c r="C6" s="47">
-        <v>302.49792280000003</v>
+        <v>512.0873775</v>
       </c>
       <c r="D6" s="27">
         <f t="shared" si="0"/>
-        <v>1204.2872967400001</v>
+        <v>1876.5486034800001</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -8335,14 +8366,14 @@
         <v>71</v>
       </c>
       <c r="B7" s="48">
-        <v>752.27831757000001</v>
+        <v>1250.9587038899999</v>
       </c>
       <c r="C7" s="48">
-        <v>130.65088157</v>
+        <v>224.68015249999999</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" si="0"/>
-        <v>621.62743599999999</v>
+        <v>1026.2785513899998</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -8350,14 +8381,14 @@
         <v>204</v>
       </c>
       <c r="B8" s="48">
-        <v>383.64015707999999</v>
+        <v>562.35492280000005</v>
       </c>
       <c r="C8" s="48">
-        <v>52.942879079999997</v>
+        <v>77.517109989999994</v>
       </c>
       <c r="D8" s="27">
         <f t="shared" si="0"/>
-        <v>330.69727799999998</v>
+        <v>484.83781281000006</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -8365,14 +8396,14 @@
         <v>175</v>
       </c>
       <c r="B9" s="47">
-        <v>1732.70458177</v>
+        <v>2729.4163217400001</v>
       </c>
       <c r="C9" s="47">
-        <v>1207.4340521300001</v>
+        <v>1939.1563059800001</v>
       </c>
       <c r="D9" s="27">
         <f t="shared" si="0"/>
-        <v>525.27052963999995</v>
+        <v>790.26001575999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -8380,14 +8411,14 @@
         <v>205</v>
       </c>
       <c r="B10" s="48">
-        <v>1371.16275774</v>
+        <v>2201.7723591099998</v>
       </c>
       <c r="C10" s="48">
-        <v>893.34532280999997</v>
+        <v>1423.8317548</v>
       </c>
       <c r="D10" s="27">
         <f t="shared" si="0"/>
-        <v>477.81743492999999</v>
+        <v>777.9406043099998</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -8395,14 +8426,14 @@
         <v>176</v>
       </c>
       <c r="B11" s="47">
-        <v>1203.6026445499999</v>
+        <v>2022.88633052</v>
       </c>
       <c r="C11" s="47">
-        <v>1426.6886535399999</v>
+        <v>2269.82641969</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" si="0"/>
-        <v>-223.08600898999998</v>
+        <v>-246.94008916999996</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -8410,14 +8441,14 @@
         <v>212</v>
       </c>
       <c r="B12" s="48">
-        <v>186.15408069</v>
+        <v>277.89006107</v>
       </c>
       <c r="C12" s="48">
-        <v>410.40748841999999</v>
+        <v>681.23333489000004</v>
       </c>
       <c r="D12" s="27">
         <f t="shared" si="0"/>
-        <v>-224.25340772999999</v>
+        <v>-403.34327382000004</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -8425,14 +8456,14 @@
         <v>213</v>
       </c>
       <c r="B13" s="48">
-        <v>168.55518856</v>
+        <v>278.63999637000001</v>
       </c>
       <c r="C13" s="48">
-        <v>177.82558041999999</v>
+        <v>263.91412875999998</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>-9.2703918599999895</v>
+        <v>14.725867610000023</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -8440,14 +8471,14 @@
         <v>214</v>
       </c>
       <c r="B14" s="48">
-        <v>141.62651867</v>
+        <v>237.14646142000001</v>
       </c>
       <c r="C14" s="48">
-        <v>227.27655566999999</v>
+        <v>339.50689375000002</v>
       </c>
       <c r="D14" s="27">
         <f t="shared" si="0"/>
-        <v>-85.650036999999998</v>
+        <v>-102.36043233000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -8455,14 +8486,14 @@
         <v>215</v>
       </c>
       <c r="B15" s="48">
-        <v>234.33700390999999</v>
+        <v>413.70484536999999</v>
       </c>
       <c r="C15" s="48">
-        <v>43.005741749999999</v>
+        <v>88.700274840000006</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>191.33126215999999</v>
+        <v>325.00457052999997</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -8470,14 +8501,14 @@
         <v>74</v>
       </c>
       <c r="B16" s="47">
-        <v>1071.0758428199999</v>
+        <v>1770.36411421</v>
       </c>
       <c r="C16" s="47">
-        <v>2707.4913193900002</v>
+        <v>3968.8562505</v>
       </c>
       <c r="D16" s="27">
         <f t="shared" si="0"/>
-        <v>-1636.4154765700002</v>
+        <v>-2198.49213629</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -8485,14 +8516,14 @@
         <v>75</v>
       </c>
       <c r="B17" s="47">
-        <v>817.57811244000004</v>
+        <v>1391.42497028</v>
       </c>
       <c r="C17" s="47">
-        <v>178.81806847999999</v>
+        <v>268.57025942000001</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>638.76004396000008</v>
+        <v>1122.8547108600001</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -8500,14 +8531,14 @@
         <v>73</v>
       </c>
       <c r="B18" s="47">
-        <v>1304.6751968799999</v>
+        <v>2157.6283789899999</v>
       </c>
       <c r="C18" s="47">
-        <v>687.25814527</v>
+        <v>974.11695552000003</v>
       </c>
       <c r="D18" s="27">
         <f t="shared" si="0"/>
-        <v>617.41705160999993</v>
+        <v>1183.51142347</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -8515,14 +8546,14 @@
         <v>207</v>
       </c>
       <c r="B19" s="48">
-        <v>335.11905289999999</v>
+        <v>490.57319502000001</v>
       </c>
       <c r="C19" s="48">
-        <v>76.667375160000006</v>
+        <v>103.15499242</v>
       </c>
       <c r="D19" s="27">
         <f t="shared" si="0"/>
-        <v>258.45167773999998</v>
+        <v>387.41820260000003</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -8530,14 +8561,14 @@
         <v>210</v>
       </c>
       <c r="B20" s="48">
-        <v>212.96472790000001</v>
+        <v>362.31211113000001</v>
       </c>
       <c r="C20" s="48">
-        <v>39.044309120000001</v>
+        <v>58.630448039999997</v>
       </c>
       <c r="D20" s="27">
         <f t="shared" si="0"/>
-        <v>173.92041878000001</v>
+        <v>303.68166309000003</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -8545,14 +8576,14 @@
         <v>211</v>
       </c>
       <c r="B21" s="48">
-        <v>160.86447251999999</v>
+        <v>259.28664493000002</v>
       </c>
       <c r="C21" s="48">
-        <v>341.33399687999997</v>
+        <v>479.11093283999998</v>
       </c>
       <c r="D21" s="27">
         <f t="shared" si="0"/>
-        <v>-180.46952435999998</v>
+        <v>-219.82428790999995</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -8560,14 +8591,14 @@
         <v>206</v>
       </c>
       <c r="B22" s="48">
-        <v>538.16199499000004</v>
+        <v>946.51444658000003</v>
       </c>
       <c r="C22" s="48">
-        <v>176.45890802</v>
+        <v>258.31680581000001</v>
       </c>
       <c r="D22" s="27">
         <f t="shared" si="0"/>
-        <v>361.70308697000007</v>
+        <v>688.19764077000002</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -8575,14 +8606,14 @@
         <v>76</v>
       </c>
       <c r="B23" s="47">
-        <v>806.12336928000002</v>
+        <v>1223.20827323</v>
       </c>
       <c r="C23" s="47">
-        <v>37.451314670000002</v>
+        <v>72.228760469999997</v>
       </c>
       <c r="D23" s="27">
         <f t="shared" si="0"/>
-        <v>768.67205461000003</v>
+        <v>1150.97951276</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -8590,14 +8621,14 @@
         <v>77</v>
       </c>
       <c r="B24" s="47">
-        <v>586.03007229000002</v>
+        <v>1114.49011032</v>
       </c>
       <c r="C24" s="47">
-        <v>41.090413150000003</v>
+        <v>100.81333033999999</v>
       </c>
       <c r="D24" s="27">
         <f t="shared" si="0"/>
-        <v>544.93965914</v>
+        <v>1013.67677998</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -8605,14 +8636,14 @@
         <v>78</v>
       </c>
       <c r="B25" s="47">
-        <v>75.301730789999993</v>
+        <v>87.561110220000003</v>
       </c>
       <c r="C25" s="47">
-        <v>33.193095450000001</v>
+        <v>69.144815120000004</v>
       </c>
       <c r="D25" s="27">
         <f t="shared" si="0"/>
-        <v>42.108635339999992</v>
+        <v>18.416295099999999</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -8620,14 +8651,14 @@
         <v>79</v>
       </c>
       <c r="B26" s="47">
-        <v>170.99937065</v>
+        <v>267.53786265999997</v>
       </c>
       <c r="C26" s="47">
-        <v>44.496689160000003</v>
+        <v>88.303249129999998</v>
       </c>
       <c r="D26" s="27">
         <f t="shared" si="0"/>
-        <v>126.50268149</v>
+        <v>179.23461352999999</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -8635,14 +8666,14 @@
         <v>80</v>
       </c>
       <c r="B27" s="49">
-        <v>1876.8735020900001</v>
+        <v>3057.96917725</v>
       </c>
       <c r="C27" s="49">
-        <v>920.36887134000006</v>
+        <v>1482.1254346999999</v>
       </c>
       <c r="D27" s="27">
         <f t="shared" si="0"/>
-        <v>956.50463075000005</v>
+        <v>1575.8437425500001</v>
       </c>
     </row>
   </sheetData>
@@ -8672,7 +8703,7 @@
         <v>172</v>
       </c>
       <c r="B2" s="43">
-        <v>13207.585358730001</v>
+        <v>21853.207608000001</v>
       </c>
       <c r="D2" s="29"/>
     </row>
@@ -8681,7 +8712,7 @@
         <v>168</v>
       </c>
       <c r="B3" s="43">
-        <v>3838.3825559400002</v>
+        <v>6178.6120975399999</v>
       </c>
       <c r="D3" s="29"/>
     </row>
@@ -8690,7 +8721,7 @@
         <v>121</v>
       </c>
       <c r="B4" s="44">
-        <v>4.3860492899999999</v>
+        <v>7.6568312000000001</v>
       </c>
       <c r="D4" s="30"/>
     </row>
@@ -8699,7 +8730,7 @@
         <v>122</v>
       </c>
       <c r="B5" s="44">
-        <v>358.34224784999998</v>
+        <v>630.60163469999998</v>
       </c>
       <c r="D5" s="30"/>
     </row>
@@ -8708,7 +8739,7 @@
         <v>123</v>
       </c>
       <c r="B6" s="44">
-        <v>34.741751530000002</v>
+        <v>73.900977810000001</v>
       </c>
       <c r="D6" s="30"/>
     </row>
@@ -8717,7 +8748,7 @@
         <v>124</v>
       </c>
       <c r="B7" s="44">
-        <v>143.80485421</v>
+        <v>218.82695206</v>
       </c>
       <c r="D7" s="30"/>
     </row>
@@ -8726,7 +8757,7 @@
         <v>125</v>
       </c>
       <c r="B8" s="44">
-        <v>78.934716230000006</v>
+        <v>135.64279291</v>
       </c>
       <c r="D8" s="30"/>
     </row>
@@ -8735,7 +8766,7 @@
         <v>126</v>
       </c>
       <c r="B9" s="44">
-        <v>2488.1987099299999</v>
+        <v>3985.3623082200002</v>
       </c>
       <c r="D9" s="30"/>
     </row>
@@ -8744,7 +8775,7 @@
         <v>127</v>
       </c>
       <c r="B10" s="44">
-        <v>405.68594094000002</v>
+        <v>671.06527274999996</v>
       </c>
       <c r="D10" s="30"/>
     </row>
@@ -8753,7 +8784,7 @@
         <v>128</v>
       </c>
       <c r="B11" s="44">
-        <v>27.567491919999998</v>
+        <v>35.68106496</v>
       </c>
       <c r="D11" s="30"/>
     </row>
@@ -8762,7 +8793,7 @@
         <v>129</v>
       </c>
       <c r="B12" s="44">
-        <v>15.39608967</v>
+        <v>23.284074100000002</v>
       </c>
       <c r="D12" s="30"/>
     </row>
@@ -8771,7 +8802,7 @@
         <v>130</v>
       </c>
       <c r="B13" s="44">
-        <v>18.001209469999999</v>
+        <v>26.273295900000001</v>
       </c>
       <c r="D13" s="30"/>
     </row>
@@ -8780,7 +8811,7 @@
         <v>131</v>
       </c>
       <c r="B14" s="44">
-        <v>216.01886056000001</v>
+        <v>317.68720475999999</v>
       </c>
       <c r="D14" s="30"/>
     </row>
@@ -8789,7 +8820,7 @@
         <v>132</v>
       </c>
       <c r="B15" s="44">
-        <v>47.30463434</v>
+        <v>52.629688170000001</v>
       </c>
       <c r="D15" s="30"/>
     </row>
@@ -8798,7 +8829,7 @@
         <v>169</v>
       </c>
       <c r="B16" s="43">
-        <v>4108.9096855199996</v>
+        <v>6750.0284991099998</v>
       </c>
       <c r="D16" s="29"/>
     </row>
@@ -8807,7 +8838,7 @@
         <v>133</v>
       </c>
       <c r="B17" s="44">
-        <v>743.04116016</v>
+        <v>1218.1314355</v>
       </c>
       <c r="D17" s="30"/>
     </row>
@@ -8816,7 +8847,7 @@
         <v>134</v>
       </c>
       <c r="B18" s="44">
-        <v>39.849933989999997</v>
+        <v>67.614102810000006</v>
       </c>
       <c r="D18" s="30"/>
     </row>
@@ -8825,7 +8856,7 @@
         <v>135</v>
       </c>
       <c r="B19" s="44">
-        <v>237.56029172000001</v>
+        <v>365.08177555999998</v>
       </c>
       <c r="D19" s="30"/>
     </row>
@@ -8834,7 +8865,7 @@
         <v>136</v>
       </c>
       <c r="B20" s="44">
-        <v>14.170199390000001</v>
+        <v>23.481003789999999</v>
       </c>
       <c r="D20" s="30"/>
     </row>
@@ -8843,7 +8874,7 @@
         <v>137</v>
       </c>
       <c r="B21" s="44">
-        <v>11.336348060000001</v>
+        <v>19.703430130000001</v>
       </c>
       <c r="D21" s="30"/>
     </row>
@@ -8852,7 +8883,7 @@
         <v>138</v>
       </c>
       <c r="B22" s="44">
-        <v>26.981322290000001</v>
+        <v>44.007000400000003</v>
       </c>
       <c r="D22" s="30"/>
     </row>
@@ -8861,7 +8892,7 @@
         <v>139</v>
       </c>
       <c r="B23" s="44">
-        <v>120.61129541</v>
+        <v>182.68527849</v>
       </c>
       <c r="D23" s="30"/>
     </row>
@@ -8870,7 +8901,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="44">
-        <v>1216.4536875700001</v>
+        <v>2073.9789836800001</v>
       </c>
       <c r="D24" s="30"/>
     </row>
@@ -8879,7 +8910,7 @@
         <v>141</v>
       </c>
       <c r="B25" s="44">
-        <v>71.898552679999995</v>
+        <v>106.14883974999999</v>
       </c>
       <c r="D25" s="30"/>
     </row>
@@ -8888,7 +8919,7 @@
         <v>142</v>
       </c>
       <c r="B26" s="44">
-        <v>141.62678188000001</v>
+        <v>225.63479645999999</v>
       </c>
       <c r="D26" s="30"/>
     </row>
@@ -8897,7 +8928,7 @@
         <v>143</v>
       </c>
       <c r="B27" s="44">
-        <v>111.2139683</v>
+        <v>175.96563567999999</v>
       </c>
       <c r="D27" s="30"/>
     </row>
@@ -8906,7 +8937,7 @@
         <v>144</v>
       </c>
       <c r="B28" s="44">
-        <v>1128.21193786</v>
+        <v>1887.6847242900001</v>
       </c>
       <c r="D28" s="30"/>
     </row>
@@ -8915,7 +8946,7 @@
         <v>145</v>
       </c>
       <c r="B29" s="44">
-        <v>47.049963599999998</v>
+        <v>71.754049539999997</v>
       </c>
       <c r="D29" s="30"/>
     </row>
@@ -8924,7 +8955,7 @@
         <v>146</v>
       </c>
       <c r="B30" s="44">
-        <v>50.140863359999997</v>
+        <v>83.504218820000006</v>
       </c>
       <c r="D30" s="30"/>
     </row>
@@ -8933,7 +8964,7 @@
         <v>147</v>
       </c>
       <c r="B31" s="44">
-        <v>18.130049110000002</v>
+        <v>29.34874619</v>
       </c>
       <c r="D31" s="30"/>
     </row>
@@ -8942,7 +8973,7 @@
         <v>148</v>
       </c>
       <c r="B32" s="44">
-        <v>130.63333014</v>
+        <v>175.30447802</v>
       </c>
       <c r="D32" s="30"/>
     </row>
@@ -8951,7 +8982,7 @@
         <v>170</v>
       </c>
       <c r="B33" s="43">
-        <v>3697.3168202500001</v>
+        <v>6087.6302882800001</v>
       </c>
       <c r="D33" s="29"/>
     </row>
@@ -8960,7 +8991,7 @@
         <v>149</v>
       </c>
       <c r="B34" s="44">
-        <v>849.9980276</v>
+        <v>1333.9643457300001</v>
       </c>
       <c r="D34" s="30"/>
     </row>
@@ -8969,7 +9000,7 @@
         <v>150</v>
       </c>
       <c r="B35" s="44">
-        <v>155.27257409000001</v>
+        <v>255.71772598000001</v>
       </c>
       <c r="D35" s="30"/>
     </row>
@@ -8978,7 +9009,7 @@
         <v>151</v>
       </c>
       <c r="B36" s="44">
-        <v>25.470443889999999</v>
+        <v>38.354973569999999</v>
       </c>
       <c r="D36" s="30"/>
     </row>
@@ -8987,7 +9018,7 @@
         <v>152</v>
       </c>
       <c r="B37" s="44">
-        <v>2.7287990299999998</v>
+        <v>4.12255064</v>
       </c>
       <c r="D37" s="30"/>
     </row>
@@ -8996,7 +9027,7 @@
         <v>153</v>
       </c>
       <c r="B38" s="44">
-        <v>67.649627609999996</v>
+        <v>101.4539458</v>
       </c>
       <c r="D38" s="30"/>
     </row>
@@ -9005,7 +9036,7 @@
         <v>154</v>
       </c>
       <c r="B39" s="44">
-        <v>16.198883989999999</v>
+        <v>25.984441180000001</v>
       </c>
       <c r="D39" s="30"/>
     </row>
@@ -9014,7 +9045,7 @@
         <v>155</v>
       </c>
       <c r="B40" s="44">
-        <v>1.43051251</v>
+        <v>1.9632358400000001</v>
       </c>
       <c r="D40" s="30"/>
     </row>
@@ -9023,7 +9054,7 @@
         <v>156</v>
       </c>
       <c r="B41" s="44">
-        <v>19.168406239999999</v>
+        <v>31.65772419</v>
       </c>
       <c r="D41" s="30"/>
     </row>
@@ -9032,7 +9063,7 @@
         <v>157</v>
       </c>
       <c r="B42" s="44">
-        <v>1053.352331</v>
+        <v>1587.7043686699999</v>
       </c>
       <c r="D42" s="30"/>
     </row>
@@ -9041,7 +9072,7 @@
         <v>158</v>
       </c>
       <c r="B43" s="44">
-        <v>298.25986130000001</v>
+        <v>576.36516614000004</v>
       </c>
       <c r="D43" s="30"/>
     </row>
@@ -9050,7 +9081,7 @@
         <v>159</v>
       </c>
       <c r="B44" s="44">
-        <v>185.25430915000001</v>
+        <v>294.64710724999998</v>
       </c>
       <c r="D44" s="30"/>
     </row>
@@ -9059,7 +9090,7 @@
         <v>160</v>
       </c>
       <c r="B45" s="44">
-        <v>751.51911275999998</v>
+        <v>1523.9142027800001</v>
       </c>
       <c r="D45" s="30"/>
     </row>
@@ -9068,7 +9099,7 @@
         <v>161</v>
       </c>
       <c r="B46" s="44">
-        <v>22.685022549999999</v>
+        <v>44.361302100000003</v>
       </c>
       <c r="D46" s="30"/>
     </row>
@@ -9077,7 +9108,7 @@
         <v>162</v>
       </c>
       <c r="B47" s="44">
-        <v>248.32890853000001</v>
+        <v>267.41919840999998</v>
       </c>
       <c r="D47" s="30"/>
     </row>
@@ -9086,7 +9117,7 @@
         <v>171</v>
       </c>
       <c r="B48" s="43">
-        <v>1562.9762970199999</v>
+        <v>2836.93672307</v>
       </c>
       <c r="D48" s="29"/>
     </row>
@@ -9095,7 +9126,7 @@
         <v>163</v>
       </c>
       <c r="B49" s="44">
-        <v>849.42092487000002</v>
+        <v>1559.89458603</v>
       </c>
       <c r="D49" s="30"/>
     </row>
@@ -9104,7 +9135,7 @@
         <v>164</v>
       </c>
       <c r="B50" s="44">
-        <v>380.88709162999999</v>
+        <v>744.01471738999999</v>
       </c>
       <c r="D50" s="30"/>
     </row>
@@ -9113,7 +9144,7 @@
         <v>165</v>
       </c>
       <c r="B51" s="44">
-        <v>9.4532592100000006</v>
+        <v>19.932383229999999</v>
       </c>
       <c r="D51" s="30"/>
     </row>
@@ -9122,7 +9153,7 @@
         <v>166</v>
       </c>
       <c r="B52" s="45">
-        <v>237.53615798999999</v>
+        <v>388.92518603000002</v>
       </c>
       <c r="D52" s="30"/>
     </row>
@@ -9131,7 +9162,7 @@
         <v>167</v>
       </c>
       <c r="B53" s="46">
-        <v>85.678863320000005</v>
+        <v>124.16985038999999</v>
       </c>
     </row>
   </sheetData>
@@ -9161,7 +9192,7 @@
         <v>177</v>
       </c>
       <c r="B2" s="29">
-        <v>10230.9320374</v>
+        <v>16345.10357168</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -9169,7 +9200,7 @@
         <v>178</v>
       </c>
       <c r="B3" s="29">
-        <v>2149.1071075599998</v>
+        <v>3375.8426948000001</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -9177,7 +9208,7 @@
         <v>179</v>
       </c>
       <c r="B4" s="30">
-        <v>1626.06836828</v>
+        <v>2486.7692147500002</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -9185,7 +9216,7 @@
         <v>180</v>
       </c>
       <c r="B5" s="30">
-        <v>231.20314798999999</v>
+        <v>365.06772862000003</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -9193,7 +9224,7 @@
         <v>181</v>
       </c>
       <c r="B6" s="30">
-        <v>291.83559129000002</v>
+        <v>524.00575143000003</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -9201,7 +9232,7 @@
         <v>182</v>
       </c>
       <c r="B7" s="29">
-        <v>3274.6054727000001</v>
+        <v>5451.1590238500003</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -9209,7 +9240,7 @@
         <v>183</v>
       </c>
       <c r="B8" s="30">
-        <v>397.57618968999998</v>
+        <v>846.49245704999998</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -9217,7 +9248,7 @@
         <v>184</v>
       </c>
       <c r="B9" s="30">
-        <v>90.548557709999997</v>
+        <v>136.29556653</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -9225,7 +9256,7 @@
         <v>185</v>
       </c>
       <c r="B10" s="30">
-        <v>151.71123872000001</v>
+        <v>244.10265992000001</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -9233,7 +9264,7 @@
         <v>186</v>
       </c>
       <c r="B11" s="30">
-        <v>2310.3730725700002</v>
+        <v>3733.1311068800001</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -9241,7 +9272,7 @@
         <v>187</v>
       </c>
       <c r="B12" s="30">
-        <v>324.39641401</v>
+        <v>491.13723347000001</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -9249,7 +9280,7 @@
         <v>188</v>
       </c>
       <c r="B13" s="29">
-        <v>294.49078997999999</v>
+        <v>431.66893614999998</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -9257,7 +9288,7 @@
         <v>189</v>
       </c>
       <c r="B14" s="30">
-        <v>36.16919438</v>
+        <v>54.94351047</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -9265,7 +9296,7 @@
         <v>190</v>
       </c>
       <c r="B15" s="30">
-        <v>258.32159560000002</v>
+        <v>376.72542568</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -9273,7 +9304,7 @@
         <v>191</v>
       </c>
       <c r="B16" s="29">
-        <v>1811.6569512200001</v>
+        <v>2894.3441279899998</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -9281,7 +9312,7 @@
         <v>192</v>
       </c>
       <c r="B17" s="30">
-        <v>722.65841826999997</v>
+        <v>1133.9802706400001</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9289,7 +9320,7 @@
         <v>193</v>
       </c>
       <c r="B18" s="30">
-        <v>123.39147755</v>
+        <v>187.76447163</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -9297,7 +9328,7 @@
         <v>194</v>
       </c>
       <c r="B19" s="30">
-        <v>965.60705540000004</v>
+        <v>1572.5993857200001</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -9305,7 +9336,7 @@
         <v>195</v>
       </c>
       <c r="B20" s="29">
-        <v>1657.2453018199999</v>
+        <v>2582.26003515</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -9313,7 +9344,7 @@
         <v>196</v>
       </c>
       <c r="B21" s="30">
-        <v>140.91804273</v>
+        <v>218.70288993</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -9321,7 +9352,7 @@
         <v>197</v>
       </c>
       <c r="B22" s="30">
-        <v>206.74287163</v>
+        <v>348.41194282999999</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -9329,7 +9360,7 @@
         <v>198</v>
       </c>
       <c r="B23" s="30">
-        <v>128.47421363000001</v>
+        <v>194.14988503000001</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -9337,7 +9368,7 @@
         <v>199</v>
       </c>
       <c r="B24" s="30">
-        <v>176.62252258999999</v>
+        <v>272.65300049000001</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -9345,7 +9376,7 @@
         <v>200</v>
       </c>
       <c r="B25" s="30">
-        <v>467.40797422999998</v>
+        <v>725.11567094999998</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -9353,7 +9384,7 @@
         <v>201</v>
       </c>
       <c r="B26" s="30">
-        <v>264.96412925999999</v>
+        <v>437.15278225999998</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -9361,7 +9392,7 @@
         <v>187</v>
       </c>
       <c r="B27" s="30">
-        <v>272.11554775000002</v>
+        <v>386.07386365999997</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -9369,7 +9400,7 @@
         <v>202</v>
       </c>
       <c r="B28" s="29">
-        <v>853.95577985</v>
+        <v>1313.11547008</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -9377,7 +9408,7 @@
         <v>173</v>
       </c>
       <c r="B29" s="38">
-        <v>189.87063427000001</v>
+        <v>296.71328366</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
"Actualizo emae-marzo26, resultado fiscal y comex (abr26)"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DB6A37-4D7D-413F-ADE8-74A76C2BB956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF46CD9E-DCF4-4787-AC76-52482510BCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -722,13 +722,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="167" formatCode="_ [$€-2]\ * #,##0.00_ ;_ [$€-2]\ * \-#,##0.00_ ;_ [$€-2]\ * &quot;-&quot;??_ "/>
     <numFmt numFmtId="168" formatCode="0.0_ ;\-0.0\ "/>
+    <numFmt numFmtId="169" formatCode="#,##0_ ;\-#,##0\ "/>
   </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
@@ -914,7 +915,7 @@
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -977,7 +978,6 @@
     <xf numFmtId="165" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -994,18 +994,20 @@
     <xf numFmtId="3" fontId="11" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="169" fontId="12" fillId="5" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="5" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="12" fillId="5" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Euro" xfId="10" xr:uid="{8CA0DC4E-5AAC-43A0-AC51-59D877AC41AF}"/>
@@ -3488,7 +3490,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -3518,10 +3520,10 @@
         <v>134.74645041349706</v>
       </c>
       <c r="C2" s="36">
-        <v>148.01098759830978</v>
+        <v>148.03259196044854</v>
       </c>
       <c r="D2" s="36">
-        <v>147.12086271528273</v>
+        <v>147.12248518161707</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3532,10 +3534,10 @@
         <v>134.23236103862521</v>
       </c>
       <c r="C3" s="36">
-        <v>147.04192648038881</v>
+        <v>147.0699078640429</v>
       </c>
       <c r="D3" s="36">
-        <v>146.54143624974256</v>
+        <v>146.54332009692405</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3546,10 +3548,10 @@
         <v>150.0878942366954</v>
       </c>
       <c r="C4" s="36">
-        <v>146.11329589755002</v>
+        <v>146.14642347701553</v>
       </c>
       <c r="D4" s="36">
-        <v>145.98963189840191</v>
+        <v>145.9912186327727</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3560,10 +3562,10 @@
         <v>153.25067436662908</v>
       </c>
       <c r="C5" s="36">
-        <v>144.91144960260394</v>
+        <v>144.8588631415312</v>
       </c>
       <c r="D5" s="36">
-        <v>145.50096500309323</v>
+        <v>145.50216986623502</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3574,10 +3576,10 @@
         <v>163.51360808690507</v>
       </c>
       <c r="C6" s="36">
-        <v>144.62489626653098</v>
+        <v>144.58234022667378</v>
       </c>
       <c r="D6" s="36">
-        <v>145.10292112863843</v>
+        <v>145.10382835195102</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3588,10 +3590,10 @@
         <v>153.66209524099784</v>
       </c>
       <c r="C7" s="36">
-        <v>144.28727796100659</v>
+        <v>144.29890359910266</v>
       </c>
       <c r="D7" s="36">
-        <v>144.81635266378433</v>
+        <v>144.81749811409966</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3602,10 +3604,10 @@
         <v>143.73110098180126</v>
       </c>
       <c r="C8" s="36">
-        <v>144.45235172541018</v>
+        <v>144.46186040008149</v>
       </c>
       <c r="D8" s="36">
-        <v>144.65327709197499</v>
+        <v>144.65594973440716</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3616,10 +3618,10 @@
         <v>143.6741026486049</v>
       </c>
       <c r="C9" s="36">
-        <v>145.52363655941912</v>
+        <v>145.52336900371643</v>
       </c>
       <c r="D9" s="36">
-        <v>144.62092576805313</v>
+        <v>144.6266492667815</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3630,10 +3632,10 @@
         <v>142.00773744282046</v>
       </c>
       <c r="C10" s="36">
-        <v>144.89712978641674</v>
+        <v>144.89720375005177</v>
       </c>
       <c r="D10" s="36">
-        <v>144.7231248780077</v>
+        <v>144.7331158955412</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3644,10 +3646,10 @@
         <v>141.13686329808141</v>
       </c>
       <c r="C11" s="36">
-        <v>145.01500612592429</v>
+        <v>145.02139649041007</v>
       </c>
       <c r="D11" s="36">
-        <v>144.95565947551708</v>
+        <v>144.97043956020906</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3658,10 +3660,10 @@
         <v>144.93832064073018</v>
       </c>
       <c r="C12" s="36">
-        <v>145.73745860567124</v>
+        <v>145.7133902031533</v>
       </c>
       <c r="D12" s="36">
-        <v>145.30662076547225</v>
+        <v>145.3262772340878</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3672,10 +3674,10 @@
         <v>142.59014516031914</v>
       </c>
       <c r="C13" s="36">
-        <v>146.95593691960002</v>
+        <v>146.96510342900294</v>
       </c>
       <c r="D13" s="36">
-        <v>145.76254941479078</v>
+        <v>145.78656218575853</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3683,13 +3685,13 @@
         <v>42736</v>
       </c>
       <c r="B14" s="17">
-        <v>136.63265948316217</v>
+        <v>136.63265948316197</v>
       </c>
       <c r="C14" s="36">
-        <v>147.28111363140778</v>
+        <v>147.23494762112568</v>
       </c>
       <c r="D14" s="36">
-        <v>146.30616240170187</v>
+        <v>146.33333771747371</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3697,13 +3699,13 @@
         <v>42767</v>
       </c>
       <c r="B15" s="17">
-        <v>132.15851633982282</v>
+        <v>132.15851633982263</v>
       </c>
       <c r="C15" s="36">
-        <v>146.93713499433917</v>
+        <v>147.00185268779848</v>
       </c>
       <c r="D15" s="36">
-        <v>146.91600896710906</v>
+        <v>146.94471653439686</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3711,13 +3713,13 @@
         <v>42795</v>
       </c>
       <c r="B16" s="17">
-        <v>152.62095855905741</v>
+        <v>152.62095855905721</v>
       </c>
       <c r="C16" s="36">
-        <v>147.75986966568857</v>
+        <v>147.76014108774692</v>
       </c>
       <c r="D16" s="36">
-        <v>147.56917267380467</v>
+        <v>147.59751892003072</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3725,13 +3727,13 @@
         <v>42826</v>
       </c>
       <c r="B17" s="17">
-        <v>151.94634480448744</v>
+        <v>151.94634480448727</v>
       </c>
       <c r="C17" s="36">
-        <v>147.625262164101</v>
+        <v>147.63096590455055</v>
       </c>
       <c r="D17" s="36">
-        <v>148.24128807548888</v>
+        <v>148.26736799772615</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3739,13 +3741,13 @@
         <v>42856</v>
       </c>
       <c r="B18" s="17">
-        <v>168.3892094693679</v>
+        <v>168.38920946936767</v>
       </c>
       <c r="C18" s="36">
-        <v>148.51681898705647</v>
+        <v>148.52167958146185</v>
       </c>
       <c r="D18" s="36">
-        <v>148.90252215418158</v>
+        <v>148.92483939642733</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3753,13 +3755,13 @@
         <v>42887</v>
       </c>
       <c r="B19" s="17">
-        <v>161.03568546945243</v>
+        <v>161.0356854694522</v>
       </c>
       <c r="C19" s="36">
-        <v>150.17273110377675</v>
+        <v>150.12442571118444</v>
       </c>
       <c r="D19" s="36">
-        <v>149.51965525841922</v>
+        <v>149.53712576798011</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3767,13 +3769,13 @@
         <v>42917</v>
       </c>
       <c r="B20" s="17">
-        <v>150.3060501239201</v>
+        <v>150.3060501239199</v>
       </c>
       <c r="C20" s="36">
-        <v>150.41984345111493</v>
+        <v>150.42452382321926</v>
       </c>
       <c r="D20" s="36">
-        <v>150.05730416267465</v>
+        <v>150.06934845722793</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3781,13 +3783,13 @@
         <v>42948</v>
       </c>
       <c r="B21" s="17">
-        <v>149.25534277384119</v>
+        <v>149.25534277384099</v>
       </c>
       <c r="C21" s="36">
-        <v>150.44687754301867</v>
+        <v>150.41158089521988</v>
       </c>
       <c r="D21" s="36">
-        <v>150.47980534569041</v>
+        <v>150.48641140604437</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3795,13 +3797,13 @@
         <v>42979</v>
       </c>
       <c r="B22" s="17">
-        <v>146.38655965775396</v>
+        <v>146.38655965775374</v>
       </c>
       <c r="C22" s="36">
-        <v>151.21992556364921</v>
+        <v>151.26823308009077</v>
       </c>
       <c r="D22" s="36">
-        <v>150.75328935366625</v>
+        <v>150.75507340134595</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3809,13 +3811,13 @@
         <v>43009</v>
       </c>
       <c r="B23" s="17">
-        <v>149.38594966601465</v>
+        <v>149.38594966601445</v>
       </c>
       <c r="C23" s="36">
-        <v>151.77525571571192</v>
+        <v>151.73469142491953</v>
       </c>
       <c r="D23" s="36">
-        <v>150.85247794964803</v>
+        <v>150.85035689592684</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3823,13 +3825,13 @@
         <v>43040</v>
       </c>
       <c r="B24" s="17">
-        <v>151.92604285202702</v>
+        <v>151.92604285202682</v>
       </c>
       <c r="C24" s="36">
-        <v>152.55842394576581</v>
+        <v>152.59226993820425</v>
       </c>
       <c r="D24" s="36">
-        <v>150.75676025442888</v>
+        <v>150.7520652202968</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3837,13 +3839,13 @@
         <v>43070</v>
       </c>
       <c r="B25" s="17">
-        <v>146.78338490922457</v>
+        <v>146.78338490922437</v>
       </c>
       <c r="C25" s="36">
-        <v>152.11344731488316</v>
+        <v>152.12139234183553</v>
       </c>
       <c r="D25" s="36">
-        <v>150.45819990243763</v>
+        <v>150.45222672541368</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3851,13 +3853,13 @@
         <v>43101</v>
       </c>
       <c r="B26" s="17">
-        <v>142.74091260617232</v>
+        <v>142.74091260617209</v>
       </c>
       <c r="C26" s="36">
-        <v>150.73320475690605</v>
+        <v>150.71792889938533</v>
       </c>
       <c r="D26" s="36">
-        <v>149.96566368423788</v>
+        <v>149.95929283420745</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3865,13 +3867,13 @@
         <v>43132</v>
       </c>
       <c r="B27" s="17">
-        <v>138.81804035165752</v>
+        <v>138.81804035165729</v>
       </c>
       <c r="C27" s="36">
-        <v>151.92718912792515</v>
+        <v>151.94087683188036</v>
       </c>
       <c r="D27" s="36">
-        <v>149.30251169045846</v>
+        <v>149.29648754360707</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3879,13 +3881,13 @@
         <v>43160</v>
       </c>
       <c r="B28" s="17">
-        <v>155.85731953576979</v>
+        <v>155.85731953576962</v>
       </c>
       <c r="C28" s="36">
-        <v>151.31327158311342</v>
+        <v>151.3386001459065</v>
       </c>
       <c r="D28" s="36">
-        <v>148.50478054472566</v>
+        <v>148.50023246777778</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3893,13 +3895,13 @@
         <v>43191</v>
       </c>
       <c r="B29" s="17">
-        <v>151.52454398394349</v>
+        <v>151.52454398394329</v>
       </c>
       <c r="C29" s="36">
-        <v>146.85430728092382</v>
+        <v>146.79524090203745</v>
       </c>
       <c r="D29" s="36">
-        <v>147.61775834167585</v>
+        <v>147.61590508743586</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3907,13 +3909,13 @@
         <v>43221</v>
       </c>
       <c r="B30" s="17">
-        <v>159.56669237791675</v>
+        <v>159.56669237791655</v>
       </c>
       <c r="C30" s="36">
-        <v>144.71989342594935</v>
+        <v>144.67702249230945</v>
       </c>
       <c r="D30" s="36">
-        <v>146.69282260219174</v>
+        <v>146.69461483510227</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3921,13 +3923,13 @@
         <v>43252</v>
       </c>
       <c r="B31" s="17">
-        <v>151.1257632334553</v>
+        <v>151.1257632334551</v>
       </c>
       <c r="C31" s="36">
-        <v>143.43166613233919</v>
+        <v>143.44436720597389</v>
       </c>
       <c r="D31" s="36">
-        <v>145.78314209846303</v>
+        <v>145.78930663291649</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -3935,13 +3937,13 @@
         <v>43282</v>
       </c>
       <c r="B32" s="17">
-        <v>145.9635244300047</v>
+        <v>145.96352443000447</v>
       </c>
       <c r="C32" s="36">
-        <v>143.86286163426718</v>
+        <v>143.83317529524027</v>
       </c>
       <c r="D32" s="36">
-        <v>144.93788535540864</v>
+        <v>144.94897637629381</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3949,13 +3951,13 @@
         <v>43313</v>
       </c>
       <c r="B33" s="17">
-        <v>146.76596003413977</v>
+        <v>146.76596003413957</v>
       </c>
       <c r="C33" s="36">
-        <v>146.70287267918201</v>
+        <v>146.73977573753155</v>
       </c>
       <c r="D33" s="36">
-        <v>144.20160832192963</v>
+        <v>144.21701514576142</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -3963,13 +3965,13 @@
         <v>43344</v>
       </c>
       <c r="B34" s="17">
-        <v>137.74656971864809</v>
+        <v>137.74656971864789</v>
       </c>
       <c r="C34" s="36">
-        <v>143.19682022408026</v>
+        <v>143.22183703333664</v>
       </c>
       <c r="D34" s="36">
-        <v>143.60495466908517</v>
+        <v>143.62308744345492</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3977,13 +3979,13 @@
         <v>43374</v>
       </c>
       <c r="B35" s="17">
-        <v>142.84327598456773</v>
+        <v>142.8432759845675</v>
       </c>
       <c r="C35" s="36">
-        <v>143.4972382881202</v>
+        <v>143.48339417996189</v>
       </c>
       <c r="D35" s="36">
-        <v>143.16169375878408</v>
+        <v>143.18038355223803</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -3991,13 +3993,13 @@
         <v>43405</v>
       </c>
       <c r="B36" s="17">
-        <v>140.59240732533573</v>
+        <v>140.59240732533553</v>
       </c>
       <c r="C36" s="36">
-        <v>141.5817162286825</v>
+        <v>141.55480044795232</v>
       </c>
       <c r="D36" s="36">
-        <v>142.87298762422233</v>
+        <v>142.88990687978861</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -4005,13 +4007,13 @@
         <v>43435</v>
       </c>
       <c r="B37" s="17">
-        <v>136.25161596905645</v>
+        <v>136.25161596905625</v>
       </c>
       <c r="C37" s="36">
-        <v>141.97558416228699</v>
+        <v>142.0496063686536</v>
       </c>
       <c r="D37" s="36">
-        <v>142.72746019426879</v>
+        <v>142.74011068149781</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -4019,13 +4021,13 @@
         <v>43466</v>
       </c>
       <c r="B38" s="17">
-        <v>134.53623985669589</v>
+        <v>134.53623985669569</v>
       </c>
       <c r="C38" s="36">
-        <v>141.75823528596922</v>
+        <v>141.81369203436475</v>
       </c>
       <c r="D38" s="36">
-        <v>142.69890452556666</v>
+        <v>142.70524575457767</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4033,13 +4035,13 @@
         <v>43497</v>
       </c>
       <c r="B39" s="17">
-        <v>132.2678886127367</v>
+        <v>132.2678886127365</v>
       </c>
       <c r="C39" s="36">
-        <v>144.16801805361411</v>
+        <v>144.2398618703196</v>
       </c>
       <c r="D39" s="36">
-        <v>142.7504499028754</v>
+        <v>142.75062969122965</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4047,13 +4049,13 @@
         <v>43525</v>
       </c>
       <c r="B40" s="17">
-        <v>144.96325495574922</v>
+        <v>144.96325495574902</v>
       </c>
       <c r="C40" s="36">
-        <v>142.61801511116187</v>
+        <v>142.61988109044677</v>
       </c>
       <c r="D40" s="36">
-        <v>142.84288102132973</v>
+        <v>142.83705874562577</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4061,13 +4063,13 @@
         <v>43556</v>
       </c>
       <c r="B41" s="17">
-        <v>149.9162214035228</v>
+        <v>149.91622140352257</v>
       </c>
       <c r="C41" s="36">
-        <v>142.59377058595626</v>
+        <v>142.54522297724586</v>
       </c>
       <c r="D41" s="36">
-        <v>142.93420960376099</v>
+        <v>142.92201598486434</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4075,13 +4077,13 @@
         <v>43586</v>
       </c>
       <c r="B42" s="17">
-        <v>164.13569907592046</v>
+        <v>164.13569907592026</v>
       </c>
       <c r="C42" s="36">
-        <v>144.62746246123709</v>
+        <v>144.51686029398829</v>
       </c>
       <c r="D42" s="36">
-        <v>142.98646106092323</v>
+        <v>142.96702028919415</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4089,13 +4091,13 @@
         <v>43617</v>
       </c>
       <c r="B43" s="17">
-        <v>150.85897174113131</v>
+        <v>150.85897174113111</v>
       </c>
       <c r="C43" s="36">
-        <v>143.72176382313401</v>
+        <v>143.62648333203899</v>
       </c>
       <c r="D43" s="36">
-        <v>142.96653648496644</v>
+        <v>142.9390000377669</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4103,13 +4105,13 @@
         <v>43647</v>
       </c>
       <c r="B44" s="17">
-        <v>146.77702964007042</v>
+        <v>146.7770296400702</v>
       </c>
       <c r="C44" s="36">
-        <v>145.57608841723237</v>
+        <v>145.57248935472896</v>
       </c>
       <c r="D44" s="36">
-        <v>142.84734942480696</v>
+        <v>142.81154657802949</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4117,13 +4119,13 @@
         <v>43678</v>
       </c>
       <c r="B45" s="17">
-        <v>141.27693468084041</v>
+        <v>141.27693468084021</v>
       </c>
       <c r="C45" s="36">
-        <v>144.5867230373083</v>
+        <v>144.62342018043961</v>
       </c>
       <c r="D45" s="36">
-        <v>142.6115037562007</v>
+        <v>142.56750628404998</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4131,13 +4133,13 @@
         <v>43709</v>
       </c>
       <c r="B46" s="17">
-        <v>134.87706647993659</v>
+        <v>134.87706647993639</v>
       </c>
       <c r="C46" s="36">
-        <v>140.45928460833969</v>
+        <v>140.48644641644498</v>
       </c>
       <c r="D46" s="36">
-        <v>142.25208700368466</v>
+        <v>142.20031686216282</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -4145,13 +4147,13 @@
         <v>43739</v>
       </c>
       <c r="B47" s="17">
-        <v>141.63933661701387</v>
+        <v>141.63933661701367</v>
       </c>
       <c r="C47" s="36">
-        <v>143.76929914815295</v>
+        <v>143.76525611707521</v>
       </c>
       <c r="D47" s="36">
-        <v>141.77251793986341</v>
+        <v>141.7140696561587</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -4159,13 +4161,13 @@
         <v>43770</v>
       </c>
       <c r="B48" s="17">
-        <v>137.77182966933154</v>
+        <v>137.77182966933131</v>
       </c>
       <c r="C48" s="36">
-        <v>140.82581612981005</v>
+        <v>140.87310912587668</v>
       </c>
       <c r="D48" s="36">
-        <v>141.18696366988326</v>
+        <v>141.1238481007837</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4173,13 +4175,13 @@
         <v>43800</v>
       </c>
       <c r="B49" s="17">
-        <v>135.7651545276351</v>
+        <v>135.76515452763491</v>
       </c>
       <c r="C49" s="36">
-        <v>140.08115057232507</v>
+        <v>140.10290445732591</v>
       </c>
       <c r="D49" s="36">
-        <v>140.52126707298086</v>
+        <v>140.45633781358129</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -4187,13 +4189,13 @@
         <v>43831</v>
       </c>
       <c r="B50" s="17">
-        <v>133.89108608957252</v>
+        <v>133.89108608957235</v>
       </c>
       <c r="C50" s="36">
-        <v>140.59146066606024</v>
+        <v>140.71252814452441</v>
       </c>
       <c r="D50" s="36">
-        <v>139.80572745278548</v>
+        <v>139.74261129934382</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -4201,13 +4203,13 @@
         <v>43862</v>
       </c>
       <c r="B51" s="17">
-        <v>128.97363874659834</v>
+        <v>128.97363874659814</v>
       </c>
       <c r="C51" s="36">
-        <v>139.32585337854485</v>
+        <v>139.35238005290518</v>
       </c>
       <c r="D51" s="36">
-        <v>139.07535965654986</v>
+        <v>139.01805511783414</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -4215,13 +4217,13 @@
         <v>43891</v>
       </c>
       <c r="B52" s="17">
-        <v>128.21106074025664</v>
+        <v>128.21106074025644</v>
       </c>
       <c r="C52" s="36">
-        <v>126.0102687562371</v>
+        <v>125.91338590990141</v>
       </c>
       <c r="D52" s="36">
-        <v>138.36706322033021</v>
+        <v>138.3194156496636</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -4229,13 +4231,13 @@
         <v>43922</v>
       </c>
       <c r="B53" s="17">
-        <v>113.29503444580129</v>
+        <v>113.29503444580112</v>
       </c>
       <c r="C53" s="36">
-        <v>106.18849056621826</v>
+        <v>106.15116639878501</v>
       </c>
       <c r="D53" s="36">
-        <v>137.71823989965426</v>
+        <v>137.68338337268341</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -4243,13 +4245,13 @@
         <v>43952</v>
       </c>
       <c r="B54" s="17">
-        <v>131.02956919734908</v>
+        <v>131.02956919734888</v>
       </c>
       <c r="C54" s="36">
-        <v>117.57694156274655</v>
+        <v>117.48924416484118</v>
       </c>
       <c r="D54" s="36">
-        <v>137.1638590138501</v>
+        <v>137.14435744012337</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -4257,13 +4259,13 @@
         <v>43983</v>
       </c>
       <c r="B55" s="17">
-        <v>132.52196526648828</v>
+        <v>132.52196526648811</v>
       </c>
       <c r="C55" s="36">
-        <v>124.69901573014316</v>
+        <v>124.62138887513295</v>
       </c>
       <c r="D55" s="36">
-        <v>136.73238309407228</v>
+        <v>136.72893144705949</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -4271,13 +4273,13 @@
         <v>44013</v>
       </c>
       <c r="B56" s="17">
-        <v>127.46368946979557</v>
+        <v>127.46368946979538</v>
       </c>
       <c r="C56" s="36">
-        <v>126.29154844608678</v>
+        <v>126.30495486357177</v>
       </c>
       <c r="D56" s="36">
-        <v>136.44366799252003</v>
+        <v>136.45479358706709</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -4285,13 +4287,13 @@
         <v>44044</v>
       </c>
       <c r="B57" s="17">
-        <v>125.18389375984724</v>
+        <v>125.18389375984702</v>
       </c>
       <c r="C57" s="36">
-        <v>128.83848661323916</v>
+        <v>128.88217104138715</v>
       </c>
       <c r="D57" s="36">
-        <v>136.31017846543881</v>
+        <v>136.33174707329843</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -4299,13 +4301,13 @@
         <v>44075</v>
       </c>
       <c r="B58" s="17">
-        <v>127.17507609335082</v>
+        <v>127.17507609335061</v>
       </c>
       <c r="C58" s="36">
-        <v>130.69241369724585</v>
+        <v>130.73468236002785</v>
       </c>
       <c r="D58" s="36">
-        <v>136.33359196995013</v>
+        <v>136.36003542140455</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -4313,13 +4315,13 @@
         <v>44105</v>
       </c>
       <c r="B59" s="17">
-        <v>131.34550189452142</v>
+        <v>131.34550189452122</v>
       </c>
       <c r="C59" s="36">
-        <v>133.27900105390182</v>
+        <v>133.28379428516581</v>
       </c>
       <c r="D59" s="36">
-        <v>136.5076983356185</v>
+        <v>136.53278399381435</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -4327,13 +4329,13 @@
         <v>44136</v>
       </c>
       <c r="B60" s="17">
-        <v>132.06865525299401</v>
+        <v>132.06865525299381</v>
       </c>
       <c r="C60" s="36">
-        <v>134.75761608382544</v>
+        <v>134.72927758000364</v>
       </c>
       <c r="D60" s="36">
-        <v>136.81700503430804</v>
+        <v>136.83548448580393</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -4341,13 +4343,13 @@
         <v>44166</v>
       </c>
       <c r="B61" s="17">
-        <v>133.85436559461567</v>
+        <v>133.85436559461547</v>
       </c>
       <c r="C61" s="36">
-        <v>136.76243997319986</v>
+        <v>136.83856286567271</v>
       </c>
       <c r="D61" s="36">
-        <v>137.24099515867724</v>
+        <v>137.24990532734935</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -4355,13 +4357,13 @@
         <v>44197</v>
       </c>
       <c r="B62" s="17">
-        <v>131.52153739734899</v>
+        <v>131.52153739734879</v>
       </c>
       <c r="C62" s="36">
-        <v>139.53110165499149</v>
+        <v>139.70457666741626</v>
       </c>
       <c r="D62" s="36">
-        <v>137.75854128313458</v>
+        <v>137.75779473374334</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -4369,13 +4371,13 @@
         <v>44228</v>
       </c>
       <c r="B63" s="17">
-        <v>126.2392669683769</v>
+        <v>126.23926696837668</v>
       </c>
       <c r="C63" s="36">
-        <v>138.17596709188399</v>
+        <v>138.16466747971225</v>
       </c>
       <c r="D63" s="36">
-        <v>138.35309338301954</v>
+        <v>138.34554082492741</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -4383,13 +4385,13 @@
         <v>44256</v>
       </c>
       <c r="B64" s="17">
-        <v>145.95690010360465</v>
+        <v>145.95690010360443</v>
       </c>
       <c r="C64" s="36">
-        <v>141.06097517355974</v>
+        <v>140.93214881658653</v>
       </c>
       <c r="D64" s="36">
-        <v>139.01403257617207</v>
+        <v>139.00251506565144</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -4397,13 +4399,13 @@
         <v>44287</v>
       </c>
       <c r="B65" s="17">
-        <v>147.28084401862384</v>
+        <v>147.28084401862364</v>
       </c>
       <c r="C65" s="36">
-        <v>139.46258508049939</v>
+        <v>139.32168396782794</v>
       </c>
       <c r="D65" s="36">
-        <v>139.73547944088494</v>
+        <v>139.72449517997134</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -4411,13 +4413,13 @@
         <v>44317</v>
       </c>
       <c r="B66" s="17">
-        <v>151.16932233869107</v>
+        <v>151.16932233869088</v>
       </c>
       <c r="C66" s="36">
-        <v>138.96189928358311</v>
+        <v>138.85334943464642</v>
       </c>
       <c r="D66" s="36">
-        <v>140.51647056125293</v>
+        <v>140.51012885766744</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -4425,13 +4427,13 @@
         <v>44348</v>
       </c>
       <c r="B67" s="17">
-        <v>148.97961710860557</v>
+        <v>148.97961710860534</v>
       </c>
       <c r="C67" s="36">
-        <v>141.53534399340631</v>
+        <v>141.49305609851737</v>
       </c>
       <c r="D67" s="36">
-        <v>141.35549240580593</v>
+        <v>141.35688684818371</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -4439,13 +4441,13 @@
         <v>44378</v>
       </c>
       <c r="B68" s="17">
-        <v>142.42591306097327</v>
+        <v>142.42591306097313</v>
       </c>
       <c r="C68" s="36">
-        <v>141.33257195041091</v>
+        <v>141.35152150148488</v>
       </c>
       <c r="D68" s="36">
-        <v>142.25463334833978</v>
+        <v>142.26480880715039</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -4453,13 +4455,13 @@
         <v>44409</v>
       </c>
       <c r="B69" s="17">
-        <v>140.9749407280367</v>
+        <v>140.9749407280365</v>
       </c>
       <c r="C69" s="36">
-        <v>143.26416810434233</v>
+        <v>143.26893353155685</v>
       </c>
       <c r="D69" s="36">
-        <v>143.21562429899168</v>
+        <v>143.23311468502996</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -4467,13 +4469,13 @@
         <v>44440</v>
       </c>
       <c r="B70" s="17">
-        <v>141.2960890894098</v>
+        <v>141.29608908940958</v>
       </c>
       <c r="C70" s="36">
-        <v>144.02331302778106</v>
+        <v>144.12924670258064</v>
       </c>
       <c r="D70" s="36">
-        <v>144.23310771308283</v>
+        <v>144.25466621351507</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -4481,13 +4483,13 @@
         <v>44470</v>
       </c>
       <c r="B71" s="17">
-        <v>139.51475869689307</v>
+        <v>139.51475869689278</v>
       </c>
       <c r="C71" s="36">
-        <v>143.40092987390815</v>
+        <v>143.42130203769142</v>
       </c>
       <c r="D71" s="36">
-        <v>145.29515450919925</v>
+        <v>145.31658660175071</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -4495,13 +4497,13 @@
         <v>44501</v>
       </c>
       <c r="B72" s="17">
-        <v>143.75187761771429</v>
+        <v>143.75187761771406</v>
       </c>
       <c r="C72" s="36">
-        <v>145.89876196548934</v>
+        <v>145.84431289987916</v>
       </c>
       <c r="D72" s="36">
-        <v>146.37689934669191</v>
+        <v>146.39426304865009</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -4509,13 +4511,13 @@
         <v>44531</v>
       </c>
       <c r="B73" s="17">
-        <v>147.22987832209441</v>
+        <v>147.22987832209424</v>
       </c>
       <c r="C73" s="36">
-        <v>149.69332822431508</v>
+        <v>149.85614630222497</v>
       </c>
       <c r="D73" s="36">
-        <v>147.44067363818939</v>
+        <v>147.45113221744668</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -4526,10 +4528,10 @@
         <v>139.63796162489982</v>
       </c>
       <c r="C74" s="36">
-        <v>148.25393324162565</v>
+        <v>148.53342518810345</v>
       </c>
       <c r="D74" s="36">
-        <v>148.44293480400648</v>
+        <v>148.44505029148579</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -4537,13 +4539,13 @@
         <v>44593</v>
       </c>
       <c r="B75" s="17">
-        <v>137.84951353039492</v>
+        <v>137.8495135303948</v>
       </c>
       <c r="C75" s="36">
-        <v>150.74905390996096</v>
+        <v>150.74492398940484</v>
       </c>
       <c r="D75" s="36">
-        <v>149.33967081502831</v>
+        <v>149.3323280608528</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -4551,13 +4553,13 @@
         <v>44621</v>
       </c>
       <c r="B76" s="17">
-        <v>153.93085077631551</v>
+        <v>153.93085077631505</v>
       </c>
       <c r="C76" s="36">
-        <v>150.53878659862093</v>
+        <v>150.39127357945512</v>
       </c>
       <c r="D76" s="36">
-        <v>150.09051948711567</v>
+        <v>150.0754352569179</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -4565,13 +4567,13 @@
         <v>44652</v>
       </c>
       <c r="B77" s="17">
-        <v>157.66169211629463</v>
+        <v>157.66169211629364</v>
       </c>
       <c r="C77" s="36">
-        <v>152.03583935458209</v>
+        <v>151.97961391938657</v>
       </c>
       <c r="D77" s="36">
-        <v>150.66598837212686</v>
+        <v>150.64689924251402</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -4579,13 +4581,13 @@
         <v>44682</v>
       </c>
       <c r="B78" s="17">
-        <v>164.68936308999244</v>
+        <v>164.68936308999193</v>
       </c>
       <c r="C78" s="36">
-        <v>152.17839451373504</v>
+        <v>151.99823712672884</v>
       </c>
       <c r="D78" s="36">
-        <v>151.04875880297126</v>
+        <v>151.03010399627965</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -4593,13 +4595,13 @@
         <v>44713</v>
       </c>
       <c r="B79" s="17">
-        <v>161.45483436245701</v>
+        <v>161.45483436245786</v>
       </c>
       <c r="C79" s="36">
-        <v>154.14485575373874</v>
+        <v>154.17057671019109</v>
       </c>
       <c r="D79" s="36">
-        <v>151.23555238684673</v>
+        <v>151.22061177468228</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -4607,13 +4609,13 @@
         <v>44743</v>
       </c>
       <c r="B80" s="17">
-        <v>152.44538769471595</v>
+        <v>152.44538769471922</v>
       </c>
       <c r="C80" s="36">
-        <v>152.47891898224907</v>
+        <v>152.4843590272539</v>
       </c>
       <c r="D80" s="36">
-        <v>151.24029427871656</v>
+        <v>151.23089937815624</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4621,13 +4623,13 @@
         <v>44774</v>
       </c>
       <c r="B81" s="17">
-        <v>151.46573902517829</v>
+        <v>151.46573902517952</v>
       </c>
       <c r="C81" s="36">
-        <v>151.65757904386837</v>
+        <v>151.6948373531994</v>
       </c>
       <c r="D81" s="36">
-        <v>151.09123715918429</v>
+        <v>151.08703011796365</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4635,13 +4637,13 @@
         <v>44805</v>
       </c>
       <c r="B82" s="17">
-        <v>149.17434933731033</v>
+        <v>149.17434933730516</v>
       </c>
       <c r="C82" s="36">
-        <v>150.76946986790088</v>
+        <v>150.78862727184716</v>
       </c>
       <c r="D82" s="36">
-        <v>150.82557137519984</v>
+        <v>150.82433398583012</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4649,13 +4651,13 @@
         <v>44835</v>
       </c>
       <c r="B83" s="17">
-        <v>146.55439498929425</v>
+        <v>146.55439498927831</v>
       </c>
       <c r="C83" s="36">
-        <v>149.29210589362691</v>
+        <v>149.26291297659591</v>
       </c>
       <c r="D83" s="36">
-        <v>150.4839717644017</v>
+        <v>150.48208706226896</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4663,13 +4665,13 @@
         <v>44866</v>
       </c>
       <c r="B84" s="17">
-        <v>148.03049443531322</v>
+        <v>148.03049443530639</v>
       </c>
       <c r="C84" s="36">
-        <v>148.59272305832613</v>
+        <v>148.50744581790943</v>
       </c>
       <c r="D84" s="36">
-        <v>150.10423203431668</v>
+        <v>150.09803027790036</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -4677,13 +4679,13 @@
         <v>44896</v>
       </c>
       <c r="B85" s="17">
-        <v>146.18080800458125</v>
+        <v>146.18080800460334</v>
       </c>
       <c r="C85" s="36">
-        <v>148.38372874076049</v>
+        <v>148.51915601579663</v>
       </c>
       <c r="D85" s="36">
-        <v>149.71925893214558</v>
+        <v>149.70569583590233</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -4691,13 +4693,13 @@
         <v>44927</v>
       </c>
       <c r="B86" s="17">
-        <v>143.03019028680231</v>
+        <v>143.03019028687322</v>
       </c>
       <c r="C86" s="36">
-        <v>149.42540329357686</v>
+        <v>149.68781431945897</v>
       </c>
       <c r="D86" s="36">
-        <v>149.35136782035747</v>
+        <v>149.32875801936962</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4705,13 +4707,13 @@
         <v>44958</v>
       </c>
       <c r="B87" s="17">
-        <v>137.26202711164171</v>
+        <v>137.26202711167147</v>
       </c>
       <c r="C87" s="36">
-        <v>149.80041668986829</v>
+        <v>149.83792215936882</v>
       </c>
       <c r="D87" s="36">
-        <v>149.0095174095525</v>
+        <v>148.97776846074467</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -4719,13 +4721,13 @@
         <v>44986</v>
       </c>
       <c r="B88" s="17">
-        <v>155.06056763777909</v>
+        <v>155.06056763767785</v>
       </c>
       <c r="C88" s="36">
-        <v>150.94516549298999</v>
+        <v>150.72559893860952</v>
       </c>
       <c r="D88" s="36">
-        <v>148.68844544834684</v>
+        <v>148.64892451373936</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -4733,13 +4735,13 @@
         <v>45017</v>
       </c>
       <c r="B89" s="17">
-        <v>150.02108492570758</v>
+        <v>150.02108492538545</v>
       </c>
       <c r="C89" s="36">
-        <v>147.40208090995787</v>
+        <v>147.35345724832627</v>
       </c>
       <c r="D89" s="36">
-        <v>148.37307500824281</v>
+        <v>148.32823404015883</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4747,13 +4749,13 @@
         <v>45047</v>
       </c>
       <c r="B90" s="17">
-        <v>153.77240570488985</v>
+        <v>153.77240570475391</v>
       </c>
       <c r="C90" s="36">
-        <v>145.7072010721923</v>
+        <v>145.65274008781518</v>
       </c>
       <c r="D90" s="36">
-        <v>148.04177512445932</v>
+        <v>147.99392557318464</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4761,13 +4763,13 @@
         <v>45078</v>
       </c>
       <c r="B91" s="17">
-        <v>152.55703188407324</v>
+        <v>152.55703188453069</v>
       </c>
       <c r="C91" s="36">
-        <v>146.22441998890517</v>
+        <v>146.23462401232104</v>
       </c>
       <c r="D91" s="36">
-        <v>147.67373495905306</v>
+        <v>147.62575922056891</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -4775,13 +4777,13 @@
         <v>45108</v>
       </c>
       <c r="B92" s="17">
-        <v>150.22297368785945</v>
+        <v>150.22297368931731</v>
       </c>
       <c r="C92" s="36">
-        <v>148.73770721655438</v>
+        <v>148.72524080197135</v>
       </c>
       <c r="D92" s="36">
-        <v>147.25561082099853</v>
+        <v>147.21026171068672</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -4789,13 +4791,13 @@
         <v>45139</v>
       </c>
       <c r="B93" s="17">
-        <v>151.94203814879756</v>
+        <v>151.94203814941196</v>
       </c>
       <c r="C93" s="36">
-        <v>150.0818844307978</v>
+        <v>150.00726396900734</v>
       </c>
       <c r="D93" s="36">
-        <v>146.78226017689644</v>
+        <v>146.74203556750248</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -4803,13 +4805,13 @@
         <v>45170</v>
       </c>
       <c r="B94" s="17">
-        <v>148.4322432701974</v>
+        <v>148.43224326812449</v>
       </c>
       <c r="C94" s="36">
-        <v>149.58382718498399</v>
+        <v>149.59810584615002</v>
       </c>
       <c r="D94" s="36">
-        <v>146.26176608811957</v>
+        <v>146.22865310169632</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4817,13 +4819,13 @@
         <v>45200</v>
       </c>
       <c r="B95" s="17">
-        <v>147.50696066044537</v>
+        <v>147.50696065384125</v>
       </c>
       <c r="C95" s="36">
-        <v>148.22226335986232</v>
+        <v>148.12592076567134</v>
       </c>
       <c r="D95" s="36">
-        <v>145.71558877455374</v>
+        <v>145.69121385227334</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -4831,13 +4833,13 @@
         <v>45231</v>
       </c>
       <c r="B96" s="17">
-        <v>146.35949533183793</v>
+        <v>146.35949532905394</v>
       </c>
       <c r="C96" s="36">
-        <v>146.58267269019237</v>
+        <v>146.56608348557839</v>
       </c>
       <c r="D96" s="36">
-        <v>145.17544035724288</v>
+        <v>145.16023078157343</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -4845,13 +4847,13 @@
         <v>45261</v>
       </c>
       <c r="B97" s="17">
-        <v>139.33576576518632</v>
+        <v>139.33576577457379</v>
       </c>
       <c r="C97" s="36">
-        <v>142.78974205810835</v>
+        <v>142.98801277026385</v>
       </c>
       <c r="D97" s="36">
-        <v>144.68575924389799</v>
+        <v>144.67835644481076</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -4859,13 +4861,13 @@
         <v>45292</v>
       </c>
       <c r="B98" s="17">
-        <v>137.54602735591297</v>
+        <v>137.54602738582324</v>
       </c>
       <c r="C98" s="36">
-        <v>143.48265454112794</v>
+        <v>143.73002234447563</v>
       </c>
       <c r="D98" s="36">
-        <v>144.29356237988557</v>
+        <v>144.29285443638179</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4873,13 +4875,13 @@
         <v>45323</v>
       </c>
       <c r="B99" s="17">
-        <v>133.63722384206051</v>
+        <v>133.6372238546686</v>
       </c>
       <c r="C99" s="36">
-        <v>144.05255219339068</v>
+        <v>143.96637419864555</v>
       </c>
       <c r="D99" s="36">
-        <v>144.04387119805276</v>
+        <v>144.04879155920639</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4887,13 +4889,13 @@
         <v>45352</v>
       </c>
       <c r="B100" s="17">
-        <v>142.56862052019582</v>
+        <v>142.56862047767686</v>
       </c>
       <c r="C100" s="36">
-        <v>142.90254208524681</v>
+        <v>142.54642488874453</v>
       </c>
       <c r="D100" s="36">
-        <v>143.97650870009548</v>
+        <v>143.98450504657345</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4901,13 +4903,13 @@
         <v>45383</v>
       </c>
       <c r="B101" s="17">
-        <v>147.26512454856004</v>
+        <v>147.26512441308907</v>
       </c>
       <c r="C101" s="36">
-        <v>140.96025044219942</v>
+        <v>140.92368699921087</v>
       </c>
       <c r="D101" s="36">
-        <v>144.11805717758716</v>
+        <v>144.12236109978107</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4915,13 +4917,13 @@
         <v>45413</v>
       </c>
       <c r="B102" s="17">
-        <v>156.7765837615064</v>
+        <v>156.77658370440048</v>
       </c>
       <c r="C102" s="36">
-        <v>142.54498400140477</v>
+        <v>142.63883411487311</v>
       </c>
       <c r="D102" s="36">
-        <v>144.47473787248018</v>
+        <v>144.46546086249469</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4929,13 +4931,13 @@
         <v>45444</v>
       </c>
       <c r="B103" s="17">
-        <v>147.36516936817389</v>
+        <v>147.3651695607501</v>
       </c>
       <c r="C103" s="36">
-        <v>143.54731240058413</v>
+        <v>143.75498601431281</v>
       </c>
       <c r="D103" s="36">
-        <v>145.03374266011252</v>
+        <v>144.99937183784681</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -4943,13 +4945,13 @@
         <v>45474</v>
       </c>
       <c r="B104" s="17">
-        <v>149.69752697536458</v>
+        <v>149.69752758894006</v>
       </c>
       <c r="C104" s="36">
-        <v>147.40216831223594</v>
+        <v>147.37653414122337</v>
       </c>
       <c r="D104" s="36">
-        <v>145.75946892808861</v>
+        <v>145.69208574365354</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -4957,13 +4959,13 @@
         <v>45505</v>
       </c>
       <c r="B105" s="17">
-        <v>147.32757348272975</v>
+        <v>147.32757374137327</v>
       </c>
       <c r="C105" s="36">
-        <v>148.11129841137603</v>
+        <v>147.97373835224366</v>
       </c>
       <c r="D105" s="36">
-        <v>146.60018857621711</v>
+        <v>146.4971186597223</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -4971,13 +4973,13 @@
         <v>45536</v>
       </c>
       <c r="B106" s="17">
-        <v>144.84378302186047</v>
+        <v>144.84378214964087</v>
       </c>
       <c r="C106" s="36">
-        <v>147.99505772220581</v>
+        <v>147.87078603835897</v>
       </c>
       <c r="D106" s="36">
-        <v>147.4957731698471</v>
+        <v>147.35997551702889</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -4985,13 +4987,13 @@
         <v>45566</v>
       </c>
       <c r="B107" s="17">
-        <v>147.99466238363041</v>
+        <v>147.99465960461652</v>
       </c>
       <c r="C107" s="36">
-        <v>148.99241120605578</v>
+        <v>148.91795097219361</v>
       </c>
       <c r="D107" s="36">
-        <v>148.38637355757476</v>
+        <v>148.22409664481577</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -4999,13 +5001,13 @@
         <v>45597</v>
       </c>
       <c r="B108" s="17">
-        <v>148.06937483613993</v>
+        <v>148.0693736646877</v>
       </c>
       <c r="C108" s="36">
-        <v>150.61267185225518</v>
+        <v>150.67943730794542</v>
       </c>
       <c r="D108" s="36">
-        <v>149.21958681063214</v>
+        <v>149.03951205065769</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -5013,13 +5015,13 @@
         <v>45627</v>
       </c>
       <c r="B109" s="17">
-        <v>148.56734190911206</v>
+        <v>148.56734585957747</v>
       </c>
       <c r="C109" s="36">
-        <v>151.05510881031032</v>
+        <v>151.28023662248589</v>
       </c>
       <c r="D109" s="36">
-        <v>149.95705141918856</v>
+        <v>149.76658666379012</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -5027,13 +5029,13 @@
         <v>45658</v>
       </c>
       <c r="B110" s="17">
-        <v>146.29580174387476</v>
+        <v>146.29581433061375</v>
       </c>
       <c r="C110" s="36">
-        <v>151.5018205088835</v>
+        <v>151.60733019823945</v>
       </c>
       <c r="D110" s="36">
-        <v>150.57471839371709</v>
+        <v>150.3790598898201</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -5041,13 +5043,13 @@
         <v>45689</v>
       </c>
       <c r="B111" s="17">
-        <v>141.2021694522208</v>
+        <v>141.20217475797378</v>
       </c>
       <c r="C111" s="36">
-        <v>153.43664475077557</v>
+        <v>153.28126184011842</v>
       </c>
       <c r="D111" s="36">
-        <v>151.064343973592</v>
+        <v>150.86631214680529</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -5055,13 +5057,13 @@
         <v>45717</v>
       </c>
       <c r="B112" s="17">
-        <v>150.40655910972941</v>
+        <v>150.40654121723682</v>
       </c>
       <c r="C112" s="36">
-        <v>150.37259728192413</v>
+        <v>149.72690968302643</v>
       </c>
       <c r="D112" s="36">
-        <v>151.43218413570568</v>
+        <v>151.23364216518962</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -5069,13 +5071,13 @@
         <v>45748</v>
       </c>
       <c r="B113" s="17">
-        <v>158.74110296645111</v>
+        <v>158.7410459584533</v>
       </c>
       <c r="C113" s="36">
-        <v>152.04459357205783</v>
+        <v>152.12611612616246</v>
       </c>
       <c r="D113" s="36">
-        <v>151.69557736720424</v>
+        <v>151.49744481721694</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -5083,13 +5085,13 @@
         <v>45778</v>
       </c>
       <c r="B114" s="17">
-        <v>164.8778979559678</v>
+        <v>164.8778739250919</v>
       </c>
       <c r="C114" s="36">
-        <v>151.67363016442619</v>
+        <v>151.92223808290362</v>
       </c>
       <c r="D114" s="36">
-        <v>151.87853516462113</v>
+        <v>151.68726574738375</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -5097,13 +5099,13 @@
         <v>45809</v>
       </c>
       <c r="B115" s="17">
-        <v>156.59401884940311</v>
+        <v>156.59409988827613</v>
       </c>
       <c r="C115" s="36">
-        <v>151.14346036788424</v>
+        <v>151.45990022602729</v>
       </c>
       <c r="D115" s="36">
-        <v>152.00690826247319</v>
+        <v>151.83958460765547</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -5111,13 +5113,13 @@
         <v>45839</v>
       </c>
       <c r="B116" s="17">
-        <v>153.90772081429063</v>
+        <v>153.90797901553967</v>
       </c>
       <c r="C116" s="36">
-        <v>151.4558141653047</v>
+        <v>151.39642049120224</v>
       </c>
       <c r="D116" s="36">
-        <v>152.10424327522946</v>
+        <v>151.99402999523531</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -5125,13 +5127,13 @@
         <v>45870</v>
       </c>
       <c r="B117" s="17">
-        <v>150.51256572733467</v>
+        <v>150.51267456824078</v>
       </c>
       <c r="C117" s="36">
-        <v>152.57027083830084</v>
+        <v>152.35274901258254</v>
       </c>
       <c r="D117" s="36">
-        <v>152.1874781401736</v>
+        <v>152.18345397817774</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -5139,13 +5141,13 @@
         <v>45901</v>
       </c>
       <c r="B118" s="17">
-        <v>151.83984439466224</v>
+        <v>151.83947735250638</v>
       </c>
       <c r="C118" s="36">
-        <v>153.53767342984943</v>
+        <v>153.34133826499504</v>
       </c>
       <c r="D118" s="36">
-        <v>152.26910227199022</v>
+        <v>152.43339517408262</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -5153,13 +5155,13 @@
         <v>45931</v>
       </c>
       <c r="B119" s="17">
-        <v>152.56798377141189</v>
+        <v>152.56490425090988</v>
       </c>
       <c r="C119" s="36">
-        <v>152.71748568104624</v>
+        <v>152.74008837138231</v>
       </c>
       <c r="D119" s="36">
-        <v>152.35630280996764</v>
+        <v>152.7594881325218</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -5167,13 +5169,13 @@
         <v>45962</v>
       </c>
       <c r="B120" s="17">
-        <v>147.69977298929118</v>
+        <v>147.69599372441905</v>
       </c>
       <c r="C120" s="36">
-        <v>152.54463449254752</v>
+        <v>152.68704430271981</v>
       </c>
       <c r="D120" s="36">
-        <v>152.45253676119401</v>
+        <v>153.17608301339749</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -5181,13 +5183,13 @@
         <v>45992</v>
       </c>
       <c r="B121" s="17">
-        <v>153.51436161199129</v>
+        <v>153.5212203973648</v>
       </c>
       <c r="C121" s="36">
-        <v>155.16117433523141</v>
+        <v>155.5184030224774</v>
       </c>
       <c r="D121" s="36">
-        <v>152.55859752385459</v>
+        <v>153.68628115401089</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -5195,27 +5197,41 @@
         <v>46023</v>
       </c>
       <c r="B122" s="17">
-        <v>148.78601868878062</v>
+        <v>148.55280173083167</v>
       </c>
       <c r="C122" s="36">
-        <v>155.70506528002818</v>
+        <v>155.16250785100169</v>
       </c>
       <c r="D122" s="36">
-        <v>152.67173720221635</v>
+        <v>154.27673098059162</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
         <v>46054</v>
       </c>
-      <c r="B123" s="41">
-        <v>138.20389337039899</v>
-      </c>
-      <c r="C123" s="42">
-        <v>151.68243919385438</v>
-      </c>
-      <c r="D123" s="42">
-        <v>152.7934630987927</v>
+      <c r="B123" s="17">
+        <v>138.34257152166515</v>
+      </c>
+      <c r="C123" s="36">
+        <v>151.03332855790745</v>
+      </c>
+      <c r="D123" s="36">
+        <v>154.9235774379822</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="4">
+        <v>46082</v>
+      </c>
+      <c r="B124" s="40">
+        <v>158.64871746521388</v>
+      </c>
+      <c r="C124" s="41">
+        <v>156.28980610599837</v>
+      </c>
+      <c r="D124" s="41">
+        <v>155.59922265893965</v>
       </c>
     </row>
   </sheetData>
@@ -7347,7 +7363,7 @@
       <c r="D78" s="10">
         <v>703987.50432157726</v>
       </c>
-      <c r="E78" s="39"/>
+      <c r="E78" s="38"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="10">
@@ -7362,7 +7378,7 @@
       <c r="D79" s="10">
         <v>737941.90937407222</v>
       </c>
-      <c r="E79" s="40"/>
+      <c r="E79" s="39"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="10">
@@ -7377,7 +7393,7 @@
       <c r="D80" s="10">
         <v>728638.58456868224</v>
       </c>
-      <c r="E80" s="40"/>
+      <c r="E80" s="39"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="10">
@@ -7523,14 +7539,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50" t="s">
+      <c r="C1" s="46"/>
+      <c r="D1" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="50"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8129,14 +8145,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="50" t="s">
+      <c r="B1" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50" t="s">
+      <c r="C1" s="46"/>
+      <c r="D1" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="50"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8307,390 +8323,390 @@
       <c r="A2" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="47">
-        <v>3642.0849776</v>
-      </c>
-      <c r="C2" s="47">
-        <v>4599.8744133099999</v>
+      <c r="B2" s="50">
+        <v>5184.6761268600003</v>
+      </c>
+      <c r="C2" s="50">
+        <v>6475.4953001000003</v>
       </c>
       <c r="D2" s="27">
         <f>B2-C2</f>
-        <v>-957.78943570999991</v>
+        <v>-1290.8191732400001</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
         <v>203</v>
       </c>
-      <c r="B3" s="48">
-        <v>2720.7819912800001</v>
-      </c>
-      <c r="C3" s="48">
-        <v>3534.7605033300001</v>
+      <c r="B3" s="44">
+        <v>3881.9424336900001</v>
+      </c>
+      <c r="C3" s="44">
+        <v>4869.7790634499997</v>
       </c>
       <c r="D3" s="27">
         <f t="shared" ref="D3:D27" si="0">B3-C3</f>
-        <v>-813.97851205000006</v>
+        <v>-987.8366297599996</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="B4" s="48">
-        <v>364.63594053000003</v>
-      </c>
-      <c r="C4" s="48">
-        <v>931.43666941000004</v>
+      <c r="B4" s="44">
+        <v>544.27488566</v>
+      </c>
+      <c r="C4" s="44">
+        <v>1418.5293560499999</v>
       </c>
       <c r="D4" s="27">
         <f t="shared" si="0"/>
-        <v>-566.80072887999995</v>
+        <v>-874.25447038999994</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="32" t="s">
         <v>209</v>
       </c>
-      <c r="B5" s="48">
-        <v>460.54735755000002</v>
-      </c>
-      <c r="C5" s="48">
-        <v>132.83453276</v>
+      <c r="B5" s="44">
+        <v>656.39092108</v>
+      </c>
+      <c r="C5" s="44">
+        <v>182.8138826</v>
       </c>
       <c r="D5" s="27">
         <f t="shared" si="0"/>
-        <v>327.71282479000001</v>
+        <v>473.57703848</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="47">
-        <v>2388.6359809800001</v>
-      </c>
-      <c r="C6" s="47">
-        <v>512.0873775</v>
+      <c r="B6" s="50">
+        <v>3791.6945303699999</v>
+      </c>
+      <c r="C6" s="50">
+        <v>724.91150055000003</v>
       </c>
       <c r="D6" s="27">
         <f t="shared" si="0"/>
-        <v>1876.5486034800001</v>
+        <v>3066.7830298199997</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="48">
-        <v>1250.9587038899999</v>
-      </c>
-      <c r="C7" s="48">
-        <v>224.68015249999999</v>
+      <c r="B7" s="44">
+        <v>2002.96056593</v>
+      </c>
+      <c r="C7" s="44">
+        <v>312.76053479000001</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" si="0"/>
-        <v>1026.2785513899998</v>
+        <v>1690.20003114</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="B8" s="48">
-        <v>562.35492280000005</v>
-      </c>
-      <c r="C8" s="48">
-        <v>77.517109989999994</v>
+      <c r="B8" s="44">
+        <v>919.74484351000001</v>
+      </c>
+      <c r="C8" s="44">
+        <v>101.28092606</v>
       </c>
       <c r="D8" s="27">
         <f t="shared" si="0"/>
-        <v>484.83781281000006</v>
+        <v>818.46391745000005</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="47">
-        <v>2729.4163217400001</v>
-      </c>
-      <c r="C9" s="47">
-        <v>1939.1563059800001</v>
+      <c r="B9" s="50">
+        <v>3758.7814747100001</v>
+      </c>
+      <c r="C9" s="50">
+        <v>2656.0205328400002</v>
       </c>
       <c r="D9" s="27">
         <f t="shared" si="0"/>
-        <v>790.26001575999999</v>
+        <v>1102.7609418699999</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="32" t="s">
         <v>205</v>
       </c>
-      <c r="B10" s="48">
-        <v>2201.7723591099998</v>
-      </c>
-      <c r="C10" s="48">
-        <v>1423.8317548</v>
+      <c r="B10" s="44">
+        <v>3093.8091247900002</v>
+      </c>
+      <c r="C10" s="44">
+        <v>1944.61581697</v>
       </c>
       <c r="D10" s="27">
         <f t="shared" si="0"/>
-        <v>777.9406043099998</v>
+        <v>1149.1933078200002</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="47">
-        <v>2022.88633052</v>
-      </c>
-      <c r="C11" s="47">
-        <v>2269.82641969</v>
+      <c r="B11" s="50">
+        <v>2696.2916236699998</v>
+      </c>
+      <c r="C11" s="50">
+        <v>3175.2879474699998</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" si="0"/>
-        <v>-246.94008916999996</v>
+        <v>-478.99632380000003</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="B12" s="48">
-        <v>277.89006107</v>
-      </c>
-      <c r="C12" s="48">
-        <v>681.23333489000004</v>
+      <c r="B12" s="44">
+        <v>394.86857359999999</v>
+      </c>
+      <c r="C12" s="44">
+        <v>976.53018064000003</v>
       </c>
       <c r="D12" s="27">
         <f t="shared" si="0"/>
-        <v>-403.34327382000004</v>
+        <v>-581.66160704000004</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="B13" s="48">
-        <v>278.63999637000001</v>
-      </c>
-      <c r="C13" s="48">
-        <v>263.91412875999998</v>
+      <c r="B13" s="44">
+        <v>361.77571188000002</v>
+      </c>
+      <c r="C13" s="44">
+        <v>356.04243484</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>14.725867610000023</v>
+        <v>5.7332770400000186</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="32" t="s">
         <v>214</v>
       </c>
-      <c r="B14" s="48">
-        <v>237.14646142000001</v>
-      </c>
-      <c r="C14" s="48">
-        <v>339.50689375000002</v>
+      <c r="B14" s="44">
+        <v>338.1297313</v>
+      </c>
+      <c r="C14" s="44">
+        <v>474.72158265000002</v>
       </c>
       <c r="D14" s="27">
         <f t="shared" si="0"/>
-        <v>-102.36043233000001</v>
+        <v>-136.59185135000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="B15" s="48">
-        <v>413.70484536999999</v>
-      </c>
-      <c r="C15" s="48">
-        <v>88.700274840000006</v>
+      <c r="B15" s="44">
+        <v>519.41292650000003</v>
+      </c>
+      <c r="C15" s="44">
+        <v>118.96263156000001</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>325.00457052999997</v>
+        <v>400.45029494000005</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="47">
-        <v>1770.36411421</v>
-      </c>
-      <c r="C16" s="47">
-        <v>3968.8562505</v>
+      <c r="B16" s="50">
+        <v>2432.6926104700001</v>
+      </c>
+      <c r="C16" s="50">
+        <v>5331.43500477</v>
       </c>
       <c r="D16" s="27">
         <f t="shared" si="0"/>
-        <v>-2198.49213629</v>
+        <v>-2898.7423942999999</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="47">
-        <v>1391.42497028</v>
-      </c>
-      <c r="C17" s="47">
-        <v>268.57025942000001</v>
+      <c r="B17" s="50">
+        <v>1936.3140979</v>
+      </c>
+      <c r="C17" s="50">
+        <v>358.63840901999998</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>1122.8547108600001</v>
+        <v>1577.6756888800001</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="B18" s="47">
-        <v>2157.6283789899999</v>
-      </c>
-      <c r="C18" s="47">
-        <v>974.11695552000003</v>
+      <c r="B18" s="50">
+        <v>3066.0885129500002</v>
+      </c>
+      <c r="C18" s="50">
+        <v>1351.3170497000001</v>
       </c>
       <c r="D18" s="27">
         <f t="shared" si="0"/>
-        <v>1183.51142347</v>
+        <v>1714.7714632500001</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="B19" s="48">
-        <v>490.57319502000001</v>
-      </c>
-      <c r="C19" s="48">
-        <v>103.15499242</v>
+      <c r="B19" s="44">
+        <v>580.35008919999996</v>
+      </c>
+      <c r="C19" s="44">
+        <v>140.81583347</v>
       </c>
       <c r="D19" s="27">
         <f t="shared" si="0"/>
-        <v>387.41820260000003</v>
+        <v>439.53425572999993</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="32" t="s">
         <v>210</v>
       </c>
-      <c r="B20" s="48">
-        <v>362.31211113000001</v>
-      </c>
-      <c r="C20" s="48">
-        <v>58.630448039999997</v>
+      <c r="B20" s="44">
+        <v>491.55269398000002</v>
+      </c>
+      <c r="C20" s="44">
+        <v>77.285400809999999</v>
       </c>
       <c r="D20" s="27">
         <f t="shared" si="0"/>
-        <v>303.68166309000003</v>
+        <v>414.26729317000002</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="32" t="s">
         <v>211</v>
       </c>
-      <c r="B21" s="48">
-        <v>259.28664493000002</v>
-      </c>
-      <c r="C21" s="48">
-        <v>479.11093283999998</v>
+      <c r="B21" s="44">
+        <v>456.01074598999998</v>
+      </c>
+      <c r="C21" s="44">
+        <v>702.65775033</v>
       </c>
       <c r="D21" s="27">
         <f t="shared" si="0"/>
-        <v>-219.82428790999995</v>
+        <v>-246.64700434000002</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="B22" s="48">
-        <v>946.51444658000003</v>
-      </c>
-      <c r="C22" s="48">
-        <v>258.31680581000001</v>
+      <c r="B22" s="44">
+        <v>1307.38461674</v>
+      </c>
+      <c r="C22" s="44">
+        <v>325.75798890999999</v>
       </c>
       <c r="D22" s="27">
         <f t="shared" si="0"/>
-        <v>688.19764077000002</v>
+        <v>981.62662782999996</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="47">
-        <v>1223.20827323</v>
-      </c>
-      <c r="C23" s="47">
-        <v>72.228760469999997</v>
+      <c r="B23" s="50">
+        <v>1637.3744370700001</v>
+      </c>
+      <c r="C23" s="50">
+        <v>135.66836939999999</v>
       </c>
       <c r="D23" s="27">
         <f t="shared" si="0"/>
-        <v>1150.97951276</v>
+        <v>1501.70606767</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="47">
-        <v>1114.49011032</v>
-      </c>
-      <c r="C24" s="47">
-        <v>100.81333033999999</v>
+      <c r="B24" s="50">
+        <v>1632.70905315</v>
+      </c>
+      <c r="C24" s="50">
+        <v>144.31502965000001</v>
       </c>
       <c r="D24" s="27">
         <f t="shared" si="0"/>
-        <v>1013.67677998</v>
+        <v>1488.3940235</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B25" s="47">
-        <v>87.561110220000003</v>
-      </c>
-      <c r="C25" s="47">
-        <v>69.144815120000004</v>
+      <c r="B25" s="50">
+        <v>105.55805049999999</v>
+      </c>
+      <c r="C25" s="50">
+        <v>82.387265009999993</v>
       </c>
       <c r="D25" s="27">
         <f t="shared" si="0"/>
-        <v>18.416295099999999</v>
+        <v>23.17078549</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B26" s="47">
-        <v>267.53786265999997</v>
-      </c>
-      <c r="C26" s="47">
-        <v>88.303249129999998</v>
+      <c r="B26" s="50">
+        <v>307.25023296000001</v>
+      </c>
+      <c r="C26" s="50">
+        <v>95.116376149999994</v>
       </c>
       <c r="D26" s="27">
         <f t="shared" si="0"/>
-        <v>179.23461352999999</v>
+        <v>212.13385681</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="49">
-        <v>3057.96917725</v>
-      </c>
-      <c r="C27" s="49">
-        <v>1482.1254346999999</v>
+      <c r="B27" s="51">
+        <v>4270.5155818599997</v>
+      </c>
+      <c r="C27" s="51">
+        <v>2012.0832006999999</v>
       </c>
       <c r="D27" s="27">
         <f t="shared" si="0"/>
-        <v>1575.8437425500001</v>
+        <v>2258.4323811599997</v>
       </c>
     </row>
   </sheetData>
@@ -8719,8 +8735,8 @@
       <c r="A2" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="43">
-        <v>21853.207608000001</v>
+      <c r="B2" s="42">
+        <v>30819.946332470001</v>
       </c>
       <c r="D2" s="29"/>
     </row>
@@ -8728,8 +8744,8 @@
       <c r="A3" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="B3" s="43">
-        <v>6178.6120975399999</v>
+      <c r="B3" s="42">
+        <v>8305.8466983399994</v>
       </c>
       <c r="D3" s="29"/>
     </row>
@@ -8737,8 +8753,8 @@
       <c r="A4" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="44">
-        <v>7.6568312000000001</v>
+      <c r="B4" s="43">
+        <v>10.89203902</v>
       </c>
       <c r="D4" s="30"/>
     </row>
@@ -8746,8 +8762,8 @@
       <c r="A5" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="44">
-        <v>630.60163469999998</v>
+      <c r="B5" s="43">
+        <v>814.48781841000005</v>
       </c>
       <c r="D5" s="30"/>
     </row>
@@ -8755,8 +8771,8 @@
       <c r="A6" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="44">
-        <v>73.900977810000001</v>
+      <c r="B6" s="43">
+        <v>113.90562789000001</v>
       </c>
       <c r="D6" s="30"/>
     </row>
@@ -8764,8 +8780,8 @@
       <c r="A7" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="44">
-        <v>218.82695206</v>
+      <c r="B7" s="43">
+        <v>278.24942086999999</v>
       </c>
       <c r="D7" s="30"/>
     </row>
@@ -8773,8 +8789,8 @@
       <c r="A8" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="44">
-        <v>135.64279291</v>
+      <c r="B8" s="43">
+        <v>208.38167605000001</v>
       </c>
       <c r="D8" s="30"/>
     </row>
@@ -8782,8 +8798,8 @@
       <c r="A9" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B9" s="44">
-        <v>3985.3623082200002</v>
+      <c r="B9" s="43">
+        <v>5394.4048729100004</v>
       </c>
       <c r="D9" s="30"/>
     </row>
@@ -8791,8 +8807,8 @@
       <c r="A10" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="44">
-        <v>671.06527274999996</v>
+      <c r="B10" s="43">
+        <v>875.40961866999999</v>
       </c>
       <c r="D10" s="30"/>
     </row>
@@ -8800,8 +8816,8 @@
       <c r="A11" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="B11" s="44">
-        <v>35.68106496</v>
+      <c r="B11" s="43">
+        <v>54.577805329999997</v>
       </c>
       <c r="D11" s="30"/>
     </row>
@@ -8809,8 +8825,8 @@
       <c r="A12" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="44">
-        <v>23.284074100000002</v>
+      <c r="B12" s="43">
+        <v>35.18868587</v>
       </c>
       <c r="D12" s="30"/>
     </row>
@@ -8818,8 +8834,8 @@
       <c r="A13" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="44">
-        <v>26.273295900000001</v>
+      <c r="B13" s="43">
+        <v>34.010485369999998</v>
       </c>
       <c r="D13" s="30"/>
     </row>
@@ -8827,8 +8843,8 @@
       <c r="A14" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B14" s="44">
-        <v>317.68720475999999</v>
+      <c r="B14" s="43">
+        <v>410.73184061000001</v>
       </c>
       <c r="D14" s="30"/>
     </row>
@@ -8836,8 +8852,8 @@
       <c r="A15" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="44">
-        <v>52.629688170000001</v>
+      <c r="B15" s="43">
+        <v>75.606807340000003</v>
       </c>
       <c r="D15" s="30"/>
     </row>
@@ -8845,8 +8861,8 @@
       <c r="A16" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B16" s="43">
-        <v>6750.0284991099998</v>
+      <c r="B16" s="42">
+        <v>9474.4234449699998</v>
       </c>
       <c r="D16" s="29"/>
     </row>
@@ -8854,8 +8870,8 @@
       <c r="A17" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="44">
-        <v>1218.1314355</v>
+      <c r="B17" s="43">
+        <v>1587.64833602</v>
       </c>
       <c r="D17" s="30"/>
     </row>
@@ -8863,8 +8879,8 @@
       <c r="A18" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="B18" s="44">
-        <v>67.614102810000006</v>
+      <c r="B18" s="43">
+        <v>91.181791079999996</v>
       </c>
       <c r="D18" s="30"/>
     </row>
@@ -8872,8 +8888,8 @@
       <c r="A19" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="44">
-        <v>365.08177555999998</v>
+      <c r="B19" s="43">
+        <v>482.15960007000001</v>
       </c>
       <c r="D19" s="30"/>
     </row>
@@ -8881,8 +8897,8 @@
       <c r="A20" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="B20" s="44">
-        <v>23.481003789999999</v>
+      <c r="B20" s="43">
+        <v>30.557581989999999</v>
       </c>
       <c r="D20" s="30"/>
     </row>
@@ -8890,8 +8906,8 @@
       <c r="A21" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="44">
-        <v>19.703430130000001</v>
+      <c r="B21" s="43">
+        <v>30.331268179999999</v>
       </c>
       <c r="D21" s="30"/>
     </row>
@@ -8899,8 +8915,8 @@
       <c r="A22" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="44">
-        <v>44.007000400000003</v>
+      <c r="B22" s="43">
+        <v>57.514141330000001</v>
       </c>
       <c r="D22" s="30"/>
     </row>
@@ -8908,8 +8924,8 @@
       <c r="A23" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B23" s="44">
-        <v>182.68527849</v>
+      <c r="B23" s="43">
+        <v>251.95402654</v>
       </c>
       <c r="D23" s="30"/>
     </row>
@@ -8917,8 +8933,8 @@
       <c r="A24" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="B24" s="44">
-        <v>2073.9789836800001</v>
+      <c r="B24" s="43">
+        <v>2982.6350197900001</v>
       </c>
       <c r="D24" s="30"/>
     </row>
@@ -8926,8 +8942,8 @@
       <c r="A25" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B25" s="44">
-        <v>106.14883974999999</v>
+      <c r="B25" s="43">
+        <v>134.31868901000001</v>
       </c>
       <c r="D25" s="30"/>
     </row>
@@ -8935,8 +8951,8 @@
       <c r="A26" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="B26" s="44">
-        <v>225.63479645999999</v>
+      <c r="B26" s="43">
+        <v>311.96963204999997</v>
       </c>
       <c r="D26" s="30"/>
     </row>
@@ -8944,8 +8960,8 @@
       <c r="A27" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="B27" s="44">
-        <v>175.96563567999999</v>
+      <c r="B27" s="43">
+        <v>244.79960692</v>
       </c>
       <c r="D27" s="30"/>
     </row>
@@ -8953,8 +8969,8 @@
       <c r="A28" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B28" s="44">
-        <v>1887.6847242900001</v>
+      <c r="B28" s="43">
+        <v>2772.0482953999999</v>
       </c>
       <c r="D28" s="30"/>
     </row>
@@ -8962,8 +8978,8 @@
       <c r="A29" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="44">
-        <v>71.754049539999997</v>
+      <c r="B29" s="43">
+        <v>97.348932500000004</v>
       </c>
       <c r="D29" s="30"/>
     </row>
@@ -8971,8 +8987,8 @@
       <c r="A30" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="B30" s="44">
-        <v>83.504218820000006</v>
+      <c r="B30" s="43">
+        <v>114.65787698</v>
       </c>
       <c r="D30" s="30"/>
     </row>
@@ -8980,8 +8996,8 @@
       <c r="A31" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="B31" s="44">
-        <v>29.34874619</v>
+      <c r="B31" s="43">
+        <v>45.24399777</v>
       </c>
       <c r="D31" s="30"/>
     </row>
@@ -8989,8 +9005,8 @@
       <c r="A32" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="B32" s="44">
-        <v>175.30447802</v>
+      <c r="B32" s="43">
+        <v>240.05464934</v>
       </c>
       <c r="D32" s="30"/>
     </row>
@@ -8998,8 +9014,8 @@
       <c r="A33" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="B33" s="43">
-        <v>6087.6302882800001</v>
+      <c r="B33" s="42">
+        <v>8618.14989522</v>
       </c>
       <c r="D33" s="29"/>
     </row>
@@ -9007,8 +9023,8 @@
       <c r="A34" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="B34" s="44">
-        <v>1333.9643457300001</v>
+      <c r="B34" s="43">
+        <v>1850.8001288</v>
       </c>
       <c r="D34" s="30"/>
     </row>
@@ -9016,8 +9032,8 @@
       <c r="A35" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B35" s="44">
-        <v>255.71772598000001</v>
+      <c r="B35" s="43">
+        <v>369.47668838999999</v>
       </c>
       <c r="D35" s="30"/>
     </row>
@@ -9025,8 +9041,8 @@
       <c r="A36" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="B36" s="44">
-        <v>38.354973569999999</v>
+      <c r="B36" s="43">
+        <v>54.008652999999995</v>
       </c>
       <c r="D36" s="30"/>
     </row>
@@ -9034,8 +9050,8 @@
       <c r="A37" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="B37" s="44">
-        <v>4.12255064</v>
+      <c r="B37" s="43">
+        <v>5.9253205600000003</v>
       </c>
       <c r="D37" s="30"/>
     </row>
@@ -9043,8 +9059,8 @@
       <c r="A38" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="B38" s="44">
-        <v>101.4539458</v>
+      <c r="B38" s="43">
+        <v>137.29049413000001</v>
       </c>
       <c r="D38" s="30"/>
     </row>
@@ -9052,8 +9068,8 @@
       <c r="A39" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B39" s="44">
-        <v>25.984441180000001</v>
+      <c r="B39" s="43">
+        <v>35.08370498</v>
       </c>
       <c r="D39" s="30"/>
     </row>
@@ -9061,8 +9077,8 @@
       <c r="A40" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="B40" s="44">
-        <v>1.9632358400000001</v>
+      <c r="B40" s="43">
+        <v>3.6218260999999998</v>
       </c>
       <c r="D40" s="30"/>
     </row>
@@ -9070,8 +9086,8 @@
       <c r="A41" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="44">
-        <v>31.65772419</v>
+      <c r="B41" s="43">
+        <v>43.316794899999998</v>
       </c>
       <c r="D41" s="30"/>
     </row>
@@ -9079,8 +9095,8 @@
       <c r="A42" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="B42" s="44">
-        <v>1587.7043686699999</v>
+      <c r="B42" s="43">
+        <v>2115.8855446100001</v>
       </c>
       <c r="D42" s="30"/>
     </row>
@@ -9088,8 +9104,8 @@
       <c r="A43" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B43" s="44">
-        <v>576.36516614000004</v>
+      <c r="B43" s="43">
+        <v>857.62822240000003</v>
       </c>
       <c r="D43" s="30"/>
     </row>
@@ -9097,8 +9113,8 @@
       <c r="A44" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="B44" s="44">
-        <v>294.64710724999998</v>
+      <c r="B44" s="43">
+        <v>409.68136580999999</v>
       </c>
       <c r="D44" s="30"/>
     </row>
@@ -9106,8 +9122,8 @@
       <c r="A45" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B45" s="44">
-        <v>1523.9142027800001</v>
+      <c r="B45" s="43">
+        <v>2376.4248511699998</v>
       </c>
       <c r="D45" s="30"/>
     </row>
@@ -9115,8 +9131,8 @@
       <c r="A46" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B46" s="44">
-        <v>44.361302100000003</v>
+      <c r="B46" s="43">
+        <v>55.773962580000003</v>
       </c>
       <c r="D46" s="30"/>
     </row>
@@ -9124,8 +9140,8 @@
       <c r="A47" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="B47" s="44">
-        <v>267.41919840999998</v>
+      <c r="B47" s="43">
+        <v>303.23233778999997</v>
       </c>
       <c r="D47" s="30"/>
     </row>
@@ -9133,8 +9149,8 @@
       <c r="A48" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="B48" s="43">
-        <v>2836.93672307</v>
+      <c r="B48" s="42">
+        <v>4421.52629394</v>
       </c>
       <c r="D48" s="29"/>
     </row>
@@ -9142,8 +9158,8 @@
       <c r="A49" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B49" s="44">
-        <v>1559.89458603</v>
+      <c r="B49" s="43">
+        <v>2600.5755681599999</v>
       </c>
       <c r="D49" s="30"/>
     </row>
@@ -9151,8 +9167,8 @@
       <c r="A50" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="B50" s="44">
-        <v>744.01471738999999</v>
+      <c r="B50" s="43">
+        <v>1066.8569785499999</v>
       </c>
       <c r="D50" s="30"/>
     </row>
@@ -9160,8 +9176,8 @@
       <c r="A51" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="B51" s="44">
-        <v>19.932383229999999</v>
+      <c r="B51" s="43">
+        <v>33.500615439999997</v>
       </c>
       <c r="D51" s="30"/>
     </row>
@@ -9169,8 +9185,8 @@
       <c r="A52" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="B52" s="45">
-        <v>388.92518603000002</v>
+      <c r="B52" s="44">
+        <v>555.05760665000003</v>
       </c>
       <c r="D52" s="30"/>
     </row>
@@ -9178,8 +9194,8 @@
       <c r="A53" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="B53" s="46">
-        <v>124.16985038999999</v>
+      <c r="B53" s="45">
+        <v>165.53552514</v>
       </c>
     </row>
   </sheetData>
@@ -9208,224 +9224,224 @@
       <c r="A2" s="33" t="s">
         <v>177</v>
       </c>
-      <c r="B2" s="29">
-        <v>16345.10357168</v>
+      <c r="B2" s="47">
+        <v>22542.675985360002</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="B3" s="29">
-        <v>3375.8426948000001</v>
+      <c r="B3" s="47">
+        <v>4517.7529110900005</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="B4" s="30">
-        <v>2486.7692147500002</v>
+      <c r="B4" s="48">
+        <v>3286.95681285</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="34" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="30">
-        <v>365.06772862000003</v>
+      <c r="B5" s="48">
+        <v>500.81195382999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="30">
-        <v>524.00575143000003</v>
+      <c r="B6" s="48">
+        <v>729.98414441</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="B7" s="29">
-        <v>5451.1590238500003</v>
+      <c r="B7" s="47">
+        <v>7697.9606936500004</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="30">
-        <v>846.49245704999998</v>
+      <c r="B8" s="48">
+        <v>1317.8545178899999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="34" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="30">
-        <v>136.29556653</v>
+      <c r="B9" s="48">
+        <v>173.75594677999999</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="30">
-        <v>244.10265992000001</v>
+      <c r="B10" s="48">
+        <v>335.70177479</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
         <v>186</v>
       </c>
-      <c r="B11" s="30">
-        <v>3733.1311068800001</v>
+      <c r="B11" s="48">
+        <v>5196.0503129199997</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B12" s="30">
-        <v>491.13723347000001</v>
+      <c r="B12" s="48">
+        <v>674.59814127000004</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="B13" s="29">
-        <v>431.66893614999998</v>
+      <c r="B13" s="47">
+        <v>577.55242461</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="B14" s="30">
-        <v>54.94351047</v>
+      <c r="B14" s="48">
+        <v>81.613303869999996</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="B15" s="30">
-        <v>376.72542568</v>
+      <c r="B15" s="48">
+        <v>495.93912074000002</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>191</v>
       </c>
-      <c r="B16" s="29">
-        <v>2894.3441279899998</v>
+      <c r="B16" s="47">
+        <v>4015.2040200599999</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="34" t="s">
         <v>192</v>
       </c>
-      <c r="B17" s="30">
-        <v>1133.9802706400001</v>
+      <c r="B17" s="48">
+        <v>1565.8439269099999</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="B18" s="30">
-        <v>187.76447163</v>
+      <c r="B18" s="48">
+        <v>230.57634225000001</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="B19" s="30">
-        <v>1572.5993857200001</v>
+      <c r="B19" s="48">
+        <v>2218.7837509000001</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
         <v>195</v>
       </c>
-      <c r="B20" s="29">
-        <v>2582.26003515</v>
+      <c r="B20" s="47">
+        <v>3560.55351277</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="34" t="s">
         <v>196</v>
       </c>
-      <c r="B21" s="30">
-        <v>218.70288993</v>
+      <c r="B21" s="48">
+        <v>292.28966401000002</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="34" t="s">
         <v>197</v>
       </c>
-      <c r="B22" s="30">
-        <v>348.41194282999999</v>
+      <c r="B22" s="48">
+        <v>489.37519828000001</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="34" t="s">
         <v>198</v>
       </c>
-      <c r="B23" s="30">
-        <v>194.14988503000001</v>
+      <c r="B23" s="48">
+        <v>286.98828068</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="34" t="s">
         <v>199</v>
       </c>
-      <c r="B24" s="30">
-        <v>272.65300049000001</v>
+      <c r="B24" s="48">
+        <v>366.13625930000001</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="34" t="s">
         <v>200</v>
       </c>
-      <c r="B25" s="30">
-        <v>725.11567094999998</v>
+      <c r="B25" s="48">
+        <v>985.58987013000001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="B26" s="30">
-        <v>437.15278225999998</v>
+      <c r="B26" s="48">
+        <v>614.21376779000002</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B27" s="30">
-        <v>386.07386365999997</v>
+      <c r="B27" s="48">
+        <v>525.96047257999999</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="B28" s="29">
-        <v>1313.11547008</v>
+      <c r="B28" s="47">
+        <v>1752.703162</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B29" s="38">
-        <v>296.71328366</v>
+      <c r="B29" s="49">
+        <v>420.94926118000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
"actualizo dato ipc mayo26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF46CD9E-DCF4-4787-AC76-52482510BCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0255C62E-AEB5-4449-BE0E-507DBB2C0604}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -994,9 +994,6 @@
     <xf numFmtId="3" fontId="11" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="169" fontId="12" fillId="5" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1008,6 +1005,9 @@
     </xf>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Euro" xfId="10" xr:uid="{8CA0DC4E-5AAC-43A0-AC51-59D877AC41AF}"/>
@@ -1339,7 +1339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H113"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="1" customWidth="1"/>
@@ -3267,6 +3267,23 @@
       </c>
       <c r="E113">
         <v>4.7</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="19">
+        <v>46143</v>
+      </c>
+      <c r="B114" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="C114">
+        <v>3.4</v>
+      </c>
+      <c r="D114">
+        <v>2.1</v>
+      </c>
+      <c r="E114">
+        <v>2.2999999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -5279,25 +5296,25 @@
         <v>112</v>
       </c>
       <c r="B2" s="37">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="C2" s="20">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="D2" s="20">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="E2" s="20">
-        <v>2.2000000000000002</v>
+        <v>2.8</v>
       </c>
       <c r="F2" s="20">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="G2" s="20">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="H2" s="16">
-        <v>2.355311683621486</v>
+        <v>2.683945290155676</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5305,25 +5322,25 @@
         <v>113</v>
       </c>
       <c r="B3" s="37">
-        <v>-0.2</v>
+        <v>0.2</v>
       </c>
       <c r="C3" s="20">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D3" s="20">
-        <v>2.2000000000000002</v>
+        <v>0.4</v>
       </c>
       <c r="E3" s="20">
-        <v>1.9</v>
+        <v>0.4</v>
       </c>
       <c r="F3" s="20">
-        <v>-1.2</v>
+        <v>-0.7</v>
       </c>
       <c r="G3" s="20">
-        <v>2.1</v>
+        <v>0.8</v>
       </c>
       <c r="H3" s="16">
-        <v>0.7135595105250081</v>
+        <v>0.30128929683261862</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5331,25 +5348,25 @@
         <v>114</v>
       </c>
       <c r="B4" s="37">
+        <v>3.6</v>
+      </c>
+      <c r="C4" s="20">
+        <v>2.8</v>
+      </c>
+      <c r="D4" s="20">
+        <v>3.1</v>
+      </c>
+      <c r="E4" s="20">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F4" s="20">
+        <v>3</v>
+      </c>
+      <c r="G4" s="20">
         <v>2.7</v>
       </c>
-      <c r="C4" s="20">
-        <v>3.1</v>
-      </c>
-      <c r="D4" s="20">
-        <v>3.5</v>
-      </c>
-      <c r="E4" s="20">
-        <v>2.6</v>
-      </c>
-      <c r="F4" s="20">
-        <v>2.7</v>
-      </c>
-      <c r="G4" s="20">
-        <v>2.5</v>
-      </c>
       <c r="H4" s="16">
-        <v>2.8197646065501569</v>
+        <v>3.1337998632663844</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5357,25 +5374,25 @@
         <v>115</v>
       </c>
       <c r="B5" s="37">
-        <v>2.7</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="C5" s="20">
-        <v>1.6</v>
+        <v>3.9</v>
       </c>
       <c r="D5" s="20">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E5" s="20">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="F5" s="20">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
       <c r="G5" s="20">
-        <v>2.9</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="H5" s="16">
-        <v>2.4095798995696471</v>
+        <v>3.7805313476907854</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5383,25 +5400,25 @@
         <v>116</v>
       </c>
       <c r="B6" s="37">
-        <v>-1.9</v>
+        <v>-5.9</v>
       </c>
       <c r="C6" s="20">
-        <v>-1.7</v>
+        <v>-5.2</v>
       </c>
       <c r="D6" s="20">
-        <v>-1.2</v>
+        <v>-2.2000000000000002</v>
       </c>
       <c r="E6" s="20">
-        <v>-3.5</v>
+        <v>-5.2</v>
       </c>
       <c r="F6" s="20">
-        <v>-4.3</v>
+        <v>-6.3</v>
       </c>
       <c r="G6" s="20">
-        <v>-3.5</v>
+        <v>-3.4</v>
       </c>
       <c r="H6" s="16">
-        <v>-2.109973494855677</v>
+        <v>-5.3366002898128091</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5409,25 +5426,25 @@
         <v>117</v>
       </c>
       <c r="B7" s="37">
-        <v>0.6</v>
+        <v>18.8</v>
       </c>
       <c r="C7" s="20">
-        <v>1.6</v>
+        <v>12.8</v>
       </c>
       <c r="D7" s="20">
-        <v>2.4</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="E7" s="20">
-        <v>-2.5</v>
+        <v>12.9</v>
       </c>
       <c r="F7" s="20">
-        <v>0.6</v>
+        <v>15.3</v>
       </c>
       <c r="G7" s="20">
-        <v>1.4</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="H7" s="16">
-        <v>0.80597515468512348</v>
+        <v>15.196813550847477</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5435,25 +5452,25 @@
         <v>118</v>
       </c>
       <c r="B8" s="37">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="C8" s="20">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="D8" s="20">
-        <v>3.2</v>
+        <v>4.2</v>
       </c>
       <c r="E8" s="20">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="F8" s="20">
-        <v>4.7</v>
+        <v>3.3</v>
       </c>
       <c r="G8" s="20">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="H8" s="16">
-        <v>3.2945735107216434</v>
+        <v>3.208517775489117</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5464,22 +5481,22 @@
         <v>2.1</v>
       </c>
       <c r="C9" s="20">
-        <v>1.3</v>
+        <v>2.5</v>
       </c>
       <c r="D9" s="20">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="E9" s="20">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="F9" s="20">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="G9" s="20">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="H9" s="16">
-        <v>1.7235024984266989</v>
+        <v>2.1193218367733468</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5487,25 +5504,25 @@
         <v>120</v>
       </c>
       <c r="B10" s="37">
-        <v>2.2999999999999998</v>
+        <v>2.7</v>
       </c>
       <c r="C10" s="20">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="D10" s="20">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="E10" s="20">
-        <v>2.8</v>
+        <v>1.7</v>
       </c>
       <c r="F10" s="20">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="G10" s="20">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="H10" s="16">
-        <v>2.5131961884953924</v>
+        <v>2.514344713912875</v>
       </c>
     </row>
   </sheetData>
@@ -5550,25 +5567,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="24">
+        <v>2.1</v>
+      </c>
+      <c r="C2" s="24">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D2" s="24">
+        <v>2</v>
+      </c>
+      <c r="E2" s="24">
         <v>2.6</v>
       </c>
-      <c r="C2" s="24">
-        <v>2.8</v>
-      </c>
-      <c r="D2" s="24">
-        <v>2.4</v>
-      </c>
-      <c r="E2" s="24">
-        <v>2.7</v>
-      </c>
       <c r="F2" s="24">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="G2" s="24">
         <v>2.1</v>
       </c>
       <c r="H2" s="24">
-        <v>2.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5576,25 +5593,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="22">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="C3" s="22">
-        <v>1.2</v>
+        <v>2.8</v>
       </c>
       <c r="D3" s="22">
-        <v>1.8</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="E3" s="22">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="F3" s="22">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="G3" s="22">
-        <v>0.4</v>
+        <v>1.9</v>
       </c>
       <c r="H3" s="22">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5602,25 +5619,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="22">
-        <v>1.9</v>
+        <v>0.8</v>
       </c>
       <c r="C4" s="22">
-        <v>2.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D4" s="22">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="E4" s="22">
-        <v>1.8</v>
+        <v>0.3</v>
       </c>
       <c r="F4" s="22">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="G4" s="22">
-        <v>2.2999999999999998</v>
+        <v>-0.2</v>
       </c>
       <c r="H4" s="22">
-        <v>2.2999999999999998</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5628,25 +5645,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="22">
-        <v>3.2</v>
+        <v>0.3</v>
       </c>
       <c r="C5" s="22">
-        <v>4.4000000000000004</v>
+        <v>-0.3</v>
       </c>
       <c r="D5" s="22">
-        <v>2.1</v>
+        <v>0.8</v>
       </c>
       <c r="E5" s="22">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="F5" s="22">
-        <v>2.4</v>
+        <v>0.3</v>
       </c>
       <c r="G5" s="22">
-        <v>3.1</v>
+        <v>0.5</v>
       </c>
       <c r="H5" s="22">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5654,25 +5671,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="22">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="C6" s="22">
-        <v>4.5999999999999996</v>
+        <v>1.8</v>
       </c>
       <c r="D6" s="22">
         <v>2.4</v>
       </c>
       <c r="E6" s="22">
-        <v>3.3</v>
+        <v>8.4</v>
       </c>
       <c r="F6" s="22">
+        <v>4</v>
+      </c>
+      <c r="G6" s="22">
         <v>3.7</v>
       </c>
-      <c r="G6" s="22">
-        <v>1.3</v>
-      </c>
       <c r="H6" s="22">
-        <v>3.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5680,25 +5697,25 @@
         <v>17</v>
       </c>
       <c r="B7" s="22">
-        <v>2.9</v>
+        <v>1.4</v>
       </c>
       <c r="C7" s="22">
-        <v>3.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D7" s="22">
-        <v>2.9</v>
+        <v>1.6</v>
       </c>
       <c r="E7" s="22">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="F7" s="22">
-        <v>2.2000000000000002</v>
+        <v>1.9</v>
       </c>
       <c r="G7" s="22">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="H7" s="22">
-        <v>3.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5706,7 +5723,7 @@
         <v>18</v>
       </c>
       <c r="B8" s="22">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="C8" s="22">
         <v>2.7</v>
@@ -5715,13 +5732,13 @@
         <v>2.5</v>
       </c>
       <c r="E8" s="22">
-        <v>2.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F8" s="22">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
       <c r="G8" s="22">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="H8" s="22">
         <v>2.2999999999999998</v>
@@ -5732,25 +5749,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="22">
-        <v>4.4000000000000004</v>
+        <v>2</v>
       </c>
       <c r="C9" s="22">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="D9" s="22">
-        <v>4.7</v>
+        <v>1.8</v>
       </c>
       <c r="E9" s="22">
-        <v>5.6</v>
+        <v>0.8</v>
       </c>
       <c r="F9" s="22">
-        <v>5.3</v>
+        <v>0.9</v>
       </c>
       <c r="G9" s="22">
-        <v>5.2</v>
+        <v>2.4</v>
       </c>
       <c r="H9" s="22">
-        <v>4.7</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5758,25 +5775,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="22">
-        <v>4.0999999999999996</v>
+        <v>3.4</v>
       </c>
       <c r="C10" s="22">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="D10" s="22">
-        <v>4.0999999999999996</v>
+        <v>2.9</v>
       </c>
       <c r="E10" s="22">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
       <c r="F10" s="22">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="G10" s="22">
-        <v>4.5</v>
+        <v>3.1</v>
       </c>
       <c r="H10" s="22">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -5784,25 +5801,25 @@
         <v>21</v>
       </c>
       <c r="B11" s="22">
-        <v>1</v>
+        <v>2.8</v>
       </c>
       <c r="C11" s="22">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="D11" s="22">
-        <v>0.1</v>
+        <v>2.6</v>
       </c>
       <c r="E11" s="22">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="F11" s="22">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
       <c r="G11" s="22">
-        <v>0.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="H11" s="22">
-        <v>1.1000000000000001</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -5810,25 +5827,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="22">
-        <v>4.2</v>
+        <v>2.9</v>
       </c>
       <c r="C12" s="22">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="D12" s="22">
-        <v>3.9</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E12" s="22">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="F12" s="22">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="G12" s="22">
-        <v>3.8</v>
+        <v>2.9</v>
       </c>
       <c r="H12" s="22">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -5836,25 +5853,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="22">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="C13" s="22">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="D13" s="22">
-        <v>2.6</v>
+        <v>1.3</v>
       </c>
       <c r="E13" s="22">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="F13" s="22">
-        <v>4.2</v>
+        <v>1.9</v>
       </c>
       <c r="G13" s="22">
-        <v>2.7</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H13" s="22">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -5865,22 +5882,22 @@
         <v>2.4</v>
       </c>
       <c r="C14" s="22">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="D14" s="22">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E14" s="22">
+        <v>2.4</v>
+      </c>
+      <c r="F14" s="22">
+        <v>2.8</v>
+      </c>
+      <c r="G14" s="22">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="H14" s="22">
         <v>1.9</v>
-      </c>
-      <c r="E14" s="22">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="F14" s="22">
-        <v>1.7</v>
-      </c>
-      <c r="G14" s="22">
-        <v>3.2</v>
-      </c>
-      <c r="H14" s="22">
-        <v>2.2999999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -5925,25 +5942,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="33">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="C2" s="33">
+        <v>33.6</v>
+      </c>
+      <c r="D2" s="33">
         <v>32.4</v>
       </c>
-      <c r="C2" s="33">
-        <v>32.6</v>
-      </c>
-      <c r="D2" s="33">
-        <v>31.9</v>
-      </c>
       <c r="E2" s="33">
-        <v>33.5</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="F2" s="33">
-        <v>32.1</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="G2" s="33">
-        <v>32.6</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="H2" s="33">
-        <v>32</v>
+        <v>32.200000000000003</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5951,25 +5968,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="34">
-        <v>30.9</v>
+        <v>33.4</v>
       </c>
       <c r="C3" s="34">
-        <v>30.4</v>
+        <v>33.5</v>
       </c>
       <c r="D3" s="34">
-        <v>31.1</v>
+        <v>33.4</v>
       </c>
       <c r="E3" s="34">
-        <v>36.299999999999997</v>
+        <v>38.200000000000003</v>
       </c>
       <c r="F3" s="34">
-        <v>32.200000000000003</v>
+        <v>34.1</v>
       </c>
       <c r="G3" s="34">
-        <v>32</v>
+        <v>33.5</v>
       </c>
       <c r="H3" s="34">
-        <v>26.2</v>
+        <v>27.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5977,25 +5994,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="34">
-        <v>23.8</v>
+        <v>24</v>
       </c>
       <c r="C4" s="34">
+        <v>24.4</v>
+      </c>
+      <c r="D4" s="34">
         <v>23.7</v>
       </c>
-      <c r="D4" s="34">
-        <v>23.5</v>
-      </c>
       <c r="E4" s="34">
-        <v>22.6</v>
+        <v>21.8</v>
       </c>
       <c r="F4" s="34">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="G4" s="34">
-        <v>24.5</v>
+        <v>23.6</v>
       </c>
       <c r="H4" s="34">
-        <v>26.6</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6003,25 +6020,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="34">
+        <v>12</v>
+      </c>
+      <c r="C5" s="34">
         <v>12.7</v>
       </c>
-      <c r="C5" s="34">
-        <v>13.3</v>
-      </c>
       <c r="D5" s="34">
-        <v>11.2</v>
+        <v>10.3</v>
       </c>
       <c r="E5" s="34">
-        <v>15.8</v>
+        <v>14.7</v>
       </c>
       <c r="F5" s="34">
-        <v>13.9</v>
+        <v>13</v>
       </c>
       <c r="G5" s="34">
-        <v>12.9</v>
+        <v>11.4</v>
       </c>
       <c r="H5" s="34">
-        <v>14.6</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -6029,25 +6046,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="34">
-        <v>47.8</v>
+        <v>48</v>
       </c>
       <c r="C6" s="34">
-        <v>45.5</v>
+        <v>43.9</v>
       </c>
       <c r="D6" s="34">
-        <v>48.2</v>
+        <v>48.7</v>
       </c>
       <c r="E6" s="34">
-        <v>56.4</v>
+        <v>67.400000000000006</v>
       </c>
       <c r="F6" s="34">
-        <v>47.5</v>
+        <v>49.6</v>
       </c>
       <c r="G6" s="34">
-        <v>46.9</v>
+        <v>50.9</v>
       </c>
       <c r="H6" s="34">
-        <v>59</v>
+        <v>54.3</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -6058,22 +6075,22 @@
         <v>23.5</v>
       </c>
       <c r="C7" s="34">
-        <v>25.5</v>
+        <v>25.1</v>
       </c>
       <c r="D7" s="34">
-        <v>22.6</v>
+        <v>22.8</v>
       </c>
       <c r="E7" s="34">
-        <v>16.3</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="F7" s="34">
-        <v>21.6</v>
+        <v>22.4</v>
       </c>
       <c r="G7" s="34">
-        <v>23.6</v>
+        <v>24</v>
       </c>
       <c r="H7" s="34">
-        <v>20.7</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6081,25 +6098,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="34">
-        <v>29.7</v>
+        <v>29.5</v>
       </c>
       <c r="C8" s="34">
-        <v>29.4</v>
+        <v>29.8</v>
       </c>
       <c r="D8" s="34">
-        <v>30.6</v>
+        <v>29.9</v>
       </c>
       <c r="E8" s="34">
-        <v>27.4</v>
+        <v>27</v>
       </c>
       <c r="F8" s="34">
-        <v>29</v>
+        <v>27.9</v>
       </c>
       <c r="G8" s="34">
-        <v>28</v>
+        <v>27.9</v>
       </c>
       <c r="H8" s="34">
-        <v>31.9</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -6107,25 +6124,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="34">
-        <v>39.9</v>
+        <v>42.1</v>
       </c>
       <c r="C9" s="34">
-        <v>40.799999999999997</v>
+        <v>43.4</v>
       </c>
       <c r="D9" s="34">
-        <v>37.6</v>
+        <v>39.700000000000003</v>
       </c>
       <c r="E9" s="34">
-        <v>34.799999999999997</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="F9" s="34">
-        <v>44</v>
+        <v>45.7</v>
       </c>
       <c r="G9" s="34">
-        <v>42.2</v>
+        <v>43.9</v>
       </c>
       <c r="H9" s="34">
-        <v>44.9</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -6133,25 +6150,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="34">
-        <v>38.299999999999997</v>
+        <v>37.4</v>
       </c>
       <c r="C10" s="34">
-        <v>40.700000000000003</v>
+        <v>39.700000000000003</v>
       </c>
       <c r="D10" s="34">
-        <v>36.700000000000003</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="E10" s="34">
         <v>34.9</v>
       </c>
       <c r="F10" s="34">
-        <v>34.700000000000003</v>
+        <v>33.9</v>
       </c>
       <c r="G10" s="34">
-        <v>37.4</v>
+        <v>37.1</v>
       </c>
       <c r="H10" s="34">
-        <v>35.799999999999997</v>
+        <v>36.799999999999997</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -6159,25 +6176,25 @@
         <v>21</v>
       </c>
       <c r="B11" s="34">
-        <v>28.5</v>
+        <v>29.8</v>
       </c>
       <c r="C11" s="34">
-        <v>28.4</v>
+        <v>30.9</v>
       </c>
       <c r="D11" s="34">
         <v>30.3</v>
       </c>
       <c r="E11" s="34">
-        <v>25.3</v>
+        <v>26.1</v>
       </c>
       <c r="F11" s="34">
-        <v>26.3</v>
+        <v>27.8</v>
       </c>
       <c r="G11" s="34">
-        <v>28</v>
+        <v>28.3</v>
       </c>
       <c r="H11" s="34">
-        <v>21.9</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -6185,25 +6202,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="34">
-        <v>41.3</v>
+        <v>42.7</v>
       </c>
       <c r="C12" s="34">
-        <v>39.4</v>
+        <v>42.5</v>
       </c>
       <c r="D12" s="34">
-        <v>39.299999999999997</v>
+        <v>40.4</v>
       </c>
       <c r="E12" s="34">
-        <v>41.6</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="F12" s="34">
-        <v>56.3</v>
+        <v>53.9</v>
       </c>
       <c r="G12" s="34">
-        <v>41.3</v>
+        <v>40.700000000000003</v>
       </c>
       <c r="H12" s="34">
-        <v>46.2</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -6211,25 +6228,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="34">
-        <v>39</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="C13" s="34">
-        <v>37.799999999999997</v>
+        <v>36.5</v>
       </c>
       <c r="D13" s="34">
-        <v>42.2</v>
+        <v>39.200000000000003</v>
       </c>
       <c r="E13" s="34">
-        <v>44</v>
+        <v>43.8</v>
       </c>
       <c r="F13" s="34">
-        <v>34.799999999999997</v>
+        <v>37.5</v>
       </c>
       <c r="G13" s="34">
-        <v>37.700000000000003</v>
+        <v>33.5</v>
       </c>
       <c r="H13" s="34">
-        <v>30.5</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -6237,25 +6254,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="34">
-        <v>31.7</v>
+        <v>31.4</v>
       </c>
       <c r="C14" s="34">
-        <v>34.6</v>
+        <v>33.9</v>
       </c>
       <c r="D14" s="34">
-        <v>30.3</v>
+        <v>30.4</v>
       </c>
       <c r="E14" s="34">
-        <v>26.3</v>
+        <v>27</v>
       </c>
       <c r="F14" s="34">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="G14" s="34">
-        <v>31.9</v>
+        <v>31.8</v>
       </c>
       <c r="H14" s="34">
-        <v>28.1</v>
+        <v>27.2</v>
       </c>
     </row>
   </sheetData>
@@ -7539,14 +7556,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46" t="s">
+      <c r="C1" s="51"/>
+      <c r="D1" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="46"/>
+      <c r="E1" s="51"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8145,14 +8162,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46" t="s">
+      <c r="C1" s="51"/>
+      <c r="D1" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="46"/>
+      <c r="E1" s="51"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8323,10 +8340,10 @@
       <c r="A2" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="50">
+      <c r="B2" s="49">
         <v>5184.6761268600003</v>
       </c>
-      <c r="C2" s="50">
+      <c r="C2" s="49">
         <v>6475.4953001000003</v>
       </c>
       <c r="D2" s="27">
@@ -8383,10 +8400,10 @@
       <c r="A6" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="50">
+      <c r="B6" s="49">
         <v>3791.6945303699999</v>
       </c>
-      <c r="C6" s="50">
+      <c r="C6" s="49">
         <v>724.91150055000003</v>
       </c>
       <c r="D6" s="27">
@@ -8428,10 +8445,10 @@
       <c r="A9" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="50">
+      <c r="B9" s="49">
         <v>3758.7814747100001</v>
       </c>
-      <c r="C9" s="50">
+      <c r="C9" s="49">
         <v>2656.0205328400002</v>
       </c>
       <c r="D9" s="27">
@@ -8458,10 +8475,10 @@
       <c r="A11" s="31" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="50">
+      <c r="B11" s="49">
         <v>2696.2916236699998</v>
       </c>
-      <c r="C11" s="50">
+      <c r="C11" s="49">
         <v>3175.2879474699998</v>
       </c>
       <c r="D11" s="27">
@@ -8533,10 +8550,10 @@
       <c r="A16" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="50">
+      <c r="B16" s="49">
         <v>2432.6926104700001</v>
       </c>
-      <c r="C16" s="50">
+      <c r="C16" s="49">
         <v>5331.43500477</v>
       </c>
       <c r="D16" s="27">
@@ -8548,10 +8565,10 @@
       <c r="A17" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="50">
+      <c r="B17" s="49">
         <v>1936.3140979</v>
       </c>
-      <c r="C17" s="50">
+      <c r="C17" s="49">
         <v>358.63840901999998</v>
       </c>
       <c r="D17" s="27">
@@ -8563,10 +8580,10 @@
       <c r="A18" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="B18" s="50">
+      <c r="B18" s="49">
         <v>3066.0885129500002</v>
       </c>
-      <c r="C18" s="50">
+      <c r="C18" s="49">
         <v>1351.3170497000001</v>
       </c>
       <c r="D18" s="27">
@@ -8638,10 +8655,10 @@
       <c r="A23" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="50">
+      <c r="B23" s="49">
         <v>1637.3744370700001</v>
       </c>
-      <c r="C23" s="50">
+      <c r="C23" s="49">
         <v>135.66836939999999</v>
       </c>
       <c r="D23" s="27">
@@ -8653,10 +8670,10 @@
       <c r="A24" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="50">
+      <c r="B24" s="49">
         <v>1632.70905315</v>
       </c>
-      <c r="C24" s="50">
+      <c r="C24" s="49">
         <v>144.31502965000001</v>
       </c>
       <c r="D24" s="27">
@@ -8668,10 +8685,10 @@
       <c r="A25" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B25" s="50">
+      <c r="B25" s="49">
         <v>105.55805049999999</v>
       </c>
-      <c r="C25" s="50">
+      <c r="C25" s="49">
         <v>82.387265009999993</v>
       </c>
       <c r="D25" s="27">
@@ -8683,10 +8700,10 @@
       <c r="A26" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B26" s="50">
+      <c r="B26" s="49">
         <v>307.25023296000001</v>
       </c>
-      <c r="C26" s="50">
+      <c r="C26" s="49">
         <v>95.116376149999994</v>
       </c>
       <c r="D26" s="27">
@@ -8698,10 +8715,10 @@
       <c r="A27" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B27" s="51">
+      <c r="B27" s="50">
         <v>4270.5155818599997</v>
       </c>
-      <c r="C27" s="51">
+      <c r="C27" s="50">
         <v>2012.0832006999999</v>
       </c>
       <c r="D27" s="27">
@@ -9224,7 +9241,7 @@
       <c r="A2" s="33" t="s">
         <v>177</v>
       </c>
-      <c r="B2" s="47">
+      <c r="B2" s="46">
         <v>22542.675985360002</v>
       </c>
     </row>
@@ -9232,7 +9249,7 @@
       <c r="A3" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="B3" s="47">
+      <c r="B3" s="46">
         <v>4517.7529110900005</v>
       </c>
     </row>
@@ -9240,7 +9257,7 @@
       <c r="A4" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="B4" s="48">
+      <c r="B4" s="47">
         <v>3286.95681285</v>
       </c>
     </row>
@@ -9248,7 +9265,7 @@
       <c r="A5" s="34" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="48">
+      <c r="B5" s="47">
         <v>500.81195382999999</v>
       </c>
     </row>
@@ -9256,7 +9273,7 @@
       <c r="A6" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="48">
+      <c r="B6" s="47">
         <v>729.98414441</v>
       </c>
     </row>
@@ -9264,7 +9281,7 @@
       <c r="A7" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="B7" s="47">
+      <c r="B7" s="46">
         <v>7697.9606936500004</v>
       </c>
     </row>
@@ -9272,7 +9289,7 @@
       <c r="A8" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="48">
+      <c r="B8" s="47">
         <v>1317.8545178899999</v>
       </c>
     </row>
@@ -9280,7 +9297,7 @@
       <c r="A9" s="34" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="48">
+      <c r="B9" s="47">
         <v>173.75594677999999</v>
       </c>
     </row>
@@ -9288,7 +9305,7 @@
       <c r="A10" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="48">
+      <c r="B10" s="47">
         <v>335.70177479</v>
       </c>
     </row>
@@ -9296,7 +9313,7 @@
       <c r="A11" s="34" t="s">
         <v>186</v>
       </c>
-      <c r="B11" s="48">
+      <c r="B11" s="47">
         <v>5196.0503129199997</v>
       </c>
     </row>
@@ -9304,7 +9321,7 @@
       <c r="A12" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B12" s="48">
+      <c r="B12" s="47">
         <v>674.59814127000004</v>
       </c>
     </row>
@@ -9312,7 +9329,7 @@
       <c r="A13" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="B13" s="47">
+      <c r="B13" s="46">
         <v>577.55242461</v>
       </c>
     </row>
@@ -9320,7 +9337,7 @@
       <c r="A14" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="B14" s="48">
+      <c r="B14" s="47">
         <v>81.613303869999996</v>
       </c>
     </row>
@@ -9328,7 +9345,7 @@
       <c r="A15" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="B15" s="48">
+      <c r="B15" s="47">
         <v>495.93912074000002</v>
       </c>
     </row>
@@ -9336,7 +9353,7 @@
       <c r="A16" s="33" t="s">
         <v>191</v>
       </c>
-      <c r="B16" s="47">
+      <c r="B16" s="46">
         <v>4015.2040200599999</v>
       </c>
     </row>
@@ -9344,7 +9361,7 @@
       <c r="A17" s="34" t="s">
         <v>192</v>
       </c>
-      <c r="B17" s="48">
+      <c r="B17" s="47">
         <v>1565.8439269099999</v>
       </c>
     </row>
@@ -9352,7 +9369,7 @@
       <c r="A18" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="B18" s="48">
+      <c r="B18" s="47">
         <v>230.57634225000001</v>
       </c>
     </row>
@@ -9360,7 +9377,7 @@
       <c r="A19" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="B19" s="48">
+      <c r="B19" s="47">
         <v>2218.7837509000001</v>
       </c>
     </row>
@@ -9368,7 +9385,7 @@
       <c r="A20" s="33" t="s">
         <v>195</v>
       </c>
-      <c r="B20" s="47">
+      <c r="B20" s="46">
         <v>3560.55351277</v>
       </c>
     </row>
@@ -9376,7 +9393,7 @@
       <c r="A21" s="34" t="s">
         <v>196</v>
       </c>
-      <c r="B21" s="48">
+      <c r="B21" s="47">
         <v>292.28966401000002</v>
       </c>
     </row>
@@ -9384,7 +9401,7 @@
       <c r="A22" s="34" t="s">
         <v>197</v>
       </c>
-      <c r="B22" s="48">
+      <c r="B22" s="47">
         <v>489.37519828000001</v>
       </c>
     </row>
@@ -9392,7 +9409,7 @@
       <c r="A23" s="34" t="s">
         <v>198</v>
       </c>
-      <c r="B23" s="48">
+      <c r="B23" s="47">
         <v>286.98828068</v>
       </c>
     </row>
@@ -9400,7 +9417,7 @@
       <c r="A24" s="34" t="s">
         <v>199</v>
       </c>
-      <c r="B24" s="48">
+      <c r="B24" s="47">
         <v>366.13625930000001</v>
       </c>
     </row>
@@ -9408,7 +9425,7 @@
       <c r="A25" s="34" t="s">
         <v>200</v>
       </c>
-      <c r="B25" s="48">
+      <c r="B25" s="47">
         <v>985.58987013000001</v>
       </c>
     </row>
@@ -9416,7 +9433,7 @@
       <c r="A26" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="B26" s="48">
+      <c r="B26" s="47">
         <v>614.21376779000002</v>
       </c>
     </row>
@@ -9424,7 +9441,7 @@
       <c r="A27" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="B27" s="48">
+      <c r="B27" s="47">
         <v>525.96047257999999</v>
       </c>
     </row>
@@ -9432,7 +9449,7 @@
       <c r="A28" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="B28" s="47">
+      <c r="B28" s="46">
         <v>1752.703162</v>
       </c>
     </row>
@@ -9440,7 +9457,7 @@
       <c r="A29" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B29" s="49">
+      <c r="B29" s="48">
         <v>420.94926118000001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
"Actualizo resultado fiscal mayo26 y el nivel de actividad al primer trimestre de 2026"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD30FEC-896F-41A8-9994-CF1572A29A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC3CD17-F080-4FAF-9713-19D12DB402DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="225">
   <si>
     <t>Período</t>
   </si>
@@ -996,9 +996,6 @@
     </xf>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1007,6 +1004,9 @@
     </xf>
     <xf numFmtId="3" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -3317,10 +3317,10 @@
         <v>84</v>
       </c>
       <c r="B2">
-        <v>599983.70014805021</v>
+        <v>599983.70014804997</v>
       </c>
       <c r="C2">
-        <v>1.3240439045926866</v>
+        <v>2.481356123815659</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3331,7 +3331,7 @@
         <v>38842.924521107714</v>
       </c>
       <c r="C3">
-        <v>16.089218460720023</v>
+        <v>18.138938518629178</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3342,7 +3342,7 @@
         <v>1545.6270924291682</v>
       </c>
       <c r="C4">
-        <v>10.567832179756099</v>
+        <v>27.45728282807076</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3353,7 +3353,7 @@
         <v>30755.076629366038</v>
       </c>
       <c r="C5">
-        <v>8.0983822641656378</v>
+        <v>12.334190997099181</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3364,7 +3364,7 @@
         <v>112761.23165011391</v>
       </c>
       <c r="C6">
-        <v>-5.0381313317373388</v>
+        <v>-1.676454111061576</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3375,7 +3375,7 @@
         <v>12673.907286977306</v>
       </c>
       <c r="C7">
-        <v>4.6886508068879618</v>
+        <v>-1.0509245571815207</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3386,7 +3386,7 @@
         <v>19017.800104434555</v>
       </c>
       <c r="C8">
-        <v>0.92123335642904092</v>
+        <v>2.5370815997647345</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3397,7 +3397,7 @@
         <v>91872.245634525272</v>
       </c>
       <c r="C9">
-        <v>-2.2069029193928613</v>
+        <v>-0.29307255440298441</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3408,7 +3408,7 @@
         <v>13022.400979766842</v>
       </c>
       <c r="C10">
-        <v>-0.66957849547361059</v>
+        <v>2.7902948421734797</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3419,7 +3419,7 @@
         <v>55633.327772916178</v>
       </c>
       <c r="C11">
-        <v>2.1967051692507011</v>
+        <v>2.2858102158443083</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3430,7 +3430,7 @@
         <v>30381.126773097683</v>
       </c>
       <c r="C12">
-        <v>17.24588178668942</v>
+        <v>7.5048032104928053</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3441,7 +3441,7 @@
         <v>85939.774708283672</v>
       </c>
       <c r="C13">
-        <v>2.0043316406221923</v>
+        <v>0.89683919333798379</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3452,7 +3452,7 @@
         <v>34900.492729780119</v>
       </c>
       <c r="C14">
-        <v>-1.0550626738513924</v>
+        <v>-1.3759391935735277</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -3463,7 +3463,7 @@
         <v>29912.893832996058</v>
       </c>
       <c r="C15">
-        <v>0.64148026369161837</v>
+        <v>5.5946826390473881E-2</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -3474,7 +3474,7 @@
         <v>23085.607234226565</v>
       </c>
       <c r="C16">
-        <v>0.28721826490549773</v>
+        <v>0.46783601580868694</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -3485,7 +3485,7 @@
         <v>15478.186568411322</v>
       </c>
       <c r="C17">
-        <v>1.0991937461104273</v>
+        <v>0.6554599397215588</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -3496,7 +3496,7 @@
         <v>4161.0766296179845</v>
       </c>
       <c r="C18">
-        <v>2.7585257742845926E-2</v>
+        <v>6.2795181172130343</v>
       </c>
     </row>
   </sheetData>
@@ -6283,7 +6283,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="11.42578125" style="10" customWidth="1"/>
@@ -6311,7 +6311,7 @@
         <v>29</v>
       </c>
       <c r="C2" s="11">
-        <v>476036.52687146427</v>
+        <v>475539.40286010271</v>
       </c>
       <c r="D2" s="11">
         <v>460369.44223294902</v>
@@ -6325,7 +6325,7 @@
         <v>30</v>
       </c>
       <c r="C3" s="11">
-        <v>470010.06614707055</v>
+        <v>470354.11948447995</v>
       </c>
       <c r="D3" s="11">
         <v>514395.68177236198</v>
@@ -6339,7 +6339,7 @@
         <v>31</v>
       </c>
       <c r="C4" s="11">
-        <v>493895.12091097509</v>
+        <v>493797.37820779701</v>
       </c>
       <c r="D4" s="11">
         <v>481151.97994350799</v>
@@ -6353,7 +6353,7 @@
         <v>32</v>
       </c>
       <c r="C5" s="11">
-        <v>500519.06692598236</v>
+        <v>500769.87964556657</v>
       </c>
       <c r="D5" s="11">
         <v>484543.67687656201</v>
@@ -6367,7 +6367,7 @@
         <v>29</v>
       </c>
       <c r="C6" s="11">
-        <v>514918.45889096794</v>
+        <v>515285.82226785243</v>
       </c>
       <c r="D6" s="11">
         <v>493602.53057785501</v>
@@ -6381,7 +6381,7 @@
         <v>30</v>
       </c>
       <c r="C7" s="11">
-        <v>527084.19831498002</v>
+        <v>526591.9714851937</v>
       </c>
       <c r="D7" s="11">
         <v>581668.24987960199</v>
@@ -6395,7 +6395,7 @@
         <v>31</v>
       </c>
       <c r="C8" s="11">
-        <v>530101.95784154162</v>
+        <v>530024.96916142374</v>
       </c>
       <c r="D8" s="11">
         <v>514697.78950542799</v>
@@ -6409,7 +6409,7 @@
         <v>32</v>
       </c>
       <c r="C9" s="11">
-        <v>540119.15496616694</v>
+        <v>540321.007099187</v>
       </c>
       <c r="D9" s="11">
         <v>522255.20005077199</v>
@@ -6423,7 +6423,7 @@
         <v>29</v>
       </c>
       <c r="C10" s="11">
-        <v>554455.77230754215</v>
+        <v>554468.16211025103</v>
       </c>
       <c r="D10" s="11">
         <v>532348.21201691695</v>
@@ -6437,7 +6437,7 @@
         <v>30</v>
       </c>
       <c r="C11" s="11">
-        <v>561157.22299964982</v>
+        <v>561434.67786953063</v>
       </c>
       <c r="D11" s="11">
         <v>614076.39260854397</v>
@@ -6451,7 +6451,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="11">
-        <v>577088.45820131898</v>
+        <v>576815.72098068486</v>
       </c>
       <c r="D12" s="11">
         <v>562978.96562687703</v>
@@ -6465,7 +6465,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="11">
-        <v>589496.16337441502</v>
+        <v>589479.05592245981</v>
       </c>
       <c r="D13" s="11">
         <v>572794.04663058801</v>
@@ -6479,7 +6479,7 @@
         <v>29</v>
       </c>
       <c r="C14" s="11">
-        <v>603483.20680705283</v>
+        <v>603416.48185863218</v>
       </c>
       <c r="D14" s="11">
         <v>576846.88569942699</v>
@@ -6493,7 +6493,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="11">
-        <v>616073.36568713211</v>
+        <v>616299.39312501706</v>
       </c>
       <c r="D15" s="11">
         <v>674620.563006485</v>
@@ -6507,7 +6507,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="11">
-        <v>624446.89492768422</v>
+        <v>624352.58868411044</v>
       </c>
       <c r="D16" s="11">
         <v>610425.69401485403</v>
@@ -6521,7 +6521,7 @@
         <v>32</v>
       </c>
       <c r="C17" s="11">
-        <v>643766.54316249432</v>
+        <v>643701.5469166023</v>
       </c>
       <c r="D17" s="11">
         <v>625876.867863597</v>
@@ -6535,7 +6535,7 @@
         <v>29</v>
       </c>
       <c r="C18" s="11">
-        <v>650003.25715436717</v>
+        <v>650062.83279971546</v>
       </c>
       <c r="D18" s="11">
         <v>616720.35706447798</v>
@@ -6549,7 +6549,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="11">
-        <v>653467.95396695228</v>
+        <v>653269.76138485561</v>
       </c>
       <c r="D19" s="11">
         <v>711405.50045523304</v>
@@ -6563,7 +6563,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="11">
-        <v>657695.28402587795</v>
+        <v>657936.93255261565</v>
       </c>
       <c r="D20" s="11">
         <v>647087.95974249404</v>
@@ -6577,7 +6577,7 @@
         <v>32</v>
       </c>
       <c r="C21" s="11">
-        <v>627538.1438176519</v>
+        <v>627435.11222766025</v>
       </c>
       <c r="D21" s="11">
         <v>613490.82170264097</v>
@@ -6591,7 +6591,7 @@
         <v>29</v>
       </c>
       <c r="C22" s="11">
-        <v>604940.28395197983</v>
+        <v>604739.79905993817</v>
       </c>
       <c r="D22" s="11">
         <v>578553.04424240498</v>
@@ -6605,7 +6605,7 @@
         <v>30</v>
       </c>
       <c r="C23" s="11">
-        <v>590529.02806835552</v>
+        <v>590902.23142847931</v>
       </c>
       <c r="D23" s="11">
         <v>631197.75186006899</v>
@@ -6619,7 +6619,7 @@
         <v>31</v>
       </c>
       <c r="C24" s="11">
-        <v>613800.25653562765</v>
+        <v>614035.54343456146</v>
       </c>
       <c r="D24" s="11">
         <v>610519.85461172694</v>
@@ -6633,7 +6633,7 @@
         <v>32</v>
       </c>
       <c r="C25" s="11">
-        <v>626221.93709553429</v>
+        <v>625813.93172851868</v>
       </c>
       <c r="D25" s="11">
         <v>615220.85493729694</v>
@@ -6647,7 +6647,7 @@
         <v>29</v>
       </c>
       <c r="C26" s="11">
-        <v>645513.99738394632</v>
+        <v>644901.88693182275</v>
       </c>
       <c r="D26" s="11">
         <v>611607.33658973</v>
@@ -6661,7 +6661,7 @@
         <v>30</v>
       </c>
       <c r="C27" s="11">
-        <v>674164.23542403907</v>
+        <v>673704.24691340048</v>
       </c>
       <c r="D27" s="11">
         <v>733730.773968903</v>
@@ -6675,7 +6675,7 @@
         <v>31</v>
       </c>
       <c r="C28" s="11">
-        <v>676995.53972733335</v>
+        <v>677196.1138942315</v>
       </c>
       <c r="D28" s="11">
         <v>668566.50948898599</v>
@@ -6689,7 +6689,7 @@
         <v>32</v>
       </c>
       <c r="C29" s="11">
-        <v>685420.94523187377</v>
+        <v>686292.47002773837</v>
       </c>
       <c r="D29" s="11">
         <v>668190.097719574</v>
@@ -6703,7 +6703,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="11">
-        <v>701686.92075505713</v>
+        <v>702715.18731246202</v>
       </c>
       <c r="D30" s="11">
         <v>662325.58597269503</v>
@@ -6717,7 +6717,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="11">
-        <v>710326.15459237562</v>
+        <v>709752.09900164558</v>
       </c>
       <c r="D31" s="11">
         <v>766332.95457161299</v>
@@ -6731,7 +6731,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="11">
-        <v>715883.91149126994</v>
+        <v>715352.50699214835</v>
       </c>
       <c r="D32" s="11">
         <v>711417.39193010505</v>
@@ -6745,7 +6745,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="11">
-        <v>715229.40204370406</v>
+        <v>715306.59557615174</v>
       </c>
       <c r="D33" s="11">
         <v>703050.45640799298</v>
@@ -6759,7 +6759,7 @@
         <v>29</v>
       </c>
       <c r="C34" s="11">
-        <v>708348.86146128085</v>
+        <v>707988.22133292514</v>
       </c>
       <c r="D34" s="11">
         <v>672685.993630504</v>
@@ -6773,7 +6773,7 @@
         <v>30</v>
       </c>
       <c r="C35" s="11">
-        <v>683593.31589575845</v>
+        <v>683985.42306130065</v>
       </c>
       <c r="D35" s="11">
         <v>730838.27259277599</v>
@@ -6787,7 +6787,7 @@
         <v>31</v>
       </c>
       <c r="C36" s="11">
-        <v>705293.74411482143</v>
+        <v>705109.9934384583</v>
       </c>
       <c r="D36" s="11">
         <v>703461.65253019601</v>
@@ -6801,7 +6801,7 @@
         <v>32</v>
       </c>
       <c r="C37" s="11">
-        <v>716708.03636393591</v>
+        <v>716860.32000311208</v>
       </c>
       <c r="D37" s="11">
         <v>706958.03908231901</v>
@@ -6815,7 +6815,7 @@
         <v>29</v>
       </c>
       <c r="C38" s="11">
-        <v>715943.73773188714</v>
+        <v>716958.91356570437</v>
       </c>
       <c r="D38" s="11">
         <v>677085.52917315101</v>
@@ -6829,7 +6829,7 @@
         <v>30</v>
       </c>
       <c r="C39" s="11">
-        <v>720882.8515662452</v>
+        <v>721290.34819069924</v>
       </c>
       <c r="D39" s="11">
         <v>776486.60279942001</v>
@@ -6843,7 +6843,7 @@
         <v>31</v>
       </c>
       <c r="C40" s="11">
-        <v>725588.38163084479</v>
+        <v>725228.86057766667</v>
       </c>
       <c r="D40" s="11">
         <v>721458.94421618199</v>
@@ -6857,7 +6857,7 @@
         <v>32</v>
       </c>
       <c r="C41" s="11">
-        <v>719213.4502822801</v>
+        <v>718150.29887718929</v>
       </c>
       <c r="D41" s="11">
         <v>706597.34502250701</v>
@@ -6871,7 +6871,7 @@
         <v>29</v>
       </c>
       <c r="C42" s="11">
-        <v>708278.97258087643</v>
+        <v>707604.64972170733</v>
       </c>
       <c r="D42" s="11">
         <v>671066.04663506302</v>
@@ -6885,7 +6885,7 @@
         <v>30</v>
       </c>
       <c r="C43" s="11">
-        <v>702914.57152322109</v>
+        <v>703288.51850467571</v>
       </c>
       <c r="D43" s="11">
         <v>760576.86834800395</v>
@@ -6899,7 +6899,7 @@
         <v>31</v>
       </c>
       <c r="C44" s="11">
-        <v>697281.49261729233</v>
+        <v>697226.21978834714</v>
       </c>
       <c r="D44" s="11">
         <v>690879.79825168301</v>
@@ -6913,7 +6913,7 @@
         <v>32</v>
       </c>
       <c r="C45" s="11">
-        <v>700749.14713207202</v>
+        <v>701104.79583873064</v>
       </c>
       <c r="D45" s="11">
         <v>686701.47061871097</v>
@@ -6927,7 +6927,7 @@
         <v>29</v>
       </c>
       <c r="C46" s="11">
-        <v>710714.75219443382</v>
+        <v>711401.44068145636</v>
       </c>
       <c r="D46" s="11">
         <v>672749.81139169901</v>
@@ -6941,7 +6941,7 @@
         <v>30</v>
       </c>
       <c r="C47" s="11">
-        <v>728934.83476324868</v>
+        <v>727767.46053102415</v>
       </c>
       <c r="D47" s="11">
         <v>791235.96554166998</v>
@@ -6955,7 +6955,7 @@
         <v>31</v>
       </c>
       <c r="C48" s="11">
-        <v>727453.63885899587</v>
+        <v>727494.47701461555</v>
       </c>
       <c r="D48" s="11">
         <v>718281.26544978202</v>
@@ -6969,7 +6969,7 @@
         <v>32</v>
       </c>
       <c r="C49" s="11">
-        <v>718845.360735483</v>
+        <v>719285.20832506299</v>
       </c>
       <c r="D49" s="11">
         <v>703681.54416900803</v>
@@ -6983,7 +6983,7 @@
         <v>29</v>
       </c>
       <c r="C50" s="11">
-        <v>713388.1069145425</v>
+        <v>712710.63575714745</v>
       </c>
       <c r="D50" s="11">
         <v>677652.08911570301</v>
@@ -6997,7 +6997,7 @@
         <v>30</v>
       </c>
       <c r="C51" s="11">
-        <v>701514.77320906788</v>
+        <v>701267.87546475301</v>
       </c>
       <c r="D51" s="11">
         <v>760703.28015165601</v>
@@ -7011,7 +7011,7 @@
         <v>31</v>
       </c>
       <c r="C52" s="11">
-        <v>703211.858554565</v>
+        <v>703825.31306672294</v>
       </c>
       <c r="D52" s="11">
         <v>694382.47577623103</v>
@@ -7025,7 +7025,7 @@
         <v>32</v>
       </c>
       <c r="C53" s="11">
-        <v>707796.65571247344</v>
+        <v>708107.57010202378</v>
       </c>
       <c r="D53" s="11">
         <v>693173.54934705805</v>
@@ -7039,7 +7039,7 @@
         <v>29</v>
       </c>
       <c r="C54" s="11">
-        <v>714701.00378393335</v>
+        <v>714000.68213478185</v>
       </c>
       <c r="D54" s="11">
         <v>681444.76611022197</v>
@@ -7053,7 +7053,7 @@
         <v>30</v>
       </c>
       <c r="C55" s="11">
-        <v>721713.65757954179</v>
+        <v>722206.78209549456</v>
       </c>
       <c r="D55" s="11">
         <v>778401.67644931702</v>
@@ -7067,7 +7067,7 @@
         <v>31</v>
       </c>
       <c r="C56" s="11">
-        <v>731047.00599477056</v>
+        <v>731022.65780373593</v>
       </c>
       <c r="D56" s="11">
         <v>721120.42685279401</v>
@@ -7081,7 +7081,7 @@
         <v>32</v>
       </c>
       <c r="C57" s="11">
-        <v>738098.12369305</v>
+        <v>738329.66901728406</v>
       </c>
       <c r="D57" s="11">
         <v>724592.92163896305</v>
@@ -7095,7 +7095,7 @@
         <v>29</v>
       </c>
       <c r="C58" s="11">
-        <v>734098.41115135164</v>
+        <v>735269.26388700691</v>
       </c>
       <c r="D58" s="11">
         <v>707324.26805721398</v>
@@ -7109,7 +7109,7 @@
         <v>30</v>
       </c>
       <c r="C59" s="11">
-        <v>703426.52003617655</v>
+        <v>702794.19038738846</v>
       </c>
       <c r="D59" s="11">
         <v>747428.29995457502</v>
@@ -7123,7 +7123,7 @@
         <v>31</v>
       </c>
       <c r="C60" s="11">
-        <v>701416.02106970118</v>
+        <v>700585.06179718161</v>
       </c>
       <c r="D60" s="11">
         <v>696101.58352180803</v>
@@ -7137,7 +7137,7 @@
         <v>32</v>
       </c>
       <c r="C61" s="11">
-        <v>690568.81966081902</v>
+        <v>690861.25584647327</v>
       </c>
       <c r="D61" s="11">
         <v>678655.62038445403</v>
@@ -7151,7 +7151,7 @@
         <v>29</v>
       </c>
       <c r="C62" s="11">
-        <v>692977.78815745737</v>
+        <v>690992.53890621837</v>
       </c>
       <c r="D62">
         <v>665848.71529970889</v>
@@ -7165,7 +7165,7 @@
         <v>30</v>
       </c>
       <c r="C63" s="11">
-        <v>696856.65350922232</v>
+        <v>697721.48697133223</v>
       </c>
       <c r="D63">
         <v>751784.46077713254</v>
@@ -7179,7 +7179,7 @@
         <v>31</v>
       </c>
       <c r="C64" s="11">
-        <v>696337.7406497316</v>
+        <v>697245.70141462015</v>
       </c>
       <c r="D64">
         <v>683900.89855257841</v>
@@ -7193,7 +7193,7 @@
         <v>32</v>
       </c>
       <c r="C65" s="11">
-        <v>686723.03203542822</v>
+        <v>686935.48705966782</v>
       </c>
       <c r="D65">
         <v>671361.13972242002</v>
@@ -7207,7 +7207,7 @@
         <v>29</v>
       </c>
       <c r="C66" s="10">
-        <v>656405.46191031951</v>
+        <v>657234.36724165711</v>
       </c>
       <c r="D66" s="10">
         <v>632389.35353461001</v>
@@ -7221,7 +7221,7 @@
         <v>30</v>
       </c>
       <c r="C67" s="10">
-        <v>563484.6621608017</v>
+        <v>562000.89823407296</v>
       </c>
       <c r="D67" s="10">
         <v>609379.98946480127</v>
@@ -7235,7 +7235,7 @@
         <v>31</v>
       </c>
       <c r="C68" s="10">
-        <v>623894.44182136783</v>
+        <v>623856.36323480471</v>
       </c>
       <c r="D68" s="10">
         <v>614192.47840422287</v>
@@ -7249,7 +7249,7 @@
         <v>32</v>
       </c>
       <c r="C69" s="10">
-        <v>654580.57870909641</v>
+        <v>655273.51589104964</v>
       </c>
       <c r="D69" s="10">
         <v>642403.32319795026</v>
@@ -7263,7 +7263,7 @@
         <v>29</v>
       </c>
       <c r="C70" s="10">
-        <v>677169.13791920443</v>
+        <v>677518.09192361217</v>
       </c>
       <c r="D70">
         <v>652831.97670632158</v>
@@ -7277,7 +7277,7 @@
         <v>30</v>
       </c>
       <c r="C71" s="10">
-        <v>679096.31371864828</v>
+        <v>678667.84323796758</v>
       </c>
       <c r="D71">
         <v>723516.62249067484</v>
@@ -7291,7 +7291,7 @@
         <v>31</v>
       </c>
       <c r="C72" s="10">
-        <v>693100.33574559912</v>
+        <v>693508.41694142157</v>
       </c>
       <c r="D72" s="10">
         <v>686756.46782667423</v>
@@ -7305,7 +7305,7 @@
         <v>32</v>
       </c>
       <c r="C73" s="10">
-        <v>709873.94875233434</v>
+        <v>709545.38403278519</v>
       </c>
       <c r="D73" s="10">
         <v>696134.66911211505</v>
@@ -7319,7 +7319,7 @@
         <v>29</v>
       </c>
       <c r="C74" s="10">
-        <v>726931.81776528095</v>
+        <v>726994.4331088519</v>
       </c>
       <c r="D74">
         <v>697625.28466635814</v>
@@ -7333,7 +7333,7 @@
         <v>30</v>
       </c>
       <c r="C75" s="10">
-        <v>741189.8641333899</v>
+        <v>741461.96753675886</v>
       </c>
       <c r="D75">
         <v>782338.62853373506</v>
@@ -7347,7 +7347,7 @@
         <v>31</v>
       </c>
       <c r="C76" s="10">
-        <v>735605.99139607733</v>
+        <v>735869.56325702253</v>
       </c>
       <c r="D76" s="10">
         <v>732662.16387550125</v>
@@ -7361,7 +7361,7 @@
         <v>32</v>
       </c>
       <c r="C77" s="10">
-        <v>721638.86160958419</v>
+        <v>721040.57100169931</v>
       </c>
       <c r="D77" s="10">
         <v>712740.45782873826</v>
@@ -7375,10 +7375,10 @@
         <v>29</v>
       </c>
       <c r="C78" s="10">
-        <v>727949.28499660653</v>
+        <v>729079.81570524594</v>
       </c>
       <c r="D78" s="10">
-        <v>703987.50432157726</v>
+        <v>704009.03517700161</v>
       </c>
       <c r="E78" s="38"/>
     </row>
@@ -7390,10 +7390,10 @@
         <v>30</v>
       </c>
       <c r="C79" s="10">
-        <v>710424.84865227621</v>
+        <v>709842.35270039842</v>
       </c>
       <c r="D79" s="10">
-        <v>737941.90937407222</v>
+        <v>738128.41122730402</v>
       </c>
       <c r="E79" s="39"/>
     </row>
@@ -7405,10 +7405,10 @@
         <v>31</v>
       </c>
       <c r="C80" s="10">
-        <v>725091.04020458832</v>
+        <v>725214.64378983236</v>
       </c>
       <c r="D80" s="10">
-        <v>728638.58456868224</v>
+        <v>728542.25584748655</v>
       </c>
       <c r="E80" s="39"/>
     </row>
@@ -7420,10 +7420,10 @@
         <v>32</v>
       </c>
       <c r="C81" s="10">
-        <v>707612.75898318249</v>
+        <v>707086.08875387569</v>
       </c>
       <c r="D81" s="10">
-        <v>700509.93457232334</v>
+        <v>700543.19869756</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -7434,10 +7434,10 @@
         <v>29</v>
       </c>
       <c r="C82" s="10">
-        <v>696039.64182027197</v>
+        <v>694486.09954866616</v>
       </c>
       <c r="D82" s="10">
-        <v>669057.73338516685</v>
+        <v>668219.6308270538</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -7448,10 +7448,10 @@
         <v>30</v>
       </c>
       <c r="C83" s="10">
-        <v>690565.59876287449</v>
+        <v>691468.75067544018</v>
       </c>
       <c r="D83">
-        <v>729947.78527455311</v>
+        <v>729909.36871982319</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -7462,10 +7462,10 @@
         <v>31</v>
       </c>
       <c r="C84" s="10">
-        <v>717175.74805169622</v>
+        <v>716166.17456055968</v>
       </c>
       <c r="D84">
-        <v>714524.36554995924</v>
+        <v>714299.21795624029</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -7476,10 +7476,10 @@
         <v>32</v>
       </c>
       <c r="C85" s="10">
-        <v>728740.35651141696</v>
+        <v>729830.51344938693</v>
       </c>
       <c r="D85" s="10">
-        <v>718991.4609365795</v>
+        <v>719523.32073093485</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -7490,10 +7490,10 @@
         <v>29</v>
       </c>
       <c r="C86" s="10">
-        <v>736261.04995951243</v>
+        <v>735468.22118616325</v>
       </c>
       <c r="D86" s="10">
-        <v>708113.80567017628</v>
+        <v>709095.12469662423</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -7504,10 +7504,10 @@
         <v>30</v>
       </c>
       <c r="C87" s="10">
-        <v>735534.38226519676</v>
+        <v>737703.22646665608</v>
       </c>
       <c r="D87" s="10">
-        <v>776528.77609078528</v>
+        <v>777482.55560690013</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -7518,10 +7518,10 @@
         <v>31</v>
       </c>
       <c r="C88" s="10">
-        <v>739903.77331731853</v>
+        <v>738582.97927448282</v>
       </c>
       <c r="D88">
-        <v>737795.74161343137</v>
+        <v>737135.06767770939</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -7532,10 +7532,24 @@
         <v>32</v>
       </c>
       <c r="C89" s="10">
-        <v>744527.7879887321</v>
+        <v>747160.42718325544</v>
       </c>
       <c r="D89">
-        <v>733788.66978506034</v>
+        <v>735202.10550800152</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="10">
+        <v>2026</v>
+      </c>
+      <c r="B90" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C90" s="10">
+        <v>752727.87372926541</v>
+      </c>
+      <c r="D90" s="10">
+        <v>725600.2445682534</v>
       </c>
     </row>
   </sheetData>
@@ -7556,14 +7570,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48" t="s">
+      <c r="C1" s="51"/>
+      <c r="D1" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="48"/>
+      <c r="E1" s="51"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8162,14 +8176,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48" t="s">
+      <c r="C1" s="51"/>
+      <c r="D1" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="48"/>
+      <c r="E1" s="51"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8752,7 +8766,7 @@
       <c r="A2" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="49">
+      <c r="B2" s="48">
         <v>40358.592053159999</v>
       </c>
       <c r="D2" s="29"/>
@@ -8761,7 +8775,7 @@
       <c r="A3" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="B3" s="49">
+      <c r="B3" s="48">
         <v>10742.82963538</v>
       </c>
       <c r="D3" s="29"/>
@@ -8770,7 +8784,7 @@
       <c r="A4" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="50">
+      <c r="B4" s="49">
         <v>13.95463872</v>
       </c>
       <c r="D4" s="30"/>
@@ -8779,7 +8793,7 @@
       <c r="A5" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="50">
+      <c r="B5" s="49">
         <v>925.60164197999995</v>
       </c>
       <c r="D5" s="30"/>
@@ -8788,7 +8802,7 @@
       <c r="A6" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="50">
+      <c r="B6" s="49">
         <v>152.02629300000001</v>
       </c>
       <c r="D6" s="30"/>
@@ -8797,7 +8811,7 @@
       <c r="A7" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="50">
+      <c r="B7" s="49">
         <v>341.09879602000001</v>
       </c>
       <c r="D7" s="30"/>
@@ -8806,7 +8820,7 @@
       <c r="A8" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="50">
+      <c r="B8" s="49">
         <v>324.02407026999998</v>
       </c>
       <c r="D8" s="30"/>
@@ -8815,7 +8829,7 @@
       <c r="A9" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B9" s="50">
+      <c r="B9" s="49">
         <v>6557.1334442699999</v>
       </c>
       <c r="D9" s="30"/>
@@ -8824,7 +8838,7 @@
       <c r="A10" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="50">
+      <c r="B10" s="49">
         <v>1708.08558193</v>
       </c>
       <c r="D10" s="30"/>
@@ -8833,7 +8847,7 @@
       <c r="A11" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="B11" s="50">
+      <c r="B11" s="49">
         <v>83.86755617</v>
       </c>
       <c r="D11" s="30"/>
@@ -8842,7 +8856,7 @@
       <c r="A12" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="50">
+      <c r="B12" s="49">
         <v>44.898907080000001</v>
       </c>
       <c r="D12" s="30"/>
@@ -8851,7 +8865,7 @@
       <c r="A13" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="50">
+      <c r="B13" s="49">
         <v>42.397263289999998</v>
       </c>
       <c r="D13" s="30"/>
@@ -8860,7 +8874,7 @@
       <c r="A14" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B14" s="50">
+      <c r="B14" s="49">
         <v>459.11204710999999</v>
       </c>
       <c r="D14" s="30"/>
@@ -8869,7 +8883,7 @@
       <c r="A15" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="50">
+      <c r="B15" s="49">
         <v>90.629395540000004</v>
       </c>
       <c r="D15" s="30"/>
@@ -8878,7 +8892,7 @@
       <c r="A16" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B16" s="49">
+      <c r="B16" s="48">
         <v>12470.11895038</v>
       </c>
       <c r="D16" s="29"/>
@@ -8887,7 +8901,7 @@
       <c r="A17" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="50">
+      <c r="B17" s="49">
         <v>2068.17821129</v>
       </c>
       <c r="D17" s="30"/>
@@ -8896,7 +8910,7 @@
       <c r="A18" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="B18" s="50">
+      <c r="B18" s="49">
         <v>122.0667815</v>
       </c>
       <c r="D18" s="30"/>
@@ -8905,7 +8919,7 @@
       <c r="A19" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="50">
+      <c r="B19" s="49">
         <v>595.02203373999998</v>
       </c>
       <c r="D19" s="30"/>
@@ -8914,7 +8928,7 @@
       <c r="A20" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="B20" s="50">
+      <c r="B20" s="49">
         <v>39.94780351</v>
       </c>
       <c r="D20" s="30"/>
@@ -8923,7 +8937,7 @@
       <c r="A21" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="50">
+      <c r="B21" s="49">
         <v>43.27242983</v>
       </c>
       <c r="D21" s="30"/>
@@ -8932,7 +8946,7 @@
       <c r="A22" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="50">
+      <c r="B22" s="49">
         <v>73.02852584</v>
       </c>
       <c r="D22" s="30"/>
@@ -8941,7 +8955,7 @@
       <c r="A23" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B23" s="50">
+      <c r="B23" s="49">
         <v>314.77157653</v>
       </c>
       <c r="D23" s="30"/>
@@ -8950,7 +8964,7 @@
       <c r="A24" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="B24" s="50">
+      <c r="B24" s="49">
         <v>3971.7894703400002</v>
       </c>
       <c r="D24" s="30"/>
@@ -8959,7 +8973,7 @@
       <c r="A25" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B25" s="50">
+      <c r="B25" s="49">
         <v>164.47925072999999</v>
       </c>
       <c r="D25" s="30"/>
@@ -8968,7 +8982,7 @@
       <c r="A26" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="B26" s="50">
+      <c r="B26" s="49">
         <v>409.54609006999999</v>
       </c>
       <c r="D26" s="30"/>
@@ -8977,7 +8991,7 @@
       <c r="A27" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="B27" s="50">
+      <c r="B27" s="49">
         <v>322.72882701999998</v>
       </c>
       <c r="D27" s="30"/>
@@ -8986,7 +9000,7 @@
       <c r="A28" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B28" s="50">
+      <c r="B28" s="49">
         <v>3712.53847206</v>
       </c>
       <c r="D28" s="30"/>
@@ -8995,7 +9009,7 @@
       <c r="A29" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="50">
+      <c r="B29" s="49">
         <v>128.95324006000001</v>
       </c>
       <c r="D29" s="30"/>
@@ -9004,7 +9018,7 @@
       <c r="A30" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="B30" s="50">
+      <c r="B30" s="49">
         <v>147.27759675999999</v>
       </c>
       <c r="D30" s="30"/>
@@ -9013,7 +9027,7 @@
       <c r="A31" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="B31" s="50">
+      <c r="B31" s="49">
         <v>56.991716140000001</v>
       </c>
       <c r="D31" s="30"/>
@@ -9022,7 +9036,7 @@
       <c r="A32" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="B32" s="50">
+      <c r="B32" s="49">
         <v>299.52692495999997</v>
       </c>
       <c r="D32" s="30"/>
@@ -9031,7 +9045,7 @@
       <c r="A33" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="B33" s="49">
+      <c r="B33" s="48">
         <v>10963.75355042</v>
       </c>
       <c r="D33" s="29"/>
@@ -9040,7 +9054,7 @@
       <c r="A34" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="B34" s="50">
+      <c r="B34" s="49">
         <v>2361.9270891900001</v>
       </c>
       <c r="D34" s="30"/>
@@ -9049,7 +9063,7 @@
       <c r="A35" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B35" s="50">
+      <c r="B35" s="49">
         <v>498.63657723</v>
       </c>
       <c r="D35" s="30"/>
@@ -9058,7 +9072,7 @@
       <c r="A36" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="B36" s="50">
+      <c r="B36" s="49">
         <v>69.397753019999996</v>
       </c>
       <c r="D36" s="30"/>
@@ -9067,7 +9081,7 @@
       <c r="A37" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="B37" s="50">
+      <c r="B37" s="49">
         <v>7.59139257</v>
       </c>
       <c r="D37" s="30"/>
@@ -9076,7 +9090,7 @@
       <c r="A38" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="B38" s="50">
+      <c r="B38" s="49">
         <v>174.5819454</v>
       </c>
       <c r="D38" s="30"/>
@@ -9085,7 +9099,7 @@
       <c r="A39" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B39" s="50">
+      <c r="B39" s="49">
         <v>43.539436969999997</v>
       </c>
       <c r="D39" s="30"/>
@@ -9094,7 +9108,7 @@
       <c r="A40" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="B40" s="50">
+      <c r="B40" s="49">
         <v>4.0489054099999997</v>
       </c>
       <c r="D40" s="30"/>
@@ -9103,7 +9117,7 @@
       <c r="A41" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="50">
+      <c r="B41" s="49">
         <v>55.587595579999999</v>
       </c>
       <c r="D41" s="30"/>
@@ -9112,7 +9126,7 @@
       <c r="A42" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="B42" s="50">
+      <c r="B42" s="49">
         <v>2534.0538823299999</v>
       </c>
       <c r="D42" s="30"/>
@@ -9121,7 +9135,7 @@
       <c r="A43" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B43" s="50">
+      <c r="B43" s="49">
         <v>1098.6494364099999</v>
       </c>
       <c r="D43" s="30"/>
@@ -9130,7 +9144,7 @@
       <c r="A44" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="B44" s="50">
+      <c r="B44" s="49">
         <v>529.39998568999999</v>
       </c>
       <c r="D44" s="30"/>
@@ -9139,7 +9153,7 @@
       <c r="A45" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B45" s="50">
+      <c r="B45" s="49">
         <v>3183.4768767599999</v>
       </c>
       <c r="D45" s="30"/>
@@ -9148,7 +9162,7 @@
       <c r="A46" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B46" s="50">
+      <c r="B46" s="49">
         <v>73.072475859999997</v>
       </c>
       <c r="D46" s="30"/>
@@ -9157,7 +9171,7 @@
       <c r="A47" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="B47" s="50">
+      <c r="B47" s="49">
         <v>329.79019799999998</v>
       </c>
       <c r="D47" s="30"/>
@@ -9166,7 +9180,7 @@
       <c r="A48" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="B48" s="49">
+      <c r="B48" s="48">
         <v>6181.8899169799997</v>
       </c>
       <c r="D48" s="29"/>
@@ -9175,7 +9189,7 @@
       <c r="A49" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B49" s="50">
+      <c r="B49" s="49">
         <v>3773.07590686</v>
       </c>
       <c r="D49" s="30"/>
@@ -9184,7 +9198,7 @@
       <c r="A50" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="B50" s="50">
+      <c r="B50" s="49">
         <v>1470.5336399299999</v>
       </c>
       <c r="D50" s="30"/>
@@ -9193,7 +9207,7 @@
       <c r="A51" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="B51" s="50">
+      <c r="B51" s="49">
         <v>42.737934950000003</v>
       </c>
       <c r="D51" s="30"/>
@@ -9202,7 +9216,7 @@
       <c r="A52" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="B52" s="50">
+      <c r="B52" s="49">
         <v>688.91321946999994</v>
       </c>
       <c r="D52" s="30"/>
@@ -9211,7 +9225,7 @@
       <c r="A53" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="B53" s="51">
+      <c r="B53" s="50">
         <v>206.62921577</v>
       </c>
     </row>

</xml_diff>

<commit_message>
"actualizo dato emae abril26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC3CD17-F080-4FAF-9713-19D12DB402DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AC08D5-75DF-4CA0-BAF2-C36B9BF50AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -3507,7 +3507,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D124"/>
+  <dimension ref="A1:D125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -3537,10 +3537,10 @@
         <v>134.74645041349706</v>
       </c>
       <c r="C2" s="36">
-        <v>148.03259196044854</v>
+        <v>147.93392530516525</v>
       </c>
       <c r="D2" s="36">
-        <v>147.12248518161707</v>
+        <v>147.05728802300575</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3551,10 +3551,10 @@
         <v>134.23236103862521</v>
       </c>
       <c r="C3" s="36">
-        <v>147.0699078640429</v>
+        <v>146.84557122133359</v>
       </c>
       <c r="D3" s="36">
-        <v>146.54332009692405</v>
+        <v>146.4791599743433</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3565,10 +3565,10 @@
         <v>150.0878942366954</v>
       </c>
       <c r="C4" s="36">
-        <v>146.14642347701553</v>
+        <v>145.96775878336345</v>
       </c>
       <c r="D4" s="36">
-        <v>145.9912186327727</v>
+        <v>145.93066633403586</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3579,10 +3579,10 @@
         <v>153.25067436662908</v>
       </c>
       <c r="C5" s="36">
-        <v>144.8588631415312</v>
+        <v>144.69616657974839</v>
       </c>
       <c r="D5" s="36">
-        <v>145.50216986623502</v>
+        <v>145.44963167660751</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3593,10 +3593,10 @@
         <v>163.51360808690507</v>
       </c>
       <c r="C6" s="36">
-        <v>144.58234022667378</v>
+        <v>144.56727263895843</v>
       </c>
       <c r="D6" s="36">
-        <v>145.10382835195102</v>
+        <v>145.06426744979953</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3607,10 +3607,10 @@
         <v>153.66209524099784</v>
       </c>
       <c r="C7" s="36">
-        <v>144.29890359910266</v>
+        <v>144.40750076903936</v>
       </c>
       <c r="D7" s="36">
-        <v>144.81749811409966</v>
+        <v>144.79569649622729</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3621,10 +3621,10 @@
         <v>143.73110098180126</v>
       </c>
       <c r="C8" s="36">
-        <v>144.46186040008149</v>
+        <v>144.60181651071224</v>
       </c>
       <c r="D8" s="36">
-        <v>144.65594973440716</v>
+        <v>144.65403542077127</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3635,10 +3635,10 @@
         <v>143.6741026486049</v>
       </c>
       <c r="C9" s="36">
-        <v>145.52336900371643</v>
+        <v>145.66149778877167</v>
       </c>
       <c r="D9" s="36">
-        <v>144.6266492667815</v>
+        <v>144.64223827479154</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3649,10 +3649,10 @@
         <v>142.00773744282046</v>
       </c>
       <c r="C10" s="36">
-        <v>144.89720375005177</v>
+        <v>144.98917021298641</v>
       </c>
       <c r="D10" s="36">
-        <v>144.7331158955412</v>
+        <v>144.75896347841521</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3663,10 +3663,10 @@
         <v>141.13686329808141</v>
       </c>
       <c r="C11" s="36">
-        <v>145.02139649041007</v>
+        <v>145.16989751944251</v>
       </c>
       <c r="D11" s="36">
-        <v>144.97043956020906</v>
+        <v>144.99665757430398</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3677,10 +3677,10 @@
         <v>144.93832064073018</v>
       </c>
       <c r="C12" s="36">
-        <v>145.7133902031533</v>
+        <v>145.77978651755154</v>
       </c>
       <c r="D12" s="36">
-        <v>145.3262772340878</v>
+        <v>145.34151040560658</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3691,10 +3691,10 @@
         <v>142.59014516031914</v>
       </c>
       <c r="C13" s="36">
-        <v>146.96510342900294</v>
+        <v>146.95099027389824</v>
       </c>
       <c r="D13" s="36">
-        <v>145.78656218575853</v>
+        <v>145.78176450559545</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3705,10 +3705,10 @@
         <v>136.63265948316197</v>
       </c>
       <c r="C14" s="36">
-        <v>147.23494762112568</v>
+        <v>147.09361189175286</v>
       </c>
       <c r="D14" s="36">
-        <v>146.33333771747371</v>
+        <v>146.30347289560493</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3719,10 +3719,10 @@
         <v>132.15851633982263</v>
       </c>
       <c r="C15" s="36">
-        <v>147.00185268779848</v>
+        <v>146.81999958929094</v>
       </c>
       <c r="D15" s="36">
-        <v>146.94471653439686</v>
+        <v>146.88879026400798</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3733,10 +3733,10 @@
         <v>152.62095855905721</v>
       </c>
       <c r="C16" s="36">
-        <v>147.76014108774692</v>
+        <v>147.63142117580773</v>
       </c>
       <c r="D16" s="36">
-        <v>147.59751892003072</v>
+        <v>147.51962090447577</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3747,10 +3747,10 @@
         <v>151.94634480448727</v>
       </c>
       <c r="C17" s="36">
-        <v>147.63096590455055</v>
+        <v>147.70171402358014</v>
       </c>
       <c r="D17" s="36">
-        <v>148.26736799772615</v>
+        <v>148.17522841474457</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3761,10 +3761,10 @@
         <v>168.38920946936767</v>
       </c>
       <c r="C18" s="36">
-        <v>148.52167958146185</v>
+        <v>148.67231109901837</v>
       </c>
       <c r="D18" s="36">
-        <v>148.92483939642733</v>
+        <v>148.82877687985808</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3775,10 +3775,10 @@
         <v>161.0356854694522</v>
       </c>
       <c r="C19" s="36">
-        <v>150.12442571118444</v>
+        <v>150.24574032624963</v>
       </c>
       <c r="D19" s="36">
-        <v>149.53712576798011</v>
+        <v>149.44932981707404</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3789,10 +3789,10 @@
         <v>150.3060501239199</v>
       </c>
       <c r="C20" s="36">
-        <v>150.42452382321926</v>
+        <v>150.47989229282791</v>
       </c>
       <c r="D20" s="36">
-        <v>150.06934845722793</v>
+        <v>150.00175591799729</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3803,10 +3803,10 @@
         <v>149.25534277384099</v>
       </c>
       <c r="C21" s="36">
-        <v>150.41158089521988</v>
+        <v>150.3849160508085</v>
       </c>
       <c r="D21" s="36">
-        <v>150.48641140604437</v>
+        <v>150.44828536486224</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3817,10 +3817,10 @@
         <v>146.38655965775374</v>
       </c>
       <c r="C22" s="36">
-        <v>151.26823308009077</v>
+        <v>151.20678120691389</v>
       </c>
       <c r="D22" s="36">
-        <v>150.75507340134595</v>
+        <v>150.75053058764885</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3831,10 +3831,10 @@
         <v>149.38594966601445</v>
       </c>
       <c r="C23" s="36">
-        <v>151.73469142491953</v>
+        <v>151.69720252270432</v>
       </c>
       <c r="D23" s="36">
-        <v>150.85035689592684</v>
+        <v>150.87798858941446</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3845,10 +3845,10 @@
         <v>151.92604285202682</v>
       </c>
       <c r="C24" s="36">
-        <v>152.59226993820425</v>
+        <v>152.63772357143588</v>
       </c>
       <c r="D24" s="36">
-        <v>150.7520652202968</v>
+        <v>150.80628666033164</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3859,10 +3859,10 @@
         <v>146.78338490922437</v>
       </c>
       <c r="C25" s="36">
-        <v>152.12139234183553</v>
+        <v>152.25539093894815</v>
       </c>
       <c r="D25" s="36">
-        <v>150.45222672541368</v>
+        <v>150.52355583017248</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3873,10 +3873,10 @@
         <v>142.74091260617209</v>
       </c>
       <c r="C26" s="36">
-        <v>150.71792889938533</v>
+        <v>150.98722525561379</v>
       </c>
       <c r="D26" s="36">
-        <v>149.95929283420745</v>
+        <v>150.03515094773516</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3887,10 +3887,10 @@
         <v>138.81804035165729</v>
       </c>
       <c r="C27" s="36">
-        <v>151.94087683188036</v>
+        <v>152.18519512030997</v>
       </c>
       <c r="D27" s="36">
-        <v>149.29648754360707</v>
+        <v>149.36311920629876</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3901,10 +3901,10 @@
         <v>155.85731953576962</v>
       </c>
       <c r="C28" s="36">
-        <v>151.3386001459065</v>
+        <v>151.5253120742554</v>
       </c>
       <c r="D28" s="36">
-        <v>148.50023246777778</v>
+        <v>148.54542503333764</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3915,10 +3915,10 @@
         <v>151.52454398394329</v>
       </c>
       <c r="C29" s="36">
-        <v>146.79524090203745</v>
+        <v>146.77368593383494</v>
       </c>
       <c r="D29" s="36">
-        <v>147.61590508743586</v>
+        <v>147.62847602367108</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3929,10 +3929,10 @@
         <v>159.56669237791655</v>
       </c>
       <c r="C30" s="36">
-        <v>144.67702249230945</v>
+        <v>144.56370636245163</v>
       </c>
       <c r="D30" s="36">
-        <v>146.69461483510227</v>
+        <v>146.66677122984348</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3943,10 +3943,10 @@
         <v>151.1257632334551</v>
       </c>
       <c r="C31" s="36">
-        <v>143.44436720597389</v>
+        <v>143.27743582661475</v>
       </c>
       <c r="D31" s="36">
-        <v>145.78930663291649</v>
+        <v>145.71784330042544</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -3957,10 +3957,10 @@
         <v>145.96352443000447</v>
       </c>
       <c r="C32" s="36">
-        <v>143.83317529524027</v>
+        <v>143.56630904676393</v>
       </c>
       <c r="D32" s="36">
-        <v>144.94897637629381</v>
+        <v>144.83517226102009</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3971,10 +3971,10 @@
         <v>146.76596003413957</v>
       </c>
       <c r="C33" s="36">
-        <v>146.73977573753155</v>
+        <v>146.5083763401191</v>
       </c>
       <c r="D33" s="36">
-        <v>144.21701514576142</v>
+        <v>144.0667550767985</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -3985,10 +3985,10 @@
         <v>137.74656971864789</v>
       </c>
       <c r="C34" s="36">
-        <v>143.22183703333664</v>
+        <v>143.17399592423629</v>
       </c>
       <c r="D34" s="36">
-        <v>143.62308744345492</v>
+        <v>143.44685177314395</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3999,10 +3999,10 @@
         <v>142.8432759845675</v>
       </c>
       <c r="C35" s="36">
-        <v>143.48339417996189</v>
+        <v>143.60656244287722</v>
       </c>
       <c r="D35" s="36">
-        <v>143.18038355223803</v>
+        <v>142.99223610249436</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -4013,10 +4013,10 @@
         <v>140.59240732533553</v>
       </c>
       <c r="C36" s="36">
-        <v>141.55480044795232</v>
+        <v>141.62161359564226</v>
       </c>
       <c r="D36" s="36">
-        <v>142.88990687978861</v>
+        <v>142.70444231322497</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -4027,10 +4027,10 @@
         <v>136.25161596905625</v>
       </c>
       <c r="C37" s="36">
-        <v>142.0496063686536</v>
+        <v>142.00720819392214</v>
       </c>
       <c r="D37" s="36">
-        <v>142.74011068149781</v>
+        <v>142.57062754953117</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -4041,10 +4041,10 @@
         <v>134.53623985669569</v>
       </c>
       <c r="C38" s="36">
-        <v>141.81369203436475</v>
+        <v>141.41909976735533</v>
       </c>
       <c r="D38" s="36">
-        <v>142.70524575457767</v>
+        <v>142.56274411876478</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4055,10 +4055,10 @@
         <v>132.2678886127365</v>
       </c>
       <c r="C39" s="36">
-        <v>144.2398618703196</v>
+        <v>143.63399679522843</v>
       </c>
       <c r="D39" s="36">
-        <v>142.75062969122965</v>
+        <v>142.64308433060683</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4069,10 +4069,10 @@
         <v>144.96325495574902</v>
       </c>
       <c r="C40" s="36">
-        <v>142.61988109044677</v>
+        <v>142.26347440308089</v>
       </c>
       <c r="D40" s="36">
-        <v>142.83705874562577</v>
+        <v>142.76985619334408</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4083,10 +4083,10 @@
         <v>149.91622140352257</v>
       </c>
       <c r="C41" s="36">
-        <v>142.54522297724586</v>
+        <v>142.5814610098206</v>
       </c>
       <c r="D41" s="36">
-        <v>142.92201598486434</v>
+        <v>142.8972437348074</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4097,10 +4097,10 @@
         <v>164.13569907592026</v>
       </c>
       <c r="C42" s="36">
-        <v>144.51686029398829</v>
+        <v>144.80047817480937</v>
       </c>
       <c r="D42" s="36">
-        <v>142.96702028919415</v>
+        <v>142.98303839742368</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4111,10 +4111,10 @@
         <v>150.85897174113111</v>
       </c>
       <c r="C43" s="36">
-        <v>143.62648333203899</v>
+        <v>144.09587933653643</v>
       </c>
       <c r="D43" s="36">
-        <v>142.9390000377669</v>
+        <v>142.99114760015667</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4125,10 +4125,10 @@
         <v>146.7770296400702</v>
       </c>
       <c r="C44" s="36">
-        <v>145.57248935472896</v>
+        <v>145.84338911769825</v>
       </c>
       <c r="D44" s="36">
-        <v>142.81154657802949</v>
+        <v>142.89375082962775</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4139,10 +4139,10 @@
         <v>141.27693468084021</v>
       </c>
       <c r="C45" s="36">
-        <v>144.62342018043961</v>
+        <v>144.80116322755515</v>
       </c>
       <c r="D45" s="36">
-        <v>142.56750628404998</v>
+        <v>142.67390042071176</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4153,10 +4153,10 @@
         <v>134.87706647993639</v>
       </c>
       <c r="C46" s="36">
-        <v>140.48644641644498</v>
+        <v>140.53903571586895</v>
       </c>
       <c r="D46" s="36">
-        <v>142.20031686216282</v>
+        <v>142.32654422761081</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -4167,10 +4167,10 @@
         <v>141.63933661701367</v>
       </c>
       <c r="C47" s="36">
-        <v>143.76525611707521</v>
+        <v>143.81839242743101</v>
       </c>
       <c r="D47" s="36">
-        <v>141.7140696561587</v>
+        <v>141.85799511764722</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -4178,13 +4178,13 @@
         <v>43770</v>
       </c>
       <c r="B48" s="17">
-        <v>137.77182966933131</v>
+        <v>137.77182966933134</v>
       </c>
       <c r="C48" s="36">
-        <v>140.87310912587668</v>
+        <v>140.87775693980214</v>
       </c>
       <c r="D48" s="36">
-        <v>141.1238481007837</v>
+        <v>141.28539477404658</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4192,13 +4192,13 @@
         <v>43800</v>
       </c>
       <c r="B49" s="17">
-        <v>135.76515452763491</v>
+        <v>135.76515452763488</v>
       </c>
       <c r="C49" s="36">
-        <v>140.10290445732591</v>
+        <v>140.11150090003781</v>
       </c>
       <c r="D49" s="36">
-        <v>140.45633781358129</v>
+        <v>140.63606308945876</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -4206,13 +4206,13 @@
         <v>43831</v>
       </c>
       <c r="B50" s="17">
-        <v>133.89108608957235</v>
+        <v>133.89108608957227</v>
       </c>
       <c r="C50" s="36">
-        <v>140.71252814452441</v>
+        <v>140.91697761884743</v>
       </c>
       <c r="D50" s="36">
-        <v>139.74261129934382</v>
+        <v>139.94160028898327</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -4220,13 +4220,13 @@
         <v>43862</v>
       </c>
       <c r="B51" s="17">
-        <v>128.97363874659814</v>
+        <v>128.97363874659808</v>
       </c>
       <c r="C51" s="36">
-        <v>139.35238005290518</v>
+        <v>139.55347026640555</v>
       </c>
       <c r="D51" s="36">
-        <v>139.01805511783414</v>
+        <v>139.23701145822935</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -4234,13 +4234,13 @@
         <v>43891</v>
       </c>
       <c r="B52" s="17">
-        <v>128.21106074025644</v>
+        <v>128.21106074025653</v>
       </c>
       <c r="C52" s="36">
-        <v>125.91338590990141</v>
+        <v>125.96973824909686</v>
       </c>
       <c r="D52" s="36">
-        <v>138.3194156496636</v>
+        <v>138.55833411203915</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -4248,13 +4248,13 @@
         <v>43922</v>
       </c>
       <c r="B53" s="17">
-        <v>113.29503444580112</v>
+        <v>113.29503444580143</v>
       </c>
       <c r="C53" s="36">
-        <v>106.15116639878501</v>
+        <v>105.99371760567273</v>
       </c>
       <c r="D53" s="36">
-        <v>137.68338337268341</v>
+        <v>137.94078869004042</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -4262,13 +4262,13 @@
         <v>43952</v>
       </c>
       <c r="B54" s="17">
-        <v>131.02956919734888</v>
+        <v>131.02956919734902</v>
       </c>
       <c r="C54" s="36">
-        <v>117.48924416484118</v>
+        <v>117.20862009281119</v>
       </c>
       <c r="D54" s="36">
-        <v>137.14435744012337</v>
+        <v>137.41736684572851</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -4276,13 +4276,13 @@
         <v>43983</v>
       </c>
       <c r="B55" s="17">
-        <v>132.52196526648811</v>
+        <v>132.52196526648763</v>
       </c>
       <c r="C55" s="36">
-        <v>124.62138887513295</v>
+        <v>124.34453609719363</v>
       </c>
       <c r="D55" s="36">
-        <v>136.72893144705949</v>
+        <v>137.01298862339578</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -4290,13 +4290,13 @@
         <v>44013</v>
       </c>
       <c r="B56" s="17">
-        <v>127.46368946979538</v>
+        <v>127.46368946979391</v>
       </c>
       <c r="C56" s="36">
-        <v>126.30495486357177</v>
+        <v>126.13173661675738</v>
       </c>
       <c r="D56" s="36">
-        <v>136.45479358706709</v>
+        <v>136.74386313284347</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -4304,13 +4304,13 @@
         <v>44044</v>
       </c>
       <c r="B57" s="17">
-        <v>125.18389375984702</v>
+        <v>125.18389375984641</v>
       </c>
       <c r="C57" s="36">
-        <v>128.88217104138715</v>
+        <v>128.86728972485162</v>
       </c>
       <c r="D57" s="36">
-        <v>136.33174707329843</v>
+        <v>136.61809092980613</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -4318,13 +4318,13 @@
         <v>44075</v>
       </c>
       <c r="B58" s="17">
-        <v>127.17507609335061</v>
+        <v>127.1750760933527</v>
       </c>
       <c r="C58" s="36">
-        <v>130.73468236002785</v>
+        <v>130.79987437384165</v>
       </c>
       <c r="D58" s="36">
-        <v>136.36003542140455</v>
+        <v>136.63583340346673</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -4332,13 +4332,13 @@
         <v>44105</v>
       </c>
       <c r="B59" s="17">
-        <v>131.34550189452122</v>
+        <v>131.34550189452784</v>
       </c>
       <c r="C59" s="36">
-        <v>133.28379428516581</v>
+        <v>133.41060851326921</v>
       </c>
       <c r="D59" s="36">
-        <v>136.53278399381435</v>
+        <v>136.79076013755875</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -4346,13 +4346,13 @@
         <v>44136</v>
       </c>
       <c r="B60" s="17">
-        <v>132.06865525299381</v>
+        <v>132.06865525299659</v>
       </c>
       <c r="C60" s="36">
-        <v>134.72927758000364</v>
+        <v>134.85001471194028</v>
       </c>
       <c r="D60" s="36">
-        <v>136.83548448580393</v>
+        <v>137.06983870593521</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -4360,13 +4360,13 @@
         <v>44166</v>
       </c>
       <c r="B61" s="17">
-        <v>133.85436559461547</v>
+        <v>133.85436559460604</v>
       </c>
       <c r="C61" s="36">
-        <v>136.83856286567271</v>
+        <v>136.96695318017814</v>
       </c>
       <c r="D61" s="36">
-        <v>137.24990532734935</v>
+        <v>137.45686112626854</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -4374,13 +4374,13 @@
         <v>44197</v>
       </c>
       <c r="B62" s="17">
-        <v>131.52153739734879</v>
+        <v>131.52153739731881</v>
       </c>
       <c r="C62" s="36">
-        <v>139.70457666741626</v>
+        <v>139.86778985546729</v>
       </c>
       <c r="D62" s="36">
-        <v>137.75779473374334</v>
+        <v>137.93577366070608</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -4388,13 +4388,13 @@
         <v>44228</v>
       </c>
       <c r="B63" s="17">
-        <v>126.23926696837668</v>
+        <v>126.23926696836405</v>
       </c>
       <c r="C63" s="36">
-        <v>138.16466747971225</v>
+        <v>138.20028013173521</v>
       </c>
       <c r="D63" s="36">
-        <v>138.34554082492741</v>
+        <v>138.49506341728181</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -4402,13 +4402,13 @@
         <v>44256</v>
       </c>
       <c r="B64" s="17">
-        <v>145.95690010360443</v>
+        <v>145.95690010364706</v>
       </c>
       <c r="C64" s="36">
-        <v>140.93214881658653</v>
+        <v>140.91577065783943</v>
       </c>
       <c r="D64" s="36">
-        <v>139.00251506565144</v>
+        <v>139.12542597753085</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -4416,13 +4416,13 @@
         <v>44287</v>
       </c>
       <c r="B65" s="17">
-        <v>147.28084401862364</v>
+        <v>147.28084401875944</v>
       </c>
       <c r="C65" s="36">
-        <v>139.32168396782794</v>
+        <v>139.26049396360543</v>
       </c>
       <c r="D65" s="36">
-        <v>139.72449517997134</v>
+        <v>139.8235460686619</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -4430,13 +4430,13 @@
         <v>44317</v>
       </c>
       <c r="B66" s="17">
-        <v>151.16932233869088</v>
+        <v>151.16932233874812</v>
       </c>
       <c r="C66" s="36">
-        <v>138.85334943464642</v>
+        <v>138.87942821950787</v>
       </c>
       <c r="D66" s="36">
-        <v>140.51012885766744</v>
+        <v>140.58828401842547</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -4444,13 +4444,13 @@
         <v>44348</v>
       </c>
       <c r="B67" s="17">
-        <v>148.97961710860534</v>
+        <v>148.97961710841227</v>
       </c>
       <c r="C67" s="36">
-        <v>141.49305609851737</v>
+        <v>141.55493596421903</v>
       </c>
       <c r="D67" s="36">
-        <v>141.35688684818371</v>
+        <v>141.41703636524801</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -4458,13 +4458,13 @@
         <v>44378</v>
       </c>
       <c r="B68" s="17">
-        <v>142.42591306097313</v>
+        <v>142.42591306035797</v>
       </c>
       <c r="C68" s="36">
-        <v>141.35152150148488</v>
+        <v>141.38117057908835</v>
       </c>
       <c r="D68" s="36">
-        <v>142.26480880715039</v>
+        <v>142.30989872852675</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -4472,13 +4472,13 @@
         <v>44409</v>
       </c>
       <c r="B69" s="17">
-        <v>140.9749407280365</v>
+        <v>140.97494072777721</v>
       </c>
       <c r="C69" s="36">
-        <v>143.26893353155685</v>
+        <v>143.29501888821403</v>
       </c>
       <c r="D69" s="36">
-        <v>143.23311468502996</v>
+        <v>143.26598461789402</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -4486,13 +4486,13 @@
         <v>44440</v>
       </c>
       <c r="B70" s="17">
-        <v>141.29608908940958</v>
+        <v>141.29608909028403</v>
       </c>
       <c r="C70" s="36">
-        <v>144.12924670258064</v>
+        <v>144.1962251789204</v>
       </c>
       <c r="D70" s="36">
-        <v>144.25466621351507</v>
+        <v>144.27799737026854</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -4500,13 +4500,13 @@
         <v>44470</v>
       </c>
       <c r="B71" s="17">
-        <v>139.51475869689278</v>
+        <v>139.51475869967888</v>
       </c>
       <c r="C71" s="36">
-        <v>143.42130203769142</v>
+        <v>143.38274230679909</v>
       </c>
       <c r="D71" s="36">
-        <v>145.31658660175071</v>
+        <v>145.3330444755376</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -4514,13 +4514,13 @@
         <v>44501</v>
       </c>
       <c r="B72" s="17">
-        <v>143.75187761771406</v>
+        <v>143.75187761888847</v>
       </c>
       <c r="C72" s="36">
-        <v>145.84431289987916</v>
+        <v>145.70199915320512</v>
       </c>
       <c r="D72" s="36">
-        <v>146.39426304865009</v>
+        <v>146.4062746613703</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -4528,13 +4528,13 @@
         <v>44531</v>
       </c>
       <c r="B73" s="17">
-        <v>147.22987832209424</v>
+        <v>147.22987831813373</v>
       </c>
       <c r="C73" s="36">
-        <v>149.85614630222497</v>
+        <v>149.70509110366692</v>
       </c>
       <c r="D73" s="36">
-        <v>147.45113221744668</v>
+        <v>147.46081171992913</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -4542,13 +4542,13 @@
         <v>44562</v>
       </c>
       <c r="B74" s="17">
-        <v>139.63796162489982</v>
+        <v>139.637961612281</v>
       </c>
       <c r="C74" s="36">
-        <v>148.53342518810345</v>
+        <v>148.55190380544317</v>
       </c>
       <c r="D74" s="36">
-        <v>148.44505029148579</v>
+        <v>148.45392567357925</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -4556,13 +4556,13 @@
         <v>44593</v>
       </c>
       <c r="B75" s="17">
-        <v>137.8495135303948</v>
+        <v>137.84951352507554</v>
       </c>
       <c r="C75" s="36">
-        <v>150.74492398940484</v>
+        <v>150.64256656224384</v>
       </c>
       <c r="D75" s="36">
-        <v>149.3323280608528</v>
+        <v>149.34073907795377</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -4570,13 +4570,13 @@
         <v>44621</v>
       </c>
       <c r="B76" s="17">
-        <v>153.93085077631505</v>
+        <v>153.9308507942531</v>
       </c>
       <c r="C76" s="36">
-        <v>150.39127357945512</v>
+        <v>150.3860254781107</v>
       </c>
       <c r="D76" s="36">
-        <v>150.0754352569179</v>
+        <v>150.08321581555236</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -4584,13 +4584,13 @@
         <v>44652</v>
       </c>
       <c r="B77" s="17">
-        <v>157.66169211629364</v>
+        <v>157.66169217344674</v>
       </c>
       <c r="C77" s="36">
-        <v>151.97961391938657</v>
+        <v>152.07758234261067</v>
       </c>
       <c r="D77" s="36">
-        <v>150.64689924251402</v>
+        <v>150.6534040255867</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -4598,13 +4598,13 @@
         <v>44682</v>
       </c>
       <c r="B78" s="17">
-        <v>164.68936308999193</v>
+        <v>164.68936311408393</v>
       </c>
       <c r="C78" s="36">
-        <v>151.99823712672884</v>
+        <v>152.10152135054884</v>
       </c>
       <c r="D78" s="36">
-        <v>151.03010399627965</v>
+        <v>151.03507926055096</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -4612,13 +4612,13 @@
         <v>44713</v>
       </c>
       <c r="B79" s="17">
-        <v>161.45483436245786</v>
+        <v>161.4548342812127</v>
       </c>
       <c r="C79" s="36">
-        <v>154.17057671019109</v>
+        <v>154.34825750063149</v>
       </c>
       <c r="D79" s="36">
-        <v>151.22061177468228</v>
+        <v>151.2247471775994</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -4626,13 +4626,13 @@
         <v>44743</v>
       </c>
       <c r="B80" s="17">
-        <v>152.44538769471922</v>
+        <v>152.44538743586068</v>
       </c>
       <c r="C80" s="36">
-        <v>152.4843590272539</v>
+        <v>152.57931165808276</v>
       </c>
       <c r="D80" s="36">
-        <v>151.23089937815624</v>
+        <v>151.23534588803642</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4640,13 +4640,13 @@
         <v>44774</v>
       </c>
       <c r="B81" s="17">
-        <v>151.46573902517952</v>
+        <v>151.46573891606155</v>
       </c>
       <c r="C81" s="36">
-        <v>151.6948373531994</v>
+        <v>151.71959575650231</v>
       </c>
       <c r="D81" s="36">
-        <v>151.08703011796365</v>
+        <v>151.09312241380925</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4654,13 +4654,13 @@
         <v>44805</v>
       </c>
       <c r="B82" s="17">
-        <v>149.17434933730516</v>
+        <v>149.17434970528168</v>
       </c>
       <c r="C82" s="36">
-        <v>150.78862727184716</v>
+        <v>150.7700560603914</v>
       </c>
       <c r="D82" s="36">
-        <v>150.82433398583012</v>
+        <v>150.8332071036196</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4668,13 +4668,13 @@
         <v>44835</v>
       </c>
       <c r="B83" s="17">
-        <v>146.55439498927831</v>
+        <v>146.55439616170329</v>
       </c>
       <c r="C83" s="36">
-        <v>149.26291297659591</v>
+        <v>149.10270937214764</v>
       </c>
       <c r="D83" s="36">
-        <v>150.48208706226896</v>
+        <v>150.49434645972877</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4682,13 +4682,13 @@
         <v>44866</v>
       </c>
       <c r="B84" s="17">
-        <v>148.03049443530639</v>
+        <v>148.03049492952468</v>
       </c>
       <c r="C84" s="36">
-        <v>148.50744581790943</v>
+        <v>148.30045235840549</v>
       </c>
       <c r="D84" s="36">
-        <v>150.09803027790036</v>
+        <v>150.11367270204204</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -4696,13 +4696,13 @@
         <v>44896</v>
       </c>
       <c r="B85" s="17">
-        <v>146.18080800460334</v>
+        <v>146.18080633796006</v>
       </c>
       <c r="C85" s="36">
-        <v>148.51915601579663</v>
+        <v>148.49540732677499</v>
       </c>
       <c r="D85" s="36">
-        <v>149.70569583590233</v>
+        <v>149.72367305158448</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -4710,13 +4710,13 @@
         <v>44927</v>
       </c>
       <c r="B86" s="17">
-        <v>143.03019028687322</v>
+        <v>143.03462349487495</v>
       </c>
       <c r="C86" s="36">
-        <v>149.68781431945897</v>
+        <v>149.96952713298742</v>
       </c>
       <c r="D86" s="36">
-        <v>149.32875801936962</v>
+        <v>149.34688054655493</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4724,13 +4724,13 @@
         <v>44958</v>
       </c>
       <c r="B87" s="17">
-        <v>137.26202711167147</v>
+        <v>137.26646276476467</v>
       </c>
       <c r="C87" s="36">
-        <v>149.83792215936882</v>
+        <v>150.10387208507404</v>
       </c>
       <c r="D87" s="36">
-        <v>148.97776846074467</v>
+        <v>148.99278837030343</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -4738,13 +4738,13 @@
         <v>44986</v>
       </c>
       <c r="B88" s="17">
-        <v>155.06056763767785</v>
+        <v>155.06501366898644</v>
       </c>
       <c r="C88" s="36">
-        <v>150.72559893860952</v>
+        <v>150.79671770186954</v>
       </c>
       <c r="D88" s="36">
-        <v>148.64892451373936</v>
+        <v>148.65736303565535</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -4752,13 +4752,13 @@
         <v>45017</v>
       </c>
       <c r="B89" s="17">
-        <v>150.02108492538545</v>
+        <v>150.05952685125044</v>
       </c>
       <c r="C89" s="36">
-        <v>147.35345724832627</v>
+        <v>147.42919171933761</v>
       </c>
       <c r="D89" s="36">
-        <v>148.32823404015883</v>
+        <v>148.32612883201449</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4766,13 +4766,13 @@
         <v>45047</v>
       </c>
       <c r="B90" s="17">
-        <v>153.77240570475391</v>
+        <v>153.81085419260503</v>
       </c>
       <c r="C90" s="36">
-        <v>145.65274008781518</v>
+        <v>145.50808199864673</v>
       </c>
       <c r="D90" s="36">
-        <v>147.99392557318464</v>
+        <v>147.97653557702176</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4780,13 +4780,13 @@
         <v>45078</v>
       </c>
       <c r="B91" s="17">
-        <v>152.55703188453069</v>
+        <v>152.59547604809092</v>
       </c>
       <c r="C91" s="36">
-        <v>146.23462401232104</v>
+        <v>146.0362071856969</v>
       </c>
       <c r="D91" s="36">
-        <v>147.62575922056891</v>
+        <v>147.58827361699645</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -4794,13 +4794,13 @@
         <v>45108</v>
       </c>
       <c r="B92" s="17">
-        <v>150.22297368931731</v>
+        <v>150.20312548190341</v>
       </c>
       <c r="C92" s="36">
-        <v>148.72524080197135</v>
+        <v>148.73013107795748</v>
       </c>
       <c r="D92" s="36">
-        <v>147.21026171068672</v>
+        <v>147.14923296818338</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -4808,13 +4808,13 @@
         <v>45139</v>
       </c>
       <c r="B93" s="17">
-        <v>151.94203814941196</v>
+        <v>151.92217935804922</v>
       </c>
       <c r="C93" s="36">
-        <v>150.00726396900734</v>
+        <v>150.0390804234014</v>
       </c>
       <c r="D93" s="36">
-        <v>146.74203556750248</v>
+        <v>146.65580516741312</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -4822,13 +4822,13 @@
         <v>45170</v>
       </c>
       <c r="B94" s="17">
-        <v>148.43224326812449</v>
+        <v>148.41237963987399</v>
       </c>
       <c r="C94" s="36">
-        <v>149.59810584615002</v>
+        <v>149.71064515367252</v>
       </c>
       <c r="D94" s="36">
-        <v>146.22865310169632</v>
+        <v>146.11778260269955</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4836,13 +4836,13 @@
         <v>45200</v>
       </c>
       <c r="B95" s="17">
-        <v>147.50696065384125</v>
+        <v>147.51381305414859</v>
       </c>
       <c r="C95" s="36">
-        <v>148.12592076567134</v>
+        <v>147.98485863929363</v>
       </c>
       <c r="D95" s="36">
-        <v>145.69121385227334</v>
+        <v>145.55865524812774</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -4850,13 +4850,13 @@
         <v>45231</v>
       </c>
       <c r="B96" s="17">
-        <v>146.35949532905394</v>
+        <v>146.36635232721147</v>
       </c>
       <c r="C96" s="36">
-        <v>146.56608348557839</v>
+        <v>146.37566723734164</v>
       </c>
       <c r="D96" s="36">
-        <v>145.16023078157343</v>
+        <v>145.01025992107282</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -4864,13 +4864,13 @@
         <v>45261</v>
       </c>
       <c r="B97" s="17">
-        <v>139.33576577457379</v>
+        <v>139.34262723777164</v>
       </c>
       <c r="C97" s="36">
-        <v>142.98801277026385</v>
+        <v>142.90845433855887</v>
       </c>
       <c r="D97" s="36">
-        <v>144.67835644481076</v>
+        <v>144.51678109590449</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -4878,13 +4878,13 @@
         <v>45292</v>
       </c>
       <c r="B98" s="17">
-        <v>137.54602738582324</v>
+        <v>137.37335120058367</v>
       </c>
       <c r="C98" s="36">
-        <v>143.73002234447563</v>
+        <v>143.57157054122101</v>
       </c>
       <c r="D98" s="36">
-        <v>144.29285443638179</v>
+        <v>144.12666448134632</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4892,13 +4892,13 @@
         <v>45323</v>
       </c>
       <c r="B99" s="17">
-        <v>133.6372238546686</v>
+        <v>133.46450581005294</v>
       </c>
       <c r="C99" s="36">
-        <v>143.96637419864555</v>
+        <v>143.69325878964582</v>
       </c>
       <c r="D99" s="36">
-        <v>144.04879155920639</v>
+        <v>143.88612523109015</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4906,13 +4906,13 @@
         <v>45352</v>
       </c>
       <c r="B100" s="17">
-        <v>142.56862047767686</v>
+        <v>142.39572385637248</v>
       </c>
       <c r="C100" s="36">
-        <v>142.54642488874453</v>
+        <v>142.2121938396119</v>
       </c>
       <c r="D100" s="36">
-        <v>143.98450504657345</v>
+        <v>143.83383928542497</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4920,13 +4920,13 @@
         <v>45383</v>
       </c>
       <c r="B101" s="17">
-        <v>147.26512441308907</v>
+        <v>147.25690008767782</v>
       </c>
       <c r="C101" s="36">
-        <v>140.92368699921087</v>
+        <v>141.13498723520038</v>
       </c>
       <c r="D101" s="36">
-        <v>144.12236109978107</v>
+        <v>143.99062537877512</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4934,13 +4934,13 @@
         <v>45413</v>
       </c>
       <c r="B102" s="17">
-        <v>156.77658370440048</v>
+        <v>156.76909889616599</v>
       </c>
       <c r="C102" s="36">
-        <v>142.63883411487311</v>
+        <v>142.70361097206074</v>
       </c>
       <c r="D102" s="36">
-        <v>144.46546086249469</v>
+        <v>144.35633880962916</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4948,13 +4948,13 @@
         <v>45444</v>
       </c>
       <c r="B103" s="17">
-        <v>147.3651695607501</v>
+        <v>147.35712151974346</v>
       </c>
       <c r="C103" s="36">
-        <v>143.75498601431281</v>
+        <v>143.77246679244459</v>
       </c>
       <c r="D103" s="36">
-        <v>144.99937183784681</v>
+        <v>144.91350117465768</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -4962,13 +4962,13 @@
         <v>45474</v>
       </c>
       <c r="B104" s="17">
-        <v>149.69752758894006</v>
+        <v>149.65170047837228</v>
       </c>
       <c r="C104" s="36">
-        <v>147.37653414122337</v>
+        <v>147.25816448563663</v>
       </c>
       <c r="D104" s="36">
-        <v>145.69208574365354</v>
+        <v>145.62760787754601</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -4976,13 +4976,13 @@
         <v>45505</v>
       </c>
       <c r="B105" s="17">
-        <v>147.32757374137327</v>
+        <v>147.28124762344183</v>
       </c>
       <c r="C105" s="36">
-        <v>147.97373835224366</v>
+        <v>147.77108034400263</v>
       </c>
       <c r="D105" s="36">
-        <v>146.4971186597223</v>
+        <v>146.45095583923919</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -4990,13 +4990,13 @@
         <v>45536</v>
       </c>
       <c r="B106" s="17">
-        <v>144.84378214964087</v>
+        <v>144.79670189548858</v>
       </c>
       <c r="C106" s="36">
-        <v>147.87078603835897</v>
+        <v>147.85494960643146</v>
       </c>
       <c r="D106" s="36">
-        <v>147.35997551702889</v>
+        <v>147.33080625379648</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -5004,13 +5004,13 @@
         <v>45566</v>
       </c>
       <c r="B107" s="17">
-        <v>147.99465960461652</v>
+        <v>148.10395140212873</v>
       </c>
       <c r="C107" s="36">
-        <v>148.91795097219361</v>
+        <v>149.03990472112946</v>
       </c>
       <c r="D107" s="36">
-        <v>148.22409664481577</v>
+        <v>148.20942501255277</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -5018,13 +5018,13 @@
         <v>45597</v>
       </c>
       <c r="B108" s="17">
-        <v>148.0693736646877</v>
+        <v>148.17873351747122</v>
       </c>
       <c r="C108" s="36">
-        <v>150.67943730794542</v>
+        <v>150.78759235875461</v>
       </c>
       <c r="D108" s="36">
-        <v>149.03951205065769</v>
+        <v>149.03728223119072</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -5032,13 +5032,13 @@
         <v>45627</v>
       </c>
       <c r="B109" s="17">
-        <v>148.56734585957747</v>
+        <v>148.67760152837457</v>
       </c>
       <c r="C109" s="36">
-        <v>151.28023662248589</v>
+        <v>151.50685869618016</v>
       </c>
       <c r="D109" s="36">
-        <v>149.76658666379012</v>
+        <v>149.77811271241328</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -5046,13 +5046,13 @@
         <v>45658</v>
       </c>
       <c r="B110" s="17">
-        <v>146.29581433061375</v>
+        <v>146.4966364505224</v>
       </c>
       <c r="C110" s="36">
-        <v>151.60733019823945</v>
+        <v>151.92199575618426</v>
       </c>
       <c r="D110" s="36">
-        <v>150.3790598898201</v>
+        <v>150.40784174193331</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -5060,13 +5060,13 @@
         <v>45689</v>
       </c>
       <c r="B111" s="17">
-        <v>141.20217475797378</v>
+        <v>141.40459964053429</v>
       </c>
       <c r="C111" s="36">
-        <v>153.28126184011842</v>
+        <v>153.37296425710733</v>
       </c>
       <c r="D111" s="36">
-        <v>150.86631214680529</v>
+        <v>150.91761287520407</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -5074,13 +5074,13 @@
         <v>45717</v>
       </c>
       <c r="B112" s="17">
-        <v>150.40654121723682</v>
+        <v>150.61015153616984</v>
       </c>
       <c r="C112" s="36">
-        <v>149.72690968302643</v>
+        <v>149.52580958425588</v>
       </c>
       <c r="D112" s="36">
-        <v>151.23364216518962</v>
+        <v>151.3132652618672</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -5088,13 +5088,13 @@
         <v>45748</v>
       </c>
       <c r="B113" s="17">
-        <v>158.7410459584533</v>
+        <v>158.93929877299897</v>
       </c>
       <c r="C113" s="36">
-        <v>152.12611612616246</v>
+        <v>152.58190688614374</v>
       </c>
       <c r="D113" s="36">
-        <v>151.49744481721694</v>
+        <v>151.6118327838486</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -5102,13 +5102,13 @@
         <v>45778</v>
       </c>
       <c r="B114" s="17">
-        <v>164.8778739250919</v>
+        <v>165.07464344720012</v>
       </c>
       <c r="C114" s="36">
-        <v>151.92223808290362</v>
+        <v>152.10509850995368</v>
       </c>
       <c r="D114" s="36">
-        <v>151.68726574738375</v>
+        <v>151.84009916066287</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -5116,13 +5116,13 @@
         <v>45809</v>
       </c>
       <c r="B115" s="17">
-        <v>156.59409988827613</v>
+        <v>156.78890416942744</v>
       </c>
       <c r="C115" s="36">
-        <v>151.45990022602729</v>
+        <v>151.51591341259004</v>
       </c>
       <c r="D115" s="36">
-        <v>151.83958460765547</v>
+        <v>152.02852454257786</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -5130,13 +5130,13 @@
         <v>45839</v>
       </c>
       <c r="B116" s="17">
-        <v>153.90797901553967</v>
+        <v>153.77022153385636</v>
       </c>
       <c r="C116" s="36">
-        <v>151.39642049120224</v>
+        <v>151.26917850671157</v>
       </c>
       <c r="D116" s="36">
-        <v>151.99402999523531</v>
+        <v>152.20647526950384</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -5144,13 +5144,13 @@
         <v>45870</v>
       </c>
       <c r="B117" s="17">
-        <v>150.51267456824078</v>
+        <v>150.37579448728511</v>
       </c>
       <c r="C117" s="36">
-        <v>152.35274901258254</v>
+        <v>152.18135872900501</v>
       </c>
       <c r="D117" s="36">
-        <v>152.18345397817774</v>
+        <v>152.39827698759578</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -5158,13 +5158,13 @@
         <v>45901</v>
       </c>
       <c r="B118" s="17">
-        <v>151.83947735250638</v>
+        <v>151.70554766622169</v>
       </c>
       <c r="C118" s="36">
-        <v>153.34133826499504</v>
+        <v>153.29642934768646</v>
       </c>
       <c r="D118" s="36">
-        <v>152.43339517408262</v>
+        <v>152.6196401859325</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -5172,13 +5172,13 @@
         <v>45931</v>
       </c>
       <c r="B119" s="17">
-        <v>152.56490425090988</v>
+        <v>152.83834864492212</v>
       </c>
       <c r="C119" s="36">
-        <v>152.74008837138231</v>
+        <v>153.03322057927417</v>
       </c>
       <c r="D119" s="36">
-        <v>152.7594881325218</v>
+        <v>152.8804146809866</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -5186,13 +5186,13 @@
         <v>45962</v>
       </c>
       <c r="B120" s="17">
-        <v>147.69599372441905</v>
+        <v>147.97168634998309</v>
       </c>
       <c r="C120" s="36">
-        <v>152.68704430271981</v>
+        <v>153.03461772858515</v>
       </c>
       <c r="D120" s="36">
-        <v>153.17608301339749</v>
+        <v>153.18672194001437</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -5200,13 +5200,13 @@
         <v>45992</v>
       </c>
       <c r="B121" s="17">
-        <v>153.5212203973648</v>
+        <v>153.84616590720057</v>
       </c>
       <c r="C121" s="36">
-        <v>155.5184030224774</v>
+        <v>155.98350628491656</v>
       </c>
       <c r="D121" s="36">
-        <v>153.68628115401089</v>
+        <v>153.54155126861306</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -5214,13 +5214,13 @@
         <v>46023</v>
       </c>
       <c r="B122" s="17">
-        <v>148.55280173083167</v>
+        <v>149.47367834853273</v>
       </c>
       <c r="C122" s="36">
-        <v>155.16250785100169</v>
+        <v>156.38624193363779</v>
       </c>
       <c r="D122" s="36">
-        <v>154.27673098059162</v>
+        <v>153.93960010835144</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -5228,27 +5228,41 @@
         <v>46054</v>
       </c>
       <c r="B123" s="17">
-        <v>138.34257152166515</v>
+        <v>139.28192710129798</v>
       </c>
       <c r="C123" s="36">
-        <v>151.03332855790745</v>
+        <v>152.22089169617513</v>
       </c>
       <c r="D123" s="36">
-        <v>154.9235774379822</v>
+        <v>154.36883960988379</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
         <v>46082</v>
       </c>
-      <c r="B124" s="40">
-        <v>158.64871746521388</v>
-      </c>
-      <c r="C124" s="41">
-        <v>156.28980610599837</v>
-      </c>
-      <c r="D124" s="41">
-        <v>155.59922265893965</v>
+      <c r="B124" s="17">
+        <v>159.96271036768385</v>
+      </c>
+      <c r="C124" s="36">
+        <v>156.88717457417997</v>
+      </c>
+      <c r="D124" s="36">
+        <v>154.81366098735921</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="4">
+        <v>46113</v>
+      </c>
+      <c r="B125" s="40">
+        <v>161.53886451705466</v>
+      </c>
+      <c r="C125" s="41">
+        <v>154.49351243562697</v>
+      </c>
+      <c r="D125" s="41">
+        <v>155.25620223242203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
"Actualizo IPC Junio y res fiscal jun26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AC08D5-75DF-4CA0-BAF2-C36B9BF50AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEE6477E-B214-4D59-8D8D-3F08F67FD215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -1339,7 +1339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="1" customWidth="1"/>
@@ -3277,12 +3277,29 @@
         <v>2.1</v>
       </c>
       <c r="C114">
+        <v>3.5</v>
+      </c>
+      <c r="D114">
+        <v>1.9</v>
+      </c>
+      <c r="E114">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="19">
+        <v>46174</v>
+      </c>
+      <c r="B115" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="C115">
         <v>3.4</v>
       </c>
-      <c r="D114">
-        <v>2.1</v>
-      </c>
-      <c r="E114">
+      <c r="D115">
+        <v>1.6</v>
+      </c>
+      <c r="E115">
         <v>2.2999999999999998</v>
       </c>
     </row>
@@ -5310,25 +5327,25 @@
         <v>112</v>
       </c>
       <c r="B2" s="37">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="C2" s="20">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="D2" s="20">
-        <v>3</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E2" s="20">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="F2" s="20">
-        <v>1.9</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G2" s="20">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="H2" s="16">
-        <v>2.683945290155676</v>
+        <v>2.3912881772367944</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5336,25 +5353,25 @@
         <v>113</v>
       </c>
       <c r="B3" s="37">
+        <v>0.1</v>
+      </c>
+      <c r="C3" s="20">
+        <v>0</v>
+      </c>
+      <c r="D3" s="20">
+        <v>0.9</v>
+      </c>
+      <c r="E3" s="20">
         <v>0.2</v>
-      </c>
-      <c r="C3" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="D3" s="20">
-        <v>0.4</v>
-      </c>
-      <c r="E3" s="20">
-        <v>0.4</v>
       </c>
       <c r="F3" s="20">
         <v>-0.7</v>
       </c>
       <c r="G3" s="20">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="H3" s="16">
-        <v>0.30128929683261862</v>
+        <v>5.5247484828879756E-2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5362,25 +5379,25 @@
         <v>114</v>
       </c>
       <c r="B4" s="37">
-        <v>3.6</v>
+        <v>0.4</v>
       </c>
       <c r="C4" s="20">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="D4" s="20">
-        <v>3.1</v>
+        <v>2.1</v>
       </c>
       <c r="E4" s="20">
-        <v>2.2000000000000002</v>
+        <v>1.7</v>
       </c>
       <c r="F4" s="20">
-        <v>3</v>
+        <v>-0.2</v>
       </c>
       <c r="G4" s="20">
-        <v>2.7</v>
+        <v>1</v>
       </c>
       <c r="H4" s="16">
-        <v>3.1337998632663844</v>
+        <v>1.0312155789434119</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5388,25 +5405,25 @@
         <v>115</v>
       </c>
       <c r="B5" s="37">
-        <v>4.0999999999999996</v>
+        <v>0.7</v>
       </c>
       <c r="C5" s="20">
-        <v>3.9</v>
+        <v>1.8</v>
       </c>
       <c r="D5" s="20">
-        <v>2.9</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="E5" s="20">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
       <c r="F5" s="20">
-        <v>4.5</v>
+        <v>0.5</v>
       </c>
       <c r="G5" s="20">
-        <v>2.2999999999999998</v>
+        <v>2.7</v>
       </c>
       <c r="H5" s="16">
-        <v>3.7805313476907854</v>
+        <v>1.3303893574575953</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5414,25 +5431,25 @@
         <v>116</v>
       </c>
       <c r="B6" s="37">
-        <v>-5.9</v>
+        <v>-2.6</v>
       </c>
       <c r="C6" s="20">
-        <v>-5.2</v>
+        <v>-3.1</v>
       </c>
       <c r="D6" s="20">
-        <v>-2.2000000000000002</v>
+        <v>-3.5</v>
       </c>
       <c r="E6" s="20">
-        <v>-5.2</v>
+        <v>-1.7</v>
       </c>
       <c r="F6" s="20">
-        <v>-6.3</v>
+        <v>-4.3</v>
       </c>
       <c r="G6" s="20">
-        <v>-3.4</v>
+        <v>-5</v>
       </c>
       <c r="H6" s="16">
-        <v>-5.3366002898128091</v>
+        <v>-2.9896060095035426</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5440,25 +5457,25 @@
         <v>117</v>
       </c>
       <c r="B7" s="37">
-        <v>18.8</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="C7" s="20">
-        <v>12.8</v>
+        <v>5.9</v>
       </c>
       <c r="D7" s="20">
-        <v>8.1999999999999993</v>
+        <v>4.7</v>
       </c>
       <c r="E7" s="20">
-        <v>12.9</v>
+        <v>3.8</v>
       </c>
       <c r="F7" s="20">
-        <v>15.3</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="G7" s="20">
-        <v>9.3000000000000007</v>
+        <v>9.4</v>
       </c>
       <c r="H7" s="16">
-        <v>15.196813550847477</v>
+        <v>7.4654649817116114</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5466,25 +5483,25 @@
         <v>118</v>
       </c>
       <c r="B8" s="37">
-        <v>3.6</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="20">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="D8" s="20">
-        <v>4.2</v>
+        <v>1.9</v>
       </c>
       <c r="E8" s="20">
-        <v>3</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F8" s="20">
-        <v>3.3</v>
+        <v>0.9</v>
       </c>
       <c r="G8" s="20">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="H8" s="16">
-        <v>3.208517775489117</v>
+        <v>1.2830523940615901</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5492,25 +5509,25 @@
         <v>119</v>
       </c>
       <c r="B9" s="37">
-        <v>2.1</v>
+        <v>-0.5</v>
       </c>
       <c r="C9" s="20">
-        <v>2.5</v>
+        <v>0.9</v>
       </c>
       <c r="D9" s="20">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="E9" s="20">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="F9" s="20">
-        <v>2.1</v>
+        <v>0.4</v>
       </c>
       <c r="G9" s="20">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
       <c r="H9" s="16">
-        <v>2.1193218367733468</v>
+        <v>0.43334628218292259</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5518,25 +5535,25 @@
         <v>120</v>
       </c>
       <c r="B10" s="37">
-        <v>2.7</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="C10" s="20">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="D10" s="20">
-        <v>3.1</v>
+        <v>1.4</v>
       </c>
       <c r="E10" s="20">
-        <v>1.7</v>
+        <v>0.9</v>
       </c>
       <c r="F10" s="20">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="G10" s="20">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="H10" s="16">
-        <v>2.514344713912875</v>
+        <v>1.4670028148804803</v>
       </c>
     </row>
   </sheetData>
@@ -5581,25 +5598,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="24">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="C2" s="24">
-        <v>2.2999999999999998</v>
+        <v>1.9</v>
       </c>
       <c r="D2" s="24">
         <v>2</v>
       </c>
       <c r="E2" s="24">
-        <v>2.6</v>
+        <v>1.9</v>
       </c>
       <c r="F2" s="24">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="G2" s="24">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
       <c r="H2" s="24">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5607,25 +5624,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="22">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="C3" s="22">
-        <v>2.8</v>
+        <v>1.2</v>
       </c>
       <c r="D3" s="22">
-        <v>2.2999999999999998</v>
+        <v>1.3</v>
       </c>
       <c r="E3" s="22">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="F3" s="22">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="G3" s="22">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="H3" s="22">
-        <v>2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5633,25 +5650,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="22">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="C4" s="22">
-        <v>1.1000000000000001</v>
+        <v>2</v>
       </c>
       <c r="D4" s="22">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="E4" s="22">
-        <v>0.3</v>
+        <v>2.4</v>
       </c>
       <c r="F4" s="22">
-        <v>0.4</v>
+        <v>2.1</v>
       </c>
       <c r="G4" s="22">
-        <v>-0.2</v>
+        <v>2.6</v>
       </c>
       <c r="H4" s="22">
-        <v>0.5</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5659,25 +5676,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="22">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="C5" s="22">
-        <v>-0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D5" s="22">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="E5" s="22">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="F5" s="22">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G5" s="22">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="H5" s="22">
-        <v>1.9</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5685,25 +5702,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="22">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="C6" s="22">
-        <v>1.8</v>
+        <v>3.9</v>
       </c>
       <c r="D6" s="22">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="E6" s="22">
-        <v>8.4</v>
+        <v>5</v>
       </c>
       <c r="F6" s="22">
-        <v>4</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="G6" s="22">
-        <v>3.7</v>
+        <v>1.5</v>
       </c>
       <c r="H6" s="22">
-        <v>0.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5711,25 +5728,25 @@
         <v>17</v>
       </c>
       <c r="B7" s="22">
+        <v>1.5</v>
+      </c>
+      <c r="C7" s="22">
+        <v>1.6</v>
+      </c>
+      <c r="D7" s="22">
+        <v>1.5</v>
+      </c>
+      <c r="E7" s="22">
+        <v>1.8</v>
+      </c>
+      <c r="F7" s="22">
         <v>1.4</v>
       </c>
-      <c r="C7" s="22">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="D7" s="22">
-        <v>1.6</v>
-      </c>
-      <c r="E7" s="22">
-        <v>1.3</v>
-      </c>
-      <c r="F7" s="22">
-        <v>1.9</v>
-      </c>
       <c r="G7" s="22">
-        <v>2.1</v>
+        <v>1.2</v>
       </c>
       <c r="H7" s="22">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5737,25 +5754,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="22">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="C8" s="22">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
       <c r="D8" s="22">
         <v>2.5</v>
       </c>
       <c r="E8" s="22">
-        <v>2.2000000000000002</v>
+        <v>3</v>
       </c>
       <c r="F8" s="22">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="G8" s="22">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="H8" s="22">
-        <v>2.2999999999999998</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5763,25 +5780,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="22">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="C9" s="22">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="D9" s="22">
-        <v>1.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E9" s="22">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="F9" s="22">
-        <v>0.9</v>
+        <v>2.1</v>
       </c>
       <c r="G9" s="22">
-        <v>2.4</v>
+        <v>0.6</v>
       </c>
       <c r="H9" s="22">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5789,25 +5806,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="22">
-        <v>3.4</v>
+        <v>0.9</v>
       </c>
       <c r="C10" s="22">
-        <v>3.7</v>
+        <v>0.3</v>
       </c>
       <c r="D10" s="22">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="E10" s="22">
-        <v>3.9</v>
+        <v>-0.1</v>
       </c>
       <c r="F10" s="22">
-        <v>3.8</v>
+        <v>1.2</v>
       </c>
       <c r="G10" s="22">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="22">
-        <v>3.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -5815,25 +5832,25 @@
         <v>21</v>
       </c>
       <c r="B11" s="22">
+        <v>4.2</v>
+      </c>
+      <c r="C11" s="22">
+        <v>4</v>
+      </c>
+      <c r="D11" s="22">
+        <v>5.2</v>
+      </c>
+      <c r="E11" s="22">
         <v>2.8</v>
       </c>
-      <c r="C11" s="22">
-        <v>3</v>
-      </c>
-      <c r="D11" s="22">
-        <v>2.6</v>
-      </c>
-      <c r="E11" s="22">
+      <c r="F11" s="22">
         <v>2.5</v>
       </c>
-      <c r="F11" s="22">
-        <v>2.8</v>
-      </c>
       <c r="G11" s="22">
-        <v>2.2000000000000002</v>
+        <v>3.4</v>
       </c>
       <c r="H11" s="22">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -5841,25 +5858,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="22">
-        <v>2.9</v>
+        <v>1.7</v>
       </c>
       <c r="C12" s="22">
-        <v>4</v>
+        <v>1.4</v>
       </c>
       <c r="D12" s="22">
-        <v>2.2000000000000002</v>
+        <v>1.4</v>
       </c>
       <c r="E12" s="22">
-        <v>0.7</v>
+        <v>2.8</v>
       </c>
       <c r="F12" s="22">
-        <v>1.2</v>
+        <v>3.5</v>
       </c>
       <c r="G12" s="22">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="H12" s="22">
-        <v>3</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -5867,25 +5884,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="22">
+        <v>1.6</v>
+      </c>
+      <c r="C13" s="22">
+        <v>1.2</v>
+      </c>
+      <c r="D13" s="22">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E13" s="22">
+        <v>1.2</v>
+      </c>
+      <c r="F13" s="22">
+        <v>1.7</v>
+      </c>
+      <c r="G13" s="22">
         <v>1.8</v>
       </c>
-      <c r="C13" s="22">
-        <v>2.1</v>
-      </c>
-      <c r="D13" s="22">
-        <v>1.3</v>
-      </c>
-      <c r="E13" s="22">
-        <v>3.2</v>
-      </c>
-      <c r="F13" s="22">
-        <v>1.9</v>
-      </c>
-      <c r="G13" s="22">
+      <c r="H13" s="22">
         <v>1.1000000000000001</v>
-      </c>
-      <c r="H13" s="22">
-        <v>1.5</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -5893,25 +5910,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="22">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="C14" s="22">
-        <v>2.4</v>
+        <v>1.9</v>
       </c>
       <c r="D14" s="22">
-        <v>2.2999999999999998</v>
+        <v>1.5</v>
       </c>
       <c r="E14" s="22">
-        <v>2.4</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F14" s="22">
-        <v>2.8</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="G14" s="22">
-        <v>2.2999999999999998</v>
+        <v>1.4</v>
       </c>
       <c r="H14" s="22">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -5956,25 +5973,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="33">
-        <v>33.200000000000003</v>
+        <v>33.5</v>
       </c>
       <c r="C2" s="33">
-        <v>33.6</v>
+        <v>33.4</v>
       </c>
       <c r="D2" s="33">
-        <v>32.4</v>
+        <v>33.4</v>
       </c>
       <c r="E2" s="33">
-        <v>35.299999999999997</v>
+        <v>36.5</v>
       </c>
       <c r="F2" s="33">
-        <v>33.200000000000003</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="G2" s="33">
-        <v>33.200000000000003</v>
+        <v>34</v>
       </c>
       <c r="H2" s="33">
-        <v>32.200000000000003</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5982,25 +5999,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="34">
-        <v>33.4</v>
+        <v>34.4</v>
       </c>
       <c r="C3" s="34">
-        <v>33.5</v>
+        <v>33.9</v>
       </c>
       <c r="D3" s="34">
-        <v>33.4</v>
+        <v>34.700000000000003</v>
       </c>
       <c r="E3" s="34">
-        <v>38.200000000000003</v>
+        <v>40.200000000000003</v>
       </c>
       <c r="F3" s="34">
-        <v>34.1</v>
+        <v>35.5</v>
       </c>
       <c r="G3" s="34">
-        <v>33.5</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="H3" s="34">
-        <v>27.7</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -6008,25 +6025,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="34">
-        <v>24</v>
+        <v>23.2</v>
       </c>
       <c r="C4" s="34">
-        <v>24.4</v>
+        <v>23.1</v>
       </c>
       <c r="D4" s="34">
-        <v>23.7</v>
+        <v>23</v>
       </c>
       <c r="E4" s="34">
-        <v>21.8</v>
+        <v>22.3</v>
       </c>
       <c r="F4" s="34">
-        <v>23.7</v>
+        <v>23.1</v>
       </c>
       <c r="G4" s="34">
-        <v>23.6</v>
+        <v>23.3</v>
       </c>
       <c r="H4" s="34">
-        <v>26.1</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6034,25 +6051,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="34">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="C5" s="34">
-        <v>12.7</v>
+        <v>13</v>
       </c>
       <c r="D5" s="34">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="E5" s="34">
-        <v>14.7</v>
+        <v>14.4</v>
       </c>
       <c r="F5" s="34">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G5" s="34">
-        <v>11.4</v>
+        <v>13.2</v>
       </c>
       <c r="H5" s="34">
-        <v>14.8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -6060,25 +6077,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="34">
-        <v>48</v>
+        <v>47.8</v>
       </c>
       <c r="C6" s="34">
-        <v>43.9</v>
+        <v>43.3</v>
       </c>
       <c r="D6" s="34">
-        <v>48.7</v>
+        <v>48.2</v>
       </c>
       <c r="E6" s="34">
-        <v>67.400000000000006</v>
+        <v>70.7</v>
       </c>
       <c r="F6" s="34">
-        <v>49.6</v>
+        <v>50.3</v>
       </c>
       <c r="G6" s="34">
-        <v>50.9</v>
+        <v>52.8</v>
       </c>
       <c r="H6" s="34">
-        <v>54.3</v>
+        <v>52.9</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -6086,25 +6103,25 @@
         <v>17</v>
       </c>
       <c r="B7" s="34">
-        <v>23.5</v>
+        <v>23.1</v>
       </c>
       <c r="C7" s="34">
-        <v>25.1</v>
+        <v>24.4</v>
       </c>
       <c r="D7" s="34">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="E7" s="34">
-        <v>16.399999999999999</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="F7" s="34">
-        <v>22.4</v>
+        <v>21.7</v>
       </c>
       <c r="G7" s="34">
-        <v>24</v>
+        <v>23.1</v>
       </c>
       <c r="H7" s="34">
-        <v>22.1</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6112,25 +6129,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="34">
-        <v>29.5</v>
+        <v>30.5</v>
       </c>
       <c r="C8" s="34">
-        <v>29.8</v>
+        <v>31</v>
       </c>
       <c r="D8" s="34">
-        <v>29.9</v>
+        <v>30.4</v>
       </c>
       <c r="E8" s="34">
-        <v>27</v>
+        <v>27.7</v>
       </c>
       <c r="F8" s="34">
-        <v>27.9</v>
+        <v>29.1</v>
       </c>
       <c r="G8" s="34">
-        <v>27.9</v>
+        <v>28.3</v>
       </c>
       <c r="H8" s="34">
-        <v>31.7</v>
+        <v>32.9</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -6141,22 +6158,22 @@
         <v>42.1</v>
       </c>
       <c r="C9" s="34">
-        <v>43.4</v>
+        <v>42.5</v>
       </c>
       <c r="D9" s="34">
-        <v>39.700000000000003</v>
+        <v>41.1</v>
       </c>
       <c r="E9" s="34">
-        <v>36.299999999999997</v>
+        <v>36</v>
       </c>
       <c r="F9" s="34">
-        <v>45.7</v>
+        <v>46.7</v>
       </c>
       <c r="G9" s="34">
-        <v>43.9</v>
+        <v>43.5</v>
       </c>
       <c r="H9" s="34">
-        <v>46.5</v>
+        <v>45.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -6164,25 +6181,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="34">
+        <v>36.1</v>
+      </c>
+      <c r="C10" s="34">
         <v>37.4</v>
       </c>
-      <c r="C10" s="34">
-        <v>39.700000000000003</v>
-      </c>
       <c r="D10" s="34">
-        <v>35.299999999999997</v>
+        <v>35.4</v>
       </c>
       <c r="E10" s="34">
-        <v>34.9</v>
+        <v>33.5</v>
       </c>
       <c r="F10" s="34">
-        <v>33.9</v>
+        <v>34.700000000000003</v>
       </c>
       <c r="G10" s="34">
-        <v>37.1</v>
+        <v>35.200000000000003</v>
       </c>
       <c r="H10" s="34">
-        <v>36.799999999999997</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -6190,25 +6207,25 @@
         <v>21</v>
       </c>
       <c r="B11" s="34">
-        <v>29.8</v>
+        <v>32</v>
       </c>
       <c r="C11" s="34">
-        <v>30.9</v>
+        <v>30.8</v>
       </c>
       <c r="D11" s="34">
-        <v>30.3</v>
+        <v>36.4</v>
       </c>
       <c r="E11" s="34">
-        <v>26.1</v>
+        <v>28.1</v>
       </c>
       <c r="F11" s="34">
-        <v>27.8</v>
+        <v>28.4</v>
       </c>
       <c r="G11" s="34">
-        <v>28.3</v>
+        <v>27.7</v>
       </c>
       <c r="H11" s="34">
-        <v>22.8</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -6216,25 +6233,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="34">
-        <v>42.7</v>
+        <v>40</v>
       </c>
       <c r="C12" s="34">
-        <v>42.5</v>
+        <v>39.299999999999997</v>
       </c>
       <c r="D12" s="34">
-        <v>40.4</v>
+        <v>36.6</v>
       </c>
       <c r="E12" s="34">
-        <v>40.799999999999997</v>
+        <v>42.3</v>
       </c>
       <c r="F12" s="34">
-        <v>53.9</v>
+        <v>51.8</v>
       </c>
       <c r="G12" s="34">
-        <v>40.700000000000003</v>
+        <v>41.3</v>
       </c>
       <c r="H12" s="34">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -6242,25 +6259,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="34">
-        <v>37.299999999999997</v>
+        <v>36.700000000000003</v>
       </c>
       <c r="C13" s="34">
-        <v>36.5</v>
+        <v>35.1</v>
       </c>
       <c r="D13" s="34">
-        <v>39.200000000000003</v>
+        <v>39.9</v>
       </c>
       <c r="E13" s="34">
-        <v>43.8</v>
+        <v>41.1</v>
       </c>
       <c r="F13" s="34">
         <v>37.5</v>
       </c>
       <c r="G13" s="34">
-        <v>33.5</v>
+        <v>32.5</v>
       </c>
       <c r="H13" s="34">
-        <v>29.9</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -6268,25 +6285,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="34">
-        <v>31.4</v>
+        <v>32.4</v>
       </c>
       <c r="C14" s="34">
-        <v>33.9</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="D14" s="34">
         <v>30.4</v>
       </c>
       <c r="E14" s="34">
-        <v>27</v>
+        <v>27.9</v>
       </c>
       <c r="F14" s="34">
-        <v>25.4</v>
+        <v>27.7</v>
       </c>
       <c r="G14" s="34">
-        <v>31.8</v>
+        <v>33</v>
       </c>
       <c r="H14" s="34">
-        <v>27.2</v>
+        <v>30.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
"Agrego emae may25 y comex junio26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEE6477E-B214-4D59-8D8D-3F08F67FD215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4921F18-139E-420D-AD54-01919946EA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -3524,7 +3524,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D125"/>
+  <dimension ref="A1:D126"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -3554,10 +3554,10 @@
         <v>134.74645041349706</v>
       </c>
       <c r="C2" s="36">
-        <v>147.93392530516525</v>
+        <v>147.90289172962787</v>
       </c>
       <c r="D2" s="36">
-        <v>147.05728802300575</v>
+        <v>147.06041914463302</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3568,10 +3568,10 @@
         <v>134.23236103862521</v>
       </c>
       <c r="C3" s="36">
-        <v>146.84557122133359</v>
+        <v>146.87869250897225</v>
       </c>
       <c r="D3" s="36">
-        <v>146.4791599743433</v>
+        <v>146.48010453906795</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3582,10 +3582,10 @@
         <v>150.0878942366954</v>
       </c>
       <c r="C4" s="36">
-        <v>145.96775878336345</v>
+        <v>145.96567107119392</v>
       </c>
       <c r="D4" s="36">
-        <v>145.93066633403586</v>
+        <v>145.92974952061303</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3596,10 +3596,10 @@
         <v>153.25067436662908</v>
       </c>
       <c r="C5" s="36">
-        <v>144.69616657974839</v>
+        <v>144.71513795719116</v>
       </c>
       <c r="D5" s="36">
-        <v>145.44963167660751</v>
+        <v>145.4474203087604</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3610,10 +3610,10 @@
         <v>163.51360808690507</v>
       </c>
       <c r="C6" s="36">
-        <v>144.56727263895843</v>
+        <v>144.57674809588957</v>
       </c>
       <c r="D6" s="36">
-        <v>145.06426744979953</v>
+        <v>145.06163776867783</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3624,10 +3624,10 @@
         <v>153.66209524099784</v>
       </c>
       <c r="C7" s="36">
-        <v>144.40750076903936</v>
+        <v>144.37905393460173</v>
       </c>
       <c r="D7" s="36">
-        <v>144.79569649622729</v>
+        <v>144.79388930864746</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3638,10 +3638,10 @@
         <v>143.73110098180126</v>
       </c>
       <c r="C8" s="36">
-        <v>144.60181651071224</v>
+        <v>144.58278827113989</v>
       </c>
       <c r="D8" s="36">
-        <v>144.65403542077127</v>
+        <v>144.65415992044788</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3652,10 +3652,10 @@
         <v>143.6741026486049</v>
       </c>
       <c r="C9" s="36">
-        <v>145.66149778877167</v>
+        <v>145.65089775486558</v>
       </c>
       <c r="D9" s="36">
-        <v>144.64223827479154</v>
+        <v>144.64490844807989</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3666,10 +3666,10 @@
         <v>142.00773744282046</v>
       </c>
       <c r="C10" s="36">
-        <v>144.98917021298641</v>
+        <v>145.01879848640064</v>
       </c>
       <c r="D10" s="36">
-        <v>144.75896347841521</v>
+        <v>144.76441821007117</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3680,10 +3680,10 @@
         <v>141.13686329808141</v>
       </c>
       <c r="C11" s="36">
-        <v>145.16989751944251</v>
+        <v>145.15354369792067</v>
       </c>
       <c r="D11" s="36">
-        <v>144.99665757430398</v>
+        <v>145.00423578331799</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3694,10 +3694,10 @@
         <v>144.93832064073018</v>
       </c>
       <c r="C12" s="36">
-        <v>145.77978651755154</v>
+        <v>145.78824914209579</v>
       </c>
       <c r="D12" s="36">
-        <v>145.34151040560658</v>
+        <v>145.3496394533513</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3708,10 +3708,10 @@
         <v>142.59014516031914</v>
       </c>
       <c r="C13" s="36">
-        <v>146.95099027389824</v>
+        <v>146.95888147081035</v>
       </c>
       <c r="D13" s="36">
-        <v>145.78176450559545</v>
+        <v>145.78841177630977</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3722,10 +3722,10 @@
         <v>136.63265948316197</v>
       </c>
       <c r="C14" s="36">
-        <v>147.09361189175286</v>
+        <v>147.08627326950506</v>
       </c>
       <c r="D14" s="36">
-        <v>146.30347289560493</v>
+        <v>146.3065815191809</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3736,10 +3736,10 @@
         <v>132.15851633982263</v>
       </c>
       <c r="C15" s="36">
-        <v>146.81999958929094</v>
+        <v>146.81395008705243</v>
       </c>
       <c r="D15" s="36">
-        <v>146.88879026400798</v>
+        <v>146.88669274545626</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3750,10 +3750,10 @@
         <v>152.62095855905721</v>
       </c>
       <c r="C16" s="36">
-        <v>147.63142117580773</v>
+        <v>147.64480930022708</v>
       </c>
       <c r="D16" s="36">
-        <v>147.51962090447577</v>
+        <v>147.51139127886813</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3764,10 +3764,10 @@
         <v>151.94634480448727</v>
       </c>
       <c r="C17" s="36">
-        <v>147.70171402358014</v>
+        <v>147.67329037105645</v>
       </c>
       <c r="D17" s="36">
-        <v>148.17522841474457</v>
+        <v>148.16108451834779</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3778,10 +3778,10 @@
         <v>168.38920946936767</v>
       </c>
       <c r="C18" s="36">
-        <v>148.67231109901837</v>
+        <v>148.67448204725812</v>
       </c>
       <c r="D18" s="36">
-        <v>148.82877687985808</v>
+        <v>148.80990363486927</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3792,10 +3792,10 @@
         <v>161.0356854694522</v>
       </c>
       <c r="C19" s="36">
-        <v>150.24574032624963</v>
+        <v>150.27199303046453</v>
       </c>
       <c r="D19" s="36">
-        <v>149.44932981707404</v>
+        <v>149.42763427653395</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3806,10 +3806,10 @@
         <v>150.3060501239199</v>
       </c>
       <c r="C20" s="36">
-        <v>150.47989229282791</v>
+        <v>150.46351778388978</v>
       </c>
       <c r="D20" s="36">
-        <v>150.00175591799729</v>
+        <v>149.97952638836915</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3820,10 +3820,10 @@
         <v>149.25534277384099</v>
       </c>
       <c r="C21" s="36">
-        <v>150.3849160508085</v>
+        <v>150.39057754222844</v>
       </c>
       <c r="D21" s="36">
-        <v>150.44828536486224</v>
+        <v>150.42776468517482</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3834,10 +3834,10 @@
         <v>146.38655965775374</v>
       </c>
       <c r="C22" s="36">
-        <v>151.20678120691389</v>
+        <v>151.21749422435974</v>
       </c>
       <c r="D22" s="36">
-        <v>150.75053058764885</v>
+        <v>150.73346509955473</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3848,10 +3848,10 @@
         <v>149.38594966601445</v>
       </c>
       <c r="C23" s="36">
-        <v>151.69720252270432</v>
+        <v>151.71275927869797</v>
       </c>
       <c r="D23" s="36">
-        <v>150.87798858941446</v>
+        <v>150.8656502006244</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3862,10 +3862,10 @@
         <v>151.92604285202682</v>
       </c>
       <c r="C24" s="36">
-        <v>152.63772357143588</v>
+        <v>152.63221481224414</v>
       </c>
       <c r="D24" s="36">
-        <v>150.80628666033164</v>
+        <v>150.79907205919287</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3876,10 +3876,10 @@
         <v>146.78338490922437</v>
       </c>
       <c r="C25" s="36">
-        <v>152.25539093894815</v>
+        <v>152.24534294207206</v>
       </c>
       <c r="D25" s="36">
-        <v>150.52355583017248</v>
+        <v>150.52073983983868</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3890,10 +3890,10 @@
         <v>142.74091260617209</v>
       </c>
       <c r="C26" s="36">
-        <v>150.98722525561379</v>
+        <v>150.97750196780996</v>
       </c>
       <c r="D26" s="36">
-        <v>150.03515094773516</v>
+        <v>150.03524574481486</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3904,10 +3904,10 @@
         <v>138.81804035165729</v>
       </c>
       <c r="C27" s="36">
-        <v>152.18519512030997</v>
+        <v>152.19147467174869</v>
       </c>
       <c r="D27" s="36">
-        <v>149.36311920629876</v>
+        <v>149.36435462115523</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3918,10 +3918,10 @@
         <v>155.85731953576962</v>
       </c>
       <c r="C28" s="36">
-        <v>151.5253120742554</v>
+        <v>151.5287558105469</v>
       </c>
       <c r="D28" s="36">
-        <v>148.54542503333764</v>
+        <v>148.54649497358778</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3932,10 +3932,10 @@
         <v>151.52454398394329</v>
       </c>
       <c r="C29" s="36">
-        <v>146.77368593383494</v>
+        <v>146.79265782593984</v>
       </c>
       <c r="D29" s="36">
-        <v>147.62847602367108</v>
+        <v>147.62845357197196</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3946,10 +3946,10 @@
         <v>159.56669237791655</v>
       </c>
       <c r="C30" s="36">
-        <v>144.56370636245163</v>
+        <v>144.56308740741699</v>
       </c>
       <c r="D30" s="36">
-        <v>146.66677122984348</v>
+        <v>146.66554660531108</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3960,10 +3960,10 @@
         <v>151.1257632334551</v>
       </c>
       <c r="C31" s="36">
-        <v>143.27743582661475</v>
+        <v>143.25908288947755</v>
       </c>
       <c r="D31" s="36">
-        <v>145.71784330042544</v>
+        <v>145.71598087635073</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -3974,10 +3974,10 @@
         <v>145.96352443000447</v>
       </c>
       <c r="C32" s="36">
-        <v>143.56630904676393</v>
+        <v>143.57920900072801</v>
       </c>
       <c r="D32" s="36">
-        <v>144.83517226102009</v>
+        <v>144.83291842509811</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3988,10 +3988,10 @@
         <v>146.76596003413957</v>
       </c>
       <c r="C33" s="36">
-        <v>146.5083763401191</v>
+        <v>146.53723087700519</v>
       </c>
       <c r="D33" s="36">
-        <v>144.0667550767985</v>
+        <v>144.06472199992993</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -4002,10 +4002,10 @@
         <v>137.74656971864789</v>
       </c>
       <c r="C34" s="36">
-        <v>143.17399592423629</v>
+        <v>143.1322414333213</v>
       </c>
       <c r="D34" s="36">
-        <v>143.44685177314395</v>
+        <v>143.44595234523834</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -4016,10 +4016,10 @@
         <v>142.8432759845675</v>
       </c>
       <c r="C35" s="36">
-        <v>143.60656244287722</v>
+        <v>143.59558509549367</v>
       </c>
       <c r="D35" s="36">
-        <v>142.99223610249436</v>
+        <v>142.99316083040782</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -4030,10 +4030,10 @@
         <v>140.59240732533553</v>
       </c>
       <c r="C36" s="36">
-        <v>141.62161359564226</v>
+        <v>141.66615037738163</v>
       </c>
       <c r="D36" s="36">
-        <v>142.70444231322497</v>
+        <v>142.70789004237591</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -4044,10 +4044,10 @@
         <v>136.25161596905625</v>
       </c>
       <c r="C37" s="36">
-        <v>142.00720819392214</v>
+        <v>141.97364875950399</v>
       </c>
       <c r="D37" s="36">
-        <v>142.57062754953117</v>
+        <v>142.57713267970016</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -4058,10 +4058,10 @@
         <v>134.53623985669569</v>
       </c>
       <c r="C38" s="36">
-        <v>141.41909976735533</v>
+        <v>141.39772924062791</v>
       </c>
       <c r="D38" s="36">
-        <v>142.56274411876478</v>
+        <v>142.57245366664446</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4072,10 +4072,10 @@
         <v>132.2678886127365</v>
       </c>
       <c r="C39" s="36">
-        <v>143.63399679522843</v>
+        <v>143.65890168370726</v>
       </c>
       <c r="D39" s="36">
-        <v>142.64308433060683</v>
+        <v>142.6556943490732</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4086,10 +4086,10 @@
         <v>144.96325495574902</v>
       </c>
       <c r="C40" s="36">
-        <v>142.26347440308089</v>
+        <v>142.25994004126758</v>
       </c>
       <c r="D40" s="36">
-        <v>142.76985619334408</v>
+        <v>142.78455876892951</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4100,10 +4100,10 @@
         <v>149.91622140352257</v>
       </c>
       <c r="C41" s="36">
-        <v>142.5814610098206</v>
+        <v>142.60578725333434</v>
       </c>
       <c r="D41" s="36">
-        <v>142.8972437348074</v>
+        <v>142.91282858001958</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4114,10 +4114,10 @@
         <v>164.13569907592026</v>
       </c>
       <c r="C42" s="36">
-        <v>144.80047817480937</v>
+        <v>144.83824997198266</v>
       </c>
       <c r="D42" s="36">
-        <v>142.98303839742368</v>
+        <v>142.99820287071864</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4128,10 +4128,10 @@
         <v>150.85897174113111</v>
       </c>
       <c r="C43" s="36">
-        <v>144.09587933653643</v>
+        <v>144.03378129578405</v>
       </c>
       <c r="D43" s="36">
-        <v>142.99114760015667</v>
+        <v>143.00474250423559</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4142,10 +4142,10 @@
         <v>146.7770296400702</v>
       </c>
       <c r="C44" s="36">
-        <v>145.84338911769825</v>
+        <v>145.83568077855986</v>
       </c>
       <c r="D44" s="36">
-        <v>142.89375082962775</v>
+        <v>142.90491277618392</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4156,10 +4156,10 @@
         <v>141.27693468084021</v>
       </c>
       <c r="C45" s="36">
-        <v>144.80116322755515</v>
+        <v>144.7905932858464</v>
       </c>
       <c r="D45" s="36">
-        <v>142.67390042071176</v>
+        <v>142.68208431588255</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4170,10 +4170,10 @@
         <v>134.87706647993639</v>
       </c>
       <c r="C46" s="36">
-        <v>140.53903571586895</v>
+        <v>140.55731399665021</v>
       </c>
       <c r="D46" s="36">
-        <v>142.32654422761081</v>
+        <v>142.33147985322461</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -4184,10 +4184,10 @@
         <v>141.63933661701367</v>
       </c>
       <c r="C47" s="36">
-        <v>143.81839242743101</v>
+        <v>143.79727407340053</v>
       </c>
       <c r="D47" s="36">
-        <v>141.85799511764722</v>
+        <v>141.85956089737351</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -4198,10 +4198,10 @@
         <v>137.77182966933134</v>
       </c>
       <c r="C48" s="36">
-        <v>140.87775693980214</v>
+        <v>140.88368953714604</v>
       </c>
       <c r="D48" s="36">
-        <v>141.28539477404658</v>
+        <v>141.28341184211027</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4212,10 +4212,10 @@
         <v>135.76515452763488</v>
       </c>
       <c r="C49" s="36">
-        <v>140.11150090003781</v>
+        <v>140.12668665666166</v>
       </c>
       <c r="D49" s="36">
-        <v>140.63606308945876</v>
+        <v>140.6304263163494</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -4226,10 +4226,10 @@
         <v>133.89108608957227</v>
       </c>
       <c r="C50" s="36">
-        <v>140.91697761884743</v>
+        <v>140.93017714538223</v>
       </c>
       <c r="D50" s="36">
-        <v>139.94160028898327</v>
+        <v>139.93237577469208</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -4240,10 +4240,10 @@
         <v>128.97363874659808</v>
       </c>
       <c r="C51" s="36">
-        <v>139.55347026640555</v>
+        <v>139.54976127560565</v>
       </c>
       <c r="D51" s="36">
-        <v>139.23701145822935</v>
+        <v>139.22448358107718</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -4254,10 +4254,10 @@
         <v>128.21106074025653</v>
       </c>
       <c r="C52" s="36">
-        <v>125.96973824909686</v>
+        <v>125.96024771330764</v>
       </c>
       <c r="D52" s="36">
-        <v>138.55833411203915</v>
+        <v>138.54271042734956</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -4268,10 +4268,10 @@
         <v>113.29503444580143</v>
       </c>
       <c r="C53" s="36">
-        <v>105.99371760567273</v>
+        <v>105.99227909223607</v>
       </c>
       <c r="D53" s="36">
-        <v>137.94078869004042</v>
+        <v>137.92242935265389</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -4282,10 +4282,10 @@
         <v>131.02956919734902</v>
       </c>
       <c r="C54" s="36">
-        <v>117.20862009281119</v>
+        <v>117.20962176752099</v>
       </c>
       <c r="D54" s="36">
-        <v>137.41736684572851</v>
+        <v>137.39712668302374</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -4296,10 +4296,10 @@
         <v>132.52196526648763</v>
       </c>
       <c r="C55" s="36">
-        <v>124.34453609719363</v>
+        <v>124.3449729358869</v>
       </c>
       <c r="D55" s="36">
-        <v>137.01298862339578</v>
+        <v>136.99165283445276</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -4310,10 +4310,10 @@
         <v>127.46368946979391</v>
       </c>
       <c r="C56" s="36">
-        <v>126.13173661675738</v>
+        <v>126.15819490838572</v>
       </c>
       <c r="D56" s="36">
-        <v>136.74386313284347</v>
+        <v>136.72209103841908</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -4324,10 +4324,10 @@
         <v>125.18389375984641</v>
       </c>
       <c r="C57" s="36">
-        <v>128.86728972485162</v>
+        <v>128.84415787500245</v>
       </c>
       <c r="D57" s="36">
-        <v>136.61809092980613</v>
+        <v>136.59679330726365</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -4338,10 +4338,10 @@
         <v>127.1750760933527</v>
       </c>
       <c r="C58" s="36">
-        <v>130.79987437384165</v>
+        <v>130.79654793201593</v>
       </c>
       <c r="D58" s="36">
-        <v>136.63583340346673</v>
+        <v>136.61536603928135</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -4352,10 +4352,10 @@
         <v>131.34550189452784</v>
       </c>
       <c r="C59" s="36">
-        <v>133.41060851326921</v>
+        <v>133.39866145682996</v>
       </c>
       <c r="D59" s="36">
-        <v>136.79076013755875</v>
+        <v>136.77112663605229</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -4366,10 +4366,10 @@
         <v>132.06865525299659</v>
       </c>
       <c r="C60" s="36">
-        <v>134.85001471194028</v>
+        <v>134.87132101698435</v>
       </c>
       <c r="D60" s="36">
-        <v>137.06983870593521</v>
+        <v>137.05076753412618</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -4380,10 +4380,10 @@
         <v>133.85436559460604</v>
       </c>
       <c r="C61" s="36">
-        <v>136.96695318017814</v>
+        <v>136.95759393151968</v>
       </c>
       <c r="D61" s="36">
-        <v>137.45686112626854</v>
+        <v>137.43790389556929</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -4394,10 +4394,10 @@
         <v>131.52153739731881</v>
       </c>
       <c r="C62" s="36">
-        <v>139.86778985546729</v>
+        <v>139.84976777699663</v>
       </c>
       <c r="D62" s="36">
-        <v>137.93577366070608</v>
+        <v>137.91642405398932</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -4408,10 +4408,10 @@
         <v>126.23926696836405</v>
       </c>
       <c r="C63" s="36">
-        <v>138.20028013173521</v>
+        <v>138.24267956970155</v>
       </c>
       <c r="D63" s="36">
-        <v>138.49506341728181</v>
+        <v>138.47503425796688</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -4422,10 +4422,10 @@
         <v>145.95690010364706</v>
       </c>
       <c r="C64" s="36">
-        <v>140.91577065783943</v>
+        <v>140.89139329828407</v>
       </c>
       <c r="D64" s="36">
-        <v>139.12542597753085</v>
+        <v>139.10476344710142</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -4436,10 +4436,10 @@
         <v>147.28084401875944</v>
       </c>
       <c r="C65" s="36">
-        <v>139.26049396360543</v>
+        <v>139.3115864823003</v>
       </c>
       <c r="D65" s="36">
-        <v>139.8235460686619</v>
+        <v>139.80273184864561</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -4450,10 +4450,10 @@
         <v>151.16932233874812</v>
       </c>
       <c r="C66" s="36">
-        <v>138.87942821950787</v>
+        <v>138.85916439674222</v>
       </c>
       <c r="D66" s="36">
-        <v>140.58828401842547</v>
+        <v>140.56795196459669</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -4464,10 +4464,10 @@
         <v>148.97961710841227</v>
       </c>
       <c r="C67" s="36">
-        <v>141.55493596421903</v>
+        <v>141.52410726823069</v>
       </c>
       <c r="D67" s="36">
-        <v>141.41703636524801</v>
+        <v>141.39767517306643</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -4478,10 +4478,10 @@
         <v>142.42591306035797</v>
       </c>
       <c r="C68" s="36">
-        <v>141.38117057908835</v>
+        <v>141.37916581108891</v>
       </c>
       <c r="D68" s="36">
-        <v>142.30989872852675</v>
+        <v>142.29185441448868</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -4492,10 +4492,10 @@
         <v>140.97494072777721</v>
       </c>
       <c r="C69" s="36">
-        <v>143.29501888821403</v>
+        <v>143.31590238415345</v>
       </c>
       <c r="D69" s="36">
-        <v>143.26598461789402</v>
+        <v>143.24949089718777</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -4506,10 +4506,10 @@
         <v>141.29608909028403</v>
       </c>
       <c r="C70" s="36">
-        <v>144.1962251789204</v>
+        <v>144.17734645091775</v>
       </c>
       <c r="D70" s="36">
-        <v>144.27799737026854</v>
+        <v>144.263236099306</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -4520,10 +4520,10 @@
         <v>139.51475869967888</v>
       </c>
       <c r="C71" s="36">
-        <v>143.38274230679909</v>
+        <v>143.35586178313645</v>
       </c>
       <c r="D71" s="36">
-        <v>145.3330444755376</v>
+        <v>145.32006310709181</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -4534,10 +4534,10 @@
         <v>143.75187761888847</v>
       </c>
       <c r="C72" s="36">
-        <v>145.70199915320512</v>
+        <v>145.71356699110419</v>
       </c>
       <c r="D72" s="36">
-        <v>146.4062746613703</v>
+        <v>146.39501768319394</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -4548,10 +4548,10 @@
         <v>147.22987831813373</v>
       </c>
       <c r="C73" s="36">
-        <v>149.70509110366692</v>
+        <v>149.72040378936583</v>
       </c>
       <c r="D73" s="36">
-        <v>147.46081171992913</v>
+        <v>147.4511533036428</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -4562,10 +4562,10 @@
         <v>139.637961612281</v>
       </c>
       <c r="C74" s="36">
-        <v>148.55190380544317</v>
+        <v>148.52454567203267</v>
       </c>
       <c r="D74" s="36">
-        <v>148.45392567357925</v>
+        <v>148.44590874633826</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -4576,10 +4576,10 @@
         <v>137.84951352507554</v>
       </c>
       <c r="C75" s="36">
-        <v>150.64256656224384</v>
+        <v>150.70922638827258</v>
       </c>
       <c r="D75" s="36">
-        <v>149.34073907795377</v>
+        <v>149.33437192086149</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -4590,10 +4590,10 @@
         <v>153.9308507942531</v>
       </c>
       <c r="C76" s="36">
-        <v>150.3860254781107</v>
+        <v>150.34672378542243</v>
       </c>
       <c r="D76" s="36">
-        <v>150.08321581555236</v>
+        <v>150.07876932527918</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -4604,10 +4604,10 @@
         <v>157.66169217344674</v>
       </c>
       <c r="C77" s="36">
-        <v>152.07758234261067</v>
+        <v>152.09770494152977</v>
       </c>
       <c r="D77" s="36">
-        <v>150.6534040255867</v>
+        <v>150.65168869920231</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -4618,10 +4618,10 @@
         <v>164.68936311408393</v>
       </c>
       <c r="C78" s="36">
-        <v>152.10152135054884</v>
+        <v>152.12668174406087</v>
       </c>
       <c r="D78" s="36">
-        <v>151.03507926055096</v>
+        <v>151.03686923587975</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -4632,10 +4632,10 @@
         <v>161.4548342812127</v>
       </c>
       <c r="C79" s="36">
-        <v>154.34825750063149</v>
+        <v>154.30297450812731</v>
       </c>
       <c r="D79" s="36">
-        <v>151.2247471775994</v>
+        <v>151.2301275132958</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -4646,10 +4646,10 @@
         <v>152.44538743586068</v>
       </c>
       <c r="C80" s="36">
-        <v>152.57931165808276</v>
+        <v>152.5581973587675</v>
       </c>
       <c r="D80" s="36">
-        <v>151.23534588803642</v>
+        <v>151.24393962017717</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4660,10 +4660,10 @@
         <v>151.46573891606155</v>
       </c>
       <c r="C81" s="36">
-        <v>151.71959575650231</v>
+        <v>151.72301499095741</v>
       </c>
       <c r="D81" s="36">
-        <v>151.09312241380925</v>
+        <v>151.10403481382463</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4674,10 +4674,10 @@
         <v>149.17434970528168</v>
       </c>
       <c r="C82" s="36">
-        <v>150.7700560603914</v>
+        <v>150.78775112517866</v>
       </c>
       <c r="D82" s="36">
-        <v>150.8332071036196</v>
+        <v>150.84526135445358</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4688,10 +4688,10 @@
         <v>146.55439616170329</v>
       </c>
       <c r="C83" s="36">
-        <v>149.10270937214764</v>
+        <v>149.08575921389939</v>
       </c>
       <c r="D83" s="36">
-        <v>150.49434645972877</v>
+        <v>150.50645589049475</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4702,10 +4702,10 @@
         <v>148.03049492952468</v>
       </c>
       <c r="C84" s="36">
-        <v>148.30045235840549</v>
+        <v>148.327566132046</v>
       </c>
       <c r="D84" s="36">
-        <v>150.11367270204204</v>
+        <v>150.12486758078268</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -4716,10 +4716,10 @@
         <v>146.18080633796006</v>
       </c>
       <c r="C85" s="36">
-        <v>148.49540732677499</v>
+        <v>148.48524371131373</v>
       </c>
       <c r="D85" s="36">
-        <v>149.72367305158448</v>
+        <v>149.73336917647515</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -4730,10 +4730,10 @@
         <v>143.03462349487495</v>
       </c>
       <c r="C86" s="36">
-        <v>149.96952713298742</v>
+        <v>149.95772966081552</v>
       </c>
       <c r="D86" s="36">
-        <v>149.34688054655493</v>
+        <v>149.35503971635941</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4744,10 +4744,10 @@
         <v>137.26646276476467</v>
       </c>
       <c r="C87" s="36">
-        <v>150.10387208507404</v>
+        <v>150.15642424124019</v>
       </c>
       <c r="D87" s="36">
-        <v>148.99278837030343</v>
+        <v>148.99990522247347</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -4758,10 +4758,10 @@
         <v>155.06501366898644</v>
       </c>
       <c r="C88" s="36">
-        <v>150.79671770186954</v>
+        <v>150.7559630178034</v>
       </c>
       <c r="D88" s="36">
-        <v>148.65736303565535</v>
+        <v>148.66373870024944</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -4772,10 +4772,10 @@
         <v>150.05952685125044</v>
       </c>
       <c r="C89" s="36">
-        <v>147.42919171933761</v>
+        <v>147.35748735405127</v>
       </c>
       <c r="D89" s="36">
-        <v>148.32612883201449</v>
+        <v>148.33221429847092</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4786,10 +4786,10 @@
         <v>153.81085419260503</v>
       </c>
       <c r="C90" s="36">
-        <v>145.50808199864673</v>
+        <v>145.5527260528016</v>
       </c>
       <c r="D90" s="36">
-        <v>147.97653557702176</v>
+        <v>147.98297145239175</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4800,10 +4800,10 @@
         <v>152.59547604809092</v>
       </c>
       <c r="C91" s="36">
-        <v>146.0362071856969</v>
+        <v>146.06326749676077</v>
       </c>
       <c r="D91" s="36">
-        <v>147.58827361699645</v>
+        <v>147.59607526377985</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -4814,10 +4814,10 @@
         <v>150.20312548190341</v>
       </c>
       <c r="C92" s="36">
-        <v>148.73013107795748</v>
+        <v>148.72466380879337</v>
       </c>
       <c r="D92" s="36">
-        <v>147.14923296818338</v>
+        <v>147.15967189693004</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -4828,10 +4828,10 @@
         <v>151.92217935804922</v>
       </c>
       <c r="C93" s="36">
-        <v>150.0390804234014</v>
+        <v>150.05694584045796</v>
       </c>
       <c r="D93" s="36">
-        <v>146.65580516741312</v>
+        <v>146.67009144248809</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -4842,10 +4842,10 @@
         <v>148.41237963987399</v>
       </c>
       <c r="C94" s="36">
-        <v>149.71064515367252</v>
+        <v>149.69824700570871</v>
       </c>
       <c r="D94" s="36">
-        <v>146.11778260269955</v>
+        <v>146.13676611930737</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4856,10 +4856,10 @@
         <v>147.51381305414859</v>
       </c>
       <c r="C95" s="36">
-        <v>147.98485863929363</v>
+        <v>148.01321137160105</v>
       </c>
       <c r="D95" s="36">
-        <v>145.55865524812774</v>
+        <v>145.5826226763221</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -4870,10 +4870,10 @@
         <v>146.36635232721147</v>
       </c>
       <c r="C96" s="36">
-        <v>146.37566723734164</v>
+        <v>146.38829854061774</v>
       </c>
       <c r="D96" s="36">
-        <v>145.01025992107282</v>
+        <v>145.03868020466888</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -4884,10 +4884,10 @@
         <v>139.34262723777164</v>
       </c>
       <c r="C97" s="36">
-        <v>142.90845433855887</v>
+        <v>142.86747030290806</v>
       </c>
       <c r="D97" s="36">
-        <v>144.51678109590449</v>
+        <v>144.54822439405362</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -4898,10 +4898,10 @@
         <v>137.37335120058367</v>
       </c>
       <c r="C98" s="36">
-        <v>143.57157054122101</v>
+        <v>143.5536731054936</v>
       </c>
       <c r="D98" s="36">
-        <v>144.12666448134632</v>
+        <v>144.15895332179335</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4912,10 +4912,10 @@
         <v>133.46450581005294</v>
       </c>
       <c r="C99" s="36">
-        <v>143.69325878964582</v>
+        <v>143.80881964781162</v>
       </c>
       <c r="D99" s="36">
-        <v>143.88612523109015</v>
+        <v>143.91670347404232</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4926,10 +4926,10 @@
         <v>142.39572385637248</v>
       </c>
       <c r="C100" s="36">
-        <v>142.2121938396119</v>
+        <v>142.11453041710828</v>
       </c>
       <c r="D100" s="36">
-        <v>143.83383928542497</v>
+        <v>143.86036158327045</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4940,10 +4940,10 @@
         <v>147.25690008767782</v>
       </c>
       <c r="C101" s="36">
-        <v>141.13498723520038</v>
+        <v>141.05611588000892</v>
       </c>
       <c r="D101" s="36">
-        <v>143.99062537877512</v>
+        <v>144.01125926444928</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4954,10 +4954,10 @@
         <v>156.76909889616599</v>
       </c>
       <c r="C102" s="36">
-        <v>142.70361097206074</v>
+        <v>142.83619727876223</v>
       </c>
       <c r="D102" s="36">
-        <v>144.35633880962916</v>
+        <v>144.37034591531875</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4968,10 +4968,10 @@
         <v>147.35712151974346</v>
       </c>
       <c r="C103" s="36">
-        <v>143.77246679244459</v>
+        <v>143.71875184087116</v>
       </c>
       <c r="D103" s="36">
-        <v>144.91350117465768</v>
+        <v>144.92087085994089</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -4982,10 +4982,10 @@
         <v>149.65170047837228</v>
       </c>
       <c r="C104" s="36">
-        <v>147.25816448563663</v>
+        <v>147.28294331306196</v>
       </c>
       <c r="D104" s="36">
-        <v>145.62760787754601</v>
+        <v>145.62950094758585</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -4996,10 +4996,10 @@
         <v>147.28124762344183</v>
       </c>
       <c r="C105" s="36">
-        <v>147.77108034400263</v>
+        <v>147.77459845486339</v>
       </c>
       <c r="D105" s="36">
-        <v>146.45095583923919</v>
+        <v>146.44979946004622</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -5010,10 +5010,10 @@
         <v>144.79670189548858</v>
       </c>
       <c r="C106" s="36">
-        <v>147.85494960643146</v>
+        <v>147.82665266807604</v>
       </c>
       <c r="D106" s="36">
-        <v>147.33080625379648</v>
+        <v>147.32966884077069</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -5024,10 +5024,10 @@
         <v>148.10395140212873</v>
       </c>
       <c r="C107" s="36">
-        <v>149.03990472112946</v>
+        <v>149.04702210828046</v>
       </c>
       <c r="D107" s="36">
-        <v>148.20942501255277</v>
+        <v>148.21264599445087</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -5038,10 +5038,10 @@
         <v>148.17873351747122</v>
       </c>
       <c r="C108" s="36">
-        <v>150.78759235875461</v>
+        <v>150.80205892011239</v>
       </c>
       <c r="D108" s="36">
-        <v>149.03728223119072</v>
+        <v>149.04951531608577</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -5052,10 +5052,10 @@
         <v>148.67760152837457</v>
       </c>
       <c r="C109" s="36">
-        <v>151.50685869618016</v>
+        <v>151.4852747475974</v>
       </c>
       <c r="D109" s="36">
-        <v>149.77811271241328</v>
+        <v>149.80399714657489</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -5066,10 +5066,10 @@
         <v>146.4966364505224</v>
       </c>
       <c r="C110" s="36">
-        <v>151.92199575618426</v>
+        <v>151.93093339871064</v>
       </c>
       <c r="D110" s="36">
-        <v>150.40784174193331</v>
+        <v>150.45108861213475</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -5080,10 +5080,10 @@
         <v>141.40459964053429</v>
       </c>
       <c r="C111" s="36">
-        <v>153.37296425710733</v>
+        <v>153.54265438189159</v>
       </c>
       <c r="D111" s="36">
-        <v>150.91761287520407</v>
+        <v>150.98034891323766</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -5094,10 +5094,10 @@
         <v>150.61015153616984</v>
       </c>
       <c r="C112" s="36">
-        <v>149.52580958425588</v>
+        <v>149.34718181686975</v>
       </c>
       <c r="D112" s="36">
-        <v>151.3132652618672</v>
+        <v>151.39565416407993</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -5108,10 +5108,10 @@
         <v>158.93929877299897</v>
       </c>
       <c r="C113" s="36">
-        <v>152.58190688614374</v>
+        <v>152.38409803081473</v>
       </c>
       <c r="D113" s="36">
-        <v>151.6118327838486</v>
+        <v>151.71206688080076</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -5122,10 +5122,10 @@
         <v>165.07464344720012</v>
       </c>
       <c r="C114" s="36">
-        <v>152.10509850995368</v>
+        <v>152.27051882633819</v>
       </c>
       <c r="D114" s="36">
-        <v>151.84009916066287</v>
+        <v>151.95539463227337</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -5136,10 +5136,10 @@
         <v>156.78890416942744</v>
       </c>
       <c r="C115" s="36">
-        <v>151.51591341259004</v>
+        <v>151.54830195145809</v>
       </c>
       <c r="D115" s="36">
-        <v>152.02852454257786</v>
+        <v>152.15179812916776</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -5150,10 +5150,10 @@
         <v>153.77022153385636</v>
       </c>
       <c r="C116" s="36">
-        <v>151.26917850671157</v>
+        <v>151.29330094897705</v>
       </c>
       <c r="D116" s="36">
-        <v>152.20647526950384</v>
+        <v>152.32498289774358</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -5164,10 +5164,10 @@
         <v>150.37579448728511</v>
       </c>
       <c r="C117" s="36">
-        <v>152.18135872900501</v>
+        <v>152.17594381036591</v>
       </c>
       <c r="D117" s="36">
-        <v>152.39827698759578</v>
+        <v>152.49533315689828</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -5178,10 +5178,10 @@
         <v>151.70554766622169</v>
       </c>
       <c r="C118" s="36">
-        <v>153.29642934768646</v>
+        <v>153.2777218239828</v>
       </c>
       <c r="D118" s="36">
-        <v>152.6196401859325</v>
+        <v>152.67467660504377</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -5192,10 +5192,10 @@
         <v>152.83834864492212</v>
       </c>
       <c r="C119" s="36">
-        <v>153.03322057927417</v>
+        <v>153.09073472926781</v>
       </c>
       <c r="D119" s="36">
-        <v>152.8804146809866</v>
+        <v>152.86703212981183</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -5206,10 +5206,10 @@
         <v>147.97168634998309</v>
       </c>
       <c r="C120" s="36">
-        <v>153.03461772858515</v>
+        <v>153.01278783725704</v>
       </c>
       <c r="D120" s="36">
-        <v>153.18672194001437</v>
+        <v>153.07496727109654</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -5220,10 +5220,10 @@
         <v>153.84616590720057</v>
       </c>
       <c r="C121" s="36">
-        <v>155.98350628491656</v>
+        <v>155.94782202617111</v>
       </c>
       <c r="D121" s="36">
-        <v>153.54155126861306</v>
+        <v>153.30179867180632</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -5231,13 +5231,13 @@
         <v>46023</v>
       </c>
       <c r="B122" s="17">
-        <v>149.47367834853273</v>
+        <v>149.429834187148</v>
       </c>
       <c r="C122" s="36">
-        <v>156.38624193363779</v>
+        <v>156.3008707103094</v>
       </c>
       <c r="D122" s="36">
-        <v>153.93960010835144</v>
+        <v>153.54792524515582</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -5245,13 +5245,13 @@
         <v>46054</v>
       </c>
       <c r="B123" s="17">
-        <v>139.28192710129798</v>
+        <v>139.31163157262827</v>
       </c>
       <c r="C123" s="36">
-        <v>152.22089169617513</v>
+        <v>152.46232518014887</v>
       </c>
       <c r="D123" s="36">
-        <v>154.36883960988379</v>
+        <v>153.81146081015922</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -5259,27 +5259,41 @@
         <v>46082</v>
       </c>
       <c r="B124" s="17">
-        <v>159.96271036768385</v>
+        <v>159.97685005773832</v>
       </c>
       <c r="C124" s="36">
-        <v>156.88717457417997</v>
+        <v>156.73111231345317</v>
       </c>
       <c r="D124" s="36">
-        <v>154.81366098735921</v>
+        <v>154.08801458161344</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
         <v>46113</v>
       </c>
-      <c r="B125" s="40">
-        <v>161.53886451705466</v>
-      </c>
-      <c r="C125" s="41">
-        <v>154.49351243562697</v>
-      </c>
-      <c r="D125" s="41">
-        <v>155.25620223242203</v>
+      <c r="B125" s="17">
+        <v>161.60721101015756</v>
+      </c>
+      <c r="C125" s="36">
+        <v>154.33640201486921</v>
+      </c>
+      <c r="D125" s="36">
+        <v>154.36994201063817</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B126" s="40">
+        <v>165.47141407640655</v>
+      </c>
+      <c r="C126" s="41">
+        <v>153.62027214485033</v>
+      </c>
+      <c r="D126" s="41">
+        <v>154.65561262723506</v>
       </c>
     </row>
   </sheetData>
@@ -8386,14 +8400,14 @@
         <v>70</v>
       </c>
       <c r="B2" s="46">
-        <v>6760.3574202399996</v>
+        <v>8481.3895971000002</v>
       </c>
       <c r="C2" s="46">
-        <v>8353.0324180600001</v>
+        <v>10358.58955208</v>
       </c>
       <c r="D2" s="27">
         <f>B2-C2</f>
-        <v>-1592.6749978200005</v>
+        <v>-1877.1999549800003</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -8401,14 +8415,14 @@
         <v>203</v>
       </c>
       <c r="B3" s="42">
-        <v>5074.5228449599999</v>
+        <v>6254.0776712200004</v>
       </c>
       <c r="C3" s="42">
-        <v>6160.8575116700003</v>
+        <v>7650.0725485599996</v>
       </c>
       <c r="D3" s="27">
         <f t="shared" ref="D3:D27" si="0">B3-C3</f>
-        <v>-1086.3346667100004</v>
+        <v>-1395.9948773399992</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -8416,14 +8430,14 @@
         <v>208</v>
       </c>
       <c r="B4" s="42">
-        <v>720.51602932000003</v>
+        <v>882.91976972999998</v>
       </c>
       <c r="C4" s="42">
-        <v>1962.3220318000001</v>
+        <v>2415.4081030100001</v>
       </c>
       <c r="D4" s="27">
         <f t="shared" si="0"/>
-        <v>-1241.8060024800002</v>
+        <v>-1532.48833328</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -8431,14 +8445,14 @@
         <v>209</v>
       </c>
       <c r="B5" s="42">
-        <v>786.42358318000004</v>
+        <v>1069.9884319400001</v>
       </c>
       <c r="C5" s="42">
-        <v>225.34801125999999</v>
+        <v>288.20453477000001</v>
       </c>
       <c r="D5" s="27">
         <f t="shared" si="0"/>
-        <v>561.07557192000002</v>
+        <v>781.78389717000005</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -8446,14 +8460,14 @@
         <v>72</v>
       </c>
       <c r="B6" s="46">
-        <v>4916.2404060999997</v>
+        <v>6114.1209186899996</v>
       </c>
       <c r="C6" s="46">
-        <v>926.04100387000005</v>
+        <v>1146.8822496400001</v>
       </c>
       <c r="D6" s="27">
         <f t="shared" si="0"/>
-        <v>3990.1994022299996</v>
+        <v>4967.2386690499998</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -8461,14 +8475,14 @@
         <v>71</v>
       </c>
       <c r="B7" s="42">
-        <v>2627.7504114600001</v>
+        <v>3279.5440918499999</v>
       </c>
       <c r="C7" s="42">
-        <v>390.88905758999999</v>
+        <v>471.02433543000001</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" si="0"/>
-        <v>2236.8613538700001</v>
+        <v>2808.5197564199998</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -8476,14 +8490,14 @@
         <v>204</v>
       </c>
       <c r="B8" s="42">
-        <v>1148.56413245</v>
+        <v>1348.9057046400001</v>
       </c>
       <c r="C8" s="42">
-        <v>126.11076921</v>
+        <v>157.82740096000001</v>
       </c>
       <c r="D8" s="27">
         <f t="shared" si="0"/>
-        <v>1022.45336324</v>
+        <v>1191.0783036800001</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -8491,14 +8505,14 @@
         <v>175</v>
       </c>
       <c r="B9" s="46">
-        <v>4887.5940500999995</v>
+        <v>5902.9134168700002</v>
       </c>
       <c r="C9" s="46">
-        <v>3378.5777676100001</v>
+        <v>4361.1140620799997</v>
       </c>
       <c r="D9" s="27">
         <f t="shared" si="0"/>
-        <v>1509.0162824899994</v>
+        <v>1541.7993547900005</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -8506,14 +8520,14 @@
         <v>205</v>
       </c>
       <c r="B10" s="42">
-        <v>3980.84028704</v>
+        <v>4858.6477084999997</v>
       </c>
       <c r="C10" s="42">
-        <v>2450.08950379</v>
+        <v>3284.0718609199998</v>
       </c>
       <c r="D10" s="27">
         <f t="shared" si="0"/>
-        <v>1530.75078325</v>
+        <v>1574.5758475799998</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -8521,14 +8535,14 @@
         <v>176</v>
       </c>
       <c r="B11" s="46">
-        <v>3543.5958568199999</v>
+        <v>4358.8776973599997</v>
       </c>
       <c r="C11" s="46">
-        <v>4101.6798812699999</v>
+        <v>5017.5170362500003</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" si="0"/>
-        <v>-558.08402445000002</v>
+        <v>-658.63933889000054</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -8536,14 +8550,14 @@
         <v>212</v>
       </c>
       <c r="B12" s="42">
-        <v>485.70343329000002</v>
+        <v>570.62108985999998</v>
       </c>
       <c r="C12" s="42">
-        <v>1240.0525508600001</v>
+        <v>1524.06350172</v>
       </c>
       <c r="D12" s="27">
         <f t="shared" si="0"/>
-        <v>-754.34911757000009</v>
+        <v>-953.44241185999999</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -8551,14 +8565,14 @@
         <v>213</v>
       </c>
       <c r="B13" s="42">
-        <v>526.35882613000001</v>
+        <v>715.86494592999998</v>
       </c>
       <c r="C13" s="42">
-        <v>438.8656244</v>
+        <v>528.95311143000004</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>87.49320173000001</v>
+        <v>186.91183449999994</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -8566,14 +8580,14 @@
         <v>214</v>
       </c>
       <c r="B14" s="42">
-        <v>428.70157697000002</v>
+        <v>516.88207270999999</v>
       </c>
       <c r="C14" s="42">
-        <v>620.79264322999995</v>
+        <v>766.57510847000003</v>
       </c>
       <c r="D14" s="27">
         <f t="shared" si="0"/>
-        <v>-192.09106625999993</v>
+        <v>-249.69303576000004</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -8581,14 +8595,14 @@
         <v>215</v>
       </c>
       <c r="B15" s="42">
-        <v>747.26877306999995</v>
+        <v>926.29658819999997</v>
       </c>
       <c r="C15" s="42">
-        <v>150.88724305</v>
+        <v>171.95748750999999</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>596.3815300199999</v>
+        <v>754.33910069000001</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -8596,14 +8610,14 @@
         <v>74</v>
       </c>
       <c r="B16" s="46">
-        <v>3938.04999632</v>
+        <v>4890.6300276399998</v>
       </c>
       <c r="C16" s="46">
-        <v>6481.3307118700004</v>
+        <v>7983.1137907000002</v>
       </c>
       <c r="D16" s="27">
         <f t="shared" si="0"/>
-        <v>-2543.2807155500004</v>
+        <v>-3092.4837630600005</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -8611,14 +8625,14 @@
         <v>75</v>
       </c>
       <c r="B17" s="46">
-        <v>2397.9217223400001</v>
+        <v>3101.0147205600001</v>
       </c>
       <c r="C17" s="46">
-        <v>452.64127581999998</v>
+        <v>562.39323972</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>1945.2804465200002</v>
+        <v>2538.62148084</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -8626,14 +8640,14 @@
         <v>73</v>
       </c>
       <c r="B18" s="46">
-        <v>3849.8118868400002</v>
+        <v>4613.0539279000004</v>
       </c>
       <c r="C18" s="46">
-        <v>1676.9590040099999</v>
+        <v>1981.40743335</v>
       </c>
       <c r="D18" s="27">
         <f t="shared" si="0"/>
-        <v>2172.8528828300005</v>
+        <v>2631.6464945500002</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -8641,14 +8655,14 @@
         <v>207</v>
       </c>
       <c r="B19" s="42">
-        <v>690.45605515</v>
+        <v>776.67251765000003</v>
       </c>
       <c r="C19" s="42">
-        <v>165.12670749</v>
+        <v>208.47525941000001</v>
       </c>
       <c r="D19" s="27">
         <f t="shared" si="0"/>
-        <v>525.32934765999994</v>
+        <v>568.19725824</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -8656,14 +8670,14 @@
         <v>210</v>
       </c>
       <c r="B20" s="42">
-        <v>655.55319564000001</v>
+        <v>798.89368889000002</v>
       </c>
       <c r="C20" s="42">
-        <v>98.943760389999994</v>
+        <v>118.69154020000001</v>
       </c>
       <c r="D20" s="27">
         <f t="shared" si="0"/>
-        <v>556.60943525000005</v>
+        <v>680.20214869000006</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -8671,14 +8685,14 @@
         <v>211</v>
       </c>
       <c r="B21" s="42">
-        <v>640.55588775000001</v>
+        <v>891.48188430000005</v>
       </c>
       <c r="C21" s="42">
-        <v>894.90727855</v>
+        <v>1032.2568432</v>
       </c>
       <c r="D21" s="27">
         <f t="shared" si="0"/>
-        <v>-254.35139079999999</v>
+        <v>-140.7749589</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -8686,14 +8700,14 @@
         <v>206</v>
       </c>
       <c r="B22" s="42">
-        <v>1558.07599291</v>
+        <v>1801.0153340700001</v>
       </c>
       <c r="C22" s="42">
-        <v>390.74539202</v>
+        <v>469.33647961000003</v>
       </c>
       <c r="D22" s="27">
         <f t="shared" si="0"/>
-        <v>1167.3306008899999</v>
+        <v>1331.6788544600001</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -8701,14 +8715,14 @@
         <v>76</v>
       </c>
       <c r="B23" s="46">
-        <v>2019.51447745</v>
+        <v>2481.4743572000002</v>
       </c>
       <c r="C23" s="46">
-        <v>177.96960652999999</v>
+        <v>217.91258299</v>
       </c>
       <c r="D23" s="27">
         <f t="shared" si="0"/>
-        <v>1841.54487092</v>
+        <v>2263.5617742100003</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -8716,14 +8730,14 @@
         <v>77</v>
       </c>
       <c r="B24" s="46">
-        <v>2095.4346260100001</v>
+        <v>2336.6136192099998</v>
       </c>
       <c r="C24" s="46">
-        <v>214.32533961999999</v>
+        <v>282.26240106</v>
       </c>
       <c r="D24" s="27">
         <f t="shared" si="0"/>
-        <v>1881.1092863900001</v>
+        <v>2054.35121815</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -8731,14 +8745,14 @@
         <v>78</v>
       </c>
       <c r="B25" s="46">
-        <v>138.51780590999999</v>
+        <v>172.32922266</v>
       </c>
       <c r="C25" s="46">
-        <v>106.6332111</v>
+        <v>116.87643165999999</v>
       </c>
       <c r="D25" s="27">
         <f t="shared" si="0"/>
-        <v>31.884594809999996</v>
+        <v>55.452791000000005</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -8746,14 +8760,14 @@
         <v>79</v>
       </c>
       <c r="B26" s="46">
-        <v>510.99229509000003</v>
+        <v>559.93835520000005</v>
       </c>
       <c r="C26" s="46">
-        <v>128.36391207</v>
+        <v>178.09884439999999</v>
       </c>
       <c r="D26" s="27">
         <f t="shared" si="0"/>
-        <v>382.62838302</v>
+        <v>381.83951080000008</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -8761,14 +8775,14 @@
         <v>80</v>
       </c>
       <c r="B27" s="47">
-        <v>5300.5615099400002</v>
+        <v>6442.1068232699999</v>
       </c>
       <c r="C27" s="47">
-        <v>2577.5686703199999</v>
+        <v>3325.2753946500002</v>
       </c>
       <c r="D27" s="27">
         <f t="shared" si="0"/>
-        <v>2722.9928396200003</v>
+        <v>3116.8314286199998</v>
       </c>
     </row>
   </sheetData>
@@ -8798,7 +8812,7 @@
         <v>172</v>
       </c>
       <c r="B2" s="48">
-        <v>40358.592053159999</v>
+        <v>49454.46268366</v>
       </c>
       <c r="D2" s="29"/>
     </row>
@@ -8807,7 +8821,7 @@
         <v>168</v>
       </c>
       <c r="B3" s="48">
-        <v>10742.82963538</v>
+        <v>12631.428010670001</v>
       </c>
       <c r="D3" s="29"/>
     </row>
@@ -8816,7 +8830,7 @@
         <v>121</v>
       </c>
       <c r="B4" s="49">
-        <v>13.95463872</v>
+        <v>16.464585719999999</v>
       </c>
       <c r="D4" s="30"/>
     </row>
@@ -8825,7 +8839,7 @@
         <v>122</v>
       </c>
       <c r="B5" s="49">
-        <v>925.60164197999995</v>
+        <v>1072.95508227</v>
       </c>
       <c r="D5" s="30"/>
     </row>
@@ -8834,7 +8848,7 @@
         <v>123</v>
       </c>
       <c r="B6" s="49">
-        <v>152.02629300000001</v>
+        <v>177.93759610000001</v>
       </c>
       <c r="D6" s="30"/>
     </row>
@@ -8843,7 +8857,7 @@
         <v>124</v>
       </c>
       <c r="B7" s="49">
-        <v>341.09879602000001</v>
+        <v>409.69851609</v>
       </c>
       <c r="D7" s="30"/>
     </row>
@@ -8852,7 +8866,7 @@
         <v>125</v>
       </c>
       <c r="B8" s="49">
-        <v>324.02407026999998</v>
+        <v>423.38260679000001</v>
       </c>
       <c r="D8" s="30"/>
     </row>
@@ -8861,7 +8875,7 @@
         <v>126</v>
       </c>
       <c r="B9" s="49">
-        <v>6557.1334442699999</v>
+        <v>7444.7477826599998</v>
       </c>
       <c r="D9" s="30"/>
     </row>
@@ -8870,7 +8884,7 @@
         <v>127</v>
       </c>
       <c r="B10" s="49">
-        <v>1708.08558193</v>
+        <v>2178.03683374</v>
       </c>
       <c r="D10" s="30"/>
     </row>
@@ -8879,7 +8893,7 @@
         <v>128</v>
       </c>
       <c r="B11" s="49">
-        <v>83.86755617</v>
+        <v>113.81617368000001</v>
       </c>
       <c r="D11" s="30"/>
     </row>
@@ -8888,7 +8902,7 @@
         <v>129</v>
       </c>
       <c r="B12" s="49">
-        <v>44.898907080000001</v>
+        <v>53.82557903</v>
       </c>
       <c r="D12" s="30"/>
     </row>
@@ -8897,7 +8911,7 @@
         <v>130</v>
       </c>
       <c r="B13" s="49">
-        <v>42.397263289999998</v>
+        <v>55.442203339999999</v>
       </c>
       <c r="D13" s="30"/>
     </row>
@@ -8906,7 +8920,7 @@
         <v>131</v>
       </c>
       <c r="B14" s="49">
-        <v>459.11204710999999</v>
+        <v>574.83523628</v>
       </c>
       <c r="D14" s="30"/>
     </row>
@@ -8915,7 +8929,7 @@
         <v>132</v>
       </c>
       <c r="B15" s="49">
-        <v>90.629395540000004</v>
+        <v>110.28581497</v>
       </c>
       <c r="D15" s="30"/>
     </row>
@@ -8924,7 +8938,7 @@
         <v>169</v>
       </c>
       <c r="B16" s="48">
-        <v>12470.11895038</v>
+        <v>15819.496350199999</v>
       </c>
       <c r="D16" s="29"/>
     </row>
@@ -8933,7 +8947,7 @@
         <v>133</v>
       </c>
       <c r="B17" s="49">
-        <v>2068.17821129</v>
+        <v>2570.6484228200002</v>
       </c>
       <c r="D17" s="30"/>
     </row>
@@ -8942,7 +8956,7 @@
         <v>134</v>
       </c>
       <c r="B18" s="49">
-        <v>122.0667815</v>
+        <v>156.63452408000001</v>
       </c>
       <c r="D18" s="30"/>
     </row>
@@ -8951,7 +8965,7 @@
         <v>135</v>
       </c>
       <c r="B19" s="49">
-        <v>595.02203373999998</v>
+        <v>731.49064919</v>
       </c>
       <c r="D19" s="30"/>
     </row>
@@ -8960,7 +8974,7 @@
         <v>136</v>
       </c>
       <c r="B20" s="49">
-        <v>39.94780351</v>
+        <v>48.8231167</v>
       </c>
       <c r="D20" s="30"/>
     </row>
@@ -8969,7 +8983,7 @@
         <v>137</v>
       </c>
       <c r="B21" s="49">
-        <v>43.27242983</v>
+        <v>58.525990210000003</v>
       </c>
       <c r="D21" s="30"/>
     </row>
@@ -8978,7 +8992,7 @@
         <v>138</v>
       </c>
       <c r="B22" s="49">
-        <v>73.02852584</v>
+        <v>91.483421500000006</v>
       </c>
       <c r="D22" s="30"/>
     </row>
@@ -8987,7 +9001,7 @@
         <v>139</v>
       </c>
       <c r="B23" s="49">
-        <v>314.77157653</v>
+        <v>403.77321796000001</v>
       </c>
       <c r="D23" s="30"/>
     </row>
@@ -8996,7 +9010,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="49">
-        <v>3971.7894703400002</v>
+        <v>5222.8086147699996</v>
       </c>
       <c r="D24" s="30"/>
     </row>
@@ -9005,7 +9019,7 @@
         <v>141</v>
       </c>
       <c r="B25" s="49">
-        <v>164.47925072999999</v>
+        <v>190.33760681999999</v>
       </c>
       <c r="D25" s="30"/>
     </row>
@@ -9014,7 +9028,7 @@
         <v>142</v>
       </c>
       <c r="B26" s="49">
-        <v>409.54609006999999</v>
+        <v>520.09811133000005</v>
       </c>
       <c r="D26" s="30"/>
     </row>
@@ -9023,7 +9037,7 @@
         <v>143</v>
       </c>
       <c r="B27" s="49">
-        <v>322.72882701999998</v>
+        <v>389.43796888999998</v>
       </c>
       <c r="D27" s="30"/>
     </row>
@@ -9032,7 +9046,7 @@
         <v>144</v>
       </c>
       <c r="B28" s="49">
-        <v>3712.53847206</v>
+        <v>4678.4785626299999</v>
       </c>
       <c r="D28" s="30"/>
     </row>
@@ -9041,7 +9055,7 @@
         <v>145</v>
       </c>
       <c r="B29" s="49">
-        <v>128.95324006000001</v>
+        <v>157.20024982999999</v>
       </c>
       <c r="D29" s="30"/>
     </row>
@@ -9050,7 +9064,7 @@
         <v>146</v>
       </c>
       <c r="B30" s="49">
-        <v>147.27759675999999</v>
+        <v>174.71465499999999</v>
       </c>
       <c r="D30" s="30"/>
     </row>
@@ -9059,7 +9073,7 @@
         <v>147</v>
       </c>
       <c r="B31" s="49">
-        <v>56.991716140000001</v>
+        <v>68.174505429999996</v>
       </c>
       <c r="D31" s="30"/>
     </row>
@@ -9068,7 +9082,7 @@
         <v>148</v>
       </c>
       <c r="B32" s="49">
-        <v>299.52692495999997</v>
+        <v>356.86673303999999</v>
       </c>
       <c r="D32" s="30"/>
     </row>
@@ -9077,7 +9091,7 @@
         <v>170</v>
       </c>
       <c r="B33" s="48">
-        <v>10963.75355042</v>
+        <v>13384.87206421</v>
       </c>
       <c r="D33" s="29"/>
     </row>
@@ -9086,7 +9100,7 @@
         <v>149</v>
       </c>
       <c r="B34" s="49">
-        <v>2361.9270891900001</v>
+        <v>2991.57088901</v>
       </c>
       <c r="D34" s="30"/>
     </row>
@@ -9095,7 +9109,7 @@
         <v>150</v>
       </c>
       <c r="B35" s="49">
-        <v>498.63657723</v>
+        <v>607.09800845999996</v>
       </c>
       <c r="D35" s="30"/>
     </row>
@@ -9104,7 +9118,7 @@
         <v>151</v>
       </c>
       <c r="B36" s="49">
-        <v>69.397753019999996</v>
+        <v>85.910532889999999</v>
       </c>
       <c r="D36" s="30"/>
     </row>
@@ -9113,7 +9127,7 @@
         <v>152</v>
       </c>
       <c r="B37" s="49">
-        <v>7.59139257</v>
+        <v>8.7954096499999999</v>
       </c>
       <c r="D37" s="30"/>
     </row>
@@ -9122,7 +9136,7 @@
         <v>153</v>
       </c>
       <c r="B38" s="49">
-        <v>174.5819454</v>
+        <v>214.91494496999999</v>
       </c>
       <c r="D38" s="30"/>
     </row>
@@ -9131,7 +9145,7 @@
         <v>154</v>
       </c>
       <c r="B39" s="49">
-        <v>43.539436969999997</v>
+        <v>53.943710869999997</v>
       </c>
       <c r="D39" s="30"/>
     </row>
@@ -9140,7 +9154,7 @@
         <v>155</v>
       </c>
       <c r="B40" s="49">
-        <v>4.0489054099999997</v>
+        <v>4.4194451199999998</v>
       </c>
       <c r="D40" s="30"/>
     </row>
@@ -9149,7 +9163,7 @@
         <v>156</v>
       </c>
       <c r="B41" s="49">
-        <v>55.587595579999999</v>
+        <v>66.158591869999995</v>
       </c>
       <c r="D41" s="30"/>
     </row>
@@ -9158,7 +9172,7 @@
         <v>157</v>
       </c>
       <c r="B42" s="49">
-        <v>2534.0538823299999</v>
+        <v>2937.4714189900001</v>
       </c>
       <c r="D42" s="30"/>
     </row>
@@ -9167,7 +9181,7 @@
         <v>158</v>
       </c>
       <c r="B43" s="49">
-        <v>1098.6494364099999</v>
+        <v>1400.86288964</v>
       </c>
       <c r="D43" s="30"/>
     </row>
@@ -9176,7 +9190,7 @@
         <v>159</v>
       </c>
       <c r="B44" s="49">
-        <v>529.39998568999999</v>
+        <v>647.06496117999995</v>
       </c>
       <c r="D44" s="30"/>
     </row>
@@ -9185,7 +9199,7 @@
         <v>160</v>
       </c>
       <c r="B45" s="49">
-        <v>3183.4768767599999</v>
+        <v>3921.32795747</v>
       </c>
       <c r="D45" s="30"/>
     </row>
@@ -9194,7 +9208,7 @@
         <v>161</v>
       </c>
       <c r="B46" s="49">
-        <v>73.072475859999997</v>
+        <v>82.83759628</v>
       </c>
       <c r="D46" s="30"/>
     </row>
@@ -9203,7 +9217,7 @@
         <v>162</v>
       </c>
       <c r="B47" s="49">
-        <v>329.79019799999998</v>
+        <v>362.49570781</v>
       </c>
       <c r="D47" s="30"/>
     </row>
@@ -9212,7 +9226,7 @@
         <v>171</v>
       </c>
       <c r="B48" s="48">
-        <v>6181.8899169799997</v>
+        <v>7618.6662585800004</v>
       </c>
       <c r="D48" s="29"/>
     </row>
@@ -9221,7 +9235,7 @@
         <v>163</v>
       </c>
       <c r="B49" s="49">
-        <v>3773.07590686</v>
+        <v>4692.6805862399997</v>
       </c>
       <c r="D49" s="30"/>
     </row>
@@ -9230,7 +9244,7 @@
         <v>164</v>
       </c>
       <c r="B50" s="49">
-        <v>1470.5336399299999</v>
+        <v>1802.6515664599999</v>
       </c>
       <c r="D50" s="30"/>
     </row>
@@ -9239,7 +9253,7 @@
         <v>165</v>
       </c>
       <c r="B51" s="49">
-        <v>42.737934950000003</v>
+        <v>55.09513304</v>
       </c>
       <c r="D51" s="30"/>
     </row>
@@ -9248,7 +9262,7 @@
         <v>166</v>
       </c>
       <c r="B52" s="49">
-        <v>688.91321946999994</v>
+        <v>825.29429833999995</v>
       </c>
       <c r="D52" s="30"/>
     </row>
@@ -9257,7 +9271,7 @@
         <v>167</v>
       </c>
       <c r="B53" s="50">
-        <v>206.62921577</v>
+        <v>242.94467449999999</v>
       </c>
     </row>
   </sheetData>
@@ -9287,7 +9301,7 @@
         <v>177</v>
       </c>
       <c r="B2" s="43">
-        <v>28575.122802149999</v>
+        <v>35531.443018580001</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -9295,7 +9309,7 @@
         <v>178</v>
       </c>
       <c r="B3" s="43">
-        <v>5680.18930654</v>
+        <v>6799.3836805999999</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -9303,7 +9317,7 @@
         <v>179</v>
       </c>
       <c r="B4" s="44">
-        <v>4049.2899463799999</v>
+        <v>4883.5781913500005</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -9311,7 +9325,7 @@
         <v>180</v>
       </c>
       <c r="B5" s="44">
-        <v>644.54279412999995</v>
+        <v>764.12688181999999</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -9319,7 +9333,7 @@
         <v>181</v>
       </c>
       <c r="B6" s="44">
-        <v>986.35656602999995</v>
+        <v>1151.6786074300001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -9327,7 +9341,7 @@
         <v>182</v>
       </c>
       <c r="B7" s="43">
-        <v>9944.4785994899994</v>
+        <v>12288.059822949999</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -9335,7 +9349,7 @@
         <v>183</v>
       </c>
       <c r="B8" s="44">
-        <v>1780.7678902600001</v>
+        <v>2178.7017841500001</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -9343,7 +9357,7 @@
         <v>184</v>
       </c>
       <c r="B9" s="44">
-        <v>241.53804482000001</v>
+        <v>292.60839814000002</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -9351,7 +9365,7 @@
         <v>185</v>
       </c>
       <c r="B10" s="44">
-        <v>403.19594374000002</v>
+        <v>482.11012384999998</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -9359,7 +9373,7 @@
         <v>186</v>
       </c>
       <c r="B11" s="44">
-        <v>6696.8891205399996</v>
+        <v>8337.3539427199994</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -9367,7 +9381,7 @@
         <v>187</v>
       </c>
       <c r="B12" s="44">
-        <v>822.08760013000006</v>
+        <v>997.28557408999995</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -9375,7 +9389,7 @@
         <v>188</v>
       </c>
       <c r="B13" s="43">
-        <v>779.41737588000001</v>
+        <v>1669.0895602000001</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -9383,7 +9397,7 @@
         <v>189</v>
       </c>
       <c r="B14" s="44">
-        <v>114.50504565</v>
+        <v>178.6497689</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -9391,7 +9405,7 @@
         <v>190</v>
       </c>
       <c r="B15" s="44">
-        <v>664.91233022999995</v>
+        <v>1490.4397913</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -9399,7 +9413,7 @@
         <v>191</v>
       </c>
       <c r="B16" s="43">
-        <v>5050.0036894200002</v>
+        <v>6144.30421019</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -9407,7 +9421,7 @@
         <v>192</v>
       </c>
       <c r="B17" s="44">
-        <v>1974.08409665</v>
+        <v>2391.5527711</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9415,7 +9429,7 @@
         <v>193</v>
       </c>
       <c r="B18" s="44">
-        <v>262.19359321000002</v>
+        <v>318.78053840000001</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -9423,7 +9437,7 @@
         <v>194</v>
       </c>
       <c r="B19" s="44">
-        <v>2813.7259995600002</v>
+        <v>3433.9709006899998</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -9431,7 +9445,7 @@
         <v>195</v>
       </c>
       <c r="B20" s="43">
-        <v>4439.4726040400001</v>
+        <v>5362.2500497299998</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -9439,7 +9453,7 @@
         <v>196</v>
       </c>
       <c r="B21" s="44">
-        <v>358.04943355</v>
+        <v>422.58905465999999</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -9447,7 +9461,7 @@
         <v>197</v>
       </c>
       <c r="B22" s="44">
-        <v>636.29293293000001</v>
+        <v>790.74661163999997</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -9455,7 +9469,7 @@
         <v>198</v>
       </c>
       <c r="B23" s="44">
-        <v>362.51033396000003</v>
+        <v>433.56903849999998</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -9463,7 +9477,7 @@
         <v>199</v>
       </c>
       <c r="B24" s="44">
-        <v>448.98838480000001</v>
+        <v>548.26871476999997</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -9471,7 +9485,7 @@
         <v>200</v>
       </c>
       <c r="B25" s="44">
-        <v>1205.3241165300001</v>
+        <v>1409.0464241100001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -9479,7 +9493,7 @@
         <v>201</v>
       </c>
       <c r="B26" s="44">
-        <v>759.16058797000005</v>
+        <v>940.87862426000004</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -9487,7 +9501,7 @@
         <v>187</v>
       </c>
       <c r="B27" s="44">
-        <v>669.14681429999996</v>
+        <v>817.15158179000002</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -9495,7 +9509,7 @@
         <v>202</v>
       </c>
       <c r="B28" s="43">
-        <v>2142.1602361300002</v>
+        <v>2597.56740356</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -9503,7 +9517,7 @@
         <v>173</v>
       </c>
       <c r="B29" s="45">
-        <v>539.40099065000004</v>
+        <v>670.78829135000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
"agrego dato ipc jul26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4921F18-139E-420D-AD54-01919946EA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB87912E-6371-4079-B50D-2DC51D993134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -1339,7 +1339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H115"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="1" customWidth="1"/>
@@ -3301,6 +3301,23 @@
       </c>
       <c r="E115">
         <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="19">
+        <v>46204</v>
+      </c>
+      <c r="B116" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="C116" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="D116">
+        <v>1.8</v>
+      </c>
+      <c r="E116">
+        <v>2.1</v>
       </c>
     </row>
   </sheetData>
@@ -5341,25 +5358,25 @@
         <v>112</v>
       </c>
       <c r="B2" s="37">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="C2" s="20">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="D2" s="20">
-        <v>2.2000000000000002</v>
+        <v>1.9</v>
       </c>
       <c r="E2" s="20">
-        <v>2.9</v>
+        <v>1.7</v>
       </c>
       <c r="F2" s="20">
-        <v>2.2999999999999998</v>
+        <v>1.8</v>
       </c>
       <c r="G2" s="20">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="H2" s="16">
-        <v>2.3912881772367944</v>
+        <v>1.8135346659637008</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5367,25 +5384,25 @@
         <v>113</v>
       </c>
       <c r="B3" s="37">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="20">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D3" s="20">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="E3" s="20">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F3" s="20">
-        <v>-0.7</v>
+        <v>-0.3</v>
       </c>
       <c r="G3" s="20">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="H3" s="16">
-        <v>5.5247484828879756E-2</v>
+        <v>0.15020439665571761</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5393,25 +5410,25 @@
         <v>114</v>
       </c>
       <c r="B4" s="37">
-        <v>0.4</v>
+        <v>3.4</v>
       </c>
       <c r="C4" s="20">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="D4" s="20">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="E4" s="20">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="F4" s="20">
-        <v>-0.2</v>
+        <v>2.4</v>
       </c>
       <c r="G4" s="20">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="H4" s="16">
-        <v>1.0312155789434119</v>
+        <v>2.5358045496943538</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5419,25 +5436,25 @@
         <v>115</v>
       </c>
       <c r="B5" s="37">
-        <v>0.7</v>
+        <v>2.6</v>
       </c>
       <c r="C5" s="20">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="D5" s="20">
+        <v>1.7</v>
+      </c>
+      <c r="E5" s="20">
+        <v>1.4</v>
+      </c>
+      <c r="F5" s="20">
+        <v>0</v>
+      </c>
+      <c r="G5" s="20">
         <v>2.2999999999999998</v>
       </c>
-      <c r="E5" s="20">
-        <v>2.1</v>
-      </c>
-      <c r="F5" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="G5" s="20">
-        <v>2.7</v>
-      </c>
       <c r="H5" s="16">
-        <v>1.3303893574575953</v>
+        <v>2.1747538305427305</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5445,25 +5462,25 @@
         <v>116</v>
       </c>
       <c r="B6" s="37">
-        <v>-2.6</v>
+        <v>7.4</v>
       </c>
       <c r="C6" s="20">
-        <v>-3.1</v>
+        <v>1.7</v>
       </c>
       <c r="D6" s="20">
-        <v>-3.5</v>
+        <v>1.3</v>
       </c>
       <c r="E6" s="20">
-        <v>-1.7</v>
+        <v>2.7</v>
       </c>
       <c r="F6" s="20">
-        <v>-4.3</v>
+        <v>-1.6</v>
       </c>
       <c r="G6" s="20">
-        <v>-5</v>
+        <v>-0.2</v>
       </c>
       <c r="H6" s="16">
-        <v>-2.9896060095035426</v>
+        <v>4.0552087145800053</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5471,25 +5488,25 @@
         <v>117</v>
       </c>
       <c r="B7" s="37">
+        <v>9</v>
+      </c>
+      <c r="C7" s="20">
+        <v>6.4</v>
+      </c>
+      <c r="D7" s="20">
+        <v>6.7</v>
+      </c>
+      <c r="E7" s="20">
+        <v>8.1</v>
+      </c>
+      <c r="F7" s="20">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="G7" s="20">
         <v>8.3000000000000007</v>
       </c>
-      <c r="C7" s="20">
-        <v>5.9</v>
-      </c>
-      <c r="D7" s="20">
-        <v>4.7</v>
-      </c>
-      <c r="E7" s="20">
-        <v>3.8</v>
-      </c>
-      <c r="F7" s="20">
-        <v>16.100000000000001</v>
-      </c>
-      <c r="G7" s="20">
-        <v>9.4</v>
-      </c>
       <c r="H7" s="16">
-        <v>7.4654649817116114</v>
+        <v>7.6784047340026973</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5497,25 +5514,25 @@
         <v>118</v>
       </c>
       <c r="B8" s="37">
-        <v>0.5</v>
+        <v>2.1</v>
       </c>
       <c r="C8" s="20">
-        <v>1.9</v>
+        <v>1</v>
       </c>
       <c r="D8" s="20">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E8" s="20">
-        <v>2.2000000000000002</v>
+        <v>1.4</v>
       </c>
       <c r="F8" s="20">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="G8" s="20">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="H8" s="16">
-        <v>1.2830523940615901</v>
+        <v>1.6333603985065226</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5523,25 +5540,25 @@
         <v>119</v>
       </c>
       <c r="B9" s="37">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="C9" s="20">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="D9" s="20">
-        <v>1.9</v>
+        <v>0.8</v>
       </c>
       <c r="E9" s="20">
-        <v>1.8</v>
+        <v>-0.6</v>
       </c>
       <c r="F9" s="20">
-        <v>0.4</v>
+        <v>-2.6</v>
       </c>
       <c r="G9" s="20">
-        <v>2.8</v>
+        <v>-0.8</v>
       </c>
       <c r="H9" s="16">
-        <v>0.43334628218292259</v>
+        <v>-0.15434022477673892</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5549,25 +5566,25 @@
         <v>120</v>
       </c>
       <c r="B10" s="37">
-        <v>1.1000000000000001</v>
+        <v>2.6</v>
       </c>
       <c r="C10" s="20">
+        <v>2.5</v>
+      </c>
+      <c r="D10" s="20">
+        <v>1.7</v>
+      </c>
+      <c r="E10" s="20">
         <v>1.8</v>
       </c>
-      <c r="D10" s="20">
-        <v>1.4</v>
-      </c>
-      <c r="E10" s="20">
-        <v>0.9</v>
-      </c>
       <c r="F10" s="20">
-        <v>1.8</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G10" s="20">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="H10" s="16">
-        <v>1.4670028148804803</v>
+        <v>2.4454493931863386</v>
       </c>
     </row>
   </sheetData>
@@ -5612,25 +5629,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="24">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="C2" s="24">
-        <v>1.9</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="D2" s="24">
         <v>2</v>
       </c>
       <c r="E2" s="24">
+        <v>2</v>
+      </c>
+      <c r="F2" s="24">
+        <v>2</v>
+      </c>
+      <c r="G2" s="24">
         <v>1.9</v>
       </c>
-      <c r="F2" s="24">
-        <v>1.7</v>
-      </c>
-      <c r="G2" s="24">
-        <v>1.6</v>
-      </c>
       <c r="H2" s="24">
-        <v>1.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5638,25 +5655,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="22">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="C3" s="22">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="D3" s="22">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="E3" s="22">
         <v>1.5</v>
       </c>
       <c r="F3" s="22">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="G3" s="22">
-        <v>1.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H3" s="22">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5664,25 +5681,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="22">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="C4" s="22">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D4" s="22">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="E4" s="22">
-        <v>2.4</v>
+        <v>1.3</v>
       </c>
       <c r="F4" s="22">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="G4" s="22">
-        <v>2.6</v>
+        <v>1.7</v>
       </c>
       <c r="H4" s="22">
-        <v>2.2000000000000002</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5690,25 +5707,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="22">
+        <v>-1.3</v>
+      </c>
+      <c r="C5" s="22">
+        <v>-3</v>
+      </c>
+      <c r="D5" s="22">
+        <v>0.1</v>
+      </c>
+      <c r="E5" s="22">
+        <v>0</v>
+      </c>
+      <c r="F5" s="22">
         <v>0.4</v>
       </c>
-      <c r="C5" s="22">
-        <v>0.1</v>
-      </c>
-      <c r="D5" s="22">
-        <v>0.7</v>
-      </c>
-      <c r="E5" s="22">
-        <v>0.7</v>
-      </c>
-      <c r="F5" s="22">
-        <v>0.1</v>
-      </c>
       <c r="G5" s="22">
-        <v>1.2</v>
+        <v>-0.7</v>
       </c>
       <c r="H5" s="22">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5716,25 +5733,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C6" s="22">
+        <v>1.5</v>
+      </c>
+      <c r="D6" s="22">
+        <v>2.6</v>
+      </c>
+      <c r="E6" s="22">
+        <v>3.9</v>
+      </c>
+      <c r="F6" s="22">
         <v>3.3</v>
       </c>
-      <c r="C6" s="22">
-        <v>3.9</v>
-      </c>
-      <c r="D6" s="22">
-        <v>2.9</v>
-      </c>
-      <c r="E6" s="22">
-        <v>5</v>
-      </c>
-      <c r="F6" s="22">
+      <c r="G6" s="22">
         <v>2.2000000000000002</v>
       </c>
-      <c r="G6" s="22">
-        <v>1.5</v>
-      </c>
       <c r="H6" s="22">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5742,22 +5759,22 @@
         <v>17</v>
       </c>
       <c r="B7" s="22">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="C7" s="22">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="D7" s="22">
-        <v>1.5</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="E7" s="22">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="F7" s="22">
-        <v>1.4</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G7" s="22">
-        <v>1.2</v>
+        <v>2.1</v>
       </c>
       <c r="H7" s="22">
         <v>1.4</v>
@@ -5768,25 +5785,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="22">
+        <v>2.5</v>
+      </c>
+      <c r="C8" s="22">
+        <v>2.4</v>
+      </c>
+      <c r="D8" s="22">
         <v>2.9</v>
       </c>
-      <c r="C8" s="22">
-        <v>3.2</v>
-      </c>
-      <c r="D8" s="22">
+      <c r="E8" s="22">
+        <v>2.7</v>
+      </c>
+      <c r="F8" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G8" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="H8" s="22">
         <v>2.5</v>
-      </c>
-      <c r="E8" s="22">
-        <v>3</v>
-      </c>
-      <c r="F8" s="22">
-        <v>2.9</v>
-      </c>
-      <c r="G8" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="H8" s="22">
-        <v>2.7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5794,25 +5811,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="22">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="C9" s="22">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="D9" s="22">
-        <v>2.2000000000000002</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E9" s="22">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="F9" s="22">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="G9" s="22">
-        <v>0.6</v>
+        <v>3.2</v>
       </c>
       <c r="H9" s="22">
-        <v>0.7</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5820,25 +5837,25 @@
         <v>20</v>
       </c>
       <c r="B10" s="22">
-        <v>0.9</v>
+        <v>2.4</v>
       </c>
       <c r="C10" s="22">
-        <v>0.3</v>
+        <v>2.6</v>
       </c>
       <c r="D10" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="E10" s="22">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F10" s="22">
         <v>2</v>
       </c>
-      <c r="E10" s="22">
-        <v>-0.1</v>
-      </c>
-      <c r="F10" s="22">
-        <v>1.2</v>
-      </c>
       <c r="G10" s="22">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="H10" s="22">
-        <v>0.3</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -5846,25 +5863,25 @@
         <v>21</v>
       </c>
       <c r="B11" s="22">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="C11" s="22">
+        <v>5.8</v>
+      </c>
+      <c r="D11" s="22">
+        <v>4.3</v>
+      </c>
+      <c r="E11" s="22">
         <v>4</v>
       </c>
-      <c r="D11" s="22">
-        <v>5.2</v>
-      </c>
-      <c r="E11" s="22">
+      <c r="F11" s="22">
+        <v>5.3</v>
+      </c>
+      <c r="G11" s="22">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="H11" s="22">
         <v>2.8</v>
-      </c>
-      <c r="F11" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="G11" s="22">
-        <v>3.4</v>
-      </c>
-      <c r="H11" s="22">
-        <v>3.2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -5872,25 +5889,25 @@
         <v>22</v>
       </c>
       <c r="B12" s="22">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="C12" s="22">
-        <v>1.4</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="D12" s="22">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="E12" s="22">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="F12" s="22">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="G12" s="22">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="H12" s="22">
-        <v>1.8</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -5898,25 +5915,25 @@
         <v>23</v>
       </c>
       <c r="B13" s="22">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="C13" s="22">
-        <v>1.2</v>
+        <v>3.3</v>
       </c>
       <c r="D13" s="22">
-        <v>2.2999999999999998</v>
+        <v>2.4</v>
       </c>
       <c r="E13" s="22">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="F13" s="22">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="G13" s="22">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="H13" s="22">
-        <v>1.1000000000000001</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -5924,25 +5941,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C14" s="22">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D14" s="22">
+        <v>2.6</v>
+      </c>
+      <c r="E14" s="22">
+        <v>1.9</v>
+      </c>
+      <c r="F14" s="22">
+        <v>1.7</v>
+      </c>
+      <c r="G14" s="22">
         <v>1.8</v>
       </c>
-      <c r="C14" s="22">
-        <v>1.9</v>
-      </c>
-      <c r="D14" s="22">
+      <c r="H14" s="22">
         <v>1.5</v>
-      </c>
-      <c r="E14" s="22">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="F14" s="22">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="G14" s="22">
-        <v>1.4</v>
-      </c>
-      <c r="H14" s="22">
-        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -5987,25 +6004,25 @@
         <v>12</v>
       </c>
       <c r="B2" s="33">
-        <v>33.5</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="C2" s="33">
-        <v>33.4</v>
+        <v>34</v>
       </c>
       <c r="D2" s="33">
         <v>33.4</v>
       </c>
       <c r="E2" s="33">
-        <v>36.5</v>
+        <v>36.9</v>
       </c>
       <c r="F2" s="33">
-        <v>33.799999999999997</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="G2" s="33">
         <v>34</v>
       </c>
       <c r="H2" s="33">
-        <v>32</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -6013,25 +6030,25 @@
         <v>13</v>
       </c>
       <c r="B3" s="34">
+        <v>34.5</v>
+      </c>
+      <c r="C3" s="34">
         <v>34.4</v>
       </c>
-      <c r="C3" s="34">
-        <v>33.9</v>
-      </c>
       <c r="D3" s="34">
-        <v>34.700000000000003</v>
+        <v>34.4</v>
       </c>
       <c r="E3" s="34">
-        <v>40.200000000000003</v>
+        <v>40.700000000000003</v>
       </c>
       <c r="F3" s="34">
-        <v>35.5</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="G3" s="34">
-        <v>35.700000000000003</v>
+        <v>34.299999999999997</v>
       </c>
       <c r="H3" s="34">
-        <v>28.2</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -6039,25 +6056,25 @@
         <v>14</v>
       </c>
       <c r="B4" s="34">
-        <v>23.2</v>
+        <v>24.2</v>
       </c>
       <c r="C4" s="34">
-        <v>23.1</v>
+        <v>24.6</v>
       </c>
       <c r="D4" s="34">
-        <v>23</v>
+        <v>23.6</v>
       </c>
       <c r="E4" s="34">
-        <v>22.3</v>
+        <v>22.9</v>
       </c>
       <c r="F4" s="34">
-        <v>23.1</v>
+        <v>23.8</v>
       </c>
       <c r="G4" s="34">
-        <v>23.3</v>
+        <v>24.7</v>
       </c>
       <c r="H4" s="34">
-        <v>25.3</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6065,25 +6082,25 @@
         <v>15</v>
       </c>
       <c r="B5" s="34">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="C5" s="34">
-        <v>13</v>
+        <v>11.4</v>
       </c>
       <c r="D5" s="34">
-        <v>10</v>
+        <v>10.7</v>
       </c>
       <c r="E5" s="34">
-        <v>14.4</v>
+        <v>13.7</v>
       </c>
       <c r="F5" s="34">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="G5" s="34">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="H5" s="34">
-        <v>14</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -6091,25 +6108,25 @@
         <v>16</v>
       </c>
       <c r="B6" s="34">
-        <v>47.8</v>
+        <v>48.9</v>
       </c>
       <c r="C6" s="34">
-        <v>43.3</v>
+        <v>44.9</v>
       </c>
       <c r="D6" s="34">
-        <v>48.2</v>
+        <v>48.5</v>
       </c>
       <c r="E6" s="34">
-        <v>70.7</v>
+        <v>72.8</v>
       </c>
       <c r="F6" s="34">
-        <v>50.3</v>
+        <v>51.7</v>
       </c>
       <c r="G6" s="34">
-        <v>52.8</v>
+        <v>52.3</v>
       </c>
       <c r="H6" s="34">
-        <v>52.9</v>
+        <v>53.1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -6117,25 +6134,25 @@
         <v>17</v>
       </c>
       <c r="B7" s="34">
-        <v>23.1</v>
+        <v>23.7</v>
       </c>
       <c r="C7" s="34">
-        <v>24.4</v>
+        <v>25</v>
       </c>
       <c r="D7" s="34">
-        <v>22.7</v>
+        <v>23.6</v>
       </c>
       <c r="E7" s="34">
-        <v>17.399999999999999</v>
+        <v>17.5</v>
       </c>
       <c r="F7" s="34">
-        <v>21.7</v>
+        <v>22.9</v>
       </c>
       <c r="G7" s="34">
-        <v>23.1</v>
+        <v>24.1</v>
       </c>
       <c r="H7" s="34">
-        <v>20.2</v>
+        <v>20.399999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6143,25 +6160,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="34">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="C8" s="34">
+        <v>32.5</v>
+      </c>
+      <c r="D8" s="34">
+        <v>32.700000000000003</v>
+      </c>
+      <c r="E8" s="34">
         <v>30.5</v>
       </c>
-      <c r="C8" s="34">
-        <v>31</v>
-      </c>
-      <c r="D8" s="34">
-        <v>30.4</v>
-      </c>
-      <c r="E8" s="34">
-        <v>27.7</v>
-      </c>
       <c r="F8" s="34">
-        <v>29.1</v>
+        <v>31.2</v>
       </c>
       <c r="G8" s="34">
-        <v>28.3</v>
+        <v>29.9</v>
       </c>
       <c r="H8" s="34">
-        <v>32.9</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -6169,25 +6186,25 @@
         <v>19</v>
       </c>
       <c r="B9" s="34">
-        <v>42.1</v>
+        <v>40.9</v>
       </c>
       <c r="C9" s="34">
-        <v>42.5</v>
+        <v>41.5</v>
       </c>
       <c r="D9" s="34">
+        <v>39.6</v>
+      </c>
+      <c r="E9" s="34">
+        <v>34.700000000000003</v>
+      </c>
+      <c r="F9" s="34">
+        <v>44.9</v>
+      </c>
+      <c r="G9" s="34">
+        <v>44.7</v>
+      </c>
+      <c r="H9" s="34">
         <v>41.1</v>
-      </c>
-      <c r="E9" s="34">
-        <v>36</v>
-      </c>
-      <c r="F9" s="34">
-        <v>46.7</v>
-      </c>
-      <c r="G9" s="34">
-        <v>43.5</v>
-      </c>
-      <c r="H9" s="34">
-        <v>45.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -6195,19 +6212,19 @@
         <v>20</v>
       </c>
       <c r="B10" s="34">
-        <v>36.1</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="C10" s="34">
-        <v>37.4</v>
+        <v>37.6</v>
       </c>
       <c r="D10" s="34">
-        <v>35.4</v>
+        <v>35.5</v>
       </c>
       <c r="E10" s="34">
-        <v>33.5</v>
+        <v>33.700000000000003</v>
       </c>
       <c r="F10" s="34">
-        <v>34.700000000000003</v>
+        <v>34.6</v>
       </c>
       <c r="G10" s="34">
         <v>35.200000000000003</v>
@@ -6221,22 +6238,22 @@
         <v>21</v>
       </c>
       <c r="B11" s="34">
-        <v>32</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="C11" s="34">
-        <v>30.8</v>
+        <v>32.5</v>
       </c>
       <c r="D11" s="34">
-        <v>36.4</v>
+        <v>33.700000000000003</v>
       </c>
       <c r="E11" s="34">
-        <v>28.1</v>
+        <v>29.4</v>
       </c>
       <c r="F11" s="34">
-        <v>28.4</v>
+        <v>31.7</v>
       </c>
       <c r="G11" s="34">
-        <v>27.7</v>
+        <v>28.9</v>
       </c>
       <c r="H11" s="34">
         <v>24.8</v>
@@ -6250,22 +6267,22 @@
         <v>40</v>
       </c>
       <c r="C12" s="34">
-        <v>39.299999999999997</v>
+        <v>40.200000000000003</v>
       </c>
       <c r="D12" s="34">
-        <v>36.6</v>
+        <v>35.200000000000003</v>
       </c>
       <c r="E12" s="34">
-        <v>42.3</v>
+        <v>45.8</v>
       </c>
       <c r="F12" s="34">
-        <v>51.8</v>
+        <v>51.1</v>
       </c>
       <c r="G12" s="34">
-        <v>41.3</v>
+        <v>40.1</v>
       </c>
       <c r="H12" s="34">
-        <v>44.4</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -6276,22 +6293,22 @@
         <v>36.700000000000003</v>
       </c>
       <c r="C13" s="34">
-        <v>35.1</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="D13" s="34">
-        <v>39.9</v>
+        <v>39.700000000000003</v>
       </c>
       <c r="E13" s="34">
-        <v>41.1</v>
+        <v>38.4</v>
       </c>
       <c r="F13" s="34">
-        <v>37.5</v>
+        <v>35.200000000000003</v>
       </c>
       <c r="G13" s="34">
-        <v>32.5</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="H13" s="34">
-        <v>27.6</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -6299,25 +6316,25 @@
         <v>24</v>
       </c>
       <c r="B14" s="34">
-        <v>32.4</v>
+        <v>32.5</v>
       </c>
       <c r="C14" s="34">
-        <v>35.299999999999997</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="D14" s="34">
-        <v>30.4</v>
+        <v>31.2</v>
       </c>
       <c r="E14" s="34">
-        <v>27.9</v>
+        <v>28.1</v>
       </c>
       <c r="F14" s="34">
-        <v>27.7</v>
+        <v>28.9</v>
       </c>
       <c r="G14" s="34">
-        <v>33</v>
+        <v>33.4</v>
       </c>
       <c r="H14" s="34">
-        <v>30.4</v>
+        <v>29.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
"Actualizo comex y res fiscal -julio26. Emae Jun26"
</commit_message>
<xml_diff>
--- a/bases/indicadores.xlsx
+++ b/bases/indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\indeco\indeco\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB87912E-6371-4079-B50D-2DC51D993134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FACEEEDE-376D-4EDF-AC87-664AD815FF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="500" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPC-Seriemensual" sheetId="1" r:id="rId1"/>
@@ -996,17 +996,17 @@
     </xf>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="11" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -3541,7 +3541,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29.140625" customWidth="1"/>
@@ -3571,10 +3571,10 @@
         <v>134.74645041349706</v>
       </c>
       <c r="C2" s="36">
-        <v>147.90289172962787</v>
+        <v>147.90228794480254</v>
       </c>
       <c r="D2" s="36">
-        <v>147.06041914463302</v>
+        <v>147.05884131449477</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -3585,10 +3585,10 @@
         <v>134.23236103862521</v>
       </c>
       <c r="C3" s="36">
-        <v>146.87869250897225</v>
+        <v>146.86931898530125</v>
       </c>
       <c r="D3" s="36">
-        <v>146.48010453906795</v>
+        <v>146.48052100056762</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3599,10 +3599,10 @@
         <v>150.0878942366954</v>
       </c>
       <c r="C4" s="36">
-        <v>145.96567107119392</v>
+        <v>145.97749833883569</v>
       </c>
       <c r="D4" s="36">
-        <v>145.92974952061303</v>
+        <v>145.93166785307798</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3613,10 +3613,10 @@
         <v>153.25067436662908</v>
       </c>
       <c r="C5" s="36">
-        <v>144.71513795719116</v>
+        <v>144.70807119513321</v>
       </c>
       <c r="D5" s="36">
-        <v>145.4474203087604</v>
+        <v>145.44994793136155</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3627,10 +3627,10 @@
         <v>163.51360808690507</v>
       </c>
       <c r="C6" s="36">
-        <v>144.57674809588957</v>
+        <v>144.62478893925029</v>
       </c>
       <c r="D6" s="36">
-        <v>145.06163776867783</v>
+        <v>145.0638187966789</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3641,10 +3641,10 @@
         <v>153.66209524099784</v>
       </c>
       <c r="C7" s="36">
-        <v>144.37905393460173</v>
+        <v>144.40593395794969</v>
       </c>
       <c r="D7" s="36">
-        <v>144.79388930864746</v>
+        <v>144.795120666016</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3655,10 +3655,10 @@
         <v>143.73110098180126</v>
       </c>
       <c r="C8" s="36">
-        <v>144.58278827113989</v>
+        <v>144.56971196835462</v>
       </c>
       <c r="D8" s="36">
-        <v>144.65415992044788</v>
+        <v>144.65413849762604</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3669,10 +3669,10 @@
         <v>143.6741026486049</v>
       </c>
       <c r="C9" s="36">
-        <v>145.65089775486558</v>
+        <v>145.62439225744868</v>
       </c>
       <c r="D9" s="36">
-        <v>144.64490844807989</v>
+        <v>144.6438070847106</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3683,10 +3683,10 @@
         <v>142.00773744282046</v>
       </c>
       <c r="C10" s="36">
-        <v>145.01879848640064</v>
+        <v>145.01346587648703</v>
       </c>
       <c r="D10" s="36">
-        <v>144.76441821007117</v>
+        <v>144.76293538516143</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3697,10 +3697,10 @@
         <v>141.13686329808141</v>
       </c>
       <c r="C11" s="36">
-        <v>145.15354369792067</v>
+        <v>145.13693619452528</v>
       </c>
       <c r="D11" s="36">
-        <v>145.00423578331799</v>
+        <v>145.00324154007509</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3711,10 +3711,10 @@
         <v>144.93832064073018</v>
       </c>
       <c r="C12" s="36">
-        <v>145.78824914209579</v>
+        <v>145.78761585131699</v>
       </c>
       <c r="D12" s="36">
-        <v>145.3496394533513</v>
+        <v>145.34973845890553</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3725,10 +3725,10 @@
         <v>142.59014516031914</v>
       </c>
       <c r="C13" s="36">
-        <v>146.95888147081035</v>
+        <v>146.95133257211731</v>
       </c>
       <c r="D13" s="36">
-        <v>145.78841177630977</v>
+        <v>145.7898359883429</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3736,13 +3736,13 @@
         <v>42736</v>
       </c>
       <c r="B14" s="17">
-        <v>136.63265948316197</v>
+        <v>136.63265948316212</v>
       </c>
       <c r="C14" s="36">
-        <v>147.08627326950506</v>
+        <v>147.10315056347034</v>
       </c>
       <c r="D14" s="36">
-        <v>146.3065815191809</v>
+        <v>146.30916445024215</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3750,13 +3750,13 @@
         <v>42767</v>
       </c>
       <c r="B15" s="17">
-        <v>132.15851633982263</v>
+        <v>132.15851633982274</v>
       </c>
       <c r="C15" s="36">
-        <v>146.81395008705243</v>
+        <v>146.83985693267059</v>
       </c>
       <c r="D15" s="36">
-        <v>146.88669274545626</v>
+        <v>146.88994972865572</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3764,13 +3764,13 @@
         <v>42795</v>
       </c>
       <c r="B16" s="17">
-        <v>152.62095855905721</v>
+        <v>152.6209585590573</v>
       </c>
       <c r="C16" s="36">
-        <v>147.64480930022708</v>
+        <v>147.67109458512658</v>
       </c>
       <c r="D16" s="36">
-        <v>147.51139127886813</v>
+        <v>147.51460995597441</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3778,13 +3778,13 @@
         <v>42826</v>
       </c>
       <c r="B17" s="17">
-        <v>151.94634480448727</v>
+        <v>151.94634480448738</v>
       </c>
       <c r="C17" s="36">
-        <v>147.67329037105645</v>
+        <v>147.66807814570066</v>
       </c>
       <c r="D17" s="36">
-        <v>148.16108451834779</v>
+        <v>148.16341792098223</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3792,13 +3792,13 @@
         <v>42856</v>
       </c>
       <c r="B18" s="17">
-        <v>168.38920946936767</v>
+        <v>168.38920946936781</v>
       </c>
       <c r="C18" s="36">
-        <v>148.67448204725812</v>
+        <v>148.68211497089837</v>
       </c>
       <c r="D18" s="36">
-        <v>148.80990363486927</v>
+        <v>148.81064989468004</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3806,13 +3806,13 @@
         <v>42887</v>
       </c>
       <c r="B19" s="17">
-        <v>161.0356854694522</v>
+        <v>161.03568546945232</v>
       </c>
       <c r="C19" s="36">
-        <v>150.27199303046453</v>
+        <v>150.26860128620675</v>
       </c>
       <c r="D19" s="36">
-        <v>149.42763427653395</v>
+        <v>149.4263530717264</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3820,13 +3820,13 @@
         <v>42917</v>
       </c>
       <c r="B20" s="17">
-        <v>150.3060501239199</v>
+        <v>150.30605012391999</v>
       </c>
       <c r="C20" s="36">
-        <v>150.46351778388978</v>
+        <v>150.45415651887882</v>
       </c>
       <c r="D20" s="36">
-        <v>149.97952638836915</v>
+        <v>149.97613834878806</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3834,13 +3834,13 @@
         <v>42948</v>
       </c>
       <c r="B21" s="17">
-        <v>149.25534277384099</v>
+        <v>149.25534277384111</v>
       </c>
       <c r="C21" s="36">
-        <v>150.39057754222844</v>
+        <v>150.39131093623385</v>
       </c>
       <c r="D21" s="36">
-        <v>150.42776468517482</v>
+        <v>150.42258328427556</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3848,13 +3848,13 @@
         <v>42979</v>
       </c>
       <c r="B22" s="17">
-        <v>146.38655965775374</v>
+        <v>146.38655965775385</v>
       </c>
       <c r="C22" s="36">
-        <v>151.21749422435974</v>
+        <v>151.21376013876639</v>
       </c>
       <c r="D22" s="36">
-        <v>150.73346509955473</v>
+        <v>150.72715127054451</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3862,13 +3862,13 @@
         <v>43009</v>
       </c>
       <c r="B23" s="17">
-        <v>149.38594966601445</v>
+        <v>149.38594966601454</v>
       </c>
       <c r="C23" s="36">
-        <v>151.71275927869797</v>
+        <v>151.69328476469425</v>
       </c>
       <c r="D23" s="36">
-        <v>150.8656502006244</v>
+        <v>150.85914085952476</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3876,13 +3876,13 @@
         <v>43040</v>
       </c>
       <c r="B24" s="17">
-        <v>151.92604285202682</v>
+        <v>151.92604285202697</v>
       </c>
       <c r="C24" s="36">
-        <v>152.63221481224414</v>
+        <v>152.61081737406121</v>
       </c>
       <c r="D24" s="36">
-        <v>150.79907205919287</v>
+        <v>150.79269365352215</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3890,13 +3890,13 @@
         <v>43070</v>
       </c>
       <c r="B25" s="17">
-        <v>146.78338490922437</v>
+        <v>146.78338490922451</v>
       </c>
       <c r="C25" s="36">
-        <v>152.24534294207206</v>
+        <v>152.23047843206538</v>
       </c>
       <c r="D25" s="36">
-        <v>150.52073983983868</v>
+        <v>150.51491752532093</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3904,13 +3904,13 @@
         <v>43101</v>
       </c>
       <c r="B26" s="17">
-        <v>142.74091260617209</v>
+        <v>142.74091260617223</v>
       </c>
       <c r="C26" s="36">
-        <v>150.97750196780996</v>
+        <v>150.97432403194165</v>
       </c>
       <c r="D26" s="36">
-        <v>150.03524574481486</v>
+        <v>150.03080673561695</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3918,13 +3918,13 @@
         <v>43132</v>
       </c>
       <c r="B27" s="17">
-        <v>138.81804035165729</v>
+        <v>138.81804035165743</v>
       </c>
       <c r="C27" s="36">
-        <v>152.19147467174869</v>
+        <v>152.21496614021012</v>
       </c>
       <c r="D27" s="36">
-        <v>149.36435462115523</v>
+        <v>149.3624332264886</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3932,13 +3932,13 @@
         <v>43160</v>
       </c>
       <c r="B28" s="17">
-        <v>155.85731953576962</v>
+        <v>155.85731953576973</v>
       </c>
       <c r="C28" s="36">
-        <v>151.5287558105469</v>
+        <v>151.54850660607454</v>
       </c>
       <c r="D28" s="36">
-        <v>148.54649497358778</v>
+        <v>148.54828673930285</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3946,13 +3946,13 @@
         <v>43191</v>
       </c>
       <c r="B29" s="17">
-        <v>151.52454398394329</v>
+        <v>151.52454398394343</v>
       </c>
       <c r="C29" s="36">
-        <v>146.79265782593984</v>
+        <v>146.80644414143845</v>
       </c>
       <c r="D29" s="36">
-        <v>147.62845357197196</v>
+        <v>147.63523092998457</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3960,13 +3960,13 @@
         <v>43221</v>
       </c>
       <c r="B30" s="17">
-        <v>159.56669237791655</v>
+        <v>159.5666923779167</v>
       </c>
       <c r="C30" s="36">
-        <v>144.56308740741699</v>
+        <v>144.58761676999234</v>
       </c>
       <c r="D30" s="36">
-        <v>146.66554660531108</v>
+        <v>146.67848734799458</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3974,13 +3974,13 @@
         <v>43252</v>
       </c>
       <c r="B31" s="17">
-        <v>151.1257632334551</v>
+        <v>151.12576323345522</v>
       </c>
       <c r="C31" s="36">
-        <v>143.25908288947755</v>
+        <v>143.27264246575626</v>
       </c>
       <c r="D31" s="36">
-        <v>145.71598087635073</v>
+        <v>145.73584383725961</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -3988,13 +3988,13 @@
         <v>43282</v>
       </c>
       <c r="B32" s="17">
-        <v>145.96352443000447</v>
+        <v>145.96352443000461</v>
       </c>
       <c r="C32" s="36">
-        <v>143.57920900072801</v>
+        <v>143.59456149815151</v>
       </c>
       <c r="D32" s="36">
-        <v>144.83291842509811</v>
+        <v>144.85986468982435</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -4002,13 +4002,13 @@
         <v>43313</v>
       </c>
       <c r="B33" s="17">
-        <v>146.76596003413957</v>
+        <v>146.76596003413968</v>
       </c>
       <c r="C33" s="36">
-        <v>146.53723087700519</v>
+        <v>146.54647689029972</v>
       </c>
       <c r="D33" s="36">
-        <v>144.06472199992993</v>
+        <v>144.09839390385193</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -4016,13 +4016,13 @@
         <v>43344</v>
       </c>
       <c r="B34" s="17">
-        <v>137.74656971864789</v>
+        <v>137.746569718648</v>
       </c>
       <c r="C34" s="36">
-        <v>143.1322414333213</v>
+        <v>143.13178589235872</v>
       </c>
       <c r="D34" s="36">
-        <v>143.44595234523834</v>
+        <v>143.48526623050319</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -4030,13 +4030,13 @@
         <v>43374</v>
       </c>
       <c r="B35" s="17">
-        <v>142.8432759845675</v>
+        <v>142.84327598456761</v>
       </c>
       <c r="C35" s="36">
-        <v>143.59558509549367</v>
+        <v>143.55929161700038</v>
       </c>
       <c r="D35" s="36">
-        <v>142.99316083040782</v>
+        <v>143.03626587801961</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -4044,13 +4044,13 @@
         <v>43405</v>
       </c>
       <c r="B36" s="17">
-        <v>140.59240732533553</v>
+        <v>140.59240732533567</v>
       </c>
       <c r="C36" s="36">
-        <v>141.66615037738163</v>
+        <v>141.61755948831191</v>
       </c>
       <c r="D36" s="36">
-        <v>142.70789004237591</v>
+        <v>142.75240421627376</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -4058,13 +4058,13 @@
         <v>43435</v>
       </c>
       <c r="B37" s="17">
-        <v>136.25161596905625</v>
+        <v>136.25161596905636</v>
       </c>
       <c r="C37" s="36">
-        <v>141.97364875950399</v>
+        <v>141.94245053564785</v>
       </c>
       <c r="D37" s="36">
-        <v>142.57713267970016</v>
+        <v>142.62030929088488</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -4072,13 +4072,13 @@
         <v>43466</v>
       </c>
       <c r="B38" s="17">
-        <v>134.53623985669569</v>
+        <v>134.5362398566958</v>
       </c>
       <c r="C38" s="36">
-        <v>141.39772924062791</v>
+        <v>141.42634449054745</v>
       </c>
       <c r="D38" s="36">
-        <v>142.57245366664446</v>
+        <v>142.61157661917866</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4086,13 +4086,13 @@
         <v>43497</v>
       </c>
       <c r="B39" s="17">
-        <v>132.2678886127365</v>
+        <v>132.26788861273661</v>
       </c>
       <c r="C39" s="36">
-        <v>143.65890168370726</v>
+        <v>143.72785091696355</v>
       </c>
       <c r="D39" s="36">
-        <v>142.6556943490732</v>
+        <v>142.68844745241501</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4100,13 +4100,13 @@
         <v>43525</v>
       </c>
       <c r="B40" s="17">
-        <v>144.96325495574902</v>
+        <v>144.96325495574916</v>
       </c>
       <c r="C40" s="36">
-        <v>142.25994004126758</v>
+        <v>142.33640443007181</v>
       </c>
       <c r="D40" s="36">
-        <v>142.78455876892951</v>
+        <v>142.80929312695918</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4114,13 +4114,13 @@
         <v>43556</v>
       </c>
       <c r="B41" s="17">
-        <v>149.91622140352257</v>
+        <v>149.91622140352271</v>
       </c>
       <c r="C41" s="36">
-        <v>142.60578725333434</v>
+        <v>142.63217066739119</v>
       </c>
       <c r="D41" s="36">
-        <v>142.91282858001958</v>
+        <v>142.92899490596105</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4128,13 +4128,13 @@
         <v>43586</v>
       </c>
       <c r="B42" s="17">
-        <v>164.13569907592026</v>
+        <v>164.1356990759204</v>
       </c>
       <c r="C42" s="36">
-        <v>144.83824997198266</v>
+        <v>144.85176283668281</v>
       </c>
       <c r="D42" s="36">
-        <v>142.99820287071864</v>
+        <v>143.00611711109545</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4142,13 +4142,13 @@
         <v>43617</v>
       </c>
       <c r="B43" s="17">
-        <v>150.85897174113111</v>
+        <v>150.85897174113128</v>
       </c>
       <c r="C43" s="36">
-        <v>144.03378129578405</v>
+        <v>144.04490409998212</v>
       </c>
       <c r="D43" s="36">
-        <v>143.00474250423559</v>
+        <v>143.00568802760029</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4156,13 +4156,13 @@
         <v>43647</v>
       </c>
       <c r="B44" s="17">
-        <v>146.7770296400702</v>
+        <v>146.77702964007034</v>
       </c>
       <c r="C44" s="36">
-        <v>145.83568077855986</v>
+        <v>145.82192292861072</v>
       </c>
       <c r="D44" s="36">
-        <v>142.90491277618392</v>
+        <v>142.90114762770563</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4170,13 +4170,13 @@
         <v>43678</v>
       </c>
       <c r="B45" s="17">
-        <v>141.27693468084021</v>
+        <v>141.27693468084036</v>
       </c>
       <c r="C45" s="36">
-        <v>144.7905932858464</v>
+        <v>144.77374425103372</v>
       </c>
       <c r="D45" s="36">
-        <v>142.68208431588255</v>
+        <v>142.67645193678277</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4184,13 +4184,13 @@
         <v>43709</v>
       </c>
       <c r="B46" s="17">
-        <v>134.87706647993639</v>
+        <v>134.87706647993653</v>
       </c>
       <c r="C46" s="36">
-        <v>140.55731399665021</v>
+        <v>140.52870612823389</v>
       </c>
       <c r="D46" s="36">
-        <v>142.33147985322461</v>
+        <v>142.32683422868618</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -4198,13 +4198,13 @@
         <v>43739</v>
       </c>
       <c r="B47" s="17">
-        <v>141.63933661701367</v>
+        <v>141.63933661701381</v>
       </c>
       <c r="C47" s="36">
-        <v>143.79727407340053</v>
+        <v>143.75161347511875</v>
       </c>
       <c r="D47" s="36">
-        <v>141.85956089737351</v>
+        <v>141.85824620693592</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -4212,13 +4212,13 @@
         <v>43770</v>
       </c>
       <c r="B48" s="17">
-        <v>137.77182966933134</v>
+        <v>137.77182966933145</v>
       </c>
       <c r="C48" s="36">
-        <v>140.88368953714604</v>
+        <v>140.81021564190533</v>
       </c>
       <c r="D48" s="36">
-        <v>141.28341184211027</v>
+        <v>141.28726807080514</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -4226,13 +4226,13 @@
         <v>43800</v>
       </c>
       <c r="B49" s="17">
-        <v>135.76515452763488</v>
+        <v>135.76515452763502</v>
       </c>
       <c r="C49" s="36">
-        <v>140.12668665666166</v>
+        <v>140.07998791005343</v>
       </c>
       <c r="D49" s="36">
-        <v>140.6304263163494</v>
+        <v>140.64135515964173</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -4240,13 +4240,13 @@
         <v>43831</v>
       </c>
       <c r="B50" s="17">
-        <v>133.89108608957227</v>
+        <v>133.89108608957241</v>
       </c>
       <c r="C50" s="36">
-        <v>140.93017714538223</v>
+        <v>140.92554601700547</v>
       </c>
       <c r="D50" s="36">
-        <v>139.93237577469208</v>
+        <v>139.9508919074238</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -4254,13 +4254,13 @@
         <v>43862</v>
       </c>
       <c r="B51" s="17">
-        <v>128.97363874659808</v>
+        <v>128.97363874659823</v>
       </c>
       <c r="C51" s="36">
-        <v>139.54976127560565</v>
+        <v>139.58431341498277</v>
       </c>
       <c r="D51" s="36">
-        <v>139.22448358107718</v>
+        <v>139.24950149986981</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -4268,13 +4268,13 @@
         <v>43891</v>
       </c>
       <c r="B52" s="17">
-        <v>128.21106074025653</v>
+        <v>128.21106074025667</v>
       </c>
       <c r="C52" s="36">
-        <v>125.96024771330764</v>
+        <v>126.02034936546131</v>
       </c>
       <c r="D52" s="36">
-        <v>138.54271042734956</v>
+        <v>138.57159350028013</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -4282,13 +4282,13 @@
         <v>43922</v>
       </c>
       <c r="B53" s="17">
-        <v>113.29503444580143</v>
+        <v>113.29503444580156</v>
       </c>
       <c r="C53" s="36">
-        <v>105.99227909223607</v>
+        <v>106.05639981841499</v>
       </c>
       <c r="D53" s="36">
-        <v>137.92242935265389</v>
+        <v>137.95177444201141</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -4296,13 +4296,13 @@
         <v>43952</v>
       </c>
       <c r="B54" s="17">
-        <v>131.02956919734902</v>
+        <v>131.02956919734916</v>
       </c>
       <c r="C54" s="36">
-        <v>117.20962176752099</v>
+        <v>117.26625454147219</v>
       </c>
       <c r="D54" s="36">
-        <v>137.39712668302374</v>
+        <v>137.42336915504214</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -4310,13 +4310,13 @@
         <v>43983</v>
       </c>
       <c r="B55" s="17">
-        <v>132.52196526648763</v>
+        <v>132.52196526648777</v>
       </c>
       <c r="C55" s="36">
-        <v>124.3449729358869</v>
+        <v>124.35972004671306</v>
       </c>
       <c r="D55" s="36">
-        <v>136.99165283445276</v>
+        <v>137.01191055029554</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -4324,13 +4324,13 @@
         <v>44013</v>
       </c>
       <c r="B56" s="17">
-        <v>127.46368946979391</v>
+        <v>127.46368946979405</v>
       </c>
       <c r="C56" s="36">
-        <v>126.15819490838572</v>
+        <v>126.14854476042942</v>
       </c>
       <c r="D56" s="36">
-        <v>136.72209103841908</v>
+        <v>136.73449987129194</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -4338,13 +4338,13 @@
         <v>44044</v>
       </c>
       <c r="B57" s="17">
-        <v>125.18389375984641</v>
+        <v>125.18389375984655</v>
       </c>
       <c r="C57" s="36">
-        <v>128.84415787500245</v>
+        <v>128.83372679932165</v>
       </c>
       <c r="D57" s="36">
-        <v>136.59679330726365</v>
+        <v>136.60088049432886</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -4352,13 +4352,13 @@
         <v>44075</v>
       </c>
       <c r="B58" s="17">
-        <v>127.1750760933527</v>
+        <v>127.17507609335286</v>
       </c>
       <c r="C58" s="36">
-        <v>130.79654793201593</v>
+        <v>130.76173160851343</v>
       </c>
       <c r="D58" s="36">
-        <v>136.61536603928135</v>
+        <v>136.61209476684212</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -4366,13 +4366,13 @@
         <v>44105</v>
       </c>
       <c r="B59" s="17">
-        <v>131.34550189452784</v>
+        <v>131.34550189452798</v>
       </c>
       <c r="C59" s="36">
-        <v>133.39866145682996</v>
+        <v>133.35013477038626</v>
       </c>
       <c r="D59" s="36">
-        <v>136.77112663605229</v>
+        <v>136.76269563502817</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -4380,13 +4380,13 @@
         <v>44136</v>
       </c>
       <c r="B60" s="17">
-        <v>132.06865525299659</v>
+        <v>132.06865525299673</v>
       </c>
       <c r="C60" s="36">
-        <v>134.87132101698435</v>
+        <v>134.79827594761082</v>
       </c>
       <c r="D60" s="36">
-        <v>137.05076753412618</v>
+        <v>137.03990402352059</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -4394,13 +4394,13 @@
         <v>44166</v>
       </c>
       <c r="B61" s="17">
-        <v>133.85436559460604</v>
+        <v>133.85436559460618</v>
       </c>
       <c r="C61" s="36">
-        <v>136.95759393151968</v>
+        <v>136.90853992586401</v>
       </c>
       <c r="D61" s="36">
-        <v>137.43790389556929</v>
+        <v>137.42718773237806</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -4408,13 +4408,13 @@
         <v>44197</v>
       </c>
       <c r="B62" s="17">
-        <v>131.52153739731881</v>
+        <v>131.52153739731895</v>
       </c>
       <c r="C62" s="36">
-        <v>139.84976777699663</v>
+        <v>139.85869931136128</v>
       </c>
       <c r="D62" s="36">
-        <v>137.91642405398932</v>
+        <v>137.90773055216602</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -4422,13 +4422,13 @@
         <v>44228</v>
       </c>
       <c r="B63" s="17">
-        <v>126.23926696836405</v>
+        <v>126.23926696836419</v>
       </c>
       <c r="C63" s="36">
-        <v>138.24267956970155</v>
+        <v>138.27778724368201</v>
       </c>
       <c r="D63" s="36">
-        <v>138.47503425796688</v>
+        <v>138.46922791775205</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -4436,13 +4436,13 @@
         <v>44256</v>
       </c>
       <c r="B64" s="17">
-        <v>145.95690010364706</v>
+        <v>145.9569001036472</v>
       </c>
       <c r="C64" s="36">
-        <v>140.89139329828407</v>
+        <v>140.94283751059339</v>
       </c>
       <c r="D64" s="36">
-        <v>139.10476344710142</v>
+        <v>139.1015222090131</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -4450,13 +4450,13 @@
         <v>44287</v>
       </c>
       <c r="B65" s="17">
-        <v>147.28084401875944</v>
+        <v>147.28084401875961</v>
       </c>
       <c r="C65" s="36">
-        <v>139.3115864823003</v>
+        <v>139.42174873428777</v>
       </c>
       <c r="D65" s="36">
-        <v>139.80273184864561</v>
+        <v>139.80063611380118</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -4464,13 +4464,13 @@
         <v>44317</v>
       </c>
       <c r="B66" s="17">
-        <v>151.16932233874812</v>
+        <v>151.16932233874826</v>
       </c>
       <c r="C66" s="36">
-        <v>138.85916439674222</v>
+        <v>138.92350185503292</v>
       </c>
       <c r="D66" s="36">
-        <v>140.56795196459669</v>
+        <v>140.56490592146289</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -4478,13 +4478,13 @@
         <v>44348</v>
       </c>
       <c r="B67" s="17">
-        <v>148.97961710841227</v>
+        <v>148.97961710841247</v>
       </c>
       <c r="C67" s="36">
-        <v>141.52410726823069</v>
+        <v>141.54410781899168</v>
       </c>
       <c r="D67" s="36">
-        <v>141.39767517306643</v>
+        <v>141.39166062844572</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -4492,13 +4492,13 @@
         <v>44378</v>
       </c>
       <c r="B68" s="17">
-        <v>142.42591306035797</v>
+        <v>142.42591306035814</v>
       </c>
       <c r="C68" s="36">
-        <v>141.37916581108891</v>
+        <v>141.35346521561027</v>
       </c>
       <c r="D68" s="36">
-        <v>142.29185441448868</v>
+        <v>142.28165460957507</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -4506,13 +4506,13 @@
         <v>44409</v>
       </c>
       <c r="B69" s="17">
-        <v>140.97494072777721</v>
+        <v>140.97494072777735</v>
       </c>
       <c r="C69" s="36">
-        <v>143.31590238415345</v>
+        <v>143.29318922352883</v>
       </c>
       <c r="D69" s="36">
-        <v>143.24949089718777</v>
+        <v>143.23502605857846</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -4520,13 +4520,13 @@
         <v>44440</v>
       </c>
       <c r="B70" s="17">
-        <v>141.29608909028403</v>
+        <v>141.29608909028411</v>
       </c>
       <c r="C70" s="36">
-        <v>144.17734645091775</v>
+        <v>144.12507279457796</v>
       </c>
       <c r="D70" s="36">
-        <v>144.263236099306</v>
+        <v>144.24592259774104</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -4534,13 +4534,13 @@
         <v>44470</v>
       </c>
       <c r="B71" s="17">
-        <v>139.51475869967888</v>
+        <v>139.51475869967891</v>
       </c>
       <c r="C71" s="36">
-        <v>143.35586178313645</v>
+        <v>143.32018242264803</v>
       </c>
       <c r="D71" s="36">
-        <v>145.32006310709181</v>
+        <v>145.30255603451579</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -4548,13 +4548,13 @@
         <v>44501</v>
       </c>
       <c r="B72" s="17">
-        <v>143.75187761888847</v>
+        <v>143.75187761888859</v>
       </c>
       <c r="C72" s="36">
-        <v>145.71356699110419</v>
+        <v>145.6282008947839</v>
       </c>
       <c r="D72" s="36">
-        <v>146.39501768319394</v>
+        <v>146.38014447859447</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -4562,13 +4562,13 @@
         <v>44531</v>
       </c>
       <c r="B73" s="17">
-        <v>147.22987831813373</v>
+        <v>147.2298783181341</v>
       </c>
       <c r="C73" s="36">
-        <v>149.72040378936583</v>
+        <v>149.65215293879575</v>
       </c>
       <c r="D73" s="36">
-        <v>147.4511533036428</v>
+        <v>147.44080755534532</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -4576,13 +4576,13 @@
         <v>44562</v>
       </c>
       <c r="B74" s="17">
-        <v>139.637961612281</v>
+        <v>139.6379616122818</v>
       </c>
       <c r="C74" s="36">
-        <v>148.52454567203267</v>
+        <v>148.50300074015578</v>
       </c>
       <c r="D74" s="36">
-        <v>148.44590874633826</v>
+        <v>148.4404600410748</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -4590,13 +4590,13 @@
         <v>44593</v>
       </c>
       <c r="B75" s="17">
-        <v>137.84951352507554</v>
+        <v>137.84951352507593</v>
       </c>
       <c r="C75" s="36">
-        <v>150.70922638827258</v>
+        <v>150.71219600987763</v>
       </c>
       <c r="D75" s="36">
-        <v>149.33437192086149</v>
+        <v>149.33271238306372</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -4604,13 +4604,13 @@
         <v>44621</v>
       </c>
       <c r="B76" s="17">
-        <v>153.9308507942531</v>
+        <v>153.93085079425231</v>
       </c>
       <c r="C76" s="36">
-        <v>150.34672378542243</v>
+        <v>150.36649250775957</v>
       </c>
       <c r="D76" s="36">
-        <v>150.07876932527918</v>
+        <v>150.07881778771394</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -4618,13 +4618,13 @@
         <v>44652</v>
       </c>
       <c r="B77" s="17">
-        <v>157.66169217344674</v>
+        <v>157.66169217344401</v>
       </c>
       <c r="C77" s="36">
-        <v>152.09770494152977</v>
+        <v>152.26721240793535</v>
       </c>
       <c r="D77" s="36">
-        <v>150.65168869920231</v>
+        <v>150.651089556285</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -4632,13 +4632,13 @@
         <v>44682</v>
       </c>
       <c r="B78" s="17">
-        <v>164.68936311408393</v>
+        <v>164.68936311408291</v>
       </c>
       <c r="C78" s="36">
-        <v>152.12668174406087</v>
+        <v>152.22665108010588</v>
       </c>
       <c r="D78" s="36">
-        <v>151.03686923587975</v>
+        <v>151.03332176495991</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -4646,13 +4646,13 @@
         <v>44713</v>
       </c>
       <c r="B79" s="17">
-        <v>161.4548342812127</v>
+        <v>161.45483428121702</v>
       </c>
       <c r="C79" s="36">
-        <v>154.30297450812731</v>
+        <v>154.32065688488396</v>
       </c>
       <c r="D79" s="36">
-        <v>151.2301275132958</v>
+        <v>151.22201815253945</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -4660,13 +4660,13 @@
         <v>44743</v>
       </c>
       <c r="B80" s="17">
-        <v>152.44538743586068</v>
+        <v>152.4453874358741</v>
       </c>
       <c r="C80" s="36">
-        <v>152.5581973587675</v>
+        <v>152.52038638813951</v>
       </c>
       <c r="D80" s="36">
-        <v>151.24393962017717</v>
+        <v>151.23059877801032</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4674,13 +4674,13 @@
         <v>44774</v>
       </c>
       <c r="B81" s="17">
-        <v>151.46573891606155</v>
+        <v>151.46573891606729</v>
       </c>
       <c r="C81" s="36">
-        <v>151.72301499095741</v>
+        <v>151.65878749519123</v>
       </c>
       <c r="D81" s="36">
-        <v>151.10403481382463</v>
+        <v>151.08612942118208</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4688,13 +4688,13 @@
         <v>44805</v>
       </c>
       <c r="B82" s="17">
-        <v>149.17434970528168</v>
+        <v>149.17434970526307</v>
       </c>
       <c r="C82" s="36">
-        <v>150.78775112517866</v>
+        <v>150.70875085496451</v>
       </c>
       <c r="D82" s="36">
-        <v>150.84526135445358</v>
+        <v>150.82457670878878</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4702,13 +4702,13 @@
         <v>44835</v>
       </c>
       <c r="B83" s="17">
-        <v>146.55439616170329</v>
+        <v>146.55439616164352</v>
       </c>
       <c r="C83" s="36">
-        <v>149.08575921389939</v>
+        <v>149.06554743419156</v>
       </c>
       <c r="D83" s="36">
-        <v>150.50645589049475</v>
+        <v>150.48557863738</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4716,13 +4716,13 @@
         <v>44866</v>
       </c>
       <c r="B84" s="17">
-        <v>148.03049492952468</v>
+        <v>148.03049492949961</v>
       </c>
       <c r="C84" s="36">
-        <v>148.327566132046</v>
+        <v>148.29221401437047</v>
       </c>
       <c r="D84" s="36">
-        <v>150.12486758078268</v>
+        <v>150.10659984539819</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -4730,13 +4730,13 @@
         <v>44896</v>
       </c>
       <c r="B85" s="17">
-        <v>146.18080633796006</v>
+        <v>146.18080633804541</v>
       </c>
       <c r="C85" s="36">
-        <v>148.48524371131373</v>
+        <v>148.43349371359295</v>
       </c>
       <c r="D85" s="36">
-        <v>149.73336917647515</v>
+        <v>149.72034836077549</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -4744,13 +4744,13 @@
         <v>44927</v>
       </c>
       <c r="B86" s="17">
-        <v>143.03462349487495</v>
+        <v>143.03462349514643</v>
       </c>
       <c r="C86" s="36">
-        <v>149.95772966081552</v>
+        <v>149.92114342631578</v>
       </c>
       <c r="D86" s="36">
-        <v>149.35503971635941</v>
+        <v>149.34922137615646</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4758,13 +4758,13 @@
         <v>44958</v>
       </c>
       <c r="B87" s="17">
-        <v>137.26646276476467</v>
+        <v>137.26646276487918</v>
       </c>
       <c r="C87" s="36">
-        <v>150.15642424124019</v>
+        <v>150.10029003096659</v>
       </c>
       <c r="D87" s="36">
-        <v>148.99990522247347</v>
+        <v>149.00211604628635</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -4772,13 +4772,13 @@
         <v>44986</v>
       </c>
       <c r="B88" s="17">
-        <v>155.06501366898644</v>
+        <v>155.06501366860087</v>
       </c>
       <c r="C88" s="36">
-        <v>150.7559630178034</v>
+        <v>150.75256289433395</v>
       </c>
       <c r="D88" s="36">
-        <v>148.66373870024944</v>
+        <v>148.67363087150412</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -4786,13 +4786,13 @@
         <v>45017</v>
       </c>
       <c r="B89" s="17">
-        <v>150.05952685125044</v>
+        <v>150.05952685002168</v>
       </c>
       <c r="C89" s="36">
-        <v>147.35748735405127</v>
+        <v>147.53224583499846</v>
       </c>
       <c r="D89" s="36">
-        <v>148.33221429847092</v>
+        <v>148.34803699709209</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4800,13 +4800,13 @@
         <v>45047</v>
       </c>
       <c r="B90" s="17">
-        <v>153.81085419260503</v>
+        <v>153.81085419208719</v>
       </c>
       <c r="C90" s="36">
-        <v>145.5527260528016</v>
+        <v>145.62328742845165</v>
       </c>
       <c r="D90" s="36">
-        <v>147.98297145239175</v>
+        <v>148.0018911303971</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4814,13 +4814,13 @@
         <v>45078</v>
       </c>
       <c r="B91" s="17">
-        <v>152.59547604809092</v>
+        <v>152.59547604983808</v>
       </c>
       <c r="C91" s="36">
-        <v>146.06326749676077</v>
+        <v>146.08926594642224</v>
       </c>
       <c r="D91" s="36">
-        <v>147.59607526377985</v>
+        <v>147.61471669119589</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -4828,13 +4828,13 @@
         <v>45108</v>
       </c>
       <c r="B92" s="17">
-        <v>150.20312548190341</v>
+        <v>150.20312548746972</v>
       </c>
       <c r="C92" s="36">
-        <v>148.72466380879337</v>
+        <v>148.6911839315234</v>
       </c>
       <c r="D92" s="36">
-        <v>147.15967189693004</v>
+        <v>147.17511504295197</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -4842,13 +4842,13 @@
         <v>45139</v>
       </c>
       <c r="B93" s="17">
-        <v>151.92217935804922</v>
+        <v>151.92217936039572</v>
       </c>
       <c r="C93" s="36">
-        <v>150.05694584045796</v>
+        <v>150.0285645140801</v>
       </c>
       <c r="D93" s="36">
-        <v>146.67009144248809</v>
+        <v>146.68020263880157</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -4856,13 +4856,13 @@
         <v>45170</v>
       </c>
       <c r="B94" s="17">
-        <v>148.41237963987399</v>
+        <v>148.41237963196167</v>
       </c>
       <c r="C94" s="36">
-        <v>149.69824700570871</v>
+        <v>149.64368007725099</v>
       </c>
       <c r="D94" s="36">
-        <v>146.13676611930737</v>
+        <v>146.14050006800522</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -4870,13 +4870,13 @@
         <v>45200</v>
       </c>
       <c r="B95" s="17">
-        <v>147.51381305414859</v>
+        <v>147.51381302893859</v>
       </c>
       <c r="C95" s="36">
-        <v>148.01321137160105</v>
+        <v>148.00946878449926</v>
       </c>
       <c r="D95" s="36">
-        <v>145.5826226763221</v>
+        <v>145.57967263807711</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -4884,13 +4884,13 @@
         <v>45231</v>
       </c>
       <c r="B96" s="17">
-        <v>146.36635232721147</v>
+        <v>146.36635231658468</v>
       </c>
       <c r="C96" s="36">
-        <v>146.38829854061774</v>
+        <v>146.35986201157135</v>
       </c>
       <c r="D96" s="36">
-        <v>145.03868020466888</v>
+        <v>145.02944531059569</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -4898,13 +4898,13 @@
         <v>45261</v>
       </c>
       <c r="B97" s="17">
-        <v>139.34262723777164</v>
+        <v>139.342627273609</v>
       </c>
       <c r="C97" s="36">
-        <v>142.86747030290806</v>
+        <v>142.8408797734873</v>
       </c>
       <c r="D97" s="36">
-        <v>144.54822439405362</v>
+        <v>144.53417943799141</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -4912,13 +4912,13 @@
         <v>45292</v>
       </c>
       <c r="B98" s="17">
-        <v>137.37335120058367</v>
+        <v>137.37335131476613</v>
       </c>
       <c r="C98" s="36">
-        <v>143.5536731054936</v>
+        <v>143.50372627874964</v>
       </c>
       <c r="D98" s="36">
-        <v>144.15895332179335</v>
+        <v>144.14240026401174</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4926,13 +4926,13 @@
         <v>45323</v>
       </c>
       <c r="B99" s="17">
-        <v>133.46450581005294</v>
+        <v>133.46450585818494</v>
       </c>
       <c r="C99" s="36">
-        <v>143.80881964781162</v>
+        <v>143.73405745303077</v>
       </c>
       <c r="D99" s="36">
-        <v>143.91670347404232</v>
+        <v>143.90035667692231</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4940,13 +4940,13 @@
         <v>45352</v>
       </c>
       <c r="B100" s="17">
-        <v>142.39572385637248</v>
+        <v>142.39572369405857</v>
       </c>
       <c r="C100" s="36">
-        <v>142.11453041710828</v>
+        <v>142.0898066454663</v>
       </c>
       <c r="D100" s="36">
-        <v>143.86036158327045</v>
+        <v>143.84698353493195</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4954,13 +4954,13 @@
         <v>45383</v>
       </c>
       <c r="B101" s="17">
-        <v>147.25690008767782</v>
+        <v>147.25689957052242</v>
       </c>
       <c r="C101" s="36">
-        <v>141.05611588000892</v>
+        <v>141.12508437171982</v>
       </c>
       <c r="D101" s="36">
-        <v>144.01125926444928</v>
+        <v>144.00290416304108</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4968,13 +4968,13 @@
         <v>45413</v>
       </c>
       <c r="B102" s="17">
-        <v>156.76909889616599</v>
+        <v>156.76909867816687</v>
       </c>
       <c r="C102" s="36">
-        <v>142.83619727876223</v>
+        <v>142.83832491106693</v>
       </c>
       <c r="D102" s="36">
-        <v>144.37034591531875</v>
+        <v>144.36812819412728</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4982,13 +4982,13 @@
         <v>45444</v>
       </c>
       <c r="B103" s="17">
-        <v>147.35712151974346</v>
+        <v>147.35712225489846</v>
       </c>
       <c r="C103" s="36">
-        <v>143.71875184087116</v>
+        <v>143.68907555762658</v>
       </c>
       <c r="D103" s="36">
-        <v>144.92087085994089</v>
+        <v>144.92532565270611</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -4996,13 +4996,13 @@
         <v>45474</v>
       </c>
       <c r="B104" s="17">
-        <v>149.65170047837228</v>
+        <v>149.65170282067913</v>
       </c>
       <c r="C104" s="36">
-        <v>147.28294331306196</v>
+        <v>147.28415957594882</v>
       </c>
       <c r="D104" s="36">
-        <v>145.62950094758585</v>
+        <v>145.63964072356882</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -5010,13 +5010,13 @@
         <v>45505</v>
       </c>
       <c r="B105" s="17">
-        <v>147.28124762344183</v>
+        <v>147.28124861080667</v>
       </c>
       <c r="C105" s="36">
-        <v>147.77459845486339</v>
+        <v>147.82949220892567</v>
       </c>
       <c r="D105" s="36">
-        <v>146.44979946004622</v>
+        <v>146.46314634054664</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -5024,13 +5024,13 @@
         <v>45536</v>
       </c>
       <c r="B106" s="17">
-        <v>144.79670189548858</v>
+        <v>144.79669856581739</v>
       </c>
       <c r="C106" s="36">
-        <v>147.82665266807604</v>
+        <v>147.86734414916225</v>
       </c>
       <c r="D106" s="36">
-        <v>147.32966884077069</v>
+        <v>147.34307891115623</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -5038,13 +5038,13 @@
         <v>45566</v>
       </c>
       <c r="B107" s="17">
-        <v>148.10395140212873</v>
+        <v>148.10394079332772</v>
       </c>
       <c r="C107" s="36">
-        <v>149.04702210828046</v>
+        <v>149.07724609103079</v>
       </c>
       <c r="D107" s="36">
-        <v>148.21264599445087</v>
+        <v>148.22246905613449</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -5052,13 +5052,13 @@
         <v>45597</v>
       </c>
       <c r="B108" s="17">
-        <v>148.17873351747122</v>
+        <v>148.17872904548861</v>
       </c>
       <c r="C108" s="36">
-        <v>150.80205892011239</v>
+        <v>150.80674041817159</v>
       </c>
       <c r="D108" s="36">
-        <v>149.04951531608577</v>
+        <v>149.05295938117266</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -5066,13 +5066,13 @@
         <v>45627</v>
       </c>
       <c r="B109" s="17">
-        <v>148.67760152837457</v>
+        <v>148.67761660915863</v>
       </c>
       <c r="C109" s="36">
-        <v>151.4852747475974</v>
+        <v>151.46158068205571</v>
       </c>
       <c r="D109" s="36">
-        <v>149.80399714657489</v>
+        <v>149.80008623128035</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -5080,13 +5080,13 @@
         <v>45658</v>
       </c>
       <c r="B110" s="17">
-        <v>146.4966364505224</v>
+        <v>146.49668450002147</v>
       </c>
       <c r="C110" s="36">
-        <v>151.93093339871064</v>
+        <v>151.9028548224955</v>
       </c>
       <c r="D110" s="36">
-        <v>150.45108861213475</v>
+        <v>150.44087661321521</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -5094,13 +5094,13 @@
         <v>45689</v>
       </c>
       <c r="B111" s="17">
-        <v>141.40459964053429</v>
+        <v>141.40461989508793</v>
       </c>
       <c r="C111" s="36">
-        <v>153.54265438189159</v>
+        <v>153.49352013447819</v>
       </c>
       <c r="D111" s="36">
-        <v>150.98034891323766</v>
+        <v>150.96654691826183</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -5108,13 +5108,13 @@
         <v>45717</v>
       </c>
       <c r="B112" s="17">
-        <v>150.61015153616984</v>
+        <v>150.61008323211774</v>
       </c>
       <c r="C112" s="36">
-        <v>149.34718181686975</v>
+        <v>149.31840483832218</v>
       </c>
       <c r="D112" s="36">
-        <v>151.39565416407993</v>
+        <v>151.38172496348201</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -5122,13 +5122,13 @@
         <v>45748</v>
       </c>
       <c r="B113" s="17">
-        <v>158.93929877299897</v>
+        <v>158.93908114668073</v>
       </c>
       <c r="C113" s="36">
-        <v>152.38409803081473</v>
+        <v>152.35852404350794</v>
       </c>
       <c r="D113" s="36">
-        <v>151.71206688080076</v>
+        <v>151.70088729461301</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -5136,13 +5136,13 @@
         <v>45778</v>
       </c>
       <c r="B114" s="17">
-        <v>165.07464344720012</v>
+        <v>165.07455171005421</v>
       </c>
       <c r="C114" s="36">
-        <v>152.27051882633819</v>
+        <v>152.12964111898245</v>
       </c>
       <c r="D114" s="36">
-        <v>151.95539463227337</v>
+        <v>151.94658597568645</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -5150,13 +5150,13 @@
         <v>45809</v>
       </c>
       <c r="B115" s="17">
-        <v>156.78890416942744</v>
+        <v>156.78921353289212</v>
       </c>
       <c r="C115" s="36">
-        <v>151.54830195145809</v>
+        <v>151.50751953044457</v>
       </c>
       <c r="D115" s="36">
-        <v>152.15179812916776</v>
+        <v>152.14393461496158</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -5164,13 +5164,13 @@
         <v>45839</v>
       </c>
       <c r="B116" s="17">
-        <v>153.77022153385636</v>
+        <v>153.77120720937</v>
       </c>
       <c r="C116" s="36">
-        <v>151.29330094897705</v>
+        <v>151.354343475533</v>
       </c>
       <c r="D116" s="36">
-        <v>152.32498289774358</v>
+        <v>152.31655807533912</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -5178,13 +5178,13 @@
         <v>45870</v>
       </c>
       <c r="B117" s="17">
-        <v>150.37579448728511</v>
+        <v>150.37620998417583</v>
       </c>
       <c r="C117" s="36">
-        <v>152.17594381036591</v>
+        <v>152.36783814947248</v>
       </c>
       <c r="D117" s="36">
-        <v>152.49533315689828</v>
+        <v>152.485181818429</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -5192,13 +5192,13 @@
         <v>45901</v>
       </c>
       <c r="B118" s="17">
-        <v>151.70554766622169</v>
+        <v>151.7041464938178</v>
       </c>
       <c r="C118" s="36">
-        <v>153.2777218239828</v>
+        <v>153.40609674320959</v>
       </c>
       <c r="D118" s="36">
-        <v>152.67467660504377</v>
+        <v>152.66272535633675</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -5206,13 +5206,13 @@
         <v>45931</v>
       </c>
       <c r="B119" s="17">
-        <v>152.83834864492212</v>
+        <v>152.83388431255179</v>
       </c>
       <c r="C119" s="36">
-        <v>153.09073472926781</v>
+        <v>153.10436298931441</v>
       </c>
       <c r="D119" s="36">
-        <v>152.86703212981183</v>
+        <v>152.85582558966763</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -5220,13 +5220,13 @@
         <v>45962</v>
       </c>
       <c r="B120" s="17">
-        <v>147.97168634998309</v>
+        <v>147.96980447689901</v>
       </c>
       <c r="C120" s="36">
-        <v>153.01278783725704</v>
+        <v>152.98368629623431</v>
       </c>
       <c r="D120" s="36">
-        <v>153.07496727109654</v>
+        <v>153.06910313427898</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -5234,13 +5234,13 @@
         <v>45992</v>
       </c>
       <c r="B121" s="17">
-        <v>153.84616590720057</v>
+        <v>153.85251211265549</v>
       </c>
       <c r="C121" s="36">
-        <v>155.94782202617111</v>
+        <v>155.89520740777738</v>
       </c>
       <c r="D121" s="36">
-        <v>153.30179867180632</v>
+        <v>153.30538384870047</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -5248,13 +5248,13 @@
         <v>46023</v>
       </c>
       <c r="B122" s="17">
-        <v>149.429834187148</v>
+        <v>149.43188619926431</v>
       </c>
       <c r="C122" s="36">
-        <v>156.3008707103094</v>
+        <v>156.36605874815257</v>
       </c>
       <c r="D122" s="36">
-        <v>153.54792524515582</v>
+        <v>153.56717850732065</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -5262,13 +5262,13 @@
         <v>46054</v>
       </c>
       <c r="B123" s="17">
-        <v>139.31163157262827</v>
+        <v>139.3365199989212</v>
       </c>
       <c r="C123" s="36">
-        <v>152.46232518014887</v>
+        <v>152.47861532335506</v>
       </c>
       <c r="D123" s="36">
-        <v>153.81146081015922</v>
+        <v>153.8599087710904</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -5276,13 +5276,13 @@
         <v>46082</v>
       </c>
       <c r="B124" s="17">
-        <v>159.97685005773832</v>
+        <v>159.9499096193297</v>
       </c>
       <c r="C124" s="36">
-        <v>156.73111231345317</v>
+        <v>156.4698201506535</v>
       </c>
       <c r="D124" s="36">
-        <v>154.08801458161344</v>
+        <v>154.18637754509663</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
@@ -5290,27 +5290,41 @@
         <v>46113</v>
       </c>
       <c r="B125" s="17">
-        <v>161.60721101015756</v>
+        <v>161.71805294443547</v>
       </c>
       <c r="C125" s="36">
-        <v>154.33640201486921</v>
+        <v>153.90332453400006</v>
       </c>
       <c r="D125" s="36">
-        <v>154.36994201063817</v>
+        <v>154.54371532399702</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
         <v>46143</v>
       </c>
-      <c r="B126" s="40">
-        <v>165.47141407640655</v>
-      </c>
-      <c r="C126" s="41">
-        <v>153.62027214485033</v>
-      </c>
-      <c r="D126" s="41">
-        <v>154.65561262723506</v>
+      <c r="B126" s="17">
+        <v>165.66808413621425</v>
+      </c>
+      <c r="C126" s="36">
+        <v>152.96249448451684</v>
+      </c>
+      <c r="D126" s="36">
+        <v>154.92890282828878</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" s="4">
+        <v>46174</v>
+      </c>
+      <c r="B127" s="40">
+        <v>161.01331908191355</v>
+      </c>
+      <c r="C127" s="41">
+        <v>154.1172638221334</v>
+      </c>
+      <c r="D127" s="41">
+        <v>155.31027391562463</v>
       </c>
     </row>
   </sheetData>
@@ -7632,14 +7646,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51" t="s">
+      <c r="C1" s="48"/>
+      <c r="D1" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="51"/>
+      <c r="E1" s="48"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8238,14 +8252,14 @@
       <c r="A1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51" t="s">
+      <c r="C1" s="48"/>
+      <c r="D1" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="51"/>
+      <c r="E1" s="48"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -8417,14 +8431,14 @@
         <v>70</v>
       </c>
       <c r="B2" s="46">
-        <v>8481.3895971000002</v>
+        <v>10131.835788459999</v>
       </c>
       <c r="C2" s="46">
-        <v>10358.58955208</v>
+        <v>12382.20280524</v>
       </c>
       <c r="D2" s="27">
         <f>B2-C2</f>
-        <v>-1877.1999549800003</v>
+        <v>-2250.367016780001</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -8432,14 +8446,14 @@
         <v>203</v>
       </c>
       <c r="B3" s="42">
-        <v>6254.0776712200004</v>
+        <v>7386.56491147</v>
       </c>
       <c r="C3" s="42">
-        <v>7650.0725485599996</v>
+        <v>9135.5407090499994</v>
       </c>
       <c r="D3" s="27">
         <f t="shared" ref="D3:D27" si="0">B3-C3</f>
-        <v>-1395.9948773399992</v>
+        <v>-1748.9757975799994</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -8447,14 +8461,14 @@
         <v>208</v>
       </c>
       <c r="B4" s="42">
-        <v>882.91976972999998</v>
+        <v>1046.4819220100001</v>
       </c>
       <c r="C4" s="42">
-        <v>2415.4081030100001</v>
+        <v>2905.88218284</v>
       </c>
       <c r="D4" s="27">
         <f t="shared" si="0"/>
-        <v>-1532.48833328</v>
+        <v>-1859.40026083</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -8462,14 +8476,14 @@
         <v>209</v>
       </c>
       <c r="B5" s="42">
-        <v>1069.9884319400001</v>
+        <v>1352.6515661799999</v>
       </c>
       <c r="C5" s="42">
-        <v>288.20453477000001</v>
+        <v>335.50739291000002</v>
       </c>
       <c r="D5" s="27">
         <f t="shared" si="0"/>
-        <v>781.78389717000005</v>
+        <v>1017.1441732699999</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -8477,14 +8491,14 @@
         <v>72</v>
       </c>
       <c r="B6" s="46">
-        <v>6114.1209186899996</v>
+        <v>7276.7667382099999</v>
       </c>
       <c r="C6" s="46">
-        <v>1146.8822496400001</v>
+        <v>1336.49858073</v>
       </c>
       <c r="D6" s="27">
         <f t="shared" si="0"/>
-        <v>4967.2386690499998</v>
+        <v>5940.2681574799999</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -8492,14 +8506,14 @@
         <v>71</v>
       </c>
       <c r="B7" s="42">
-        <v>3279.5440918499999</v>
+        <v>3787.38927302</v>
       </c>
       <c r="C7" s="42">
-        <v>471.02433543000001</v>
+        <v>522.54152991000001</v>
       </c>
       <c r="D7" s="27">
         <f t="shared" si="0"/>
-        <v>2808.5197564199998</v>
+        <v>3264.84774311</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -8507,14 +8521,14 @@
         <v>204</v>
       </c>
       <c r="B8" s="42">
-        <v>1348.9057046400001</v>
+        <v>1741.6900650600001</v>
       </c>
       <c r="C8" s="42">
-        <v>157.82740096000001</v>
+        <v>175.76956447000001</v>
       </c>
       <c r="D8" s="27">
         <f t="shared" si="0"/>
-        <v>1191.0783036800001</v>
+        <v>1565.9205005900001</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -8522,14 +8536,14 @@
         <v>175</v>
       </c>
       <c r="B9" s="46">
-        <v>5902.9134168700002</v>
+        <v>7243.4021109400001</v>
       </c>
       <c r="C9" s="46">
-        <v>4361.1140620799997</v>
+        <v>5225.90957196</v>
       </c>
       <c r="D9" s="27">
         <f t="shared" si="0"/>
-        <v>1541.7993547900005</v>
+        <v>2017.4925389800001</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -8537,14 +8551,14 @@
         <v>205</v>
       </c>
       <c r="B10" s="42">
-        <v>4858.6477084999997</v>
+        <v>5970.7614276200002</v>
       </c>
       <c r="C10" s="42">
-        <v>3284.0718609199998</v>
+        <v>3967.0999705899999</v>
       </c>
       <c r="D10" s="27">
         <f t="shared" si="0"/>
-        <v>1574.5758475799998</v>
+        <v>2003.6614570300003</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -8552,14 +8566,14 @@
         <v>176</v>
       </c>
       <c r="B11" s="46">
-        <v>4358.8776973599997</v>
+        <v>5199.1678182699998</v>
       </c>
       <c r="C11" s="46">
-        <v>5017.5170362500003</v>
+        <v>5782.4787789499997</v>
       </c>
       <c r="D11" s="27">
         <f t="shared" si="0"/>
-        <v>-658.63933889000054</v>
+        <v>-583.31096067999988</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -8567,14 +8581,14 @@
         <v>212</v>
       </c>
       <c r="B12" s="42">
-        <v>570.62108985999998</v>
+        <v>659.46119262000002</v>
       </c>
       <c r="C12" s="42">
-        <v>1524.06350172</v>
+        <v>1798.04473865</v>
       </c>
       <c r="D12" s="27">
         <f t="shared" si="0"/>
-        <v>-953.44241185999999</v>
+        <v>-1138.58354603</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -8582,14 +8596,14 @@
         <v>213</v>
       </c>
       <c r="B13" s="42">
-        <v>715.86494592999998</v>
+        <v>923.75633140000002</v>
       </c>
       <c r="C13" s="42">
-        <v>528.95311143000004</v>
+        <v>593.88788952000004</v>
       </c>
       <c r="D13" s="27">
         <f t="shared" si="0"/>
-        <v>186.91183449999994</v>
+        <v>329.86844187999998</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -8597,14 +8611,14 @@
         <v>214</v>
       </c>
       <c r="B14" s="42">
-        <v>516.88207270999999</v>
+        <v>597.18803424999999</v>
       </c>
       <c r="C14" s="42">
-        <v>766.57510847000003</v>
+        <v>878.77091515999996</v>
       </c>
       <c r="D14" s="27">
         <f t="shared" si="0"/>
-        <v>-249.69303576000004</v>
+        <v>-281.58288090999997</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -8612,14 +8626,14 @@
         <v>215</v>
       </c>
       <c r="B15" s="42">
-        <v>926.29658819999997</v>
+        <v>1135.45100806</v>
       </c>
       <c r="C15" s="42">
-        <v>171.95748750999999</v>
+        <v>190.25197933000001</v>
       </c>
       <c r="D15" s="27">
         <f t="shared" si="0"/>
-        <v>754.33910069000001</v>
+        <v>945.19902873000001</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -8627,14 +8641,14 @@
         <v>74</v>
       </c>
       <c r="B16" s="46">
-        <v>4890.6300276399998</v>
+        <v>5589.1728557099996</v>
       </c>
       <c r="C16" s="46">
-        <v>7983.1137907000002</v>
+        <v>9494.7219496399994</v>
       </c>
       <c r="D16" s="27">
         <f t="shared" si="0"/>
-        <v>-3092.4837630600005</v>
+        <v>-3905.5490939299998</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -8642,14 +8656,14 @@
         <v>75</v>
       </c>
       <c r="B17" s="46">
-        <v>3101.0147205600001</v>
+        <v>3684.9481077599999</v>
       </c>
       <c r="C17" s="46">
-        <v>562.39323972</v>
+        <v>649.82246679000002</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>2538.62148084</v>
+        <v>3035.1256409699999</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -8657,14 +8671,14 @@
         <v>73</v>
       </c>
       <c r="B18" s="46">
-        <v>4613.0539279000004</v>
+        <v>5318.7616484999999</v>
       </c>
       <c r="C18" s="46">
-        <v>1981.40743335</v>
+        <v>2310.8556745300002</v>
       </c>
       <c r="D18" s="27">
         <f t="shared" si="0"/>
-        <v>2631.6464945500002</v>
+        <v>3007.9059739699996</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -8672,14 +8686,14 @@
         <v>207</v>
       </c>
       <c r="B19" s="42">
-        <v>776.67251765000003</v>
+        <v>863.06267104999995</v>
       </c>
       <c r="C19" s="42">
-        <v>208.47525941000001</v>
+        <v>238.04602537</v>
       </c>
       <c r="D19" s="27">
         <f t="shared" si="0"/>
-        <v>568.19725824</v>
+        <v>625.01664568000001</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -8687,14 +8701,14 @@
         <v>210</v>
       </c>
       <c r="B20" s="42">
-        <v>798.89368889000002</v>
+        <v>909.10152768</v>
       </c>
       <c r="C20" s="42">
-        <v>118.69154020000001</v>
+        <v>134.54632391000001</v>
       </c>
       <c r="D20" s="27">
         <f t="shared" si="0"/>
-        <v>680.20214869000006</v>
+        <v>774.55520376999993</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -8702,14 +8716,14 @@
         <v>211</v>
       </c>
       <c r="B21" s="42">
-        <v>891.48188430000005</v>
+        <v>991.09674127999995</v>
       </c>
       <c r="C21" s="42">
-        <v>1032.2568432</v>
+        <v>1185.1922510899999</v>
       </c>
       <c r="D21" s="27">
         <f t="shared" si="0"/>
-        <v>-140.7749589</v>
+        <v>-194.09550980999995</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -8717,14 +8731,14 @@
         <v>206</v>
       </c>
       <c r="B22" s="42">
-        <v>1801.0153340700001</v>
+        <v>2104.22535883</v>
       </c>
       <c r="C22" s="42">
-        <v>469.33647961000003</v>
+        <v>570.53177382000001</v>
       </c>
       <c r="D22" s="27">
         <f t="shared" si="0"/>
-        <v>1331.6788544600001</v>
+        <v>1533.6935850099999</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -8732,14 +8746,14 @@
         <v>76</v>
       </c>
       <c r="B23" s="46">
-        <v>2481.4743572000002</v>
+        <v>2974.4506729999998</v>
       </c>
       <c r="C23" s="46">
-        <v>217.91258299</v>
+        <v>268.65412280999999</v>
       </c>
       <c r="D23" s="27">
         <f t="shared" si="0"/>
-        <v>2263.5617742100003</v>
+        <v>2705.7965501899998</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -8747,14 +8761,14 @@
         <v>77</v>
       </c>
       <c r="B24" s="46">
-        <v>2336.6136192099998</v>
+        <v>2576.3643842800002</v>
       </c>
       <c r="C24" s="46">
-        <v>282.26240106</v>
+        <v>367.98612315999998</v>
       </c>
       <c r="D24" s="27">
         <f t="shared" si="0"/>
-        <v>2054.35121815</v>
+        <v>2208.3782611200004</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -8762,14 +8776,14 @@
         <v>78</v>
       </c>
       <c r="B25" s="46">
-        <v>172.32922266</v>
+        <v>199.64993278</v>
       </c>
       <c r="C25" s="46">
-        <v>116.87643165999999</v>
+        <v>126.95507979999999</v>
       </c>
       <c r="D25" s="27">
         <f t="shared" si="0"/>
-        <v>55.452791000000005</v>
+        <v>72.694852980000007</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -8777,14 +8791,14 @@
         <v>79</v>
       </c>
       <c r="B26" s="46">
-        <v>559.93835520000005</v>
+        <v>606.94943167999998</v>
       </c>
       <c r="C26" s="46">
-        <v>178.09884439999999</v>
+        <v>201.79184792000001</v>
       </c>
       <c r="D26" s="27">
         <f t="shared" si="0"/>
-        <v>381.83951080000008</v>
+        <v>405.15758375999997</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -8792,14 +8806,14 @@
         <v>80</v>
       </c>
       <c r="B27" s="47">
-        <v>6442.1068232699999</v>
+        <v>7563.7167973200003</v>
       </c>
       <c r="C27" s="47">
-        <v>3325.2753946500002</v>
+        <v>4137.7659778699999</v>
       </c>
       <c r="D27" s="27">
         <f t="shared" si="0"/>
-        <v>3116.8314286199998</v>
+        <v>3425.9508194500004</v>
       </c>
     </row>
   </sheetData>
@@ -8828,8 +8842,8 @@
       <c r="A2" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="48">
-        <v>49454.46268366</v>
+      <c r="B2" s="49">
+        <v>58365.18628691</v>
       </c>
       <c r="D2" s="29"/>
     </row>
@@ -8837,8 +8851,8 @@
       <c r="A3" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="B3" s="48">
-        <v>12631.428010670001</v>
+      <c r="B3" s="49">
+        <v>14749.46763087</v>
       </c>
       <c r="D3" s="29"/>
     </row>
@@ -8846,8 +8860,8 @@
       <c r="A4" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="49">
-        <v>16.464585719999999</v>
+      <c r="B4" s="50">
+        <v>18.157807630000001</v>
       </c>
       <c r="D4" s="30"/>
     </row>
@@ -8855,8 +8869,8 @@
       <c r="A5" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="49">
-        <v>1072.95508227</v>
+      <c r="B5" s="50">
+        <v>1256.8318682199999</v>
       </c>
       <c r="D5" s="30"/>
     </row>
@@ -8864,8 +8878,8 @@
       <c r="A6" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="49">
-        <v>177.93759610000001</v>
+      <c r="B6" s="50">
+        <v>201.09731998000001</v>
       </c>
       <c r="D6" s="30"/>
     </row>
@@ -8873,8 +8887,8 @@
       <c r="A7" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="49">
-        <v>409.69851609</v>
+      <c r="B7" s="50">
+        <v>470.26634000000001</v>
       </c>
       <c r="D7" s="30"/>
     </row>
@@ -8882,8 +8896,8 @@
       <c r="A8" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="49">
-        <v>423.38260679000001</v>
+      <c r="B8" s="50">
+        <v>509.21601561</v>
       </c>
       <c r="D8" s="30"/>
     </row>
@@ -8891,8 +8905,8 @@
       <c r="A9" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B9" s="49">
-        <v>7444.7477826599998</v>
+      <c r="B9" s="50">
+        <v>8762.7264263800007</v>
       </c>
       <c r="D9" s="30"/>
     </row>
@@ -8900,8 +8914,8 @@
       <c r="A10" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="49">
-        <v>2178.03683374</v>
+      <c r="B10" s="50">
+        <v>2444.2489930800002</v>
       </c>
       <c r="D10" s="30"/>
     </row>
@@ -8909,8 +8923,8 @@
       <c r="A11" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="B11" s="49">
-        <v>113.81617368000001</v>
+      <c r="B11" s="50">
+        <v>156.34153777</v>
       </c>
       <c r="D11" s="30"/>
     </row>
@@ -8918,8 +8932,8 @@
       <c r="A12" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="49">
-        <v>53.82557903</v>
+      <c r="B12" s="50">
+        <v>60.934622490000002</v>
       </c>
       <c r="D12" s="30"/>
     </row>
@@ -8927,8 +8941,8 @@
       <c r="A13" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="49">
-        <v>55.442203339999999</v>
+      <c r="B13" s="50">
+        <v>71.689543749999999</v>
       </c>
       <c r="D13" s="30"/>
     </row>
@@ -8936,8 +8950,8 @@
       <c r="A14" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B14" s="49">
-        <v>574.83523628</v>
+      <c r="B14" s="50">
+        <v>670.09803132000002</v>
       </c>
       <c r="D14" s="30"/>
     </row>
@@ -8945,8 +8959,8 @@
       <c r="A15" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="49">
-        <v>110.28581497</v>
+      <c r="B15" s="50">
+        <v>127.85912464</v>
       </c>
       <c r="D15" s="30"/>
     </row>
@@ -8954,8 +8968,8 @@
       <c r="A16" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B16" s="48">
-        <v>15819.496350199999</v>
+      <c r="B16" s="49">
+        <v>18910.693595339999</v>
       </c>
       <c r="D16" s="29"/>
     </row>
@@ -8963,8 +8977,8 @@
       <c r="A17" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="49">
-        <v>2570.6484228200002</v>
+      <c r="B17" s="50">
+        <v>3097.1531389400002</v>
       </c>
       <c r="D17" s="30"/>
     </row>
@@ -8972,8 +8986,8 @@
       <c r="A18" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="B18" s="49">
-        <v>156.63452408000001</v>
+      <c r="B18" s="50">
+        <v>181.72376378999999</v>
       </c>
       <c r="D18" s="30"/>
     </row>
@@ -8981,8 +8995,8 @@
       <c r="A19" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="49">
-        <v>731.49064919</v>
+      <c r="B19" s="50">
+        <v>854.0703671</v>
       </c>
       <c r="D19" s="30"/>
     </row>
@@ -8990,8 +9004,8 @@
       <c r="A20" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="B20" s="49">
-        <v>48.8231167</v>
+      <c r="B20" s="50">
+        <v>57.90506328</v>
       </c>
       <c r="D20" s="30"/>
     </row>
@@ -8999,8 +9013,8 @@
       <c r="A21" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="49">
-        <v>58.525990210000003</v>
+      <c r="B21" s="50">
+        <v>69.489123500000005</v>
       </c>
       <c r="D21" s="30"/>
     </row>
@@ -9008,8 +9022,8 @@
       <c r="A22" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="49">
-        <v>91.483421500000006</v>
+      <c r="B22" s="50">
+        <v>109.83325639</v>
       </c>
       <c r="D22" s="30"/>
     </row>
@@ -9017,8 +9031,8 @@
       <c r="A23" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B23" s="49">
-        <v>403.77321796000001</v>
+      <c r="B23" s="50">
+        <v>474.87592073000002</v>
       </c>
       <c r="D23" s="30"/>
     </row>
@@ -9026,8 +9040,8 @@
       <c r="A24" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="B24" s="49">
-        <v>5222.8086147699996</v>
+      <c r="B24" s="50">
+        <v>6315.0275704100004</v>
       </c>
       <c r="D24" s="30"/>
     </row>
@@ -9035,8 +9049,8 @@
       <c r="A25" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B25" s="49">
-        <v>190.33760681999999</v>
+      <c r="B25" s="50">
+        <v>222.67925025</v>
       </c>
       <c r="D25" s="30"/>
     </row>
@@ -9044,8 +9058,8 @@
       <c r="A26" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="B26" s="49">
-        <v>520.09811133000005</v>
+      <c r="B26" s="50">
+        <v>620.26536309000005</v>
       </c>
       <c r="D26" s="30"/>
     </row>
@@ -9053,8 +9067,8 @@
       <c r="A27" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="B27" s="49">
-        <v>389.43796888999998</v>
+      <c r="B27" s="50">
+        <v>436.22027859000002</v>
       </c>
       <c r="D27" s="30"/>
     </row>
@@ -9062,8 +9076,8 @@
       <c r="A28" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B28" s="49">
-        <v>4678.4785626299999</v>
+      <c r="B28" s="50">
+        <v>5592.0888350599998</v>
       </c>
       <c r="D28" s="30"/>
     </row>
@@ -9071,8 +9085,8 @@
       <c r="A29" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="49">
-        <v>157.20024982999999</v>
+      <c r="B29" s="50">
+        <v>181.02550357999999</v>
       </c>
       <c r="D29" s="30"/>
     </row>
@@ -9080,8 +9094,8 @@
       <c r="A30" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="B30" s="49">
-        <v>174.71465499999999</v>
+      <c r="B30" s="50">
+        <v>205.02960447000001</v>
       </c>
       <c r="D30" s="30"/>
     </row>
@@ -9089,8 +9103,8 @@
       <c r="A31" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="B31" s="49">
-        <v>68.174505429999996</v>
+      <c r="B31" s="50">
+        <v>78.771963679999999</v>
       </c>
       <c r="D31" s="30"/>
     </row>
@@ -9098,8 +9112,8 @@
       <c r="A32" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="B32" s="49">
-        <v>356.86673303999999</v>
+      <c r="B32" s="50">
+        <v>414.53459248000001</v>
       </c>
       <c r="D32" s="30"/>
     </row>
@@ -9107,8 +9121,8 @@
       <c r="A33" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="B33" s="48">
-        <v>13384.87206421</v>
+      <c r="B33" s="49">
+        <v>15553.555421290001</v>
       </c>
       <c r="D33" s="29"/>
     </row>
@@ -9116,8 +9130,8 @@
       <c r="A34" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="B34" s="49">
-        <v>2991.57088901</v>
+      <c r="B34" s="50">
+        <v>3533.0068182999998</v>
       </c>
       <c r="D34" s="30"/>
     </row>
@@ -9125,8 +9139,8 @@
       <c r="A35" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B35" s="49">
-        <v>607.09800845999996</v>
+      <c r="B35" s="50">
+        <v>735.04779130999998</v>
       </c>
       <c r="D35" s="30"/>
     </row>
@@ -9134,8 +9148,8 @@
       <c r="A36" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="B36" s="49">
-        <v>85.910532889999999</v>
+      <c r="B36" s="50">
+        <v>101.79144912</v>
       </c>
       <c r="D36" s="30"/>
     </row>
@@ -9143,8 +9157,8 @@
       <c r="A37" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="B37" s="49">
-        <v>8.7954096499999999</v>
+      <c r="B37" s="50">
+        <v>10.22030971</v>
       </c>
       <c r="D37" s="30"/>
     </row>
@@ -9152,8 +9166,8 @@
       <c r="A38" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="B38" s="49">
-        <v>214.91494496999999</v>
+      <c r="B38" s="50">
+        <v>244.06434983</v>
       </c>
       <c r="D38" s="30"/>
     </row>
@@ -9161,8 +9175,8 @@
       <c r="A39" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B39" s="49">
-        <v>53.943710869999997</v>
+      <c r="B39" s="50">
+        <v>61.774884800000002</v>
       </c>
       <c r="D39" s="30"/>
     </row>
@@ -9170,8 +9184,8 @@
       <c r="A40" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="B40" s="49">
-        <v>4.4194451199999998</v>
+      <c r="B40" s="50">
+        <v>5.2625535000000001</v>
       </c>
       <c r="D40" s="30"/>
     </row>
@@ -9179,8 +9193,8 @@
       <c r="A41" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="49">
-        <v>66.158591869999995</v>
+      <c r="B41" s="50">
+        <v>76.379257499999994</v>
       </c>
       <c r="D41" s="30"/>
     </row>
@@ -9188,8 +9202,8 @@
       <c r="A42" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="B42" s="49">
-        <v>2937.4714189900001</v>
+      <c r="B42" s="50">
+        <v>3237.7422759599999</v>
       </c>
       <c r="D42" s="30"/>
     </row>
@@ -9197,8 +9211,8 @@
       <c r="A43" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B43" s="49">
-        <v>1400.86288964</v>
+      <c r="B43" s="50">
+        <v>1660.5043017999999</v>
       </c>
       <c r="D43" s="30"/>
     </row>
@@ -9206,8 +9220,8 @@
       <c r="A44" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="B44" s="49">
-        <v>647.06496117999995</v>
+      <c r="B44" s="50">
+        <v>774.47669218999999</v>
       </c>
       <c r="D44" s="30"/>
     </row>
@@ -9215,8 +9229,8 @@
       <c r="A45" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B45" s="49">
-        <v>3921.32795747</v>
+      <c r="B45" s="50">
+        <v>4621.4257138399998</v>
       </c>
       <c r="D45" s="30"/>
     </row>
@@ -9224,8 +9238,8 @@
       <c r="A46" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B46" s="49">
-        <v>82.83759628</v>
+      <c r="B46" s="50">
+        <v>103.31335292</v>
       </c>
       <c r="D46" s="30"/>
     </row>
@@ -9233,8 +9247,8 @@
       <c r="A47" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="B47" s="49">
-        <v>362.49570781</v>
+      <c r="B47" s="50">
+        <v>388.54567050999998</v>
       </c>
       <c r="D47" s="30"/>
     </row>
@@ -9242,8 +9256,8 @@
       <c r="A48" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="B48" s="48">
-        <v>7618.6662585800004</v>
+      <c r="B48" s="49">
+        <v>9151.4696394099992</v>
       </c>
       <c r="D48" s="29"/>
     </row>
@@ -9251,8 +9265,8 @@
       <c r="A49" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B49" s="49">
-        <v>4692.6805862399997</v>
+      <c r="B49" s="50">
+        <v>5722.2773933500002</v>
       </c>
       <c r="D49" s="30"/>
     </row>
@@ -9260,8 +9274,8 @@
       <c r="A50" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="B50" s="49">
-        <v>1802.6515664599999</v>
+      <c r="B50" s="50">
+        <v>2139.9432461699998</v>
       </c>
       <c r="D50" s="30"/>
     </row>
@@ -9269,8 +9283,8 @@
       <c r="A51" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="B51" s="49">
-        <v>55.09513304</v>
+      <c r="B51" s="50">
+        <v>75.096219039999994</v>
       </c>
       <c r="D51" s="30"/>
     </row>
@@ -9278,8 +9292,8 @@
       <c r="A52" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="B52" s="49">
-        <v>825.29429833999995</v>
+      <c r="B52" s="42">
+        <v>932.30774222000002</v>
       </c>
       <c r="D52" s="30"/>
     </row>
@@ -9287,8 +9301,8 @@
       <c r="A53" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="B53" s="50">
-        <v>242.94467449999999</v>
+      <c r="B53" s="51">
+        <v>281.84503862999998</v>
       </c>
     </row>
   </sheetData>
@@ -9318,7 +9332,7 @@
         <v>177</v>
       </c>
       <c r="B2" s="43">
-        <v>35531.443018580001</v>
+        <v>42285.6429794</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -9326,7 +9340,7 @@
         <v>178</v>
       </c>
       <c r="B3" s="43">
-        <v>6799.3836805999999</v>
+        <v>7966.5527909100001</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -9334,7 +9348,7 @@
         <v>179</v>
       </c>
       <c r="B4" s="44">
-        <v>4883.5781913500005</v>
+        <v>5703.72560419</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -9342,7 +9356,7 @@
         <v>180</v>
       </c>
       <c r="B5" s="44">
-        <v>764.12688181999999</v>
+        <v>897.51211365999995</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -9350,7 +9364,7 @@
         <v>181</v>
       </c>
       <c r="B6" s="44">
-        <v>1151.6786074300001</v>
+        <v>1365.31507306</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -9358,7 +9372,7 @@
         <v>182</v>
       </c>
       <c r="B7" s="43">
-        <v>12288.059822949999</v>
+        <v>14713.917361530001</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -9366,7 +9380,7 @@
         <v>183</v>
       </c>
       <c r="B8" s="44">
-        <v>2178.7017841500001</v>
+        <v>2620.4116493299998</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -9374,7 +9388,7 @@
         <v>184</v>
       </c>
       <c r="B9" s="44">
-        <v>292.60839814000002</v>
+        <v>360.11411499000002</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -9382,7 +9396,7 @@
         <v>185</v>
       </c>
       <c r="B10" s="44">
-        <v>482.11012384999998</v>
+        <v>577.07729746999996</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -9390,7 +9404,7 @@
         <v>186</v>
       </c>
       <c r="B11" s="44">
-        <v>8337.3539427199994</v>
+        <v>9948.1876556099996</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -9398,7 +9412,7 @@
         <v>187</v>
       </c>
       <c r="B12" s="44">
-        <v>997.28557408999995</v>
+        <v>1208.1266441299999</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -9406,7 +9420,7 @@
         <v>188</v>
       </c>
       <c r="B13" s="43">
-        <v>1669.0895602000001</v>
+        <v>2298.2558634400002</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -9414,7 +9428,7 @@
         <v>189</v>
       </c>
       <c r="B14" s="44">
-        <v>178.6497689</v>
+        <v>229.38295342999999</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -9422,7 +9436,7 @@
         <v>190</v>
       </c>
       <c r="B15" s="44">
-        <v>1490.4397913</v>
+        <v>2068.8729100099999</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -9430,7 +9444,7 @@
         <v>191</v>
       </c>
       <c r="B16" s="43">
-        <v>6144.30421019</v>
+        <v>7227.0718579900004</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -9438,7 +9452,7 @@
         <v>192</v>
       </c>
       <c r="B17" s="44">
-        <v>2391.5527711</v>
+        <v>2773.1099563900002</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9446,7 +9460,7 @@
         <v>193</v>
       </c>
       <c r="B18" s="44">
-        <v>318.78053840000001</v>
+        <v>375.03283696</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -9454,7 +9468,7 @@
         <v>194</v>
       </c>
       <c r="B19" s="44">
-        <v>3433.9709006899998</v>
+        <v>4078.92906464</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -9462,7 +9476,7 @@
         <v>195</v>
       </c>
       <c r="B20" s="43">
-        <v>5362.2500497299998</v>
+        <v>6251.3278832100004</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -9470,7 +9484,7 @@
         <v>196</v>
       </c>
       <c r="B21" s="44">
-        <v>422.58905465999999</v>
+        <v>484.15647494000001</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -9478,7 +9492,7 @@
         <v>197</v>
       </c>
       <c r="B22" s="44">
-        <v>790.74661163999997</v>
+        <v>928.84081617000004</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -9486,7 +9500,7 @@
         <v>198</v>
       </c>
       <c r="B23" s="44">
-        <v>433.56903849999998</v>
+        <v>4.7688800000000005E-3</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -9494,7 +9508,7 @@
         <v>199</v>
       </c>
       <c r="B24" s="44">
-        <v>548.26871476999997</v>
+        <v>510.76962545999999</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -9502,7 +9516,7 @@
         <v>200</v>
       </c>
       <c r="B25" s="44">
-        <v>1409.0464241100001</v>
+        <v>644.35921371999996</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -9510,7 +9524,7 @@
         <v>201</v>
       </c>
       <c r="B26" s="44">
-        <v>940.87862426000004</v>
+        <v>1610.9767362600001</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -9518,28 +9532,28 @@
         <v>187</v>
       </c>
       <c r="B27" s="44">
-        <v>817.15158179000002</v>
+        <v>1114.6196868300001</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="B28" s="43">
-        <v>2597.56740356</v>
+      <c r="B28" s="44">
+        <v>957.60056095000004</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B29" s="45">
-        <v>670.78829135000001</v>
+      <c r="B29" s="43">
+        <v>3045.5730030099999</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B30">
-        <v>845.88280497999995</v>
+      <c r="B30" s="45">
+        <v>782.94421930999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>